<commit_message>
Dividir Excel en 3 partes para cubrir todas las etiquetas
</commit_message>
<xml_diff>
--- a/work/from_google/novedades.xlsx
+++ b/work/from_google/novedades.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Traduccion" sheetId="1" r:id="rId1"/>
+    <sheet name=" Traducción" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -409,1137 +409,1137 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Hi,\n\nCitizens for Prosperity needs help moving supplies around one of our outposts. The boxes need to be picked up from &lt;EM4&gt;{0} and taken to &lt;EM4&gt;{1} \n\nDoesn’t sound too difficult, does it? Just make sure you’re wearing a comfy pair of shoes. Also, to make your life easier, I'd bring a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; with you. \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 200 / 400 / 800</v>
+        <v> Hola,\n\nCiudadanos por la Prosperidad necesita ayuda para trasladar suministros en uno de nuestros puestos avanzados. Las cajas deben recogerse en &lt;EM4&gt;{0} y llevarse a &lt;EM4&gt;{1}. \n\nNo parece muy difícil, ¿verdad? Solo asegúrate de llevar un par de zapatos cómodos. Además, para facilitarte la vida, te recomiendo que traigas un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt;. \n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 200 / 400 / 800</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Hey, \n\nOne of our veteran haulers got sick and backed out of a run that we desperately needed. {0} stepped up and offered to do it. I was hesitant to give it to ‘em because it’s riskier than the routes they normally do. Seems like my concern was warranted. Last update we got from ‘em was near {1} which is XenoThreat territory.\n\nCan’t have this hanging over my head much longer. Any chance you’d be willing to head to their last known location and see if you can find out what happened? It’d mean a lot to me and others. Not only to know the status of {2} but also the cargo, which is really needed at {3} If you find it and complete the delivery, it would be a huge help to the CFP members there.   \n\nFly safe out there,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 3,200</v>
+        <v>Hola, \n\nUno de nuestros transportistas veteranos se enfermó y canceló un viaje que necesitábamos desesperadamente. {0} se ofreció a hacerlo. Dudé en dárselo porque es más arriesgado que las rutas que normalmente hacen. Parece que mi preocupación estaba justificada. La última actualización que recibimos de él fue cerca de {1} que es territorio XenoThreat.\n\nNo puedo tener esto en la cabeza por mucho más tiempo. ¿Hay alguna posibilidad de que estés dispuesto a ir a su última ubicación conocida y ver si puedes averiguar qué pasó? Significará mucho para mí y para otros. No solo para saber el estado de {2} sino también la carga, que realmente se necesita en {3} Si la encuentras y completas la entrega, sería una gran ayuda para los miembros de CFP allí. \n\nVuela seguro ahí fuera,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 3200</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Hey,\n\nI’ve been tracking Headhunters activity at {0} Recently, they stocked it with supplies we believe were stolen from one of our cargo convoys. {1} offered to go get our goods back but hasn’t checked in since. Really need to know what happened to them and if our supplies are there.\n\nThink this is something you could handle? You’ll probably have to deal with Headhunters forces to get to the bottom of this. Also, any goods you grab should go to {2} once you’re out of there.\n\nThanks, \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 800</v>
+        <v>Hola,\n\nHe estado siguiendo la actividad de los Cazadores de Cabezas en {0}. Recientemente, lo abastecieron con suministros que creemos que fueron robados de uno de nuestros convoyes de carga. {1} se ofreció a recuperar nuestra mercancía, pero no se ha comunicado desde entonces. Realmente necesito saber qué les pasó y si nuestros suministros están allí.\n\n¿Crees que podrías encargarte de esto? Probablemente tendrás que lidiar con las fuerzas de los Cazadores de Cabezas para llegar al fondo del asunto. Además, cualquier mercancía que tomes debe ir a {2} una vez que salgas de allí.\n\nGracias,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 800</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Hey,\n\nWondering if you can help me. I’ve lost touch with a dedicated CFP volunteer named {0} who was tracking down supplies taken by XenoThreat. Their last comm said they believed our stuff was being held at {1} I told them to be careful, but haven’t heard anything since.\n\nAny chance you can head out and try to locate {2} While there, if you spot the supplies, please bring them to {3} I’ll give you the same warning I gave {4} that spot is a known Xeno stronghold. Better be prepared. Would hate for you to disappear too after visiting that spot. \n\nBe Safe, \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 1,500</v>
+        <v>Hola,\n\nMe pregunto si podrías ayudarme. He perdido el contacto con un voluntario dedicado de CFP llamado {0} que estaba rastreando suministros tomados por XenoThreat. Su última comunicación decía que creía que nuestras cosas estaban retenidas en {1}. Le dije que tuviera cuidado, pero no he vuelto a saber nada.\n\n¿Hay alguna posibilidad de que puedas ir e intentar localizar {2}? Una vez allí, si ves los suministros, por favor tráelos a {3}. Te daré la misma advertencia que le di a {4}: ese lugar es un conocido bastión Xeno. Mejor prepárate. No me gustaría que desaparecieras también después de visitar ese lugar.\n\nCuídate,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 1500</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Hi,\n\nGot a tough assignment here. There’s a small, satellite outpost near {0} that needs to be investigated. I received intel that it’s housing some of our stolen supplies and sent {1} to retrieve them. Haven’t heard anything from them in a while and am worried they ran into trouble.\n\nXenoThreat controls that location, but I hoped {2} could slip in and out without getting noticed. Seems like that spot might be more heavily guarded than expected. Looking for someone to take a look and see what happened to {3} Also, if any of our supplies are found there, I need them taken to {4} \n\nDo you think you can give it a shot? I’m guessing that the Xenos are entrenched there. Prepare accordingly and don’t expect them to make this easy on you.  \n\nThanks, \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 800</v>
+        <v>Hola,\n\nTengo una misión difícil. Hay un pequeño puesto de avanzada satélite cerca de {0} que necesita ser investigado. Recibí información de que alberga algunos de nuestros suministros robados y envié a {1} a recuperarlos. No he tenido noticias de ellos en un tiempo y me preocupa que hayan tenido problemas.\n\nXenoThreat controla esa ubicación, pero esperaba que {2} pudiera entrar y salir sin ser detectado. Parece que ese lugar podría estar más vigilado de lo esperado. Busco a alguien que eche un vistazo y vea qué le pasó a {3}. Además, si se encuentra alguno de nuestros suministros allí, necesito que se los lleven a {4}.\n\n¿Crees que puedes intentarlo? Supongo que los Xenos están atrincherados allí. Prepárate en consecuencia y no esperes que te lo pongan fácil. \n\nGracias, \n\nLima Endicott\nOperadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 800</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>More and more CFP ships are being targeted lately, and despite our best efforts to keep our trading routes quiet, we're still losing haulers to outlaw attacks.\n\nOur pilot over at &lt;EM4&gt;{0} is the latest casualty. It pains me to think about how much we've lost, but as long as there are people who need our help, we have to keep on fighting.\n\nIf you have a ship that can carry &lt;EM4&gt;{1} cargo containers&lt;/EM4&gt; and a &lt;EM4&gt;heavy-duty tractor beam&lt;/EM4&gt;, we need you to head to the above location and recover that cargo.\n\nThis won't be easy, the pilot was one of our best and wouldn't go down without a fight. Let's not underestimate these outlaws, bring a trustworthy crew and watch each other's backs.\n\nOnce you've got the cargo, deliver it to the freight elevator at &lt;EM4&gt;{2} and I'll get it processed.\n\nGood luck and take care,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- P8-SC SMG\n- C54 SMG\n- S71 Rifle\n- ORC-mkX Arms Woodland\n- ORC-mkX Legs Woodland\n- ORC-mkX Core Woodland\n- ORC-mkX Helmet Woodland\n- ORC-mkV Arms Woodland\n- ORC-mkV Legs Woodland\n- ORC-mkV Core Woodland\n- G-2 Helmet Woodland\n- P8-SC SMG Magazine (45 cap)\n- C54 SMG Magazine (50 cap)\n- S71 Rifle Magazine (30 cap)\n</v>
+        <v>Cada vez más naves de la CFP están siendo atacadas últimamente, y a pesar de nuestros mejores esfuerzos por mantener nuestras rutas comerciales tranquilas, seguimos perdiendo transportistas en ataques de forajidos.\n\nNuestro piloto en &lt;EM4&gt;{0} es la última víctima. Me duele pensar en todo lo que hemos perdido, pero mientras haya gente que necesite nuestra ayuda, tenemos que seguir luchando.\n\nSi tienes una nave que pueda transportar &lt;EM4&gt;{1} contenedores de carga&lt;/EM4&gt; y un &lt;EM4&gt;rayo tractor de alta potencia&lt;/EM4&gt;, necesitamos que te dirijas a la ubicación mencionada y recuperes esa carga.\n\nEsto no será fácil, el piloto era uno de los mejores y no se rendiría sin luchar. No subestimemos a estos forajidos, traigan una tripulación de confianza y cuídense las espaldas.\n\nUna vez que tengan la carga, entréguenla al montacargas en &lt;EM4&gt;{2} y yo me encargaré de procesarla.\n\nBuena suerte y cuídense,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Subfusil P8-SC\n- Subfusil C54\n- Rifle S71\n- Brazos ORC-mkX Woodland\n- Piernas ORC-mkX Woodland\n- Núcleo ORC-mkX Woodland\n- Casco ORC-mkX Woodland\n- Brazos ORC-mkV Woodland\n- Piernas ORC-mkV Woodland\n- ORC-mkV Core Woodland\n- Casco G-2 Woodland\n- Cargador de subfusil P8-SC (capacidad 45)\n- Cargador de subfusil C54 (capacidad 50)\n- Cargador de rifle S71 (capacidad 30)\n</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Hi,\n\nSomeone knocked out one of our supply ships and towed it to {0} We really need the cargo onboard. You available to head over there and recover that cargo? \n\nOnce you’ve got the goods, we need them taken to their original destination at {1} Did a little digging into this group, and let’s just say, they don’t come off as very professional. Shouldn’t give you too much resistance, but still best to show up ready to throw down.\n\nAlso, to make your life easier, I'd make sure you have a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; with you. \n\nFly Safe, \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 100</v>
+        <v>Hola,\n\nAlguien ha inutilizado uno de nuestros barcos de suministro y lo ha remolcado hasta {0}. Necesitamos urgentemente la carga a bordo. ¿Estás disponible para ir allí y recuperarla? \n\nUna vez que tengas la mercancía, necesitamos que la lleves a su destino original en {1}. He investigado un poco sobre este grupo y, digamos, no parecen muy profesionales. No deberías encontrar mucha resistencia, pero aun así es mejor que te presentes preparado para la batalla.\n\nAdemás, para facilitarte la vida, asegúrate de llevar contigo un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt;. \n\nVuela seguro, \n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 100</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Hey,\n\nOutlaws in the system have been getting aggressive lately, targeting more of our convoys. They recently ambushed one of our cargo ships and stole supplies desperately needed by our operations. If we don’t get it back, we’re worried that the locals will start losing faith. They need to know that Citizens for Prosperity can’t just be bullied out of operation.\n\nWe managed to track the outlaws to {0} Now we need someone who isn’t afraid of crossing these criminals to recover the shipment and deliver it to {1} \n\nAlso, to make your life easier, I'd make sure you have a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; with you. \n\nSo, do you think you could make the run for us?\n\nThanks,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 1,200</v>
+        <v>Hola,\n\nLos forajidos del sistema se han vuelto agresivos últimamente, atacando a más de nuestros convoyes. Recientemente emboscaron uno de nuestros barcos de carga y robaron suministros que nuestras operaciones necesitan desesperadamente. Si no los recuperamos, nos preocupa que los lugareños empiecen a perder la fe. Necesitan saber que Ciudadanos por la Prosperidad no se dejará intimidar hasta que deje de operar.\n\nLogramos rastrear a los forajidos hasta {0}. Ahora necesitamos a alguien que no tenga miedo de enfrentarse a estos criminales para recuperar el cargamento y entregarlo a {1}.\n\nAdemás, para facilitarte la vida, asegúrate de tener un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt; contigo. \n\nEntonces, ¿crees que podrías hacer la carrera por nosotros?\n\nGracias,\n\nLima Endicott\nOperadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 1200</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Hey,\n\nOutlaws used a fake distress beacon to lure one of our cargo ships into a trap and steal the supplies onboard. Thankfully, we placed trackers in the cargo containers, because the stuff is valuable mining and construction materials needed at {0} \n\nLooks like the goods ended up at {1} Need someone to head there, reclaim the supplies, and take them to {2} Doubt they’ll make it easy for you, but if it helps, they didn’t show any mercy to our ship crew. Reclaiming those supplies will not only help the CFP but ensure that our crew didn’t die in vain.   \n\nAlso, to make your life easier, I'd make sure you have a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; with you. \n\nThanks,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 150</v>
+        <v>Hola,\n\nUnos forajidos usaron una baliza de socorro falsa para atraer a uno de nuestros barcos de carga a una trampa y robar los suministros a bordo. Por suerte, colocamos rastreadores en los contenedores de carga, porque se trata de valiosos materiales de minería y construcción necesarios en {0}. \n\nParece que la mercancía terminó en {1}. Necesitamos a alguien que vaya allí, recupere los suministros y los lleve a {2}. Dudo que te lo pongan fácil, pero si te sirve de algo, no tuvieron piedad con la tripulación de nuestro barco. Recuperar esos suministros no solo ayudará a la CFP, sino que también asegurará que nuestra tripulación no murió en vano. \n\nAdemás, para facilitarte la vida, asegúrate de tener un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt; contigo. \n\nGracias,\n\nLima Endicott\nOperadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 150</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Hey,\n\nOne of our supply ships fell prey to a XenoThreat ambush. I’ll spare you the grisly details, but all that really remains is the cargo our people were carrying to {0} Trackers hidden within the cargo shows that XenoThreat collected the goods and then took them to a few locations spread out across {1} \nWe can’t let the XenoThreat get away with what they did to our crew and keep all those goods too. That’s why we want to strike back on both fronts. We need someone who can raid that location, retrieve the stolen cargo, and teach the Xenos that there will be consequences for their horrendous actions. Can you help us fight back?\n\nAlso, to make your life easier, I'd make sure you have a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; with you. \n\nThanks,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 2,400</v>
+        <v>Hola,\n\nUna de nuestras naves de suministro cayó presa de una emboscada de XenoThreat. Te ahorraré los detalles espeluznantes, pero todo lo que queda es la carga que nuestra gente llevaba a {0}. Los rastreadores ocultos en la carga muestran que XenoThreat recogió los bienes y luego los llevó a varias ubicaciones dispersas por {1}. \nNo podemos permitir que XenoThreat se salga con la suya con lo que le hicieron a nuestra tripulación y que además se quede con todos esos bienes. Por eso queremos contraatacar en ambos frentes. Necesitamos a alguien que pueda asaltar esa ubicación, recuperar la carga robada y enseñarles a los Xenos que habrá consecuencias por sus horribles acciones. ¿Puedes ayudarnos a contraatacar?\n\nAdemás, para facilitarte la vida, asegúrate de que tengas un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt; contigo. \n\nGracias,\n\nLima Endicott\nOperadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 2400</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Hi,\n\nIt appears an electrical issue caused us to lose track of a {0} carrying medical supplies. Thankfully, I received word that the ship was found at {1} We really need someone to get out there and recover the supplies onboard before someone else does. Those provisions are desperately needed at {2} Any chance you could grab them and complete the delivery? \n\nMakes me nervous seeing that the ship is at a lagrange point. Lots of folks scour them for stuff like this. Would be smart to come prepared to defend yourself if someone else comes looking to steal it.\n\nAlso, to make your life easier, I'd make sure you have a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; with you.    \n\nThanks,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 100</v>
+        <v>Hola,\n\nParece que un problema eléctrico nos hizo perder el rastro de una {0} que transportaba suministros médicos. Por suerte, me informaron de que la nave fue encontrada en {1}. Necesitamos urgentemente que alguien vaya allí y recupere los suministros a bordo antes de que lo haga otra persona. Esas provisiones son desesperadamente necesarias en {2}. ¿Hay alguna posibilidad de que puedas recogerlas y completar la entrega? \n\nMe preocupa que la nave esté en un punto de Lagrange. Mucha gente los rastrea en busca de este tipo de cosas. Sería inteligente que vinieras preparado para defenderte si alguien viene a robarlo.\n\nAdemás, para facilitarte la vida, asegúrate de llevar contigo un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt;. \n\nGracias,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 100</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Hey,\n\nI’m concerned a {0} moving medical supplies for us might’ve come under attack. The signal was lost around {1} which has seen a spike in outlaw activity recently. Losing that ship alone would be bad enough, but it’ll be even worse if those supplies don’t make it to {2} \n\nWe would need you to search for the ship at its last known position, recover the supplies, and then take them to {3} Your help would make a bad situation better. \n\nAlso, to make your life easier, I'd make sure you have a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; with you. \n\nThanks,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 150</v>
+        <v>Hola,\n\nMe preocupa que una {0} que transportaba suministros médicos para nosotros haya sido atacada. La señal se perdió cerca de {1}, donde recientemente se ha registrado un aumento en la actividad delictiva. Perder esa nave ya sería bastante malo, pero sería aún peor si esos suministros no llegan a {2}. \n\nNecesitamos que busques la nave en su última posición conocida, recuperes los suministros y los lleves a {3}. Tu ayuda mejoraría una situación difícil. \n\nAdemás, para facilitarte las cosas, asegúrate de que tengas un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt; contigo. \n\nGracias,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 150</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Violence is never our first choice, but sometimes it must be used as a preventative measure.\n\nWe’re planning a strike on a Headhunter controlled outpost and need your help.\n\nWe need to make sure that if something goes wrong they won’t be able to call for backup and escalate the situation. That’s where you come in. We need you to head over to &lt;EM4&gt;{0} and disable the communication towers. There should be a &lt;EM4&gt;control panel located at the top&lt;/EM4&gt; of each tower that you can use to deactivate them.\n\nIf you’re able to do this, Citizens for Prosperity will be able to gain some vital ground in Pyro.\n\nIt’s also worth keeping in mind for future contracts that you can choose to take out the comms towers instead of risking a fight with reinforcement dropships.\n\nStay alert and stay safe.\n\nThank you,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 75</v>
+        <v>La violencia nunca es nuestra primera opción, pero a veces debe usarse como medida preventiva.\n\nEstamos planeando un ataque a un puesto avanzado controlado por Headhunters y necesitamos tu ayuda.\n\nDebemos asegurarnos de que si algo sale mal, no puedan pedir refuerzos y la situación se agrave. Ahí es donde entras tú. Necesitamos que vayas a &lt;EM4&gt;{0} y desactives las torres de comunicación. Debería haber un panel de control en la parte superior de cada torre que puedes usar para desactivarlas.\n\nSi logras hacerlo, Ciudadanos por la Prosperidad podrá ganar terreno vital en Pyro.\n\nTambién es importante tener en cuenta para futuros contratos que puedes optar por destruir las torres de comunicaciones en lugar de arriesgarte a una pelea con las naves de refuerzo.\n\nMantente alerta y a salvo.\n\nGracias,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\nReputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 75</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Citizens for Prosperity are eager to help the people of Pyro, and it starts with freeing them from the grasp of XenoThreat.\n\nWe’re preparing a team to infiltrate one of their outposts, but we need someone to go in ahead to take out their communication towers first. Once those towers are offline, they won’t be able to call for reinforcements and we can proceed with our plan.\n\nHead to &lt;EM4&gt;{0} and find the towers. At the &lt;EM4&gt;top is a control panel&lt;/EM4&gt; that can be used to disable them.\n\nAlso, it’s worth noting that most outposts use a similar system, so you’ll know how to disable the comms towers rather than risk fighting reinforcement dropships when you’re doing other jobs.\n\nGood luck,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 75 / 100</v>
+        <v>Ciudadanos por la Prosperidad están ansiosos por ayudar a la gente de Pyro, y todo comienza con liberarlos del yugo de XenoThreat.\n\nEstamos preparando un equipo para infiltrarse en uno de sus puestos de avanzada, pero necesitamos que alguien se adelante para destruir primero sus torres de comunicación. Una vez que esas torres estén fuera de servicio, no podrán pedir refuerzos y podremos continuar con nuestro plan.\n\nDirígete a &lt;EM4&gt;{0} y encuentra las torres. En la parte superior hay un panel de control que se puede usar para desactivarlos.\n\nAdemás, cabe destacar que la mayoría de los puestos avanzados usan un sistema similar, así que sabrás cómo desactivar las torres de comunicaciones en lugar de arriesgarte a luchar contra las naves de refuerzo mientras realizas otras tareas.\n\nBuena suerte,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 75 / 100</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Hi,\n\nHere's the situation. After spending an hour on comms talking to the hauler, trying to help them diagnose what's wrong with their ship, it's been decided that we now need to get someone to head over to &lt;EM4&gt;{0} and complete the delivery.\n\nThis is a pretty big one. You'll need a ship that can store &lt;EM4&gt;{1} cargo containers&lt;/EM4&gt; and unless you're super strong a &lt;EM4&gt;heavy-duty tractor beam&lt;/EM4&gt; to shift it all.\n\nI would really appreciate if we could just get this one done. Take the cargo to the freight elevator at &lt;EM4&gt;{2} and we can put this all behind us.\n\n{3} Tieno \nJr. Logistics Coordinator \nCovalex Shipping   \n'Anything you need, anywhere you need it.' \n\n\n\n\n\n\n\nCovalex Shipping is a limited liability corporation. To encourage timely deliveries and prevent fraud on cargo hauls, Covalex Shipping will set a delivery time limit and upon expiration, any undelivered cargo will be considered stolen and treated as such. Total payment will be prorated according to the percentage of cargo successfully delivered.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>Hola,\n\nEsta es la situación. Después de pasar una hora en comunicaciones hablando con el transportista, tratando de ayudarlos a diagnosticar qué le pasa a su barco, se ha decidido que ahora necesitamos que alguien vaya a &lt;EM4&gt;{0} y complete la entrega.\n\nEste es un envío bastante grande. Necesitarás un barco que pueda almacenar &lt;EM4&gt;{1} contenedores de carga&lt;/EM4&gt; y, a menos que seas súper fuerte, una &lt;EM4&gt;raya tractora de alta resistencia&lt;/EM4&gt; para moverlo todo.\n\nRealmente agradecería que pudiéramos hacer esto. Lleva la carga al montacargas en &lt;EM4&gt;{2} y podremos dejar todo esto atrás.\n\n{3} Tieno \nJr. Coordinador de Logística \nCovalex Shipping \n'Todo lo que necesites, donde lo necesites.' \n\n\n\n\n\n\n\nCovalex Shipping es una corporación de responsabilidad limitada. Para fomentar las entregas puntuales y prevenir el fraude en el transporte de carga, Covalex Shipping establecerá un plazo límite de entrega y, una vez transcurrido dicho plazo, cualquier carga no entregada se considerará robada y se tratará como tal. El pago total se prorrateará según el porcentaje de carga entregada con éxito.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Call me Twitch. I run the Dead Saints. \n\nI doubt this is the first time you've heard of us, but in case you haven't, we do a lot of things, but one of them is transporting goods that need discreet handling. \n\nI got your info from one of my contacts. They say you've got the stuff we like in a hauler, which works for me, because we're looking for one. \n\nHere's my proposal – we're offering creds to the pilot that can transport some special cargo for us. Your ship’s hold will need room for &lt;EM4&gt;{0} cargo containers&lt;/EM4&gt;, and you'll need a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; for loading and unloading. All you have to do is get everything from &lt;EM4&gt;{1} to &lt;EM4&gt;{2} without getting security involved. \n \nIf you can pull the job off, the Saints will have more contracts for you down the line. \n\n-Twitch\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100</v>
+        <v>Llámame Twitch. Dirijo los Santos Muertos. \n\nDudo que sea la primera vez que oyes hablar de nosotros, pero por si acaso, hacemos muchas cosas, entre ellas, transportar mercancías que requieren un manejo discreto. \n\nObtuve tu información de uno de mis contactos. Dicen que tienes lo que buscamos en una nave de transporte, lo cual me viene bien, porque estamos buscando una. \n\nEsta es mi propuesta: ofrecemos créditos al piloto que pueda transportar una carga especial para nosotros. La bodega de tu nave necesitará espacio para &lt;EM4&gt;{0} contenedores de carga&lt;/EM4&gt;, y necesitarás un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt; para cargar y descargar. Todo lo que tienes que hacer es llevar todo de &lt;EM4&gt;{1} a &lt;EM4&gt;{2} sin llamar la atención de la seguridad. \n \nSi logras completar el trabajo, los Santos tendrán más contratos para ti en el futuro. \n\n-Twitch\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>We got a situation. Some gang that no one’s heard of are trying to make a name for themselves by targeting our transport ships. They think they can make a big show of how tough they are raiding our haulers and acting like they’re big shots. Amateurs.\n\nProblem is, they got lucky during their last attack. Our pilot barely made it out alive, but their ship is still sitting full of supplies over at &lt;EM4&gt;{0} a crew you can trust and your &lt;EM4&gt;heavy-duty tractor beam&lt;/EM4&gt; and get your ass over there.\n\nAfter, drop the gear off at the freight elevator in &lt;EM4&gt;{1} You do this for me and I’ll give you a good cut of the sale.\n\n-Twitch\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>Tenemos un problema. Una banda desconocida está intentando hacerse famosa atacando nuestros barcos de transporte. Creen que pueden alardear de su dureza asaltando nuestros cargueros y comportándose como si fueran peces gordos. Unos aficionados.\n\nEl problema es que tuvieron suerte en su último ataque. Nuestro piloto apenas sobrevivió, pero su nave sigue llena de suministros en &lt;EM4&gt;{0}. Necesitas una tripulación de confianza y tu &lt;EM4&gt;rayo tractor de alta potencia&lt;/EM4&gt; y ven para allá.\n\nDespués, deja el equipo en el montacargas de &lt;EM4&gt;{1}. Si haces esto por mí, te daré una buena parte de la venta.\n\n-Twitch\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ECKHART SECURITY, LLC.\nCONTRACTS &amp; DISPATCH\n\nCONTRACT TYPE: Recover Cargo\nApproval code: = {0} IMMEDIATE PROCESSING\n\nCalling for a skilled contractor to recover a displaced shipment located at &lt;EM4&gt;{1} Client's hauler was transporting some high value cargo when they decided to respond to a distress beacon and got ambushed by a group of outlaws. The client believes their pilot is gone but their cargo could still be recovered.\n\nThe information we have so far is that you'll need a ship that can carry &lt;EM4&gt;{2} cargo containers&lt;/EM4&gt;, a &lt;EM4&gt;heavy-duty tractor beam&lt;/EM4&gt; for shifting the goods, as well as your support ships to help deal with the outlaws at the location. \n\nClient will be expecting the completed delivery to be made to the freight elevator at &lt;EM4&gt;{3} contract is non-negotiable.\n\nThis message may contain confidential, proprietary, privileged and/or private information. The information is intended to be for the use of the individual or entity designated above.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>ECKHART SECURITY, LLC.\nCONTRATOS Y DESPACHO\n\nTIPO DE CONTRATO: Recuperación de carga\nCódigo de aprobación: = {0} PROCESAMIENTO INMEDIATO\n\nSe solicita un contratista especializado para recuperar un envío desplazado ubicado en &lt;EM4&gt;{1}. El transportista del cliente transportaba carga de alto valor cuando decidió responder a una señal de socorro y fue emboscado por un grupo de forajidos. El cliente cree que su piloto ha desaparecido, pero su carga aún podría recuperarse.\n\nLa información que tenemos hasta ahora es que necesitará un barco que pueda transportar &lt;EM4&gt;{2} contenedores de carga&lt;/EM4&gt;, un &lt;EM4&gt;rayo tractor de alta resistencia&lt;/EM4&gt; para mover la mercancía, así como sus barcos de apoyo para ayudar a lidiar con los forajidos en la ubicación. El cliente espera que la entrega completa se realice en el montacargas ubicado en &lt;EM4&gt;{3}. El contrato no es negociable. Este mensaje puede contener información confidencial, de propiedad exclusiva, privilegiada y/o privada. La información está destinada al uso de la persona o entidad designada anteriormente. Reputación otorgada (por dificultad): 50/200</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>AVAILABLE FTL CONTRACT\nFOR IMMEDIATE ASSIGNMENT\n\n**CONTRACT DETAILS** \nA reliable and hardworking entry-level courier is needed to ferry a delivery in Stanton.\nYou will be responsible for providing your own transportation.\nInterested contractors need the &lt;EM4&gt;ability to lift up to .25 SCU boxes&lt;/EM4&gt;.\nContractors are employed on an independent basis and therefore not covered by FTL's company insurance.\n\n{0} Awarded (by difficulty):&lt;/EM4&gt; 100 / 500\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Colossus (Quantum Drive)\n- Huracan (Quantum Drive)\n- Agni (Quantum Drive)\n- Defiant (Powerplant)\n- Endurance (Powerplant)\n- Sedulity (Powerplant)\n</v>
+        <v>CONTRATO FTL DISPONIBLE\nPARA ASIGNACIÓN INMEDIATA\n\n**DETALLES DEL CONTRATO** \nSe necesita un mensajero confiable y trabajador de nivel básico para transportar una entrega en Stanton.\nUsted será responsable de proporcionar su propio transporte.\nLos contratistas interesados deben tener la &lt;EM4&gt;capacidad de levantar cajas de hasta 0.25 SCU&lt;/EM4&gt;.\nLos contratistas son empleados de forma independiente y, por lo tanto, no están cubiertos por el seguro de la empresa FTL.\n\n{0} Adjudicado (por dificultad):&lt;/EM4&gt; 100 / 500\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Colossus (Quantum Drive)\n- Huracan (Quantum Drive)\n- Agni (Quantum Drive)\n- Defiant (Powerplant)\n- Endurance (Powerplant)\n- Sedulity (Powerplant)\n</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Following the brutal attack on Pyro and our efforts to combat the vigilante group the Frontier Fighters, our strategic reserves across the system are at an all-time low. Citizens for Prosperity are eager to replenish our stocks before we reach a point of desperation. \n\nTo that end, we were hoping that you would be able to resupply&lt;EM4&gt; {0} with detatrine. &lt;/EM4&gt;\n\nThis rare chemical compound is a key ingredient in several vital medical supplies, so it is important that replace what we used up treating local civilians and CFP members injured in the wake of the Frontier Fighter assault.\n\nNormally we would direct you to reputable sources to acquire detatrine, but our contacts have informed us that several &lt;EM4&gt;depots&lt;/EM4&gt; around the system have suddenly decided to sell the chemical at a significantly reduced price. In fact, it’s inexpensive enough that I suspect it will draw some unwanted attention. If you decide to seek out this potentially deadly deal, please do so with caution.\n\nYour support of our efforts is much appreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Tras el brutal ataque a Pyro y nuestros esfuerzos por combatir al grupo justiciero Frontier Fighters, nuestras reservas estratégicas en todo el sistema están en su nivel más bajo. Ciudadanos por la Prosperidad están ansiosos por reabastecer nuestras existencias antes de que lleguemos a un punto de desesperación. \n\nCon ese fin, esperábamos que pudieras reabastecer a &lt;EM4&gt; {0} con detatrina. &lt;/EM4&gt;\n\nEste raro compuesto químico es un ingrediente clave en varios suministros médicos vitales, por lo que es importante reemplazar lo que consumimos tratando a los civiles locales y a los miembros de CFP heridos tras el ataque de Frontier Fighters.\n\nNormalmente te dirigiríamos a fuentes confiables para adquirir detatrina, pero nuestros contactos nos han informado que varios depósitos de &lt;EM4&gt; en todo el sistema han decidido repentinamente vender el químico a un precio significativamente reducido. De hecho, es tan barato que sospecho que atraerá atención no deseada. Si decide buscar esta oferta potencialmente mortal, hágalo con precaución.\n\nAgradecemos mucho su apoyo a nuestros esfuerzos.\n\nLima Endicott\nOperadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Following the brutal attack on Pyro and our efforts to combat the vigilante group the Frontier Fighters, our strategic reserves across the system are at an all-time low. Citizens for Prosperity are eager to replenish our stocks before we reach a point of desperation. \n\nTo that end, we were hoping that you would recruit a full fleet to resupply&lt;EM4&gt; {0} with detatrine. &lt;/EM4&gt;\n\nThis rare chemical compound is a key ingredient in several vital medical supplies, so it is important that replace what we used up treating local civilians and CFP members injured in the wake of the Frontier Fighter assault.\n\nNormally we would direct you to reputable sources to acquire detatrine, but our contacts have informed us that several &lt;EM4&gt;depots&lt;/EM4&gt; around the system have suddenly decided to sell the chemical at a significantly reduced price. In fact, it’s inexpensive enough that I suspect it will draw some unwanted attention. If you decide to seek out this potentially deadly deal, please do so with caution.\n\nYour support of our efforts is much appreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Tras el brutal ataque a Pyro y nuestros esfuerzos por combatir al grupo justiciero de los Frontier Fighters, nuestras reservas estratégicas en todo el sistema están en su nivel más bajo. Ciudadanos por la Prosperidad está ansioso por reabastecer nuestras existencias antes de que lleguemos a un punto de desesperación. \n\nCon ese fin, esperábamos que reclutaras una flota completa para reabastecer &lt;EM4&gt; {0} con detatrina. &lt;/EM4&gt;\n\nEste raro compuesto químico es un ingrediente clave en varios suministros médicos vitales, por lo que es importante reemplazar lo que consumimos tratando a los civiles locales y a los miembros de CFP heridos tras el ataque de los Frontier Fighters.\n\nNormalmente te dirigiríamos a fuentes confiables para adquirir detatrina, pero nuestros contactos nos han informado que varios depósitos de &lt;EM4&gt; en todo el sistema han decidido repentinamente vender el químico a un precio significativamente reducido. De hecho, es tan barato que sospecho que atraerá atención no deseada. Si decide buscar esta oferta potencialmente mortal, hágalo con precaución.\n\nAgradecemos mucho su apoyo a nuestros esfuerzos.\n\nLima Endicott\nOperadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Following the brutal attack on Pyro and our efforts to combat the vigilante group the Frontier Fighters, our strategic reserves across the system are at an all-time low. Citizens for Prosperity are eager to replenish our stocks before we reach a point of desperation. \n\nTo that end, we were hoping that you and a team of your choosing would be able to resupply&lt;EM4&gt; {0} with detatrine. &lt;/EM4&gt;  \n\nThis rare chemical compound is a key ingredient in several vital medical supplies, so it is important that replace what we used up treating local civilians and CFP members injured in the wake of the Frontier Fighter assault.\n\nNormally we would direct you to reputable sources to acquire detatrine, but our contacts have informed us that several &lt;EM4&gt;depots&lt;/EM4&gt; around the system have suddenly decided to sell the chemical at a significantly reduced price. In fact, it’s inexpensive enough that I suspect it will draw some unwanted attention. If you decide to seek out this potentially deadly deal, please do so with caution.\n\nYour support of our efforts is much appreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Tras el brutal ataque a Pyro y nuestros esfuerzos por combatir al grupo justiciero Frontier Fighters, nuestras reservas estratégicas en todo el sistema están en su nivel más bajo. Ciudadanos por la Prosperidad deseamos reabastecer nuestras existencias antes de llegar a un punto de desesperación. \n\nCon ese fin, esperábamos que usted y un equipo de su elección pudieran reabastecer a &lt;EM4&gt; {0} con detatrina. &lt;/EM4&gt; \n\nEste raro compuesto químico es un ingrediente clave en varios suministros médicos vitales, por lo que es importante reemplazar lo que consumimos tratando a los civiles locales y a los miembros de CFP heridos tras el ataque de Frontier Fighters.\n\nNormalmente, le dirigiríamos a fuentes confiables para adquirir detatrina, pero nuestros contactos nos han informado que varios depósitos de &lt;EM4&gt; en todo el sistema han decidido repentinamente vender el químico a un precio significativamente reducido. De hecho, es tan barato que sospecho que atraerá atención no deseada. Si decide buscar esta oferta potencialmente mortal, hágalo con precaución.\n\nAgradecemos mucho su apoyo a nuestros esfuerzos.\n\nLima Endicott\nOperadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Kicking the crap out of those Frontier Fighter bastards seriously depleted our supplies and now our stash of detatrine is practically out of stock. \n\nThat’s why you’re going to do a detatrine resupply run to&lt;EM4&gt; {0} &lt;/EM4&gt;\n\nNot sure if you’re familiar with it, but the chemical’s what we use to make our batches of sludge. We can’t really afford to let our sales of the stuff dry up right now. Not when we need credits so bad.\n\nThe good news is that &lt;EM4&gt;depots&lt;/EM4&gt; across the system are offering detatrine and rock-bottom prices. Hell if I know why they’re doing it, all I know is that everyone with a lick of sense is trying to get their hands on the stuff so be ready for fierce competition. \n\nI’m trustin’ you to get it done,\nStows  \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Darles una paliza a esos bastardos de Frontier Fighter agotó seriamente nuestros suministros y ahora nuestro alijo de detatrina está prácticamente agotado. \n\nPor eso vas a hacer una carrera de reabastecimiento de detatrina a &lt;EM4&gt; {0} &lt;/EM4&gt;\n\nNo sé si estás familiarizado con ella, pero el químico es lo que usamos para hacer nuestros lotes de lodo. Realmente no podemos permitirnos que nuestras ventas de esa cosa se agoten ahora mismo. No cuando necesitamos créditos tan desesperadamente.\n\nLa buena noticia es que los depósitos de &lt;EM4&gt; en todo el sistema están ofreciendo detatrina a precios bajísimos. Ni idea de por qué lo hacen, lo único que sé es que todo el mundo con un mínimo de sentido común está intentando hacerse con ella, así que prepárate para una competencia feroz. \n\nConfío en que lo harás,\nStows \n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Kicking the crap out of those Frontier Fighter bastards seriously depleted our supplies and now our stash of detatrine is practically out of stock. \n\nThat’s why you’re going to put together a full fleet to do a detatrine resupply run to&lt;EM4&gt; {0} &lt;/EM4&gt;\n\nNot sure if you’re familiar with it, but the chemical’s what we use to make our batches of sludge. We can’t really afford to let our sales of the stuff dry up right now. Not when we need credits so bad.\n\nThe good news is that &lt;EM4&gt;depots&lt;/EM4&gt; across the system are offering detatrine and rock-bottom prices. Hell if I know why they’re doing it, all I know is that everyone with a lick of sense is trying to get their hands on the stuff so be ready for fierce competition. \n\nI’m trustin’ you to get it done,\nStows  \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Darles una paliza a esos bastardos de Frontier Fighter agotó seriamente nuestros suministros y ahora nuestro alijo de detatrina está prácticamente agotado. \n\nPor eso vas a reunir una flota completa para hacer una misión de reabastecimiento de detatrina a &lt;EM4&gt; {0} &lt;/EM4&gt;\n\nNo sé si estás familiarizado con ella, pero el químico es lo que usamos para hacer nuestros lotes de lodo. Realmente no podemos permitirnos que nuestras ventas de esa cosa se agoten ahora mismo. No cuando necesitamos créditos tan desesperadamente.\n\nLa buena noticia es que los depósitos de &lt;EM4&gt;&lt;/EM4&gt; en todo el sistema están ofreciendo detatrina a precios bajísimos. Ni idea de por qué lo hacen, lo único que sé es que todo el mundo con un mínimo de sentido común está intentando hacerse con ella, así que prepárate para una competencia feroz. \n\nConfío en que lo harás,\nStows \n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Kicking the crap out of those Frontier Fighter bastards seriously depleted our supplies and now our stash of detatrine is practically out of stock.\n\nThat’s why you and whoever else you want to bring along are going to do a detatrine resupply run to&lt;EM4&gt; {0} &lt;/EM4&gt;\n\nNot sure if you’re familiar with it, but the chemical’s what we use to make our batches of sludge. We can’t really afford to let our sales of the stuff dry up right now. Not when we need credits so bad.\n\nThe good news is that &lt;EM4&gt;depots&lt;/EM4&gt; across the system are offering detatrine and rock-bottom prices. Hell if I know why they’re doing it, all I know is that everyone with a lick of sense is trying to get their hands on the stuff so be ready for fierce competition. \n\nI’m trustin’ you to get it done,\nStows  \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Darles una paliza a esos bastardos de Frontier Fighter agotó seriamente nuestros suministros y ahora nuestro alijo de detatrina está prácticamente agotado.\n\nPor eso tú y quien quieras traer van a hacer una carrera de reabastecimiento de detatrina a &lt;EM4&gt; {0} &lt;/EM4&gt;\n\nNo sé si estás familiarizado con ella, pero el químico es lo que usamos para hacer nuestros lotes de lodo. Realmente no podemos permitirnos que nuestras ventas de esa cosa se agoten ahora mismo. No cuando necesitamos créditos tan desesperadamente.\n\nLa buena noticia es que los depósitos de &lt;EM4&gt; en todo el sistema están ofreciendo detatrina a precios bajísimos. Ni idea de por qué lo hacen, lo único que sé es que todo el mundo con un mínimo de sentido común está intentando hacerse con ella, así que prepárate para una competencia feroz. \n\nConfío en que lo harás,\nStows \n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>We need a contractor to provide convoy and protection services at &lt;EM4&gt;{0} One of our elite clients' are under attack from a band of outlaws targeting their &lt;EM4&gt;{1} and ships&lt;/EM4&gt;. You'll need to keep the crew safe as they traverse the area, as well as make sure the assets stay as intact. These thugs look like they can do some real damage, so be sure you engage them with caution or the client might not be the only one to take heavy losses.\n\nIf you manage to nail this to the Foxwell standards, we’re offering &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt; as compensation to the main contractor. \n\nGood luck,\n\nKevin Walton\nDispatcher, Foxwell Enforcement\n'Security, Your Way'\n\nFoxwell Enforcement is a bonded security specialist licensed to operate throughout the UEE. We are always looking for new operators to join our family. If you or anyone you know is interested, please reach out to one of our contract representatives.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 100\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: nyx, Nyx III, Nyx System&lt;/EM4&gt;\n- Frost-Star SL (Cooler)\n- Fridan (Cooler)\n- Tepilo (Cooler)\n- Frost-Star (Cooler)\n- ArcticStorm (Cooler)\n- Berian (Cooler)\n- Gelid (Cooler)\n- Frost-Star EX (Cooler)\n- ColdSnap (Cooler)\n- Aufeis (Cooler)\n- Graupel (Cooler)\n- Frost-Star XL (Cooler)\n- FrostBurn (Cooler)\n- Draug (Cooler)\n- Elsen (Cooler)\n- Kragen (Cooler)\n\n&lt;EM4&gt;[Regional Variants] example locations: Pyro I, Checkmate Clinic, RAB-FOXTROT&lt;/EM4&gt;\n- IonWave (Powerplant)\n- Radix (Powerplant)\n- IonBurst (Powerplant)\n- PowerBolt (Powerplant)\n- LightBlossom (Powerplant)\n- MagnaBloom (Powerplant)\n- FullForce (Powerplant)\n- IonSurge (Powerplant)\n- DayBreak (Powerplant)\n- Radiance (Powerplant)\n- FullForce Pro (Powerplant)\n- IonSurge Pro (Powerplant)\n- Celestial (Powerplant)\n- NewDawn (Powerplant)\n\n&lt;EM4&gt;[Regional Variants] example locations: Aberdeen, Magda, Arial&lt;/EM4&gt;\n- 7SA (Shield)\n- INK (Shield)\n- 7MA 'Lorica' (Shield)\n- RPEL (Shield)\n- 7CA 'Nargun' (Shield)\n- HAVEN (Shield)\n</v>
+        <v>Necesitamos un contratista para brindar servicios de convoy y protección en &lt;EM4&gt;{0}. Uno de nuestros clientes de élite está siendo atacado por una banda de forajidos que tienen como objetivo sus &lt;EM4&gt;{1} y barcos&lt;/EM4&gt;. Deberá mantener a la tripulación a salvo mientras atraviesan el área, así como asegurarse de que los activos permanezcan intactos. Estos matones parecen poder causar daños reales, así que asegúrese de enfrentarlos con precaución o el cliente podría no ser el único en sufrir grandes pérdidas.\n\nSi logra cumplir con los estándares de Foxwell, ofrecemos &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt; como compensación al contratista principal.\n\nBuena suerte,\n\nKevin Walton\nDespachador, Foxwell Enforcement\n'Seguridad, a su manera'\n\nFoxwell Enforcement es un especialista en seguridad con fianza y licencia para operar en toda la UEE. Siempre estamos buscando nuevos operadores para unirse a nuestra familia. Si usted o alguien que conoce está interesado, comuníquese con uno de nuestros representantes de contratos.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 100\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: nyx, Nyx III, Nyx System&lt;/EM4&gt;\n- Frost-Star SL (Cooler)\n- Fridan (Cooler)\n- Tepilo (Cooler)\n- Frost-Star (Cooler)\n- ArcticStorm (Cooler)\n- Berian (Cooler)\n- Gelid (Cooler)\n- Frost-Star EX (Cooler)\n- ColdSnap (Cooler)\n- Aufeis (Cooler)\n- Graupel (Cooler)\n- Frost-Star XL (Cooler)\n- FrostBurn (Cooler)\n- Draug (Cooler)\n- Elsen (Cooler)\n- Kragen (Cooler)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Pyro I, Checkmate Clinic, RAB-FOXTROT&lt;/EM4&gt;\n- IonWave (Planta de energía)\n- Radix (Planta de energía)\n- IonBurst (Planta de energía)\n- PowerBolt (Planta de energía)\n- LightBlossom (Planta de energía)\n- MagnaBloom (Planta de energía)\n- FullForce (Planta de energía)\n- IonSurge (Planta de energía)\n- DayBreak (Planta de energía)\n- Radiance (Planta de energía)\n- FullForce Pro (Planta de energía)\n- IonSurge Pro (Planta de energía)\n- Celestial (Planta de energía)\n- NewDawn (Planta de energía)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Aberdeen, Magda, Arial&lt;/EM4&gt;\n- 7SA (Escudo)\n- TINTA (Escudo)\n- 7MA 'Lorica' (Escudo)\n- RPEL (Escudo)\n- 7CA 'Nargun' (Escudo)\n- REFUGIO (Escudo)\n</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Crew managing one of our client's operations at &lt;EM4&gt;{0} have reported that they're under attack from a criminal gang targeting the &lt;EM4&gt;{1} and ships&lt;/EM4&gt; in the area. It will be your job to keep both safe at all costs. I don't have all the facts yet, but I reckon this will be a tough mission – these outlaws seem determined to do some real carnage. \n\nIf it were me, I would &lt;EM&gt;bring backup&lt;/EM4&gt; to deal with them. And if you manage to protect everyone, we’re offering a well-earned &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt; to the main contractor who deals with these lowlife's successfully. \n\nBest of luck,\n\nKevin Walton\nDispatcher, Foxwell Enforcement\n'Security, Your Way'\n\nFoxwell Enforcement is a bonded security specialist licensed to operate throughout the UEE. We are always looking for new operators to join our family. If you or anyone you know is interested, please reach out to one of our contract representatives.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 200\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Nyx III, Nyx System, Nyx II&lt;/EM4&gt;\n- Frost-Star SL (Cooler)\n- Fridan (Cooler)\n- Tepilo (Cooler)\n- Frost-Star (Cooler)\n- ArcticStorm (Cooler)\n- Berian (Cooler)\n- Gelid (Cooler)\n- Frost-Star EX (Cooler)\n- ColdSnap (Cooler)\n- Aufeis (Cooler)\n- Graupel (Cooler)\n- Frost-Star XL (Cooler)\n- FrostBurn (Cooler)\n- Draug (Cooler)\n- Elsen (Cooler)\n- Kragen (Cooler)\n\n&lt;EM4&gt;[Regional Variants] example locations: nyx, Nyx System, Nyx III&lt;/EM4&gt;\n- CF-117 Bulldog Repeater\n- CF-227 Badger Repeater\n- CF-337 Panther Repeater\n- CF-447 Rhino Repeater\n- CF-557 Galdereen Repeater\n- CF-667 Mammoth Repeater\n- V60-26 (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: Patch City, RAB-NOVEMBER, Checkmate Clinic&lt;/EM4&gt;\n- IonWave (Powerplant)\n- Radix (Powerplant)\n- IonBurst (Powerplant)\n- PowerBolt (Powerplant)\n- LightBlossom (Powerplant)\n- MagnaBloom (Powerplant)\n- FullForce (Powerplant)\n- IonSurge (Powerplant)\n- DayBreak (Powerplant)\n- Radiance (Powerplant)\n- FullForce Pro (Powerplant)\n- IonSurge Pro (Powerplant)\n- Celestial (Powerplant)\n- NewDawn (Powerplant)\n\n&lt;EM4&gt;[Regional Variants] example locations: Cluster NBD-102, RAB-FOXTROT, RAB-ROTH&lt;/EM4&gt;\n- Glacier (Cooler)\n- Avalanche (Cooler)\n- Blizzard (Cooler)\n- DR Model-XJ1 Repeater\n- DR Model-XJ2 Repeater\n- DR Model-XJ3 Repeater\n\n&lt;EM4&gt;[Regional Variants] example locations: Ita, Arial, Aberdeen&lt;/EM4&gt;\n- 7SA (Shield)\n- INK (Shield)\n- 7MA 'Lorica' (Shield)\n- RPEL (Shield)\n- 7CA 'Nargun' (Shield)\n- HAVEN (Shield)\n\n&lt;EM4&gt;[Regional Variants] example locations: Magda, Arial, Ita&lt;/EM4&gt;\n- Attrition-4 Repeater\n- Attrition-5 Repeater\n- Attrition-6 Repeater\n- FR-86 (Shield)\n- Sens (Radar)\n- Tige (Radar)\n</v>
+        <v>La tripulación que gestiona las operaciones de uno de nuestros clientes en &lt;EM4&gt;{0} ha informado que están siendo atacados por una banda criminal que tiene como objetivo el &lt;EM4&gt;{1} y los barcos&lt;/EM4&gt; en la zona. Será su trabajo mantenerlos a salvo a toda costa. Todavía no tengo todos los datos, pero creo que será una misión difícil; estos forajidos parecen decididos a causar una verdadera carnicería. \n\nSi fuera yo, &lt;EM&gt;traería refuerzos&lt;/EM4&gt; para lidiar con ellos. Y si logra proteger a todos, ofrecemos un merecido &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt; al contratista principal que se encargue con éxito de estos maleantes. \n\nMucha suerte,\n\nKevin Walton\nDespachador, Foxwell Enforcement\n'Seguridad, a su manera'\n\nFoxwell Enforcement es un especialista en seguridad con fianza y licencia para operar en toda la UEE. Siempre estamos buscando nuevos operadores para unirse a nuestra familia. Si usted o alguien que conoce está interesado, comuníquese con uno de nuestros representantes de contratos.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 200\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx III, Nyx System, Nyx II&lt;/EM4&gt;\n- Frost-Star SL (enfriador)\n- Fridan (enfriador)\n- Tepilo (enfriador)\n- Frost-Star (enfriador)\n- ArcticStorm (enfriador)\n- Berian (enfriador)\n- Gelid (enfriador)\n- Frost-Star EX (enfriador)\n- ColdSnap (enfriador)\n- Aufeis (enfriador)\n- Graupel (enfriador)\n- Frost-Star XL (enfriador)\n- FrostBurn (enfriador)\n- Draug (enfriador)\n- Elsen (Cooler)\n- Kragen (Cooler)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: nyx, Nyx System, Nyx III&lt;/EM4&gt;\n- Repetidor Bulldog CF-117\n- Repetidor Tejón CF-227\n- Repetidor Pantera CF-337\n- Repetidor Rinoceronte CF-447\n- Repetidor Galdereen CF-557\n- Repetidor Mamut CF-667\n- V60-26 (Radar)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Patch City, RAB-NOVEMBER, Clínica Checkmate&lt;/EM4&gt;\n- Onda iónica (Planta de energía)\n- Radix (Planta de energía)\n- Explosión iónica (Planta de energía)\n- Rayo de energía (Planta de energía)\n- Flor de luz (Planta de energía)\n- Magnaflor (Planta de energía)\n- Fuerza total (Planta de energía)\n- IonSurge (Planta de energía)\n- DayBreak (Planta de energía)\n- Radiance (Planta de energía)\n- FullForce Pro (Planta de energía)\n- IonSurge Pro (Planta de energía)\n- Celestial (Planta de energía)\n- NewDawn (Planta de energía)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Cluster NBD-102, RAB-FOXTROT, RAB-ROTH&lt;/EM4&gt;\n- Glacier (Enfriador)\n- Avalanche (Enfriador)\n- Blizzard (Enfriador)\n- Repetidor DR Model-XJ1\n- Repetidor DR Model-XJ2\n- Repetidor DR Model-XJ3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Ita, Arial, Aberdeen&lt;/EM4&gt;\n- 7SA (Escudo)\n- INK (Escudo)\n- 7MA 'Lorica' (Escudo)\n- RPEL (Escudo)\n- 7CA 'Nargun' (Escudo)\n- HAVEN (Escudo)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Magda, Arial, Ita&lt;/EM4&gt;\n- Repetidor Attrition-4\n- Repetidor Attrition-5\n- Repetidor Attrition-6\n- FR-86 (Escudo)\n- Sens (Radar)\n- Tige (Radar)\n</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>We need a contractor to provide convoy and protection services at &lt;EM4&gt;{0} One of our elite clients' are under attack from a band of outlaws targeting their &lt;EM4&gt;{1} and ships&lt;/EM4&gt;. You'll need to keep the crew safe as they traverse the area, as well as make sure the assets stay as intact. These thugs look like they can do some real damage, so be sure you engage them with caution or the client might not be the only one to take heavy losses.\n\nIf you manage to nail this to the Foxwell standards, we’re offering &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt; as compensation to the main contractor. \n\nGood luck,\n\nKevin Walton\nDispatcher, Foxwell Enforcement\n'Security, Your Way'\n\nFoxwell Enforcement is a bonded security specialist licensed to operate throughout the UEE. We are always looking for new operators to join our family. If you or anyone you know is interested, please reach out to one of our contract representatives.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 150\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Nyx I, nyx, Nyx&lt;/EM4&gt;\n- Frost-Star SL (Cooler)\n- Fridan (Cooler)\n- Tepilo (Cooler)\n- Frost-Star (Cooler)\n- ArcticStorm (Cooler)\n- Berian (Cooler)\n- Gelid (Cooler)\n- Frost-Star EX (Cooler)\n- ColdSnap (Cooler)\n- Aufeis (Cooler)\n- Graupel (Cooler)\n- Frost-Star XL (Cooler)\n- FrostBurn (Cooler)\n- Draug (Cooler)\n- Elsen (Cooler)\n- Kragen (Cooler)\n\n&lt;EM4&gt;[Regional Variants] example locations: Patch City, Cluster NBD-102, RAB-ALPHA&lt;/EM4&gt;\n- IonWave (Powerplant)\n- Radix (Powerplant)\n- IonBurst (Powerplant)\n- PowerBolt (Powerplant)\n- LightBlossom (Powerplant)\n- MagnaBloom (Powerplant)\n- FullForce (Powerplant)\n- IonSurge (Powerplant)\n- DayBreak (Powerplant)\n- Radiance (Powerplant)\n- FullForce Pro (Powerplant)\n- IonSurge Pro (Powerplant)\n- Celestial (Powerplant)\n- NewDawn (Powerplant)\n\n&lt;EM4&gt;[Regional Variants] example locations: Ita, Hurston, Magda&lt;/EM4&gt;\n- 7SA (Shield)\n- INK (Shield)\n- 7MA 'Lorica' (Shield)\n- RPEL (Shield)\n- 7CA 'Nargun' (Shield)\n- HAVEN (Shield)\n</v>
+        <v>Necesitamos un contratista para brindar servicios de convoy y protección en &lt;EM4&gt;{0}. Uno de nuestros clientes de élite está siendo atacado por una banda de forajidos que tienen como objetivo sus &lt;EM4&gt;{1} y barcos&lt;/EM4&gt;. Deberá mantener a la tripulación a salvo mientras atraviesan el área, así como asegurarse de que los activos permanezcan intactos. Estos matones parecen poder causar daños reales, así que asegúrese de enfrentarlos con precaución o el cliente podría no ser el único en sufrir grandes pérdidas.\n\nSi logra cumplir con los estándares de Foxwell, ofrecemos &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt; como compensación al contratista principal.\n\nBuena suerte,\n\nKevin Walton\nDespachador, Foxwell Enforcement\n'Seguridad, a su manera'\n\nFoxwell Enforcement es un especialista en seguridad con fianza y licencia para operar en toda la UEE. Siempre estamos buscando nuevos operadores para unirse a nuestra familia. Si usted o alguien que conoce está interesado, comuníquese con uno de nuestros representantes de contratos.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 150\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx I, nyx, Nyx&lt;/EM4&gt;\n- Frost-Star SL (Cooler)\n- Fridan (Cooler)\n- Tepilo (Cooler)\n- Frost-Star (Cooler)\n- ArcticStorm (Cooler)\n- Berian (Cooler)\n- Gelid (Cooler)\n- Frost-Star EX (Cooler)\n- ColdSnap (Cooler)\n- Aufeis (Cooler)\n- Graupel (Cooler)\n- Frost-Star XL (Cooler)\n- FrostBurn (Cooler)\n- Draug (Cooler)\n- Elsen (Cooler)\n- Kragen (Cooler)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Patch City, Cluster NBD-102, RAB-ALPHA&lt;/EM4&gt;\n- IonWave (Planta de energía)\n- Radix (Planta de energía)\n- IonBurst (Planta de energía)\n- PowerBolt (Planta de energía)\n- LightBlossom (Planta de energía)\n- MagnaBloom (Planta de energía)\n- FullForce (Planta de energía)\n- IonSurge (Planta de energía)\n- DayBreak (Planta de energía)\n- Radiance (Planta de energía)\n- FullForce Pro (Planta de energía)\n- IonSurge Pro (Planta de energía)\n- Celestial (Planta de energía)\n- NewDawn (Planta de energía)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Ita, Hurston, Magda&lt;/EM4&gt;\n- 7SA (Escudo)\n- INK (Escudo)\n- 7MA 'Lorica' (Escudo)\n- RPEL (Escudo)\n- 7CA 'Nargun' (Escudo)\n- HAVEN (Escudo)\n</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>An emergency SOS just came through from a maintenance crew under the employ of one of Foxwell's VIP clients. If available, we urge you to get to &lt;EM4&gt;{0} as soon as possible. While engaging with the attackers, you'll be expected to protect the client’s  &lt;EM4&gt;{1} and of their ships that may need assistance&lt;/EM4&gt;. \n\nThis is far from the first we've seen from these particular outlaws, so believe me when I say these pilots are not to be taken lightly. I strongly recommend that you arrange a &lt;EM&gt;highly competent backup force&lt;/EM&gt; to fly with you to the site.\n\nIf you manage to successfully defend the client's interests, we’re offering &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt; as compensation to the main contractor brave enough to take this job on. \n\nStay safe, and good luck,\n\nKevin Walton\nDispatcher, Foxwell Enforcement\n'Security, Your Way'\n\nFoxwell Enforcement is a bonded security specialist licensed to operate throughout the UEE. We are always looking for new operators to join our family. If you or anyone you know is interested, please reach out to one of our contract representatives.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 300\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: nyx, Nyx III, Nyx System&lt;/EM4&gt;\n- Frost-Star SL (Cooler)\n- Fridan (Cooler)\n- Tepilo (Cooler)\n- Frost-Star (Cooler)\n- ArcticStorm (Cooler)\n- Berian (Cooler)\n- Gelid (Cooler)\n- Frost-Star EX (Cooler)\n- ColdSnap (Cooler)\n- Aufeis (Cooler)\n- Graupel (Cooler)\n- Frost-Star XL (Cooler)\n- FrostBurn (Cooler)\n- Draug (Cooler)\n- Elsen (Cooler)\n- Kragen (Cooler)\n\n&lt;EM4&gt;[Regional Variants] example locations: Nyx II, Nyx System, Nyx I&lt;/EM4&gt;\n- CF-117 Bulldog Repeater\n- CF-227 Badger Repeater\n- CF-337 Panther Repeater\n- CF-447 Rhino Repeater\n- CF-557 Galdereen Repeater\n- CF-667 Mammoth Repeater\n- V60-26 (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-KILO, RAB-IGNITION, RAB-TUNG&lt;/EM4&gt;\n- IonWave (Powerplant)\n- Radix (Powerplant)\n- IonBurst (Powerplant)\n- PowerBolt (Powerplant)\n- LightBlossom (Powerplant)\n- MagnaBloom (Powerplant)\n- FullForce (Powerplant)\n- IonSurge (Powerplant)\n- DayBreak (Powerplant)\n- Radiance (Powerplant)\n- FullForce Pro (Powerplant)\n- IonSurge Pro (Powerplant)\n- Celestial (Powerplant)\n- NewDawn (Powerplant)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-TUNG, Checkmate, RAB-BRAVO&lt;/EM4&gt;\n- Glacier (Cooler)\n- Avalanche (Cooler)\n- Blizzard (Cooler)\n- DR Model-XJ1 Repeater\n- DR Model-XJ2 Repeater\n- DR Model-XJ3 Repeater\n\n&lt;EM4&gt;[Regional Variants] example locations: Ita, Arial, Aberdeen&lt;/EM4&gt;\n- 7SA (Shield)\n- INK (Shield)\n- 7MA 'Lorica' (Shield)\n- RPEL (Shield)\n- 7CA 'Nargun' (Shield)\n- HAVEN (Shield)\n\n&lt;EM4&gt;[Regional Variants] example locations: Ita, Aberdeen, Hurston&lt;/EM4&gt;\n- Attrition-4 Repeater\n- Attrition-5 Repeater\n- Attrition-6 Repeater\n- FR-86 (Shield)\n- Sens (Radar)\n- Tige (Radar)\n</v>
+        <v>Acaba de llegar una señal de socorro de emergencia de un equipo de mantenimiento empleado por uno de los clientes VIP de Foxwell. Si está disponible, le instamos a que llegue a &lt;EM4&gt;{0} lo antes posible. Mientras se enfrenta a los atacantes, se espera que proteja el &lt;EM4&gt;{1} del cliente y sus naves que puedan necesitar asistencia&lt;/EM4&gt;. \n\nEsta no es la primera vez que vemos a estos forajidos en particular, así que créame cuando le digo que no hay que subestimar a estos pilotos. Le recomiendo encarecidamente que organice una &lt;EM&gt;fuerza de apoyo altamente competente&lt;/EM&gt; para que vuele con usted al sitio.\n\nSi logra defender con éxito los intereses del cliente, ofrecemos &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt; como compensación al contratista principal lo suficientemente valiente como para aceptar este trabajo. \n\nManténgase a salvo y buena suerte,\n\nKevin Walton\nOperador, Foxwell Enforcement\n'Seguridad, a su manera'\n\nFoxwell Enforcement es una empresa de seguridad especializada, con licencia para operar en toda la UEE. Siempre estamos buscando nuevos operadores para unirse a nuestra familia. Si usted o alguien que conoce está interesado, comuníquese con uno de nuestros representantes de contratos.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 300\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: nyx, Nyx III, Nyx System&lt;/EM4&gt;\n- Frost-Star SL (Cooler)\n- Fridan (Cooler)\n- Tepilo (Cooler)\n- Frost-Star (Cooler)\n- ArcticStorm (Cooler)\n- Berian (Cooler)\n- Gelid (Cooler)\n- Frost-Star EX (Cooler)\n- ColdSnap (Cooler)\n- Aufeis (Cooler)\n- Graupel (Cooler)\n- Frost-Star XL (Cooler)\n- FrostBurn (Cooler)\n- Draug (Cooler)\n- Elsen (Cooler)\n- Kragen (Cooler)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx II, Nyx System, Nyx I&lt;/EM4&gt;\n- Repetidor Bulldog CF-117\n- Repetidor Badger CF-227\n- Repetidor Panther CF-337\n- Repetidor Rhino CF-447\n- Repetidor Galdereen CF-557\n- Repetidor Mammoth CF-667\n- V60-26 (Radar)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-KILO, RAB-IGNITION, RAB-TUNG&lt;/EM4&gt;\n- Onda iónica (Planta de energía)\n- Radix (Planta de energía)\n- IonBurst (Planta de energía)\n- PowerBolt (Planta de energía)\n- LightBlossom (Planta de energía)\n- MagnaBloom (Planta de energía)\n- FullForce (Planta de energía)\n- IonSurge (Planta de energía)\n- DayBreak (Planta de energía)\n- Radiance (Planta de energía)\n- FullForce Pro (Planta de energía)\n- IonSurge Pro (Planta de energía)\n- Celestial (Planta de energía)\n- NewDawn (Planta de energía)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-TUNG, Checkmate, RAB-BRAVO&lt;/EM4&gt;\n- Glacier (Enfriador)\n- Avalanche (Enfriador)\n- Blizzard (Enfriador)\n- DR Model-XJ1 Repeater\n- DR Model-XJ2 Repeater\n- DR Model-XJ3 Repeater\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Ita, Arial, Aberdeen&lt;/EM4&gt;\n- 7SA (Escudo)\n- INK (Escudo)\n- 7MA 'Lorica' (Escudo)\n- RPEL (Escudo)\n- 7CA 'Nargun' (Escudo)\n- HAVEN (Escudo)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Ita, Aberdeen, Hurston&lt;/EM4&gt;\n- Repetidor Attrition-4\n- Repetidor Attrition-5\n- Repetidor Attrition-6\n- FR-86 (Escudo)\n- Sens (Radar)\n- Tige (Radar)\n</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>For any pilots in the area – a group of bandits is targeting one of our clients at &lt;EM4&gt;{0} specifically their &lt;EM4&gt;{1} and the maintenance ships that manage them. From our intel, it's only a few outlaws trying to make some quick credits, but they're also the type to cause some real damage if you get in their way.\n\nIf you take care of them and relocate the client's ship and crew safely, we’re offering &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt; to the main contractor. \n\nGood luck,\n\nKevin Walton\nDispatcher, Foxwell Enforcement\n'Security, Your Way'\n\nFoxwell Enforcement is a bonded security specialist licensed to operate throughout the UEE. We are always looking for new operators to join our family. If you or anyone you know is interested, please reach out to one of our contract representatives.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 100\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Nyx System, Nyx I, nyx&lt;/EM4&gt;\n- Frost-Star SL (Cooler)\n- Fridan (Cooler)\n- Tepilo (Cooler)\n- Frost-Star (Cooler)\n- ArcticStorm (Cooler)\n- Berian (Cooler)\n- Gelid (Cooler)\n- Frost-Star EX (Cooler)\n- ColdSnap (Cooler)\n- Aufeis (Cooler)\n- Graupel (Cooler)\n- Frost-Star XL (Cooler)\n- FrostBurn (Cooler)\n- Draug (Cooler)\n- Elsen (Cooler)\n- Kragen (Cooler)\n\n&lt;EM4&gt;[Regional Variants] example locations: Monox, Checkmate, Checkmate Clinic&lt;/EM4&gt;\n- IonWave (Powerplant)\n- Radix (Powerplant)\n- IonBurst (Powerplant)\n- PowerBolt (Powerplant)\n- LightBlossom (Powerplant)\n- MagnaBloom (Powerplant)\n- FullForce (Powerplant)\n- IonSurge (Powerplant)\n- DayBreak (Powerplant)\n- Radiance (Powerplant)\n- FullForce Pro (Powerplant)\n- IonSurge Pro (Powerplant)\n- Celestial (Powerplant)\n- NewDawn (Powerplant)\n\n&lt;EM4&gt;[Regional Variants] example locations: Aberdeen, Arial, Ita&lt;/EM4&gt;\n- 7SA (Shield)\n- INK (Shield)\n- 7MA 'Lorica' (Shield)\n- RPEL (Shield)\n- 7CA 'Nargun' (Shield)\n- HAVEN (Shield)\n</v>
+        <v>Para cualquier piloto en la zona: un grupo de bandidos está atacando a uno de nuestros clientes en &lt;EM4&gt;{0} específicamente su &lt;EM4&gt;{1} y las naves de mantenimiento que las gestionan. Según nuestra información, se trata solo de unos pocos forajidos que intentan ganar unos créditos rápidos, pero también son del tipo que pueden causar daños reales si te interpones en su camino.\n\nSi te encargas de ellos y reubicas la nave y la tripulación del cliente de forma segura, ofrecemos &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt; al contratista principal. \n\nBuena suerte,\n\nKevin Walton\nDespachador, Foxwell Enforcement\n'Seguridad, a tu manera'\n\nFoxwell Enforcement es un especialista en seguridad con fianza y licencia para operar en toda la UEE. Siempre estamos buscando nuevos operadores para unirse a nuestra familia. Si usted o alguien que conoce está interesado, comuníquese con uno de nuestros representantes de contratos.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 100\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx System, Nyx I, nyx&lt;/EM4&gt;\n- Frost-Star SL (enfriador)\n- Fridan (enfriador)\n- Tepilo (enfriador)\n- Frost-Star (enfriador)\n- ArcticStorm (enfriador)\n- Berian (enfriador)\n- Gelid (enfriador)\n- Frost-Star EX (enfriador)\n- ColdSnap (enfriador)\n- Aufeis (enfriador)\n- Graupel (enfriador)\n- Frost-Star XL (enfriador)\n- FrostBurn (enfriador)\n- Draug (enfriador)\n- Elsen (Cooler)\n- Kragen (Cooler)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Monox, Checkmate, Checkmate Clinic&lt;/EM4&gt;\n- IonWave (Planta de energía)\n- Radix (Planta de energía)\n- IonBurst (Planta de energía)\n- PowerBolt (Planta de energía)\n- LightBlossom (Planta de energía)\n- MagnaBloom (Planta de energía)\n- FullForce (Planta de energía)\n- IonSurge (Planta de energía)\n- DayBreak (Planta de energía)\n- Radiance (Planta de energía)\n- FullForce Pro (Planta de energía)\n- IonSurge Pro (Planta de energía)\n- Celestial (Planta de energía)\n- NewDawn (Planta de energía)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Aberdeen, Arial, Ita&lt;/EM4&gt;\n- 7SA (Escudo)\n- INK (Escudo)\n- 7MA 'Lorica' (Escudo)\n- RPEL (Escudo)\n- 7CA 'Nargun' (Escudo)\n- HAVEN (Escudo)\n</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Urgent ship aid needed at &lt;EM4&gt;{0} A band of destructive criminal outlaws that have been trying to make a name for themselves recently has struck hard against one of our high priority clients, &lt;EM4&gt;attacking their ships and targeting the client's {1} It will be your job to keep everyone and everything safe – though it won't be an easy feat.\n\nI cannot stress enough how dangerous these attackers are, so be sure to &lt;EM&gt;bring backup&lt;/EM&gt; to deal with them. If you, the crew, and the infrastructures make it out intact, we’re offering a generous sum of &lt;EM4&gt;{2}  MG Scrip&lt;/EM4&gt; to the main contractor. \n\nBest of luck,\n\nKevin Walton\nDispatcher, Foxwell Enforcement\n'Security, Your Way'\n\nFoxwell Enforcement is a bonded security specialist licensed to operate throughout the UEE. We are always looking for new operators to join our family. If you or anyone you know is interested, please reach out to one of our contract representatives.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 250\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Nyx II, Nyx I, Nyx&lt;/EM4&gt;\n- Frost-Star SL (Cooler)\n- Fridan (Cooler)\n- Tepilo (Cooler)\n- Frost-Star (Cooler)\n- ArcticStorm (Cooler)\n- Berian (Cooler)\n- Gelid (Cooler)\n- Frost-Star EX (Cooler)\n- ColdSnap (Cooler)\n- Aufeis (Cooler)\n- Graupel (Cooler)\n- Frost-Star XL (Cooler)\n- FrostBurn (Cooler)\n- Draug (Cooler)\n- Elsen (Cooler)\n- Kragen (Cooler)\n\n&lt;EM4&gt;[Regional Variants] example locations: Nyx I, Nyx II, nyx&lt;/EM4&gt;\n- CF-117 Bulldog Repeater\n- CF-227 Badger Repeater\n- CF-337 Panther Repeater\n- CF-447 Rhino Repeater\n- CF-557 Galdereen Repeater\n- CF-667 Mammoth Repeater\n- V60-26 (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-FOXTROT, Monox, Patch City&lt;/EM4&gt;\n- IonWave (Powerplant)\n- Radix (Powerplant)\n- IonBurst (Powerplant)\n- PowerBolt (Powerplant)\n- LightBlossom (Powerplant)\n- MagnaBloom (Powerplant)\n- FullForce (Powerplant)\n- IonSurge (Powerplant)\n- DayBreak (Powerplant)\n- Radiance (Powerplant)\n- FullForce Pro (Powerplant)\n- IonSurge Pro (Powerplant)\n- Celestial (Powerplant)\n- NewDawn (Powerplant)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-TUNG, RAB-FOXTROT, Checkmate Clinic&lt;/EM4&gt;\n- Glacier (Cooler)\n- Avalanche (Cooler)\n- Blizzard (Cooler)\n- DR Model-XJ1 Repeater\n- DR Model-XJ2 Repeater\n- DR Model-XJ3 Repeater\n\n&lt;EM4&gt;[Regional Variants] example locations: Aberdeen, Ita, Arial&lt;/EM4&gt;\n- 7SA (Shield)\n- INK (Shield)\n- 7MA 'Lorica' (Shield)\n- RPEL (Shield)\n- 7CA 'Nargun' (Shield)\n- HAVEN (Shield)\n\n&lt;EM4&gt;[Regional Variants] example locations: Aberdeen, Arial, Hurston&lt;/EM4&gt;\n- Attrition-4 Repeater\n- Attrition-5 Repeater\n- Attrition-6 Repeater\n- FR-86 (Shield)\n- Sens (Radar)\n- Tige (Radar)\n</v>
+        <v>Se necesita ayuda urgente para el barco en &lt;EM4&gt;{0} Una banda de destructivos forajidos criminales que han estado tratando de hacerse un nombre recientemente ha atacado duramente a uno de nuestros clientes de alta prioridad, &lt;EM4&gt;atacando sus barcos y apuntando al cliente {1} Será tu trabajo mantener a todos y todo a salvo, aunque no será una hazaña fácil.\n\nNo puedo enfatizar lo suficiente lo peligrosos que son estos atacantes, así que asegúrate de &lt;EM&gt;traer refuerzos&lt;/EM&gt; para lidiar con ellos. Si tú, la tripulación y las infraestructuras salen intactos, estamos ofreciendo una generosa suma de &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt; al contratista principal. \n\nBuena suerte,\n\nKevin Walton\nDespachador, Foxwell Enforcement\n'Seguridad, a tu manera'\n\nFoxwell Enforcement es un especialista en seguridad afianzado con licencia para operar en toda la UEE. Siempre estamos buscando nuevos operadores para unirse a nuestra familia. Si usted o alguien que conoce está interesado, comuníquese con uno de nuestros representantes de contratos.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 250\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx II, Nyx I, Nyx&lt;/EM4&gt;\n- Frost-Star SL (más frío)\n- Fridan (más frío)\n- Tepilo (más frío)\n- Frost-Star (más frío)\n- ArcticStorm (más frío)\n- Berian (más frío)\n- Gelid (más frío)\n- Frost-Star EX (más frío)\n- ColdSnap (más frío)\n- Aufeis (más frío)\n- Graupel (más frío)\n- Frost-Star XL (más frío)\n- FrostBurn (más frío)\n- Draug (más frío)\n- Elsen (Cooler)\n- Kragen (Cooler)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx I, Nyx II, nyx&lt;/EM4&gt;\n- Repetidor Bulldog CF-117\n- Repetidor Tejón CF-227\n- Repetidor Pantera CF-337\n- Repetidor Rinoceronte CF-447\n- Repetidor Galdereen CF-557\n- Repetidor Mamut CF-667\n- V60-26 (Radar)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-FOXTROT, Monox, Patch City&lt;/EM4&gt;\n- Onda iónica (Planta de energía)\n- Radix (Planta de energía)\n- Explosión iónica (Planta de energía)\n- Rayo de energía (Planta de energía)\n- Flor de luz (Planta de energía)\n- MagnaFlor (Planta de energía)\n- Fuerza total (Planta de energía)\n- IonSurge (Planta de energía)\n- DayBreak (Planta de energía)\n- Radiance (Planta de energía)\n- FullForce Pro (Planta de energía)\n- IonSurge Pro (Planta de energía)\n- Celestial (Planta de energía)\n- NewDawn (Planta de energía)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-TUNG, RAB-FOXTROT, Checkmate Clinic&lt;/EM4&gt;\n- Glacier (Enfriador)\n- Avalanche (Enfriador)\n- Blizzard (Enfriador)\n- DR Model-XJ1 Repeater\n- DR Model-XJ2 Repeater\n- DR Model-XJ3 Repeater\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Aberdeen, Ita, Arial&lt;/EM4&gt;\n- 7SA (Escudo)\n- INK (Escudo)\n- 7MA 'Lorica' (Escudo)\n- RPEL (Escudo)\n- 7CA 'Nargun' (Escudo)\n- HAVEN (Escudo)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Aberdeen, Arial, Hurston&lt;/EM4&gt;\n- Repetidor Attrition-4\n- Repetidor Attrition-5\n- Repetidor Attrition-6\n- FR-86 (Escudo)\n- Sens (Radar)\n- Tige (Radar)\n</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Looking for a consummate professional to handle a high-stakes job. We’ve got VIP clients at &lt;EM4&gt;{0} who are facing extremely aggressive and motivated outlaws targeting ships around their location. Exact details on the attack are still rolling in, but it appears to be a wide ranging, multi-pronged operation. \n\nIf you’re available, I highly recommend that you bring additional combat support ships, plenty of supplies, and your A-game. Get this right, and we’ll reward the main contractor with a bonus payment of &lt;EM4&gt;{1} MG Scrip&lt;/EM4&gt;.\n\nGood luck,\n\nKevin Walton\nDispatcher, Foxwell Enforcement\n'Security, Your Way'\n\nFoxwell Enforcement is a bonded security specialist licensed to operate throughout the UEE. We are always looking for new operators to join our family. If you or anyone you know is interested, please reach out to one of our contract representatives.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 300 / 16,000\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Parallax "Shock Trooper" Energy Assault Rifle\n- Antium Arms Storm\n- Antium Core Storm\n- Antium Legs Storm\n- Antium Helmet Storm\n- Parallax Rifle Battery (80 Cap)\n</v>
+        <v>Buscamos un profesional consumado para manejar un trabajo de alto riesgo. Tenemos clientes VIP en &lt;EM4&gt;{0} que se enfrentan a forajidos extremadamente agresivos y motivados que atacan naves alrededor de su ubicación. Los detalles exactos del ataque aún están llegando, pero parece ser una operación amplia y multifacética. \n\nSi está disponible, le recomiendo encarecidamente que traiga naves de apoyo de combate adicionales, muchos suministros y su mejor desempeño. Si lo hace bien, recompensaremos al contratista principal con un pago adicional de &lt;EM4&gt;{1} MG Scrip&lt;/EM4&gt;.\n\nBuena suerte,\n\nKevin Walton\nDespachador, Foxwell Enforcement\n'Seguridad, a su manera'\n\nFoxwell Enforcement es un especialista en seguridad con fianza y licencia para operar en toda la UEE. Siempre estamos buscando nuevos operadores para unirse a nuestra familia. Si usted o alguien que conoce está interesado, póngase en contacto con uno de nuestros representantes contractuales.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 300 / 16.000\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Fusil de asalto de energía Parallax "Shock Trooper"\n- Tormenta de brazos Antium\n- Tormenta de núcleo Antium\n- Tormenta de piernas Antium\n- Tormenta de casco Antium\n- Batería de rifle Parallax (capacidad 80)\n</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Foxwell has been tracking a &lt;EM4&gt;{0} used by outlaws and discovered a pattern to its movements. The ship should be passing by &lt;EM4&gt;{1} soon.\n\nLooking for a contractor willing to hustle there, hide in the emission cloud, and then spring the trap when the time is right. There’s usually escort ships with the &lt;EM4&gt;{2} Careful not to jump the gun and blow your cover. The element of surprise is crucial from what I’ve read.\n\nPull this off and we'll give the main contractor a bonus payment of &lt;EM4&gt;{3} MG Scrip&lt;/EM4&gt;.\n\nGood luck,\n\nKevin Walton\nDispatcher, Foxwell Enforcement\n'Security, Your Way'\n\nFoxwell Enforcement is a bonded security specialist licensed to operate throughout the UEE. We are always looking for new operators to join our family. If you or anyone you know is interested, please reach out to one of our contract representatives.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 150 / 2,000\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Parallax "Sunstone" Energy Assault Rifle\n- Antium Arms Jet\n- Antium Core Jet\n- Antium Legs Jet\n- Parallax Rifle Battery (80 Cap)\n</v>
+        <v>Foxwell ha estado rastreando un &lt;EM4&gt;{0} utilizado por forajidos y ha descubierto un patrón en sus movimientos. El barco debería pasar pronto por &lt;EM4&gt;{1}.\n\nBuscamos un contratista dispuesto a ir rápidamente allí, esconderse en la nube de emisión y luego activar la trampa cuando sea el momento adecuado. Normalmente hay barcos de escolta con el &lt;EM4&gt;{2}. Tenga cuidado de no precipitarse y revelar su identidad. El elemento sorpresa es crucial por lo que he leído.\n\nSi lo logra, le daremos al contratista principal un pago de bonificación de &lt;EM4&gt;{3} MG Scrip&lt;/EM4&gt;.\n\nBuena suerte,\n\nKevin Walton\nDespachador, Foxwell Enforcement\n'Seguridad, a su manera'\n\nFoxwell Enforcement es un especialista en seguridad con fianza y licencia para operar en toda la UEE. Siempre estamos buscando nuevos operadores para unirse a nuestra familia. Si usted o alguien que conoce está interesado, comuníquese con uno de nuestros representantes de contratos.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 150 / 2000\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Fusil de asalto de energía Parallax "Sunstone"\n- Jet de brazos Antium\n- Jet de núcleo Antium\n- Jet de piernas Antium\n- Batería de rifle Parallax (capacidad de 80)\n</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Care to help us ghost a bad guy? \n\nWe’ve been hired to hunt down an outlaw flying a &lt;EM4&gt;{0} Shouldn’t be too hard since they take the same flightpath each day. That makes them a prime target for an ambush if I ever saw one. I’ve analyzed the route and determined that &lt;EM4&gt;{1} is the ideal spot to strike. There’s an emission cloud there that’ll be perfect to hide your ship’s signature while you wait.   \n\nJob is simple if you’re interested. Head to the location, hide out, power down, and then wait for them to fly by. Sometimes they roll alone but they often have other single-seat ships with them. Shouldn’t be too hard to handle for a pro. Plus, we’ll still have reinforcements nearby and ready to deploy once it pops off.\n\nPull this off and we'll give the main contractor a bonus payment of &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt;.\n\nGood luck,\n\n\nKevin Walton\nDispatcher, Foxwell Enforcement\n'Security, Your Way'\n\nFoxwell Enforcement is a bonded security specialist licensed to operate throughout the UEE. We are always looking for new operators to join our family. If you or anyone you know is interested, please reach out to one of our contract representatives.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 500\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Parallax "Sunstone" Energy Assault Rifle\n- Antium Arms Jet\n- Antium Core Jet\n- Antium Legs Jet\n- Parallax Rifle Battery (80 Cap)\n</v>
+        <v>¿Te gustaría ayudarnos a eliminar a un tipo malo? \n\nNos han contratado para dar caza a un forajido que vuela una &lt;EM4&gt;{0}. No debería ser muy difícil, ya que toman la misma ruta de vuelo todos los días. Eso los convierte en un objetivo perfecto para una emboscada, si es que alguna vez vi una. He analizado la ruta y he determinado que &lt;EM4&gt;{1} es el lugar ideal para atacar. Hay una nube de emisión allí que será perfecta para ocultar la firma de tu nave mientras esperas. \n\nEl trabajo es simple si te interesa. Dirígete a la ubicación, escóndete, apaga la energía y luego espera a que pasen volando. A veces vuelan solos, pero a menudo tienen otras naves monoplaza con ellos. No debería ser demasiado difícil de manejar para un profesional. Además, seguiremos teniendo refuerzos cerca y listos para desplegarse una vez que comience.\n\nSi lo logramos, le daremos al contratista principal un pago de bonificación de &lt;EM4&gt;{2} MG Scrip&lt;/EM4&gt;.\n\nBuena suerte,\n\n\nKevin Walton\nDespachador, Foxwell Enforcement\n'Seguridad, a tu manera'\n\nFoxwell Enforcement es un especialista en seguridad con fianza y licencia para operar en todo el UEE. Siempre estamos buscando nuevos operadores para unirse a nuestra familia. Si usted o alguien que conoce está interesado, póngase en contacto con uno de nuestros representantes contractuales.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 500\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Fusil de asalto de energía Parallax "Sunstone"\n- Jet de brazos Antium\n- Jet de núcleo Antium\n- Jet de piernas Antium\n- Batería de rifle Parallax (capacidad de 80)\n</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>I was having a shite day, and it just got worse. Our interests over at &lt;EM4&gt;{0} comm'd to let me know that their  &lt;EM&gt;{1} are under attack by these no-name hoods looking to stake a claim.\n\nYou're gonna go there for me and protect the place, including any &lt;EM4&gt;friendly ships&lt;/EM4&gt; unfortunate enough to be caught in the crossfire. Don't think putting these wannabees in their place will be too tricky for someone like you. \n\nAlso, I’ll sweeten the pot by giving the main contractor &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; just to show my appreciation. \n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 100\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Nyx System, Nyx I, nyx&lt;/EM4&gt;\n- Cryo-Star SL (Cooler)\n- Winter-Star SL (Cooler)\n- Kelvid (Cooler)\n- Cryo-Star (Cooler)\n- Winter-Star (Cooler)\n- BlastChill (Cooler)\n- FlashFreeze (Cooler)\n- Endo (Cooler)\n- Cryo-Star EX (Cooler)\n- Winter-Star EX (Cooler)\n- FullFrost (Cooler)\n- WhiteOut (Cooler)\n- Taiga (Cooler)\n- Cryo-Star XL (Cooler)\n- Winter-Star XL (Cooler)\n- ColdSurge (Cooler)\n- FrostBite (Cooler)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-TUNG, Patch City, RAB-ALPHA&lt;/EM4&gt;\n- DuraJet (Powerplant)\n- ZapJet (Powerplant)\n- WhiteRose (Powerplant)\n- SparkJet (Powerplant)\n- Lotus (Powerplant)\n- SparkJet Pro (Powerplant)\n- TigerLilly (Powerplant)\n\n&lt;EM4&gt;[Regional Variants] example locations: Ita, Arial, Magda&lt;/EM4&gt;\n- PIN (Shield)\n- 5SA 'Rhada' (Shield)\n- 6SA (Shield)\n- HEX (Shield)\n- WEB (Shield)\n- 5MA 'Chimalli' (Shield)\n- 6MA 'Kozane' (Shield)\n- BLOC (Shield)\n- STOP (Shield)\n- 5CA 'Akura' (Shield)\n- 6CA 'Bila' (Shield)\n- ARMOR (Shield)\n- GUARD (Shield)\n</v>
+        <v>Estaba teniendo un día de mierda, y solo empeoró. Nuestros intereses en &lt;EM4&gt;{0} me comunicaron que su &lt;EM&gt;{1} está siendo atacado por estos matones sin nombre que buscan reclamar territorio.\n\nVas a ir allí por mí y proteger el lugar, incluyendo cualquier &lt;EM4&gt;nave amiga&lt;/EM4&gt; que tenga la mala suerte de quedar atrapada en el fuego cruzado. No creo que poner a estos aspirantes a serlo sea demasiado difícil para alguien como tú.\n\nAdemás, endulzaré la oferta dándole al contratista principal &lt;EM4&gt;{2} Certificado del Consejo&lt;/EM4&gt; solo para mostrar mi agradecimiento. \n\nSe guarda.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 100\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx System, Nyx I, nyx&lt;/EM4&gt;\n- Cryo-Star SL (enfriador)\n- Winter-Star SL (enfriador)\n- Kelvid (enfriador)\n- Cryo-Star (enfriador)\n- Winter-Star (enfriador)\n- BlastChill (enfriador)\n- FlashFreeze (enfriador)\n- Endo (enfriador)\n- Cryo-Star EX (enfriador)\n- Winter-Star EX (enfriador)\n- FullFrost (enfriador)\n- WhiteOut (enfriador)\n- Taiga (enfriador)\n- Cryo-Star XL (enfriador)\n- Winter-Star XL (Cooler)\n- ColdSurge (Cooler)\n- FrostBite (Cooler)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-TUNG, Patch City, RAB-ALPHA&lt;/EM4&gt;\n- DuraJet (Planta de energía)\n- ZapJet (Planta de energía)\n- WhiteRose (Planta de energía)\n- SparkJet (Planta de energía)\n- Lotus (Planta de energía)\n- SparkJet Pro (Planta de energía)\n- TigerLilly (Planta de energía)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Ita, Arial, Magda&lt;/EM4&gt;\n- PIN (Escudo)\n- 5SA 'Rhada' (Escudo)\n- 6SA (Escudo)\n- HEX (Escudo)\n- WEB (Escudo)\n- 5MA 'Chimalli' (Escudo)\n- 6MA 'Kozane' (Escudo)\n- BLOQUE (Escudo)\n- STOP (Escudo)\n- 5CA 'Akura' (Escudo)\n- 6CA 'Bila' (Escudo)\n- ARMADURA (Escudo)\n- GUARDIA (Escudo)\n</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>There's this small gang that continues to be a thorn in our side, and the bastards have just ambushed some friends over at &lt;EM4&gt;{0} Seems like they're doing their best to destroy the &lt;EM4&gt;{1} there.\n\nI need you and whatever &lt;EM4&gt;crew you can muster&lt;/EM4&gt; on site stopping these mungers from blowing everything up and protecting any &lt;EM4&gt;friendly ships&lt;/EM4&gt; that need a hand.\n\nHandle this right and I’ll give the main contractor  &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt;.\n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 200\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Nyx System, nyx, Nyx III&lt;/EM4&gt;\n- Cryo-Star SL (Cooler)\n- Winter-Star SL (Cooler)\n- Kelvid (Cooler)\n- Cryo-Star (Cooler)\n- Winter-Star (Cooler)\n- BlastChill (Cooler)\n- FlashFreeze (Cooler)\n- Endo (Cooler)\n- Cryo-Star EX (Cooler)\n- Winter-Star EX (Cooler)\n- FullFrost (Cooler)\n- WhiteOut (Cooler)\n- Taiga (Cooler)\n- Cryo-Star XL (Cooler)\n- Winter-Star XL (Cooler)\n- ColdSurge (Cooler)\n- FrostBite (Cooler)\n\n&lt;EM4&gt;[Regional Variants] example locations: Nyx III, nyx, Nyx&lt;/EM4&gt;\n- Tarantula GT-870 Mark 1 Cannon\n- Tarantula GT-870 Mark 2 Cannon\n- Tarantula GT-870 Mark 3 Cannon\n- YellowJacket GT-210 Gatling\n- Scorpion GT-215 Gatling\n- Mantis GT-220 Gatling\n- V880 (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-ROTH, Checkmate Clinic, RAB-NOVEMBER&lt;/EM4&gt;\n- DuraJet (Powerplant)\n- ZapJet (Powerplant)\n- WhiteRose (Powerplant)\n- SparkJet (Powerplant)\n- Lotus (Powerplant)\n- SparkJet Pro (Powerplant)\n- TigerLilly (Powerplant)\n\n&lt;EM4&gt;[Regional Variants] example locations: Patch City Clinic, Pyro I, Patch City&lt;/EM4&gt;\n- AD4B Ballistic Gatling\n- AD5B Ballistic Gatling\n- AD6B Ballistic Gatling\n- V801-11 (Radar)\n- V801-12 (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: Hurston, Aberdeen, Magda&lt;/EM4&gt;\n- PIN (Shield)\n- 5SA 'Rhada' (Shield)\n- 6SA (Shield)\n- HEX (Shield)\n- WEB (Shield)\n- 5MA 'Chimalli' (Shield)\n- 6MA 'Kozane' (Shield)\n- BLOC (Shield)\n- STOP (Shield)\n- 5CA 'Akura' (Shield)\n- 6CA 'Bila' (Shield)\n- ARMOR (Shield)\n- GUARD (Shield)\n\n&lt;EM4&gt;[Regional Variants] example locations: Hurston, Arial, Magda&lt;/EM4&gt;\n- SW16BR1 “Buzzsaw” Repeater\n- SW16BR2 “Sawbuck” Repeater\n- SW16BR3 “Shredder” Repeater\n- Vigilance (Radar)\n- Devoue (Radar)\n- Tige (Radar)\n</v>
+        <v>Hay una pequeña banda que sigue siendo una espina clavada en nuestro costado, y esos bastardos acaban de emboscar a unos amigos en &lt;EM4&gt;{0}. Parece que están haciendo todo lo posible por destruir el &lt;EM4&gt;{1} de allí.\n\nNecesito que tú y cualquier &lt;EM4&gt;tripulación que puedas reunir&lt;/EM4&gt; estén en el lugar para detener a estos desgraciados antes de que lo hagan volar todo por los aires y proteger cualquier &lt;EM4&gt;nave amiga&lt;/EM4&gt; que necesite ayuda.\n\nSi lo haces bien, le daré al contratista principal un &lt;EM4&gt;{2} Consejo&lt;/EM4&gt;.\n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 200\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Sistema Nyx, nyx, Nyx III&lt;/EM4&gt;\n- Cryo-Star SL (Cooler)\n- Winter-Star SL (Cooler)\n- Kelvid (Cooler)\n- Cryo-Star (Cooler)\n- Winter-Star (Cooler)\n- BlastChill (Cooler)\n- FlashFreeze (Cooler)\n- Endo (Cooler)\n- Cryo-Star EX (Cooler)\n- Winter-Star EX (Cooler)\n- FullFrost (Cooler)\n- WhiteOut (Cooler)\n- Taiga (Cooler)\n- Cryo-Star XL (Cooler)\n- Winter-Star XL (Cooler)\n- ColdSurge (Cooler)\n- FrostBite (Cooler)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx III, nyx, Nyx&lt;/EM4&gt;\n- Tarantula GT-870 Mark 1 Cannon\n- Tarantula GT-870 Mark 2 Cannon\n- Cañón Tarantula GT-870 Mark 3\n- Ametralladora Gatling YellowJacket GT-210\n- Ametralladora Gatling Scorpion GT-215\n- Ametralladora Gatling Mantis GT-220\n- V880 (Radar)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-ROTH, Clínica Checkmate, RAB-NOVIEMBRE&lt;/EM4&gt;\n- DuraJet (Planta de energía)\n- ZapJet (Planta de energía)\n- WhiteRose (Planta de energía)\n- SparkJet (Planta de energía)\n- Lotus (Planta de energía)\n- SparkJet Pro (Planta de energía)\n- TigerLilly (Planta de energía)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Clínica Patch City, Pyro I, Patch City&lt;/EM4&gt;\n- Ametralladora Gatling balística AD4B\n- Ametralladora Gatling balística AD5B\n- Ametralladora Gatling balística AD6B\n- V801-11 (Radar)\n- V801-12 (Radar)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Hurston, Aberdeen, Magda&lt;/EM4&gt;\n- PIN (Escudo)\n- 5SA 'Rhada' (Escudo)\n- 6SA (Escudo)\n- HEX (Escudo)\n- WEB (Escudo)\n- 5MA 'Chimalli' (Escudo)\n- 6MA 'Kozane' (Escudo)\n- BLOC (Escudo)\n- STOP (Escudo)\n- 5CA 'Akura' (Escudo)\n- 6CA 'Bila' (Escudo)\n- ARMOR (Escudo)\n- GUARD (Escudo)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Hurston, Arial, Magda&lt;/EM4&gt;\n- SW16BR1 “Buzzsaw” Repetidor\n- Repetidor SW16BR2 “Sawbuck”\n- Repetidor SW16BR3 “Shredder”\n- Vigilance (Radar)\n- Devoue (Radar)\n- Tige (Radar)\n</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>A new gang who is proving to be a real pain in the ass for the Headhunters just upped the stakes by attacking the &lt;EM4&gt;{0} at &lt;EM4&gt;{1} Never a good thing since we got interest in the welfare of the folks there, but doubly so because if they do too much damage it might royally screw an upcoming operation.\n\nHead over there as soon as you're able and stop the attack before they can do any lasting damage. And if any &lt;EM4&gt;friendly ships&lt;/EM4&gt; need a hand, I want you to look out for them too. Don't expect this gang to be pushovers but you should still be able to deal with them if you keep your head on.\n \nIf you need any extra motivation, I’m adding &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; for the main contractor.\n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 150 / 2,000\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Nyx I, Nyx, Nyx II&lt;/EM4&gt;\n- Cryo-Star SL (Cooler)\n- Winter-Star SL (Cooler)\n- Kelvid (Cooler)\n- Cryo-Star (Cooler)\n- Winter-Star (Cooler)\n- BlastChill (Cooler)\n- FlashFreeze (Cooler)\n- Endo (Cooler)\n- Cryo-Star EX (Cooler)\n- Winter-Star EX (Cooler)\n- FullFrost (Cooler)\n- WhiteOut (Cooler)\n- Taiga (Cooler)\n- Cryo-Star XL (Cooler)\n- Winter-Star XL (Cooler)\n- ColdSurge (Cooler)\n- FrostBite (Cooler)\n\n&lt;EM4&gt;[Regional Variants] example locations: Monox, RAB-FOXTROT, RAB-ALPHA&lt;/EM4&gt;\n- DuraJet (Powerplant)\n- ZapJet (Powerplant)\n- WhiteRose (Powerplant)\n- SparkJet (Powerplant)\n- Lotus (Powerplant)\n- SparkJet Pro (Powerplant)\n- TigerLilly (Powerplant)\n\n&lt;EM4&gt;[Regional Variants] example locations: Magda, Ita, Hurston&lt;/EM4&gt;\n- PIN (Shield)\n- 5SA 'Rhada' (Shield)\n- 6SA (Shield)\n- HEX (Shield)\n- WEB (Shield)\n- 5MA 'Chimalli' (Shield)\n- 6MA 'Kozane' (Shield)\n- BLOC (Shield)\n- STOP (Shield)\n- 5CA 'Akura' (Shield)\n- 6CA 'Bila' (Shield)\n- ARMOR (Shield)\n- GUARD (Shield)\n</v>
+        <v>Una nueva banda que está demostrando ser una verdadera molestia para los Headhunters acaba de subir la apuesta atacando el &lt;EM4&gt;{0} en &lt;EM4&gt;{1}. Nunca es buena señal, ya que nos interesa el bienestar de la gente de allí, pero más aún porque si causan demasiado daño, podría arruinar por completo una operación próxima.\n\nDirígete allí tan pronto como puedas y detén el ataque antes de que puedan causar daños permanentes. Y si alguna nave &lt;EM4&gt;amiga&lt;/EM4&gt; necesita ayuda, quiero que también estés pendiente de ella. No esperes que esta pandilla sea fácil de vencer, pero aún así deberías poder lidiar con ellos si mantienes la cabeza fría.\n \nSi necesitas motivación adicional, estoy agregando &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; para el contratista principal.\n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 150 / 2000\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx I, Nyx, Nyx II&lt;/EM4&gt;\n- Cryo-Star SL (Cooler)\n- Winter-Star SL (Cooler)\n- Kelvid (Cooler)\n- Cryo-Star (Cooler)\n- Winter-Star (Cooler)\n- BlastChill (Cooler)\n- FlashFreeze (Cooler)\n- Endo (Cooler)\n- Cryo-Star EX (Cooler)\n- Winter-Star EX (Cooler)\n- FullFrost (Cooler)\n- WhiteOut (Cooler)\n- Taiga (Cooler)\n- Cryo-Star XL (Cooler)\n- Winter-Star XL (Cooler)\n- ColdSurge (Cooler)\n- FrostBite (Cooler)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Monox, RAB-FOXTROT, RAB-ALPHA&lt;/EM4&gt;\n- DuraJet (Planta motriz)\n- ZapJet (Planta motriz)\n- WhiteRose (Planta motriz)\n- SparkJet (Planta motriz)\n- Lotus (Planta motriz)\n- SparkJet Pro (Planta motriz)\n- TigerLilly (Planta motriz)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Magda, Ita, Hurston&lt;/EM4&gt;\n- PIN (Escudo)\n- 5SA 'Rhada' (Escudo)\n- 6SA (Escudo)\n- HEX (Escudo)\n- WEB (Escudo)\n- 5MA 'Chimalli' (Escudo)\n- 6MA 'Kozane' (Escudo)\n- BLOC (Escudo)\n- STOP (Escudo)\n- 5CA 'Akura' (Escudo)\n- 6CA 'Bila' (Escudo)\n- ARMOR (Escudo)\n- GUARD (Escudo)\n</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>The maintenance and reliable function of &lt;EM4&gt;{0} is pretty darn important to the Headhunters, but this rival crew seems determined knock it out of contention. They're on site now, targeting &lt;EM4&gt;{1} there. \n\nProtecting the site, and any &lt;EM4&gt;friendly ships&lt;/EM4&gt;, in the area is important enough that I want you to bring some &lt;EM4&gt;reliable backup along&lt;/EM4&gt; when you go and terminate these nullbrains. \n\nTo prove just how serious we are about getting this done right, the main contractor will earn &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; for making sure absolutely nothing goes wrong.\n\n- Stow\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 300\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Nyx II, nyx, Nyx III&lt;/EM4&gt;\n- Cryo-Star SL (Cooler)\n- Winter-Star SL (Cooler)\n- Kelvid (Cooler)\n- Cryo-Star (Cooler)\n- Winter-Star (Cooler)\n- BlastChill (Cooler)\n- FlashFreeze (Cooler)\n- Endo (Cooler)\n- Cryo-Star EX (Cooler)\n- Winter-Star EX (Cooler)\n- FullFrost (Cooler)\n- WhiteOut (Cooler)\n- Taiga (Cooler)\n- Cryo-Star XL (Cooler)\n- Winter-Star XL (Cooler)\n- ColdSurge (Cooler)\n- FrostBite (Cooler)\n\n&lt;EM4&gt;[Regional Variants] example locations: Nyx III, Nyx, nyx&lt;/EM4&gt;\n- Tarantula GT-870 Mark 1 Cannon\n- Tarantula GT-870 Mark 2 Cannon\n- Tarantula GT-870 Mark 3 Cannon\n- YellowJacket GT-210 Gatling\n- Scorpion GT-215 Gatling\n- Mantis GT-220 Gatling\n- V880 (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-IGNITION, RAB-NOVEMBER, RAB-TUNG&lt;/EM4&gt;\n- DuraJet (Powerplant)\n- ZapJet (Powerplant)\n- WhiteRose (Powerplant)\n- SparkJet (Powerplant)\n- Lotus (Powerplant)\n- SparkJet Pro (Powerplant)\n- TigerLilly (Powerplant)\n\n&lt;EM4&gt;[Regional Variants] example locations: Monox, RAB-NOVEMBER, RAB-ROTH&lt;/EM4&gt;\n- AD4B Ballistic Gatling\n- AD5B Ballistic Gatling\n- AD6B Ballistic Gatling\n- V801-11 (Radar)\n- V801-12 (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: Hurston, Arial, Magda&lt;/EM4&gt;\n- PIN (Shield)\n- 5SA 'Rhada' (Shield)\n- 6SA (Shield)\n- HEX (Shield)\n- WEB (Shield)\n- 5MA 'Chimalli' (Shield)\n- 6MA 'Kozane' (Shield)\n- BLOC (Shield)\n- STOP (Shield)\n- 5CA 'Akura' (Shield)\n- 6CA 'Bila' (Shield)\n- ARMOR (Shield)\n- GUARD (Shield)\n\n&lt;EM4&gt;[Regional Variants] example locations: Hurston, Magda, Arial&lt;/EM4&gt;\n- SW16BR1 “Buzzsaw” Repeater\n- SW16BR2 “Sawbuck” Repeater\n- SW16BR3 “Shredder” Repeater\n- Vigilance (Radar)\n- Devoue (Radar)\n- Tige (Radar)\n</v>
+        <v>El mantenimiento y el funcionamiento fiable de &lt;EM4&gt;{0} es de suma importancia para los Headhunters, pero esta tripulación rival parece decidida a eliminarlo. Ya están en el lugar, apuntando a &lt;EM4&gt;{1}. \n\nProteger el sitio y cualquier &lt;EM4&gt;nave amiga&lt;/EM4&gt; en la zona es tan importante que quiero que traigas algún &lt;EM4&gt;refuerzo fiable&lt;/EM4&gt; cuando vayas a eliminar a estos cerebros nulos. \n\nPara demostrar lo serios que nos tomamos esto para que todo salga bien, el contratista principal ganará &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; por asegurarse de que absolutamente nada salga mal.\n\n- Stow\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 300\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx II, nyx, Nyx III&lt;/EM4&gt;\n- Cryo-Star SL (Cooler)\n- Winter-Star SL (Cooler)\n- Kelvid (Cooler)\n- Cryo-Star (Cooler)\n- Winter-Star (Cooler)\n- BlastChill (Cooler)\n- FlashFreeze (Cooler)\n- Endo (Cooler)\n- Cryo-Star EX (Cooler)\n- Winter-Star EX (Cooler)\n- FullFrost (Cooler)\n- WhiteOut (Cooler)\n- Taiga (Cooler)\n- Cryo-Star XL (Cooler)\n- Winter-Star XL (Cooler)\n- ColdSurge (Cooler)\n- FrostBite (Cooler)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx III, Nyx, nyx&lt;/EM4&gt;\n- Tarantula GT-870 Mark 1 Cannon\n- Tarantula GT-870 Mark 2 Cannon\n- Tarantula GT-870 Mark 3 Cannon\n- YellowJacket GT-210 Gatling\n- Scorpion GT-215 Gatling\n- Mantis GT-220 Gatling\n- V880 (Radar)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-IGNITION, RAB-NOVEMBER, RAB-TUNG&lt;/EM4&gt;\n- DuraJet (Planta motriz)\n- ZapJet (Planta motriz)\n- WhiteRose (Planta motriz)\n- SparkJet (Planta motriz)\n- Lotus (Planta motriz)\n- SparkJet Pro (Planta motriz)\n- TigerLilly (Planta motriz)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Monox, RAB-NOVIEMBRE, RAB-ROTH&lt;/EM4&gt;\n- AD4B Ballistic Gatling\n- AD5B Ballistic Gatling\n- AD6B Ballistic Gatling\n- V801-11 (Radar)\n- V801-12 (Radar)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Hurston, Arial, Magda&lt;/EM4&gt;\n- PIN (Escudo)\n- 5SA 'Rhada' (Escudo)\n- 6SA (Escudo)\n- HEX (Escudo)\n- WEB (Escudo)\n- 5MA 'Chimalli' (Escudo)\n- 6MA 'Kozane' (Escudo)\n- BLOC (Escudo)\n- STOP (Escudo)\n- 5CA 'Akura' (Escudo)\n- 6CA 'Bila' (Escudo)\n- ARMOR (Escudo)\n- GUARD (Escudo)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Hurston, Magda, Arial&lt;/EM4&gt;\n- SW16BR1 Repetidor “Buzzsaw”\n- SW16BR2 Repetidor “Sawbuck”\n- SW16BR3 Repetidor “Shredder”\n- Vigilance (Radar)\n- Devoue (Radar)\n- Tige (Radar)\n</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>I won't bore you with the nitty gritty, but trust me when I say that &lt;EM4&gt;{0} is important to the Headhunters. So imagine how pissed I am to learn that they're being harassed by some aggressive upstarts who are hellbent on taking out their &lt;EM&gt;{1} It won't stand.   \n\nGet there and provide some protection before everything gets destroyed, including &lt;EM4&gt;any friendly ships&lt;/EM4&gt; in the area. Nullbrains like these hopefully won't pose too much of a challenge to a rising star like yourself.\n\nClear ‘em all out I’ll throw &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; to whoever accepted this gig.\n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 100\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Nyx System, Nyx, nyx&lt;/EM4&gt;\n- Cryo-Star SL (Cooler)\n- Winter-Star SL (Cooler)\n- Kelvid (Cooler)\n- Cryo-Star (Cooler)\n- Winter-Star (Cooler)\n- BlastChill (Cooler)\n- FlashFreeze (Cooler)\n- Endo (Cooler)\n- Cryo-Star EX (Cooler)\n- Winter-Star EX (Cooler)\n- FullFrost (Cooler)\n- WhiteOut (Cooler)\n- Taiga (Cooler)\n- Cryo-Star XL (Cooler)\n- Winter-Star XL (Cooler)\n- ColdSurge (Cooler)\n- FrostBite (Cooler)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-ALPHA, Patch City, RAB-FOXTROT&lt;/EM4&gt;\n- DuraJet (Powerplant)\n- ZapJet (Powerplant)\n- WhiteRose (Powerplant)\n- SparkJet (Powerplant)\n- Lotus (Powerplant)\n- SparkJet Pro (Powerplant)\n- TigerLilly (Powerplant)\n\n&lt;EM4&gt;[Regional Variants] example locations: Aberdeen, Ita, Hurston&lt;/EM4&gt;\n- PIN (Shield)\n- 5SA 'Rhada' (Shield)\n- 6SA (Shield)\n- HEX (Shield)\n- WEB (Shield)\n- 5MA 'Chimalli' (Shield)\n- 6MA 'Kozane' (Shield)\n- BLOC (Shield)\n- STOP (Shield)\n- 5CA 'Akura' (Shield)\n- 6CA 'Bila' (Shield)\n- ARMOR (Shield)\n- GUARD (Shield)\n</v>
+        <v>No te aburriré con los detalles, pero créeme cuando te digo que &lt;EM4&gt;{0} es importante para los Headhunters. Así que imagina lo cabreado que estoy al enterarme de que están siendo acosados por unos advenedizos agresivos que están empeñados en acabar con su &lt;EM&gt;{1}. No lo permitiré. \n\nLlega allí y proporciona protección antes de que todo sea destruido, incluyendo &lt;EM4&gt;cualquier nave amiga&lt;/EM4&gt; en la zona. Esperemos que los cerebros nulos como estos no representen un gran desafío para una estrella en ascenso como tú.\n\nEliminadlos a todos. Daré &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; a quien haya aceptado este trabajo.\n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 100\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Sistema Nyx, Nyx, nyx&lt;/EM4&gt;\n- Cryo-Star SL (enfriador)\n- Winter-Star SL (enfriador)\n- Kelvid (enfriador)\n- Cryo-Star (enfriador)\n- Winter-Star (enfriador)\n- BlastChill (enfriador)\n- FlashFreeze (enfriador)\n- Endo (enfriador)\n- Cryo-Star EX (enfriador)\n- Winter-Star EX (Cooler)\n- FullFrost (Cooler)\n- WhiteOut (Cooler)\n- Taiga (Cooler)\n- Cryo-Star XL (Cooler)\n- Winter-Star XL (Cooler)\n- ColdSurge (Cooler)\n- FrostBite (Cooler)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-ALPHA, Patch City, RAB-FOXTROT&lt;/EM4&gt;\n- DuraJet (Planta de energía)\n- ZapJet (Planta de energía)\n- WhiteRose (Planta de energía)\n- SparkJet (Planta de energía)\n- Lotus (Planta de energía)\n- SparkJet Pro (Planta de energía)\n- TigerLilly (Planta de energía)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Aberdeen, Ita, Hurston&lt;/EM4&gt;\n- PIN (Escudo)\n- 5SA 'Rhada' (Escudo)\n- 6SA (Escudo)\n- HEX (Escudo)\n- WEB (Escudo)\n- 5MA 'Chimalli' (Escudo)\n- 6MA 'Kozane' (Escudo)\n- BLOC (Escudo)\n- STOP (Escudo)\n- 5CA 'Akura' (Escudo)\n- 6CA 'Bila' (Escudo)\n- ARMOR (Escudo)\n- GUARD (Escudo)\n</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>So, I thought we had done a good job of keeping things on the quiet side, but looks like the fact &lt;EM4&gt;{0} has Headhunters ties has gotten out. Now there are some heavy operators causing major problems there, targeting the &lt;EM&gt;{1} and generally causing me a massive headache.\n\nWith the amount of firepower these interlopers are packing, you're gonna need to bring along a &lt;EM4&gt;crew of your own&lt;/EM4&gt; to pull this off. Especially since I need you to be protecting any &lt;EM4&gt;friendly ships&lt;/EM4&gt; that need help.\n\nThis op needs to go off without a hitch, so I’m offering the main contractor &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; for a job well done. \n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 250\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Nyx I, Nyx, Nyx System&lt;/EM4&gt;\n- Cryo-Star SL (Cooler)\n- Winter-Star SL (Cooler)\n- Kelvid (Cooler)\n- Cryo-Star (Cooler)\n- Winter-Star (Cooler)\n- BlastChill (Cooler)\n- FlashFreeze (Cooler)\n- Endo (Cooler)\n- Cryo-Star EX (Cooler)\n- Winter-Star EX (Cooler)\n- FullFrost (Cooler)\n- WhiteOut (Cooler)\n- Taiga (Cooler)\n- Cryo-Star XL (Cooler)\n- Winter-Star XL (Cooler)\n- ColdSurge (Cooler)\n- FrostBite (Cooler)\n\n&lt;EM4&gt;[Regional Variants] example locations: Nyx System, nyx, Nyx III&lt;/EM4&gt;\n- Tarantula GT-870 Mark 1 Cannon\n- Tarantula GT-870 Mark 2 Cannon\n- Tarantula GT-870 Mark 3 Cannon\n- YellowJacket GT-210 Gatling\n- Scorpion GT-215 Gatling\n- Mantis GT-220 Gatling\n- V880 (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-KILO, Pyro I, RAB-BRAVO&lt;/EM4&gt;\n- DuraJet (Powerplant)\n- ZapJet (Powerplant)\n- WhiteRose (Powerplant)\n- SparkJet (Powerplant)\n- Lotus (Powerplant)\n- SparkJet Pro (Powerplant)\n- TigerLilly (Powerplant)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-TUNG, Cluster NBD-102, Checkmate Clinic&lt;/EM4&gt;\n- AD4B Ballistic Gatling\n- AD5B Ballistic Gatling\n- AD6B Ballistic Gatling\n- V801-11 (Radar)\n- V801-12 (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: Ita, Hurston, Arial&lt;/EM4&gt;\n- PIN (Shield)\n- 5SA 'Rhada' (Shield)\n- 6SA (Shield)\n- HEX (Shield)\n- WEB (Shield)\n- 5MA 'Chimalli' (Shield)\n- 6MA 'Kozane' (Shield)\n- BLOC (Shield)\n- STOP (Shield)\n- 5CA 'Akura' (Shield)\n- 6CA 'Bila' (Shield)\n- ARMOR (Shield)\n- GUARD (Shield)\n\n&lt;EM4&gt;[Regional Variants] example locations: Ita, Arial, Magda&lt;/EM4&gt;\n- SW16BR1 “Buzzsaw” Repeater\n- SW16BR2 “Sawbuck” Repeater\n- SW16BR3 “Shredder” Repeater\n- Vigilance (Radar)\n- Devoue (Radar)\n- Tige (Radar)\n</v>
+        <v>Así que pensé que habíamos hecho un buen trabajo manteniendo las cosas en secreto, pero parece que se ha filtrado el hecho de que &lt;EM4&gt;{0} tiene vínculos con los Cazadores de Cabezas. Ahora hay algunos operadores pesados causando grandes problemas allí, apuntando a &lt;EM&gt;{1} y en general causándome un gran dolor de cabeza.\n\nCon la cantidad de potencia de fuego que tienen estos intrusos, vas a necesitar traer una &lt;EM4&gt;tripulación propia&lt;/EM4&gt; para lograr esto. Especialmente porque necesito que protejas cualquier &lt;EM4&gt;nave amiga&lt;/EM4&gt; que necesite ayuda.\n\nEsta operación tiene que salir sin problemas, así que le ofrezco al contratista principal &lt;EM4&gt;{2} Consejo&lt;/EM4&gt; por un trabajo bien hecho. \n\nSe guarda.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 250\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx I, Nyx, Nyx System&lt;/EM4&gt;\n- Cryo-Star SL (enfriador)\n- Winter-Star SL (enfriador)\n- Kelvid (enfriador)\n- Cryo-Star (enfriador)\n- Winter-Star (enfriador)\n- BlastChill (enfriador)\n- FlashFreeze (enfriador)\n- Endo (enfriador)\n- Cryo-Star EX (enfriador)\n- Winter-Star EX (enfriador)\n- FullFrost (enfriador)\n- WhiteOut (enfriador)\n- Taiga (enfriador)\n- Cryo-Star XL (enfriador)\n- Winter-Star XL (Cooler)\n- ColdSurge (Cooler)\n- FrostBite (Cooler)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx System, nyx, Nyx III&lt;/EM4&gt;\n- Tarantula GT-870 Mark 1 Cannon\n- Tarantula GT-870 Mark 2 Cannon\n- Tarantula GT-870 Mark 3 Cannon\n- YellowJacket GT-210 Gatling\n- Scorpion GT-215 Gatling\n- Mantis GT-220 Gatling\n- V880 (Radar)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-KILO, Pyro I, RAB-BRAVO&lt;/EM4&gt;\n- DuraJet (Planta de energía)\n- ZapJet (Planta de energía)\n- WhiteRose (Planta de energía)\n- SparkJet (Planta de energía)\n- Lotus (Planta de energía)\n- SparkJet Pro (Planta motriz)\n- TigerLilly (Planta motriz)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-TUNG, Cluster NBD-102, Checkmate Clinic&lt;/EM4&gt;\n- AD4B Ballistic Gatling\n- AD5B Ballistic Gatling\n- AD6B Ballistic Gatling\n- V801-11 (Radar)\n- V801-12 (Radar)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Ita, Hurston, Arial&lt;/EM4&gt;\n- PIN (Escudo)\n- 5SA 'Rhada' (Escudo)\n- 6SA (Escudo)\n- HEX (Escudo)\n- WEB (Escudo)\n- 5MA 'Chimalli' (Escudo)\n- 6MA 'Kozane' (Escudo)\n- BLOC (Escudo)\n- STOP (Escudo)\n- 5CA 'Akura' (Escudo)\n- 6CA 'Bila' (Escudo)\n- ARMADURA (Escudo)\n- GUARDIA (Escudo)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Ita, Arial, Magda&lt;/EM4&gt;\n- SW16BR1 Repetidor “Buzzsaw”\n- SW16BR2 Repetidor “Sawbuck”\n- SW16BR3 Repetidor “Shredder”\n- Vigilancia (Radar)\n- Devoue (Radar)\n- Tige (Radar)\n</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Here’s the thing, I got a situation over at &lt;EM4&gt;{0} and need someone with a brain between their ears to sort it out for me. Former pilot of mine thought he could cut a deal with another gang and unsurprisingly it didn’t work out for him. Now my cargo is sitting idle and being guarded by a whole bunch of nullbrains waiting for their hauler to come pick it up.\n\nNeed you to head there with a &lt;EM4&gt;heavy-duty tractor beam&lt;/EM4&gt; and a strong crew to get my shit back before its gone for good.\n\nTake it all to the freight elevator at &lt;EM4&gt;{1} and I’ll give you a generous cut of the takings.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>Verás, tengo un problema en &lt;EM4&gt;{0} y necesito a alguien con cerebro para que me lo solucione. Mi antiguo piloto pensó que podía llegar a un acuerdo con otra banda y, como era de esperar, no le salió bien. Ahora mi carga está parada, custodiada por un montón de idiotas que esperan a que su transportista venga a recogerla.\n\nNecesito que vayas allí con un &lt;EM4&gt;rayo tractor de alta resistencia&lt;/EM4&gt; y una tripulación fuerte para recuperar mi mierda antes de que se pierda para siempre.\n\nLlévalo todo al montacargas en &lt;EM4&gt;{1} y te daré una buena parte de las ganancias.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Any interest in taking out a &lt;EM4&gt;{0} for us? \n\nShouldn’t be too much trouble. We’ve already done the legwork and figured out that they're scheduled to pass by &lt;EM4&gt;{1} soon. Just go dark in the nearby emission cloud and you’ll get a good jump on ‘em.  \n\nThey might roll through solo or with some friends. All would be single-seaters but they can hold their own in a dogfight. We’ll drop some forces in the region who can provide support once the fun starts.\n\nYou pull this off and I'll toss &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; to the main contractor for a job well done.\n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 1,000</v>
+        <v>¿Te interesa eliminar un &lt;EM4&gt;{0} por nosotros? \n\nNo debería ser demasiado problema. Ya hemos hecho el trabajo preliminar y hemos averiguado que pasarán cerca de &lt;EM4&gt;{1} pronto. Simplemente ocultándote en la nube de emisión cercana, les sacarás ventaja. \n\nPodrían pasar solos o con algunos amigos. Todos serían monoplazas, pero pueden defenderse bien en un combate aéreo. Desplegaremos algunas fuerzas en la región que podrán brindar apoyo una vez que comience la acción.\n\nSi lo logras, le daré un &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; al contratista principal por un trabajo bien hecho.\n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 1000</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>A squad of ships recently shanked one of our convoys, and ten credits says they’re gonna try and do it again. Looking for someone to launch a reprisal attack before that can happen.  \n\nWe’ve ID’d the idiots as consisting of several large craft and a sizable escort. We believe the leader is flying a &lt;EM4&gt;{0} and set that ship as the primary target. Since it’s a sizable and aggressive squad, a surprise attack seems like a smart play. They often pass by &lt;EM4&gt;{1} which has an emission cloud to hide in. Be smart and patient then strike when the time is right. \n\nUnless you fancy yourself a real ace, it’s probably best to bring some friends. Maybe you can entice folks by letting them know they can pick through the wreckage for valuables once the deed is done.\n\nAnd on top of that, I'll give the main contractor a bonus &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; to sweeten the pot.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 200 / 2,000</v>
+        <v>Un escuadrón de naves atacó recientemente uno de nuestros convoyes, y apuesto diez créditos a que intentarán hacerlo de nuevo. Buscamos a alguien que lance un ataque de represalia antes de que eso suceda. \n\nHemos identificado a los idiotas como varias naves grandes y una escolta considerable. Creemos que el líder está pilotando una &lt;EM4&gt;{0} y hemos establecido esa nave como objetivo principal. Dado que es un escuadrón considerable y agresivo, un ataque sorpresa parece una jugada inteligente. Suelen pasar cerca de &lt;EM4&gt;{1}, que tiene una nube de emisión en la que esconderse. Sé inteligente y paciente, y ataca cuando sea el momento adecuado. \n\nA menos que te creas un verdadero as, probablemente sea mejor traer algunos amigos. Tal vez puedas atraer a la gente haciéndoles saber que pueden rebuscar entre los escombros en busca de objetos de valor una vez que se haya hecho el trabajo.\n\nY además, le daré al contratista principal una bonificación de &lt;EM4&gt;{2} Certificados del Consejo&lt;/EM4&gt; para endulzar la oferta.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 200 / 2000</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Got an opportunity for someone eager to show off their flying skills. Headhunters have been running afoul of this numbrain flying a&lt;EM4&gt;{0} and we’re gonna put a stop to it once and for all.\n\nYou’re gonna help us set a trap for them. See, there’s an &lt;EM4&gt;emission cloud&lt;/EM4&gt; near &lt;EM4&gt;{1} that they fly by frequently. \n\nHead there, hide inside the cloud by powering down your ship, and attack the asshole as soon as you see ‘em and other single-seaters dumb enough to fly with them. It’ll be all you for that first hit, but we’ll put some support ships nearby to help finish the job. \n\nAnd in honor of this being your first surprise attack for us, there's a bonus of &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; for the main contractor at the end of the job. \n\nStows out.\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 500</v>
+        <v>Tenemos una oportunidad para alguien ansioso por mostrar sus habilidades de vuelo. Los cazadores de cabezas han estado teniendo problemas con este numbrain que vuela un&lt;EM4&gt;{0} y vamos a ponerle fin de una vez por todas.\n\nNos ayudarás a tenderles una trampa. Verás, hay una nube de emisión de &lt;EM4&gt;&lt;/EM4&gt; cerca de &lt;EM4&gt;{1} por la que vuelan con frecuencia. \n\nDirígete allí, escóndete dentro de la nube apagando tu nave y ataca al imbécil tan pronto como lo veas y a otros monoplazas lo suficientemente tontos como para volar con él. Serás tú solo para ese primer golpe, pero pondremos algunas naves de apoyo cerca para ayudar a terminar el trabajo. \n\nY en honor a que este sea tu primer ataque sorpresa para nosotros, hay una bonificación de &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; para el contratista principal al final del trabajo. \n\nSe oculta.\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 500</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>One of our Clips put out a kill order on a &lt;EM4&gt;{0} Feel like making ‘em happy by taking it out?\n\nHere’s what you need to know. The target and their escort are scheduled to pass by &lt;EM4&gt;{1} Looks like there’s an emission cloud nearby that can hide your ship’s sig. Wait there until you’re ready to strike. \n\nThe Clip only cares about wiping out the target. Anything of value you find floating in the wreckage is all yours. \n\nAnd on top of that, I'll give the main contractor a bonus &lt;EM4&gt;{2} Council Scrip to sweeten the pot. \n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 150 / 2,000</v>
+        <v>Uno de nuestros Clips emitió una orden de eliminación contra un &lt;EM4&gt;{0}. ¿Te apetece complacerlos eliminándolo?\n\nEsto es lo que necesitas saber. El objetivo y su escolta tienen previsto pasar por &lt;EM4&gt;{1}. Parece que hay una nube de emisión cerca que puede ocultar la firma de tu nave. Espera allí hasta que estés listo para atacar. \n\nAl Clip solo le importa eliminar al objetivo. Todo lo de valor que encuentres flotando entre los restos es tuyo. \n\nY además, le daré al contratista principal un bono de &lt;EM4&gt;{2} Council Scrip para endulzar la oferta. \n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 150 / 2000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Headhunters are looking for someone with the skills and crew to execute an elite op. A military frigate and escort ships are stalking one of our Clips around the system. Don’t know their intentions but it can’t be good. Figure while they’ve got their eyes focused on their prize, we get someone to gather a crew to hit ‘em.  \n\nAlready got a spot picked out. If you get to &lt;EM4&gt;{0} there’s an emission cloud that’s exactly what we need. Head there with friends, power down your ships, and wait for the &lt;EM4&gt;{1} and its escorts to pass by. \n\nWith a bonus of &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; for the main contractor, payment alone should make this worth your while, but you can also keep anything you scrounge from the wreckage.\n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 300 / 16,000</v>
+        <v>Los cazatalentos buscan a alguien con las habilidades y la tripulación necesarias para ejecutar una operación de élite. Una fragata militar y naves de escolta están siguiendo a uno de nuestros Clips por todo el sistema. Desconocemos sus intenciones, pero no pueden ser buenas. Pensemos que mientras tienen la vista puesta en su objetivo, podemos conseguir que alguien reúna una tripulación para atacarlos. \n\nYa tenemos un lugar elegido. Si llegas a &lt;EM4&gt;{0} hay una nube de emisión que es justo lo que necesitamos. Dirígete allí con tus amigos, apaga tus naves y espera a que pase la &lt;EM4&gt;{1} y sus escoltas. \n\nCon una bonificación de &lt;EM4&gt;{2} Certificados del Consejo&lt;/EM4&gt; para el contratista principal, el pago por sí solo debería hacer que esto valga la pena, pero también puedes quedarte con todo lo que encuentres entre los restos.\n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 300 / 16,000</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Some numskull flying a &lt;EM4&gt;{0} was caught spying on our ops. We ran ‘em off with a warning only to spot ‘em doing the same shit someplace else. Since they didn’t get the message, seems we gotta send a stronger one.    \n\nThere’s an emission cloud near &lt;EM4&gt;{1} that they fly by frequently. Primo place to power down, hide, and launch a surprise attack. Sometimes they fly solo, sometimes there’s other single-seaters with them. It’ll be all you for that first hit, but we’ll put some support ships nearby to help finish the job. \n\nAnd if you needed some extra motivation, there's a bonus of &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; for the main contractor at the end of the job. \n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 500</v>
+        <v>Un imbécil que volaba una &lt;EM4&gt;{0} fue sorprendido espiando nuestras operaciones. Lo ahuyentamos con una advertencia, solo para verlo haciendo la misma mierda en otro lugar. Como no entendieron el mensaje, parece que tenemos que enviar uno más fuerte. \n\nHay una nube de emisión cerca de &lt;EM4&gt;{1} por la que vuelan con frecuencia. Un lugar privilegiado para apagar la potencia, esconderse y lanzar un ataque sorpresa. A veces vuelan solos, a veces hay otros monoplazas con ellos. Serás tú el único responsable del primer impacto, pero pondremos algunas naves de apoyo cerca para ayudar a terminar el trabajo. \n\nY si necesitabas motivación extra, hay una bonificación de &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; para el contratista principal al final del trabajo. \n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 500</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Some folks don’t seem happy with us. Got word that several sub-capital ships and a number of escorts are targeting our ops. Figured the best way to keep ‘em from causing us trouble is to hit them before they hit us. \n\nWe got eyes on a &lt;EM4&gt;{0} that’s part of this squad, and it looks like they regularly pass by &lt;EM4&gt;{1} a spot tailor made for a surprise attack. A nearby emission cloud can hide you and anyone you bring along for muscle.\n\nNo sugarcoating it. This ain’t gonna be easy. But the payoff should make it worth your while. Finish the job and the main contractor gets a bonus &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt;. \n\nPlus, who knows what kinda good stuff you’ll find floating in all that wreckage.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 250 / 8,000</v>
+        <v>Parece que a algunos no les agrada nuestra presencia. Nos enteramos de que varias naves subcapitales y varias escoltas están atacando nuestras operaciones. Pensamos que la mejor manera de evitar problemas es atacarlos antes de que nos ataquen. \n\nTenemos a la vista una &lt;EM4&gt;{0} que forma parte de este escuadrón, y parece que pasan regularmente por &lt;EM4&gt;{1}, un lugar ideal para un ataque sorpresa. Una nube de emisión cercana puede ocultarte a ti y a cualquiera que traigas como refuerzo.\n\nNo hay que andarse con rodeos. Esto no va a ser fácil. Pero la recompensa debería valer la pena. Si terminas el trabajo, el contratista principal recibe una bonificación de &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt;. \n\nAdemás, quién sabe qué cosas buenas encontrarás flotando entre todos esos restos.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 250 / 8000</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Our friends at &lt;EM4&gt;{0} have been compromised. A new gang in the area  are threatening them by targeting their &lt;EM4&gt;{1}  \n\nIf those get destroyed its going to be seriously bad for business, so I want you over there pronto on protection duty.  \n \nIf you need any extra motivation, I’m adding &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; for the main contractor.\n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 150 / 2,000</v>
+        <v>Nuestros amigos de &lt;EM4&gt;{0} han sido comprometidos. Una nueva banda en la zona los está amenazando atacando su &lt;EM4&gt;{1} \n\nSi esos son destruidos, será muy malo para el negocio, así que quiero que vayas allí de inmediato para protegerlos. \n \nSi necesitas alguna motivación adicional, estoy agregando &lt;EM4&gt;{2} Council Scrip&lt;/EM4&gt; para el contratista principal.\n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 150 / 2,000</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Some idiots with a deathwish are attacking our ships around &lt;EM4&gt;{0} Can’t let ‘em do that without paying the price. Want to do the honors?\n\nIf so, head out and get after ‘em. The crew there is tracking the attacker’s movements and I’ll pass along situational updates as they come in. \n\nAlso, I’ll sweeten the pot by giving the main contractor a bonus of &lt;EM4&gt;{1} Council Scrip&lt;/EM4&gt; just to show my appreciation. \n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 1,000</v>
+        <v> Unos idiotas con ganas de morir están atacando nuestros barcos cerca de &lt;EM4&gt;{0}. No podemos permitir que lo hagan sin pagar las consecuencias. ¿Quieres encargarte de ello?\n\nSi es así, sal y atácalos. La tripulación está siguiendo los movimientos del atacante y te informaré de las novedades. \n\nAdemás, para mostrar mi agradecimiento, le daré al contratista principal una bonificación de &lt;EM4&gt;{1} Sellos del Consejo&lt;/EM4&gt;. \n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 1000</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Got word that Headhunters ships heading to &lt;EM4&gt;{0} are coming under attack. Scans have revealed enemy forces in the wider region intent on targeting our ops. \n\nThere’s enough of them that it’s gonna take more than one person to clear away all that trash. If you can grab your gear and a few friends, I could really use you out there.  \n\nThe specific attack areas and targets are evolving. Don’t worry about the details now. Just get there and I’ll let you know where you’re needed.  \n\nHandle this right and I’ll give the main contractor a bonus &lt;EM4&gt;{1} Council Scrip&lt;/EM4&gt;.\n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 200 / 2,000</v>
+        <v>Me han informado de que las naves de Headhunters que se dirigen a &lt;EM4&gt;{0} están siendo atacadas. Los escaneos han revelado fuerzas enemigas en la región con la intención de atacar nuestras operaciones. \n\nHay suficientes como para que se necesite más de una persona para eliminar toda esa basura. Si puedes traer tu equipo y a algunos amigos, realmente te necesitaría allí. \n\nLas zonas de ataque y los objetivos específicos están cambiando. No te preocupes por los detalles ahora. Simplemente llega allí y te haré saber dónde se te necesita. \n\nSi manejas esto bien, le daré al contratista principal una bonificación de &lt;EM4&gt;{1} Council Scrip&lt;/EM4&gt;.\n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 200 / 2000</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Our airspace around &lt;EM4&gt;{0} has been compromised. Enemy ships are threatening the base and any of our ships in the area. Gotta put a stop to this immediately, so get your shit in order and get over there. Just get going and I’ll update you with any relevant info on where you’re needed. \n \nIf you need any extra motivation, I’m adding a bonus &lt;EM4&gt;{1} Council Scrip&lt;/EM4&gt; for the main contractor.\n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 150 / 2,000</v>
+        <v>Nuestro espacio aéreo alrededor de &lt;EM4&gt;{0} ha sido comprometido. Naves enemigas amenazan la base y cualquiera de nuestras naves en la zona. Hay que detener esto inmediatamente, así que prepárate y ve para allá. Ponte en marcha y te informaré sobre dónde se te necesita. \n \nSi necesitas motivación adicional, añadiré un bono de &lt;EM4&gt;{1} Council Scrip&lt;/EM4&gt; para el contratista principal.\n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 150 / 2000</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Our crew at &lt;EM4&gt;{0} needs help. Enemy ships are swarming the area and attacking anything and everything they can find. That’d be bad enough as is, but this site has some absolutely crucial gear and personnel that we can’t have destroyed or compromised. \n\nConsidering the size and scale of the attack, you’re gonna need a fully supplied ship and some reliable wingmen. Gather your crew, fly out to the site, and I’ll send you specifics on where you’re needed most.\n\nTo prove just how serious we are about getting this done right, the main contractor will earn a bonus &lt;EM4&gt;{1} Council Scrip&lt;/EM4&gt; for making sure absolutely nothing goes wrong.\n\n- Stow\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 300 / 16,000</v>
+        <v>Nuestro equipo en &lt;EM4&gt;{0} necesita ayuda. Naves enemigas están invadiendo la zona y atacando todo lo que encuentran. Eso ya sería bastante malo, pero este sitio tiene equipo y personal absolutamente cruciales que no podemos permitir que sean destruidos o comprometidos. \n\nConsiderando el tamaño y la escala del ataque, necesitarás una nave completamente equipada y algunos compañeros de ala confiables. Reúne a tu equipo, vuela al sitio y te enviaré detalles sobre dónde se te necesita más.\n\nPara demostrar lo serios que nos tomamos esto para que salga bien, el contratista principal ganará un bono de &lt;EM4&gt;{1} Council Scrip&lt;/EM4&gt; por asegurarse de que absolutamente nada salga mal.\n\n- Stow\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 300 / 16,000</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Headhunters flying in and out of &lt;EM4&gt;{0} are being harassed by some aggressive upstarts. Need them dealt with before they become a real pain in the ass.   \n\nGet there and I’ll update you on what these pests are doing so you can hunt ‘em down. \n\nClear ‘em all out I’ll throw &lt;EM4&gt;{1} Council Scrip&lt;/EM4&gt; to whoever accepted this gig as a bonus.\n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 500</v>
+        <v>Los cazatalentos que entran y salen de &lt;EM4&gt;{0} están siendo acosados por unos advenedizos agresivos. Hay que acabar con ellos antes de que se conviertan en una verdadera molestia. \n\nLlega allí y te informaré de lo que están haciendo estas plagas para que puedas darles caza. \n\nEliminadlos a todos y daré un &lt;EM4&gt;{1} Council Scrip&lt;/EM4&gt; como bonificación a quien haya aceptado este trabajo.\n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 500</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Looking for someone who can not only dogfight but recruit others to the Headhunters cause. Our operations center at &lt;EM4&gt;{0} along with any ships going to and from it, are being targeted by hostile forces. We need support there pronto. \n\nNot gonna lie, but there’s lots of heat around there. That’s why you’ll need to be fully supplied and find some trustworthy friends to fly at your wing. When you get your crew together, head out there and I’ll update you if there’s any flare ups in the area that need your attention.\n\nThis op needs to go off without a hitch, so I’m offering the main contractor a bonus &lt;EM4&gt;{1} Council Scrip&lt;/EM4&gt; for a job well done. \n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 250 / 8,000</v>
+        <v>Buscamos a alguien que no solo pueda participar en combates aéreos, sino también reclutar a otros para la causa de los Headhunters. Nuestro centro de operaciones en &lt;EM4&gt;{0}, junto con cualquier nave que se dirija hacia o desde allí, está siendo atacado por fuerzas hostiles. Necesitamos apoyo allí urgentemente. \n\nNo voy a mentir, hay mucha tensión por allí. Por eso necesitarás estar completamente abastecido y encontrar algunos amigos de confianza que vuelen contigo. Cuando tengas a tu tripulación, dirígete hacia allá y te informaré si hay algún incidente en la zona que requiera tu atención.\n\nEsta operación debe salir a la perfección, así que le ofrezco al contratista principal una bonificación de &lt;EM4&gt;{1} Council Scrip&lt;/EM4&gt; por un trabajo bien hecho. \n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 250 / 8000</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Got a bunch of boxes sitting at &lt;EM4&gt;{0} that have to be moved to &lt;EM4&gt;{1} Seems easy enough, right? Well, guess it ain’t. \n\nThe idiot who was supposed to move these things threw out his back trying to carry all of ‘em at once. So, you know, maybe bring a &lt;EM4&gt; handheld tractor beam&lt;/EM4&gt; and try taking ‘em one at a time like a normal person. But, hey, don’t let me tell you how to do your job. Just get it done. \n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 200 / 400 / 800</v>
+        <v>Tengo un montón de cajas en &lt;EM4&gt;{0} que hay que mover a &lt;EM4&gt;{1}. Parece bastante fácil, ¿verdad? Pues parece que no. \n\nEl idiota que se suponía que iba a mover estas cosas se lesionó la espalda intentando cargarlas todas a la vez. Así que, ya sabes, quizás deberías traer un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt; e intentar moverlas una por una como una persona normal. Pero bueno, no dejes que te diga cómo hacer tu trabajo. Simplemente hazlo. \n\nSe oculta.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 200 / 400 / 800</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>CFP think they’re safe over at &lt;EM4&gt;{0} but we got big plans for them. You’re gonna pave the way for us by heading there and shutting down their comm towers.\n\nThere should be a &lt;EM4&gt;control terminal at the top&lt;/EM4&gt; that you can use to shut the tower down. You get that sorted and they won’t be able to call for backup. Then we can show those skags who this system belongs to.\n\nMost outposts use the same system, so this’ll come in handy next time you want to make sure reinforcements don’t mess with you.\n\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 75</v>
+        <v>CFP cree que están a salvo en &lt;EM4&gt;{0}, pero tenemos grandes planes para ellos. Nos allanarás el camino dirigiéndote allí y desactivando sus torres de comunicaciones.\n\nDebería haber una terminal de control &lt;EM4&gt;en la parte superior&lt;/EM4&gt; que puedes usar para desactivar la torre. Si lo consigues, no podrán pedir refuerzos. Entonces podremos mostrarles a esos skags a quién pertenece este sistema.\n\nLa mayoría de los puestos de avanzada usan el mismo sistema, así que esto te será útil la próxima vez que quieras asegurarte de que los refuerzos no te molesten.\n\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 75</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>We’re making a play to hit some XenoThreat assholes where it hurts but need to be smart about it. That’s why we’re sending you in first to take out their comm towers so they can’t call for backup. You do that and we can be in and out before they know it.\n\nHead to &lt;EM4&gt;{0} and climb the comm towers there. Should be a &lt;EM4&gt;control panel at the top&lt;/EM4&gt; you can use to switch them off.\n\nIn fact, same goes for most other outposts. Rather than having to deal with reinforcements, you can just turn off the comm towers. But hey, if you wanna ring the bell to ghost a few more Xenothreat I ain’t complaining.\n\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 75 / 100</v>
+        <v>Estamos intentando atacar a esos malditos XenoThreat donde más les duele, pero tenemos que ser inteligentes. Por eso te enviamos primero para que destruyas sus torres de comunicación y no puedan pedir refuerzos. Si lo haces, entraremos y saldremos antes de que se den cuenta.\n\nDirígete a &lt;EM4&gt;{0} y sube a las torres de comunicación. Debería haber un &lt;EM4&gt;panel de control en la parte superior&lt;/EM4&gt; que puedes usar para apagarlas.\n\nDe hecho, lo mismo se aplica a la mayoría de los demás puestos avanzados. En lugar de tener que lidiar con refuerzos, puedes simplemente apagar las torres de comunicación. Pero bueno, si quieres tocar la campana para eliminar a unos cuantos XenoThreat más, no me quejo.\n\n\nSe despide.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 75 / 100</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Headhunters have been expanding, but still need help getting a lay of our new territory. I’ve got a run to check spots we want scanned ready to go. \n\nThis one kicks off at the &lt;EM4&gt;location marker&lt;/EM4&gt; on your HUD and will look at a few more locations after that, but I’ll update you as we clear them out. Not expecting you to run into any trouble but no guarantees. Trouble seems to follow us.\n\nGet this done and I'll toss the main contractor &lt;EM4&gt;{0} Council Scrip&lt;/EM4&gt; as a thanks.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 1,000</v>
+        <v>Los reclutadores se han expandido, pero aún necesitan ayuda para familiarizarse con nuestro nuevo territorio. Tengo una misión lista para escanear los lugares que queremos explorar. \n\nEsta misión comienza en el marcador de ubicación &lt;EM4&gt; en tu HUD y luego revisará algunos lugares más, pero te mantendré informado a medida que los vayamos completando. No espero que tengas problemas, pero no hay garantías. Los problemas parecen perseguirnos.\n\nSi terminas esto, te daré el bono del Consejo &lt;EM4&gt;{0}&lt;/EM4&gt; del contratista principal como agradecimiento.\n\nSe despide.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 1000</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>I’ve noticed an uptick in attacks on Headhunter ships and it's got me feelin' jumpy. Got an important resupply shipment that we can’t afford to lose, and need help determining what route to send it. I’ve strung together a few potential spots that I’d set up in if I was gonna hit ‘em. Any chance you could visit and clear out any lowlifes that may be hiding there? \n\nThe route starts at the &lt;EM4&gt;location marker&lt;/EM4&gt; on your HUD. After you scan it and clear whatever’s there, I’ll send you to a few other areas that could work. I’ve been hearing people have been rolling through these spots, so would be smart to &lt;EM4&gt;bring a friend&lt;/EM4&gt; to watch your back.\n\nYou make it to the end and I'll give the main contractor a bonus &lt;EM4&gt;{0} Council Scrip&lt;/EM4&gt; as thanks. \n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 200 / 2,000</v>
+        <v>He notado un aumento en los ataques a las naves Headhunter y me tiene nervioso. Tenemos un envío de reabastecimiento importante que no podemos permitirnos perder, y necesito ayuda para determinar qué ruta enviar. He juntado algunos lugares potenciales donde me establecería si fuera a atacarlos. ¿Hay alguna posibilidad de que puedas visitarlos y eliminar a cualquier maleante que pueda estar escondido allí? \n\nLa ruta comienza en el marcador de ubicación &lt;EM4&gt;&lt;/EM4&gt; en tu HUD. Después de escanearlo y eliminar lo que haya allí, te enviaré a algunas otras áreas que podrían funcionar. He oído que la gente ha estado pasando por estos lugares, así que sería inteligente &lt;EM4&gt;traer a un amigo&lt;/EM4&gt; para que te cubra las espaldas.\n\nSi llegas al final, le daré al contratista principal una bonificación de &lt;EM4&gt;{0} Council Scrip&lt;/EM4&gt; como agradecimiento. \n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 200 / 2.000</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>The local Clip wants current intel on several of our sectors. Not sure what they’re looking for but I’m not about to ask. My job is to find someone willing to swing through and scan these locations. You available? \n\nAll you need to do is head to the &lt;EM4&gt;location marker&lt;/EM4&gt; on your HUD, run a scan, and if it’s clear, move to the next spot. If you run into any issues, take care of it. \n\nAin’t sound too tough now does it? Plus, I'll give the main contractor a bonus &lt;EM4&gt;{0} Council Scrip&lt;/EM4&gt; as thanks. \n\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 150 / 2,000</v>
+        <v>El Clip local quiere información actualizada sobre varios de nuestros sectores. No estoy seguro de qué buscan, pero no voy a preguntar. Mi trabajo es encontrar a alguien dispuesto a pasarse y escanear estas ubicaciones. ¿Estás disponible? \n\nSolo tienes que dirigirte al marcador de ubicación &lt;EM4&gt; en tu HUD, realizar un escaneo y, si está despejado, pasar al siguiente lugar. Si encuentras algún problema, soluciónalo. \n\nNo suena tan difícil, ¿verdad? Además, le daré al contratista principal un bono de &lt;EM4&gt;{0} Council Scrip&lt;/EM4&gt; como agradecimiento. \n\n\nSe despide.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 150 / 2000</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Got some asshole’s trying to push us out of the system. You up for pushing back?\n\nSee, there are some folks who really don’t want us here, and have started sending out hunting parties of five to seven ships, often with a bigger gun ship, to places where we’re building up our presence. Time for us to show that we’re here to stay.  \n\nI’ve strung together a few spots starting at the &lt;EM4&gt;location marker&lt;/EM4&gt; on your HUD where we’re seeing the most hostile encounters. Need you to visit each one and scan to see if we can bait them into a fight.\n\nKnow this is going to be a hard one, so don't be cocky and try to go it alone. If I were you, I'd bring at least &lt;EM4&gt;three friends&lt;/EM4&gt; onboard for support. To make it worth your while, I'm promising a bonus of &lt;EM4&gt;{0} Council Scrip&lt;/EM4&gt; to the main contractor that pulls it off. \n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 300 / 16,000</v>
+        <v>Hay unos imbéciles que intentan echarnos del sistema. ¿Estás listo para contraatacar?\n\nVerás, hay gente que no nos quiere aquí y ha empezado a enviar grupos de caza de cinco a siete naves, a menudo con una nave de combate más grande, a lugares donde estamos estableciendo nuestra presencia. Es hora de demostrar que estamos aquí para quedarnos. \n\nHe conectado algunos puntos a partir del marcador de ubicación &lt;EM4&gt;&lt;/EM4&gt; en tu HUD donde estamos viendo los encuentros más hostiles. Necesito que visites cada uno y escanees para ver si podemos atraerlos a una pelea.\n\nSé que esto va a ser difícil, así que no seas arrogante e intentes hacerlo solo. Si yo fuera tú, traería al menos &lt;EM4&gt;tres amigos&lt;/EM4&gt; a bordo para que te apoyen. Para que valga la pena, prometo una bonificación de &lt;EM4&gt;{0} Council Scrip&lt;/EM4&gt; al contratista principal que lo consiga. \n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 300 / 16.000</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Headhunters want some intel on what’s happening around territory. We’ve already set up some monitoring satellites, but nothing beats a good ol’ patrol. You up for it?\n\nIf so, get on over to the &lt;EM4&gt;location marker&lt;/EM4&gt; on your HUD. Start by scanning that region and then we’ll guide you to a few more spots that we want info on. \n\nAnd if you needed some extra motivation, there's a bonus of &lt;EM4&gt;{0} Council Scrip&lt;/EM4&gt; for the main contractor at the end of the job. \n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 500</v>
+        <v>Los reclutadores quieren información sobre lo que está sucediendo en el territorio. Ya hemos instalado algunos satélites de vigilancia, pero nada supera una buena patrulla. ¿Te animas?\n\nSi es así, dirígete al marcador de ubicación &lt;EM4&gt; en tu HUD. Empieza escaneando esa región y luego te guiaremos a algunos lugares más sobre los que necesitamos información. \n\nY si necesitabas un incentivo adicional, hay una bonificación de &lt;EM4&gt;{0} Council Scrip&lt;/EM4&gt; para el contratista principal al final del trabajo. \n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 500</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>We’re getting pushback from folks who don’t seem happy that we’re here. Folks have gotten keen to our haunts and started sending out squads to hit our ships. You down to visit a few of those spots to show that we won’t be scared off? \n\nIf so, start by seeing what’s around the &lt;EM4&gt;location marker&lt;/EM4&gt; on your HUD. From there I’ll guide you to a few other hotspots that we need checked. Better get your shit in order before heading out. I'd recommend loading up on ammo and convincing &lt;EM4&gt;two friends&lt;/EM4&gt; to join the patrol.\n\nYou do this for the Headhunters and I'll see to it that the main contractor gets a bonus of &lt;EM4&gt;{0} Council Scrip&lt;/EM4&gt;. \n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 250 / 8,000</v>
+        <v>Estamos recibiendo resistencia de gente que no parece contenta con nuestra presencia. Algunos se han interesado por nuestros lugares y han empezado a enviar escuadrones para atacar nuestras naves. ¿Te animas a visitar algunos de esos lugares para demostrar que no nos asustaremos? \n\nSi es así, empieza por ver qué hay alrededor del marcador de ubicación &lt;EM4&gt; en tu HUD. Desde ahí te guiaré a otros puntos clave que debemos revisar. Mejor prepárate antes de salir. Te recomiendo que te cargues de munición y convenzas a &lt;EM4&gt;dos amigos&lt;/EM4&gt; para que se unan a la patrulla.\n\nHaces esto por los Headhunters y me aseguraré de que el contratista principal reciba una bonificación de &lt;EM4&gt;{0} Council Scrip&lt;/EM4&gt;. \n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 250 / 8000</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>XenoThreat are on the warpath right now. They’ve launched simultaneous attacks on several Headhunters sites and stretched our fighters thin. Got word they’re planning to storm {0} next, and we can’t get anyone there to defend it. \n\nI’m looking to pay someone to pull together a crew, gather supplies, and mount a strong defense for us. Gonna be honest with you, this is shaping up to be a hell of a fight. Xenos are sending some of their most experienced forces there. Not much else I can say except that they’ll probably stagger the arrival of their forces, wipe them all out and you’ll be paid handsomely. \n\nThink you can rise to the occasion?  \n\n-Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Atzkav Sniper Rifle\n- Atzkav "Igniter" Sniper Rifle\n- Atzkav "Mirage" Sniper Rifle\n- Calico Arms Tactical\n- Calico Core Tactical\n- Calico Legs Tactical\n- Calico Helmet Tactical\n- Atzkav Sniper Rifle Battery (8 cap)\n</v>
+        <v>XenoThreat está en pie de guerra ahora mismo. Han lanzado ataques simultáneos contra varios sitios de Headhunters y han agotado a nuestros combatientes. Nos han dicho que planean asaltar {0} a continuación, y no podemos enviar a nadie para defenderlo. \n\nBusco a alguien que reúna un equipo, consiga suministros y organice una defensa sólida para nosotros. Para serte sincero, esto se perfila como una batalla épica. Los xenos están enviando algunas de sus fuerzas más experimentadas. No puedo decir mucho más, excepto que probablemente escalonarán la llegada de sus fuerzas, las aniquilarán a todas y te pagarán generosamente. \n\n¿Crees que puedes estar a la altura de las circunstancias? \n\n-Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Fusil de francotirador Atzkav\n- Fusil de francotirador Atzkav "Igniter"\n- Fusil de francotirador Atzkav "Mirage"\n- Armas tácticas Calico\n- Núcleo táctico Calico\n- Piernas tácticas Calico\n- Casco táctico Calico\n- Batería de fusil de francotirador Atzkav (8 unidades)\n</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>A client has contacted us about resolving a &lt;EM4&gt;{0} infestation issue before it gets any worse. Several locations around &lt;EM4&gt;{1} are currently beset by the creatures. There’s a growing concern that if this goes on for too much longer, then the natural habit will be ravaged beyond repair. Are you available to take care of this issue?\n\nYou can refer to &lt;EM4&gt;"The Guide to Stanton Wildlife"&lt;/EM4&gt; in your Journal for more specific information on the targeted creature.\n\nBest,\n\nWanda Werkheiser\nContract Manager\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 2,000 / 4,000</v>
+        <v>Un cliente se ha puesto en contacto con nosotros para resolver un problema de infestación de &lt;EM4&gt;{0} antes de que empeore. Varias zonas alrededor de &lt;EM4&gt;{1} están actualmente infestadas por estas criaturas. Existe una creciente preocupación de que, si esto continúa por mucho más tiempo, el hábitat natural quede devastado sin posibilidad de recuperación. ¿Están disponibles para solucionar este problema?\n\nPuede consultar &lt;EM4&gt;"La guía de la fauna silvestre de Stanton"&lt;/EM4&gt; en su Diario para obtener información más específica sobre la criatura en cuestión.\n\nSaludos cordiales,\n\nWanda Werkheiser\nGerente de Contratos\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 2000 / 4000</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Highpoint Wilderness is seeking a contractor to cull a pack of kopions that are threatening to overrun one of Citizens for Prosperity's outposts. After an initial assessment, it has been decided that relocation is impossible and a culling of them is the only viable option. If you're interested, head to &lt;EM4&gt;{0}  and once we've received confirmation that the task is complete we will send payment.\n\nBest,\n\nWanda Werkheiser\nContract Manager\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 75 / 100</v>
+        <v>Highpoint Wilderness busca un contratista para eliminar una manada de kopions que amenaza con invadir uno de los puestos de avanzada de Citizens for Prosperity. Tras una evaluación inicial, se ha decidido que la reubicación es imposible y que la eliminación selectiva es la única opción viable. Si está interesado, diríjase a &lt;EM4&gt;{0} y, una vez que recibamos la confirmación de que la tarea se ha completado, le enviaremos el pago.\n\nSaludos cordiales,\n\nWanda Werkheiser\nGerente de Contratos\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 75 / 100</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Members of the group Citizens for Prosperity were recently ambushed by several packs of kopions at &lt;EM4&gt;{0} and have requested Highpoint's services in dealing with them. For the safety of everyone trying to settle in the area, we require the immediate services of someone who can deal with this on our behalf.\n\nExpect a large number of animals and prepare yourself accordingly.\n\nBest,\n\nWanda Werkheiser\nContract Manager\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 300</v>
+        <v>Miembros del grupo Ciudadanos por la Prosperidad fueron emboscados recientemente por varias manadas de kopions en &lt;EM4&gt;{0} y han solicitado los servicios de Highpoint para lidiar con ellos. Para la seguridad de todos los que intentan establecerse en la zona, necesitamos los servicios inmediatos de alguien que pueda encargarse de esto en nuestro nombre.\n\nEspere una gran cantidad de animales y prepárese en consecuencia.\n\nSaludos cordiales,\n\nWanda Werkheiser\nGerente de Contratos\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 300</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>We’re putting out a contract for anyone who is capable of hunting animals responsibly. Citizens for Prosperity needs a group of aggressive kopions who have been harassing their people culled from &lt;EM4&gt;{0} After some initial monitoring, it looked as if they may on, but unfortunately we’ve been forced to take action. This is a relatively straightforward job, but when dealing with dangerous animals, cautious is always advised.\n\nBest,\n\nWanda Werkheiser\nContract Manager\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 75 / 100</v>
+        <v>Estamos publicando un contrato para cualquier persona capaz de cazar animales de forma responsable. Citizens for Prosperity necesita un grupo de kopions agresivos que han estado acosando a su gente, eliminados de &lt;EM4&gt;{0}. Después de un monitoreo inicial, parecía que podrían seguir, pero desafortunadamente nos hemos visto obligados a tomar medidas. Este es un trabajo relativamente sencillo, pero cuando se trata de animales peligrosos, siempre se recomienda precaución.\n\nSaludos cordiales,\n\nWanda Werkheiser\nGerente de Contratos\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 75 / 100</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Citizens for Prosperity recently reported to us that one of their scouts was injured by kopions during a routine exploration mission. According to them, this isn't the first time this particular pack has posed a problem, so they've requested our services to clear out the area. The report shows they were last seen at &lt;EM4&gt;{0} behavior is typical of kopions looking to expand their territory, so it is highly likely that you will be dealing with more kopions than initially observed. Caution is advised. \n\nBest,\n\nWanda Werkheiser\nContract Manager\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50 / 100 / 150</v>
+        <v>Citizens for Prosperity nos informó recientemente que uno de sus exploradores resultó herido por kopions durante una misión de exploración rutinaria. Según ellos, no es la primera vez que esta manada en particular ha causado problemas, por lo que han solicitado nuestros servicios para despejar la zona. El informe indica que fueron vistos por última vez en &lt;EM4&gt;{0}. Este comportamiento es típico de los kopions que buscan expandir su territorio, por lo que es muy probable que se encuentre con más kopions de los observados inicialmente. Se recomienda precaución. \n\nSaludos cordiales,\n\nWanda Werkheiser\nGerente de Contratos\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50 / 100 / 150</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Highpoint Wilderness needs someone to exterminate an overpopulated pack of kopions that's threatening one of CFP's settlements. This pack can be found at &lt;EM4&gt;{0} Remember to exhibit caution when approaching them and arm yourself accordingly.\n\nBest,\n\nWanda Werkheiser\nContract Manager\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 75 / 100</v>
+        <v>Highpoint Wilderness necesita a alguien que extermine una manada superpoblada de kopions que amenaza uno de los asentamientos de CFP. Esta manada se encuentra en &lt;EM4&gt;{0}. Recuerde tener precaución al acercarse y armarse adecuadamente.\n\nSaludos cordiales,\n\nWanda Werkheiser\nGerente de Contratos\nEspecialistas en Highpoint Wilderness\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 75 / 100</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Citizens for Prosperity have approached us with information that multiple groups of kopions have been attacking people at &lt;EM4&gt;{0} without provocation. Currently, no deaths have been reported, but they are concerned their most vulnerable will be at risk if these kopions continue running rampant.\n\nEnsure you are prepared adequately, kopions hunt in packs and it is easy to become overwhelmed by their sheer numbers.\n\nBest,\n\nWanda Werkheiser\nContract Manager\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 150</v>
+        <v> Ciudadanos por la Prosperidad se han puesto en contacto con nosotros para informarnos de que varios grupos de kopions han estado atacando a personas en &lt;EM4&gt;{0} sin provocación. Actualmente, no se han reportado muertes, pero les preocupa que las personas más vulnerables corran peligro si estos kopions siguen actuando sin control.\n\nAsegúrese de estar bien preparado, los kopions cazan en manada y es fácil verse superado por su gran número.\n\nSaludos cordiales,\n\nWanda Werkheiser\nGerente de Contratos\nHighpoint Wilderness Specialists\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 150</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Hockrow Agency \nCase File #MP12854\nLead Investigator: Arken Mallor\n\nCase Summary:\nWe have been asked to track down two contractors who work for a client of ours after they lost contact with them. They were last known to be traveling together in {0} Until their exact situation can be assessed, our client is stuck in a waiting pattern. \n\nContract Investigator Actions:\nLocate &lt;EM4&gt;{1} at &lt;EM4&gt;{2} and confirm their status. \n\nIf they are deceased, examine the body closely so we can verify their death via your mobiGlas.\n\nAdditional Notes:\nYou'll be heading into what is regarded as a particularly dangerous spot. Backup is highly recommended for this encounter.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>Agencia Hockrow \nExpediente n.° MP12854\nInvestigador principal: Arken Mallor\n\nResumen del caso:\nSe nos ha solicitado localizar a dos contratistas que trabajan para un cliente nuestro después de que perdimos el contacto con ellos. Se sabe que la última vez que se les vio fue viajando juntos en {0}. Hasta que se pueda evaluar su situación exacta, nuestro cliente se encuentra en una situación de espera. \n\nAcciones del investigador de contratistas:\nLocalizar a &lt;EM4&gt;{1} en &lt;EM4&gt;{2} y confirmar su estado. \n\nSi han fallecido, examinar el cuerpo detenidamente para que podamos verificar su muerte a través de su mobiGlas.\n\nNotas adicionales:\nSe dirigirá a lo que se considera un lugar particularmente peligroso. Se recomienda encarecidamente contar con refuerzos para este encuentro.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Hey,\n\nNeed a reliable contractor to help us out with a bit of a situation.\n\nOur of our haulers has dropped out mid-contract and now our client's cargo is stuck in transit. Think they were trying to negotiate a better rate with us, but that's not how Ling does business. Anyway, they're done and we desperately need the shipment finished.\n\nPetra and I have been working with this client for years now and have built up a good rapport. Be a shame to throw that all a way because of an unreliable hauler. Can you head to &lt;EM4&gt;{0} and collect the shipment? You'll need a &lt;EM4&gt;heavy-duty tractor beam&lt;/EM4&gt; and a ship that can carry &lt;EM4&gt;{1} cargo containers&lt;/EM4&gt;.\n\nTake the shipment to the freight elevator over at &lt;EM4&gt;{2} and we'll get you paid as soon as. We'd really appreciate your help with this and I'm sure our client would too.\n\nThanks,  \nReyes Ling \nCargo Logistics Coordinator \nLing Family Hauling \n\n\n\n\n\n\n\nLing Family Hauling knows it’s a dangerous and unpredictable universe and has established several protocols to protect both you and our client’s cargo. To ensure you aren’t punished for circumstances outside of your control, total payment will be prorated to the percentage of cargo successfully delivered. A delivery timer will be set for each haul. Any cargo that remains undelivered upon its expiration will be flagged as stolen and treated as such. All pick-ups and deliveries must be autoloaded or done at a freight elevator.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>Hola,\n\nNecesitamos un contratista confiable que nos ayude con un pequeño problema.\n\nNuestro transportista se ha retirado a mitad del contrato y ahora la carga de nuestro cliente está atascada en tránsito. Creo que estaban tratando de negociar una mejor tarifa con nosotros, pero así no es como Ling hace negocios. En fin, se han ido y necesitamos desesperadamente que el envío se complete.\n\nPetra y yo hemos estado trabajando con este cliente durante años y hemos construido una buena relación. Sería una lástima echarlo todo a perder por un transportista poco confiable. ¿Puedes ir a &lt;EM4&gt;{0} y recoger el envío? Necesitarás una &lt;EM4&gt;viga tractora de alta resistencia&lt;/EM4&gt; y un barco que pueda transportar &lt;EM4&gt;{1} contenedores de carga&lt;/EM4&gt;.\n\nLleva el envío al montacargas en &lt;EM4&gt;{2} y te pagaremos tan pronto como. Agradeceríamos mucho su ayuda con esto y estoy seguro de que nuestro cliente también.\n\nGracias, \nReyes Ling \nCoordinador de Logística de Carga \nLing Family Hauling \n\n\n\n\n\n\n\nLing Family Hauling sabe que es un universo peligroso e impredecible y ha establecido varios protocolos para proteger tanto su carga como la de nuestro cliente. Para garantizar que no sea penalizado por circunstancias fuera de su control, el pago total se prorrateará según el porcentaje de carga entregada con éxito. Se establecerá un temporizador de entrega para cada transporte. Cualquier carga que permanezca sin entregar al expirar el plazo se marcará como robada y se tratará como tal. Todas las recogidas y entregas deben realizarse mediante carga automática o en un elevador de carga.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Following the brutal attack on Pyro and our efforts to combat the vigilante group the Frontier Fighters, our strategic reserves across the system are at an all-time low. Citizens for Prosperity are eager to replenish our stocks before we reach a point of desperation. \n\nTo that end, we were hoping that you could resupply&lt;EM4&gt; {0} &lt;/EM4&gt;\n\nI leave it up to you to decide how best to procure and refine the resources, but the asteroid clusters near LaGrange points might be a good place to start mining.\n\nYour support of our efforts is much appreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Tras el brutal ataque a Pyro y nuestros esfuerzos por combatir al grupo justiciero Frontier Fighters, nuestras reservas estratégicas en todo el sistema están en su nivel más bajo. Ciudadanos por la Prosperidad están ansiosos por reabastecer nuestras existencias antes de que lleguemos a un punto de desesperación. \n\nPara ello, esperábamos que pudieras reabastecernos&lt;EM4&gt; {0} &lt;/EM4&gt;\n\nTe dejo a ti la decisión de la mejor manera de obtener y refinar los recursos, pero los cúmulos de asteroides cerca de los puntos de Lagrange podrían ser un buen lugar para comenzar la minería.\n\nAgradecemos mucho tu apoyo a nuestros esfuerzos,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Following the brutal attack on Pyro and our efforts to combat the vigilante group the Frontier Fighters, our strategic reserves across the system are at an all-time low. Citizens for Prosperity are eager to replenish our stocks before we reach a point of desperation. \n\nTo that end, we were hoping that you would recruit a full fleet to resupply&lt;EM4&gt; {0} &lt;/EM4&gt;\n\nI leave it up to you to decide how best to procure and refine the resources, but the asteroid clusters near LaGrange points might be a good place to start mining.\n\nYour support of our efforts is much appreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Tras el brutal ataque a Pyro y nuestros esfuerzos por combatir al grupo justiciero Frontier Fighters, nuestras reservas estratégicas en todo el sistema están en su nivel más bajo. Ciudadanos por la Prosperidad están ansiosos por reabastecer nuestras existencias antes de que lleguemos a un punto de desesperación. \n\nPara ello, esperábamos que reclutaran una flota completa para reabastecernos&lt;EM4&gt; {0} &lt;/EM4&gt;\n\nLes dejo a ustedes la decisión de cómo obtener y refinar mejor los recursos, pero los cúmulos de asteroides cerca de los puntos de Lagrange podrían ser un buen lugar para comenzar la minería.\n\nAgradecemos mucho su apoyo a nuestros esfuerzos.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Following the brutal attack on Pyro and our efforts to combat the vigilante group the Frontier Fighters, our strategic reserves across the system are at an all-time low. Citizens for Prosperity are eager to replenish our stocks before we reach a point of desperation. \n\nTo that end, we were hoping that you and a team of your choosing could resupply&lt;EM4&gt; {0} &lt;/EM4&gt;\n\nI leave it up to you to decide how best to procure and refine the resources, but the asteroid clusters near LaGrange points might be a good place to start mining.\n\nYour support of our efforts is much appreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Tras el brutal ataque a Pyro y nuestros esfuerzos por combatir al grupo justiciero Frontier Fighters, nuestras reservas estratégicas en todo el sistema están en su nivel más bajo. Ciudadanos por la Prosperidad están ansiosos por reabastecer nuestras existencias antes de que lleguemos a un punto de desesperación. \n\nPara ello, esperábamos que usted y un equipo de su elección pudieran reabastecernos&lt;EM4&gt; {0} &lt;/EM4&gt;\n\nLe dejo a su criterio la mejor manera de obtener y refinar los recursos, pero los cúmulos de asteroides cerca de los puntos de Lagrange podrían ser un buen lugar para comenzar la minería.\n\nAgradecemos mucho su apoyo a nuestros esfuerzos,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Following the brutal attack on Pyro and our efforts to combat the vigilante group the Frontier Fighters, our strategic reserves across the system are at an all-time low. Citizens for Prosperity are eager to replenish our stocks before we reach a point of desperation. \n\nTo that end, we were hoping that you could deliver the needed supplies to&lt;EM4&gt; {0} &lt;/EM4&gt;We have arranged shipment to Pyro from there.\n\nI leave it up to you to decide how best to procure and refine the resources, but Daymar or Aberdeen might be good places to start mining.\n\nYour support of our efforts is much appreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400</v>
+        <v>Tras el brutal ataque a Pyro y nuestros esfuerzos por combatir al grupo justiciero Frontier Fighters, nuestras reservas estratégicas en todo el sistema se encuentran en su nivel más bajo. Ciudadanos por la Prosperidad deseamos reponer nuestras existencias antes de llegar a un punto de desesperación. \n\nPara ello, esperábamos que pudieras entregar los suministros necesarios a &lt;EM4&gt; {0} &lt;/EM4&gt;. Hemos organizado el envío a Pyro desde allí.\n\nTe dejo a ti la decisión de cómo obtener y refinar mejor los recursos, pero Daymar o Aberdeen podrían ser buenos lugares para comenzar la minería.\n\nAgradecemos mucho tu apoyo a nuestros esfuerzos.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Following the brutal attack on Pyro and our efforts to combat the vigilante group the Frontier Fighters, our strategic reserves across the system are at an all-time low. Citizens for Prosperity are eager to replenish our stocks before we reach a point of desperation. \n\nTo that end, we were hoping that you would recruit a full fleet to deliver the supplies to &lt;EM4&gt; {0} &lt;/EM4&gt; We have arranged shipment to Pyro from there.\n\nI leave it up to you to decide how best to procure and refine the resources, but Daymar or Aberdeen might be good places to start mining.\n\nYour support of our efforts is much appreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400</v>
+        <v>Tras el brutal ataque a Pyro y nuestros esfuerzos por combatir al grupo justiciero Frontier Fighters, nuestras reservas estratégicas en todo el sistema se encuentran en su nivel más bajo. Ciudadanos por la Prosperidad deseamos reponer nuestras existencias antes de llegar a un punto de desesperación. \n\nPara ello, esperábamos que reclutara una flota completa para entregar los suministros a &lt;EM4&gt; {0} &lt;/EM4&gt;. Hemos organizado el envío a Pyro desde allí.\n\nLe dejo a su criterio la mejor manera de obtener y refinar los recursos, pero Daymar o Aberdeen podrían ser buenos lugares para comenzar la minería.\n\nAgradecemos enormemente su apoyo a nuestros esfuerzos.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Following the brutal attack on Pyro and our efforts to combat the vigilante group the Frontier Fighters, our strategic reserves across the system are at an all-time low. Citizens for Prosperity are eager to replenish our stocks before we reach a point of desperation. \n\nTo that end, we were hoping that you and a team of your choosing could deliver the needed supplies to&lt;EM4&gt; {0} &lt;/EM4&gt;We have arranged shipment to Pyro from there.\n\nI leave it up to you to decide how best to procure and refine the resources, but Daymar or Aberdeen might be good places to start mining.\n\nYour support of our efforts is much appreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400</v>
+        <v>Tras el brutal ataque a Pyro y nuestros esfuerzos por combatir al grupo justiciero Frontier Fighters, nuestras reservas estratégicas en todo el sistema se encuentran en su nivel más bajo. Ciudadanos por la Prosperidad están ansiosos por reponer nuestras existencias antes de que lleguemos a un punto de desesperación. \n\nCon ese fin, esperábamos que usted y un equipo de su elección pudieran entregar los suministros necesarios a &lt;EM4&gt; {0} &lt;/EM4&gt;. Hemos organizado el envío a Pyro desde allí.\n\nLe dejo a su criterio la mejor manera de obtener y refinar los recursos, pero Daymar o Aberdeen podrían ser buenos lugares para comenzar la minería.\n\nAgradecemos mucho su apoyo a nuestros esfuerzos.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Following the brutal attack on Pyro and our efforts to combat the vigilante group the Frontier Fighters, our strategic reserves across the system are at an all-time low. Citizens for Prosperity are eager to replenish our stocks before we reach a point of desperation. \n\nTo that end, we were hoping that you could resupply&lt;EM4&gt; {0} with salvaged materials.&lt;/EM4&gt; It would go a long way in helping us rebuild what was lost in the attacks.\n\nI leave it up to you to decide how best to acquire what we need, but should be able to find some wrecks to scavenge orbiting around most planets. \n\nYour support of our efforts is much appreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Tras el brutal ataque a Pyro y nuestros esfuerzos por combatir al grupo justiciero Frontier Fighters, nuestras reservas estratégicas en todo el sistema se encuentran en su nivel más bajo. Ciudadanos por la Prosperidad deseamos reabastecer nuestras existencias antes de llegar a un punto de desesperación. \n\nPara ello, esperábamos que pudieras reabastecernos con materiales recuperados. Sería de gran ayuda para reconstruir lo perdido en los ataques.\n\nTe dejo a ti la decisión de cómo adquirir lo que necesitamos, pero deberías poder encontrar algunos restos de naves para saquear orbitando alrededor de la mayoría de los planetas. \n\nAgradecemos enormemente tu apoyo a nuestros esfuerzos.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n\nReputación otorgada (por dificultad): -190.500 / 400 / 2.400</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Following the brutal attack on Pyro and our efforts to combat the vigilante group the Frontier Fighters, our strategic reserves across the system are at an all-time low. Citizens for Prosperity are eager to replenish our stocks before we reach a point of desperation. \n\nTo that end, we were hoping that you could recruit a full fleet to resupply&lt;EM4&gt; {0} with salvaged materials.&lt;/EM4&gt; It would go a long way in helping us rebuild what was lost in the attacks.\n\nI leave it up to you to decide how best to acquire what we need, but should be able to find some wrecks to scavenge orbiting around most planets.\n\nYour support of our efforts is much appreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Tras el brutal ataque a Pyro y nuestros esfuerzos por combatir al grupo paramilitar Frontier Fighters, nuestras reservas estratégicas en todo el sistema se encuentran en su nivel más bajo. Ciudadanos por la Prosperidad están ansiosos por reponer nuestras reservas antes de que lleguemos a una situación desesperada. \n\nCon ese fin, esperábamos que pudieras reclutar una flota completa para reabastecer&lt;EM4&gt; {0} con materiales recuperados.&lt;/EM4&gt; Sería de gran ayuda para reconstruir lo que se perdió en los ataques.\n\nTe dejo a ti la decisión de cómo adquirir mejor lo que necesitamos, pero deberías poder encontrar algunos restos de naves para saquear orbitando alrededor de la mayoría de los planetas.\n\nAgradecemos mucho tu apoyo a nuestros esfuerzos.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Following the brutal attack on Pyro and our efforts to combat the vigilante group the Frontier Fighters, our strategic reserves across the system are at an all-time low. Citizens for Prosperity are eager to replenish our stocks before we reach a point of desperation. \n\nTo that end, we were hoping that you and a team of your choosing could resupply&lt;EM4&gt; {0} with salvaged materials.&lt;/EM4&gt; It would go a long way in helping us rebuild what was lost in the attacks.\n\nI leave it up to you to decide how best to acquire what we need, but should be able to find some wrecks to scavenge orbiting around most planets. \n\nYour support of our efforts is much appreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Tras el brutal ataque a Pyro y nuestros esfuerzos por combatir al grupo justiciero Frontier Fighters, nuestras reservas estratégicas en todo el sistema están en su nivel más bajo. Ciudadanos por la Prosperidad están ansiosos por reabastecer nuestras existencias antes de que lleguemos a un punto de desesperación. \n\nCon ese fin, esperábamos que usted y un equipo de su elección pudieran reabastecer&lt;EM4&gt; {0} con materiales recuperados.&lt;/EM4&gt; Sería de gran ayuda para reconstruir lo que se perdió en los ataques.\n\nLe dejo a usted la decisión de cómo obtener mejor lo que necesitamos, pero debería poder encontrar algunos restos de naves para saquear orbitando alrededor de la mayoría de los planetas. \n\nAgradecemos enormemente su apoyo a nuestros esfuerzos,\n\nLima Endicott\nOperadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Kicking the crap out of those Frontier Fighter bastards seriously depleted our supplies and now our stash of resources is practically out of stock. \n\nThat’s why you’re going to do a resupply run to&lt;EM4&gt; {0} &lt;/EM4&gt;\n\nUp to you how you get the stuff. Mine it, steal it, buy it from a trader - I don’t care as long as I get what I need refined and delivered. Might be worth checking the asteroid clusters near LaGrange points to start.\n\nI’m trustin’ you to get it done,\nStows  \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Darles una paliza a esos bastardos de Frontier Fighter agotó seriamente nuestros suministros y ahora nuestras reservas de recursos están prácticamente agotadas. \n\nPor eso vas a hacer una misión de reabastecimiento a &lt;EM4&gt; {0} &lt;/EM4&gt;\n\nTú decides cómo conseguir las cosas. Mínalas, róbalas, cómpralas a un comerciante; no me importa con tal de obtener lo que necesito refinado y entregado. Quizás valga la pena revisar los cúmulos de asteroides cerca de los puntos de Lagrange para empezar.\n\nConfío en que lo harás,\nStows \n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Kicking the crap out of those Frontier Fighter bastards seriously depleted our supplies and now our stash of resources is practically out of stock. \n\nThat’s why you and whoever else you want to bring along are going to do a resupply run to&lt;EM4&gt; {0} &lt;/EM4&gt;\n\nUp to you how you get the stuff. Mine it, steal it, buy it from a trader - I don’t care as long as I get what I need refined and delivered. Might be worth checking the asteroid clusters near LaGrange points to start.\n\nI’m trustin’ you to get it done,\nStows  \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Darles una paliza a esos bastardos de Frontier Fighter agotó seriamente nuestros suministros y ahora nuestras reservas de recursos están prácticamente agotadas. \n\nPor eso tú y quien quieras traer contigo van a hacer una misión de reabastecimiento a &lt;EM4&gt; {0} &lt;/EM4&gt;\n\nTú decides cómo conseguir las cosas. Mínalas, róbalas, cómpralas a un comerciante; no me importa con tal de obtener lo que necesito refinado y entregado. Quizás valga la pena revisar los cúmulos de asteroides cerca de los puntos de Lagrange para empezar.\n\nConfío en que lo harás,\nStows \n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Kicking the crap out of those Frontier Fighter bastards seriously depleted our supplies and now our stash of resources is practically out of stock. \n\nThat’s why you’re going to put together a full fleet to do a resupply run to&lt;EM4&gt; {0} &lt;/EM4&gt;\n\nUp to you how you get the stuff. Mine it, steal it, buy it from a trader - I don’t care as long as I get what I need refined and delivered. Might be worth checking the asteroid clusters near LaGrange points to start.\n\nI’m trustin’ you to get it done,\nStows  \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Darles una paliza a esos bastardos de Frontier Fighter agotó seriamente nuestros suministros y ahora nuestras reservas de recursos están prácticamente agotadas. \n\nPor eso vas a reunir una flota completa para hacer una misión de reabastecimiento a &lt;EM4&gt; {0} &lt;/EM4&gt;\n\nTú decides cómo conseguir las cosas. Mínalas, róbalas, cómpralas a un comerciante; no me importa con tal de obtener lo que necesito refinado y entregado. Quizás valga la pena revisar los cúmulos de asteroides cerca de los puntos de Lagrange para empezar.\n\nConfío en que lo harás,\nStows \n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Kicking the crap out of those Frontier Fighter bastards seriously depleted our supplies and now our stash of resources is practically out of stock. \n\nThat’s why you’re going to drop off the supplies at&lt;EM4&gt; {0} &lt;/EM4&gt;I have ship waiting to take it to Pyro from there.\n\nUp to you how you get the stuff. Mine it, steal it, buy it from a trader - I don’t care as long as I get what I need refined and delivered. Might be worth checking Daymar or Aberdeen to start.\n\nI’m trustin’ you to get it done,\nStows  \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400</v>
+        <v>Darles una paliza a esos bastardos de Frontier Fighter agotó seriamente nuestros suministros y ahora nuestras reservas de recursos están prácticamente agotadas. \n\nPor eso vas a dejar los suministros en &lt;EM4&gt; {0} &lt;/EM4&gt;. Tengo una nave esperando para llevarlos a Pyro desde allí.\n\nTú decides cómo conseguir las cosas. Mínalas, róbalas, cómpralas a un comerciante; no me importa con tal de obtener lo que necesito refinado y entregado. Quizás valga la pena revisar Daymar o Aberdeen para empezar.\n\nConfío en que lo harás,\nStows \n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Kicking the crap out of those Frontier Fighter bastards seriously depleted our supplies and now our stash of resources is practically out of stock. \n\nThat’s why you and whoever else you want to bring along are going to drop off the supplies at&lt;EM4&gt; {0} &lt;/EM4&gt;I have ship waiting to take it to Pyro from there.\n\nUp to you how you get the stuff. Mine it, steal it, buy it from a trader - I don’t care as long as I get what I need refined and delivered. Might be worth checking Daymar or Aberdeen to start.\n\nI’m trustin’ you to get it done,\nStows  \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400</v>
+        <v>Darles una paliza a esos bastardos de Frontier Fighter agotó seriamente nuestros suministros y ahora nuestras reservas de recursos están prácticamente agotadas. \n\nPor eso tú y quien quieras traer van a dejar los suministros en &lt;EM4&gt; {0} &lt;/EM4&gt;Tengo una nave esperando para llevarlos a Pyro desde allí.\n\nDepende de ti cómo consigas las cosas. Mínalas, róbalas, cómpralas a un comerciante; no me importa con tal de obtener lo que necesito refinado y entregado. Quizás valga la pena revisar Daymar o Aberdeen para empezar.\n\nConfío en que lo harás,\nStows \n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Kicking the crap out of those Frontier Fighter bastards seriously depleted our supplies and now our stash of resources is practically out of stock. \n\nThat’s why you’re going to put together a full fleet to deliver the supplies to&lt;EM4&gt; {0} &lt;/EM4&gt;I have ship waiting to take it to Pyro from there.\n\nUp to you how you get the stuff. Mine it, steal it, buy it from a trader - I don’t care as long as I get what I need refined and delivered. Might be worth checking Daymar or Aberdeen to start.\n\nI’m trustin’ you to get it done,\nStows  \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400</v>
+        <v>Darles una paliza a esos bastardos de Frontier Fighter agotó seriamente nuestros suministros y ahora nuestras reservas de recursos están prácticamente agotadas. \n\nPor eso vas a reunir una flota completa para entregar los suministros a &lt;EM4&gt; {0} &lt;/EM4&gt;. Tengo una nave esperando para llevarlos a Pyro desde allí.\n\nTú decides cómo conseguir las cosas. Mínalas, róbalas, cómpralas a un comerciante; no me importa con tal de obtener lo que necesito refinado y entregado. Quizás valga la pena revisar Daymar o Aberdeen para empezar.\n\nConfío en que lo harás,\nStows \n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Kicking the crap out of those Frontier Fighter bastards seriously depleted our supplies and now our stash is practically out of stock. \n\nThat’s why you’re going to do a resupply run to&lt;EM4&gt; {0} and bring them the salvaged materials. &lt;/EM4&gt;\n\nScrap it yourself or take it off some unsuspecting scav. Should be able to find some wrecks orbiting around most planets. Your call. Either way, as soon as we get the supplies, we’ll put it to good use building back up everything we lost.\n\nI’m trustin’ you to get it done,\nStows  \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Darles una paliza a esos bastardos de Frontier Fighter agotó seriamente nuestros suministros y ahora nuestro alijo está prácticamente vacío. \n\nPor eso vas a hacer una misión de reabastecimiento a &lt;EM4&gt; {0} y traerles los materiales recuperados. &lt;/EM4&gt;\n\nDesguazalo tú mismo o quítaselo a algún carroñero desprevenido. Deberías poder encontrar algunos restos orbitando alrededor de la mayoría de los planetas. Tú decides. De cualquier manera, tan pronto como tengamos los suministros, les daremos un buen uso para reconstruir todo lo que perdimos.\n\nConfío en que lo harás,\nStows \n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Kicking the crap out of those Frontier Fighter bastards seriously depleted our supplies and now our stash is practically out of stock. \n\nThat’s why you’re going to put together a full fleet to do a resupply run to&lt;EM4&gt; {0} and bring them the salvaged materials. &lt;/EM4&gt;\n\nScrap it yourself or take it off some unsuspecting scav. Should be able to find some wrecks orbiting around most planets. Your call. Either way, as soon as we get the supplies, we’ll put it to good use building back up everything we lost.\n\nI’m trustin’ you to get it done,\nStows  \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Darles una paliza a esos bastardos de Frontier Fighter agotó seriamente nuestros suministros y ahora nuestras reservas están prácticamente agotadas. \n\nPor eso vas a reunir una flota completa para hacer una misión de reabastecimiento a &lt;EM4&gt; {0} y traerles los materiales recuperados. &lt;/EM4&gt;\n\nDesguazalo tú mismo o quítaselo a algún carroñero desprevenido. Deberías poder encontrar algunos restos orbitando alrededor de la mayoría de los planetas. Tú decides. De cualquier manera, tan pronto como tengamos los suministros, les daremos un buen uso para reconstruir todo lo que perdimos.\n\nConfío en que lo harás,\nStows \n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Kicking the crap out of those Frontier Fighter bastards seriously depleted our supplies and now our stash is practically out of stock. \n\nThat’s why you and whoever else you want to bring along are going to do a resupply run to&lt;EM4&gt; {0} and bring them the salvaged materials. &lt;/EM4&gt;\n\nScrap it yourself or take it off some unsuspecting scav. Should be able to find some wrecks orbiting around most planets. Your call. Either way, as soon as we get the supplies, we’ll put it to good use building back up everything we lost.\n\nI’m trustin’ you to get it done,\nStows out\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; -190,500 / 400 / 2,400</v>
+        <v>Darles una paliza a esos bastardos de Frontier Fighter agotó seriamente nuestros suministros y ahora nuestro alijo está prácticamente vacío. \n\nPor eso tú y quien quieras traer contigo haréis una misión de reabastecimiento a &lt;EM4&gt; {0} y les traeréis los materiales recuperados. &lt;/EM4&gt;\n\nDesguazadlo vosotros mismos o quitárselo a algún carroñero desprevenido. Deberíais poder encontrar algunos restos orbitando alrededor de la mayoría de los planetas. Tú decides. En cualquier caso, en cuanto tengamos los suministros, les daremos un buen uso para reconstruir todo lo que perdimos.\n\nConfío en que lo conseguiréis.\nStows se despide\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; -190.500 / 400 / 2.400</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>To all available contractors,\n\nRayari scientists are hard at work trying to solve the issues with failing regen tech. Currently, their efforts are hindered by a lack of materials which they believe could be essential for their experiments.  \n\nIn particular, our scientists at &lt;EM4&gt;{0} have had to put their work on hold after running out of those resources. With a restock from our normal provider not possible for months owing to short supply, we’ll pay a premium to anyone who can assist with restocking the materials.\n\nFor more information on the animals in question, refer to "Explorer's Guide to Harvestables" in your Journal.\n\nTogether we can make the universe better for all.\n\nNarina Lerrem\nSenior Manager\nClinical Research Outsourcing\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 200\n&lt;EM4&gt;Multiple Blueprint Pools (Yormandi Eye Only)&lt;/EM4&gt;\n&lt;EM4&gt;Pool 1&lt;/EM4&gt;\n- P8-AR Rifle\n- Palatino Arms\n- Palatino Core\n- Palatino Legs\n- Palatino Helmet\n- Palatino Arms Moonfall\n- Palatino Core Moonfall\n- Palatino Legs Moonfall\n- Palatino Helmet Moonfall\n- P8-ARM Rifle Magazine (30 cap)\n\n&lt;EM4&gt;Pool 2&lt;/EM4&gt;\n- Prism "Deep Sea" Laser Shotgun\n- Prism "Bonedust" Laser Shotgun\n- Prism "Firesteel" Laser Shotgun\n- Prism Laser Shotgun\n- Stirling Exploration Suit\n- Siebe Helmet\n- Prism Laser Shotgun Battery (20 cap)\n</v>
+        <v> todos los contratistas disponibles:\n\nLos científicos de Rayari están trabajando arduamente para resolver los problemas con la tecnología de regeneración defectuosa. Actualmente, sus esfuerzos se ven obstaculizados por la falta de materiales que consideran esenciales para sus experimentos.\n\nEn particular, nuestros científicos en &lt;EM4&gt;{0} han tenido que suspender su trabajo tras agotarse dichos recursos. Dado que no será posible reabastecernos de nuestro proveedor habitual durante meses debido a la escasez de suministros, pagaremos una prima a cualquiera que pueda ayudarnos a reabastecer los materiales.\n\nPara obtener más información sobre los animales en cuestión, consulte la "Guía del explorador para la recolección" en su Diario.\n\nJuntos podemos hacer del universo un lugar mejor para todos.\n\nNarina Lerrem\nGerente sénior\nSubcontratación de investigación clínica\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 200\n&lt;EM4&gt;Múltiples grupos de planos (solo ojo de Yormandi)&lt;/EM4&gt;\n&lt;EM4&gt;Grupo 1&lt;/EM4&gt;\n- Rifle P8-AR\n- Brazos Palatino\n- Núcleo Palatino\n- Piernas Palatino\n- Casco Palatino\n- Caída de la Luna de Brazos Palatino\n- Caída de la Luna de Núcleo Palatino\n- Caída de la Luna de Piernas Palatino\n- Caída de la Luna de Casco Palatino\n- Cargador de rifle P8-ARM (30 cápsulas)\n\n&lt;EM4&gt;Piscina 2&lt;/EM4&gt;\n- Escopeta láser Prism "Deep Sea"\n- Escopeta láser Prism "Bonedust"\n- Escopeta láser Prism "Firesteel"\n- Escopeta láser Prism\n- Traje de exploración Stirling\n- Casco Siebe\n- Batería para escopeta láser Prism (20 cápsulas)\n</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>To all available contractors,\n\nOur research team at at &lt;EM4&gt;{0} is working tirelessly on solving the current ‘Regen Crisis’ and addressing the issue of unstable imprints. Their work has produced promising results, but a lack of a key resource is impeding their ability to run further experiments. \n\nWe’ve received word from our supplier that increased demand combined with lower mining yields means that we won’t receive our scheduled shipment for another few months. Our research team can’t wait that long, and we’re hoping you can help.      \n\nThe resource is hard to come by, but we have it on good authority that the old Hathor mining facilities were built in areas with a high concentration of the ore. Since Hathor went defunct not long after establishing their operations in- system, there’s a good chance that activating one of these mining lasers could provide you with what we need.\n\nTogether we can make the universe better for all.\n\nNarina Lerrem\nSenior Manager\nClinical Research Outsourcing\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 150\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Pulse Laser Pistol\n- Pulse "Blacklist" Pistol\n- Pulse "Rouge" Pistol\n- Quartz Energy SMG\n- Quartz "Deadfall" Energy SMG\n- Quartz "Black Op" Energy SMG\n- Quartz "Lumen" Energy SMG\n- Quartz Energy SMG Battery (45 cap)\n- Pulse Laser Pistol Battery (60 Cap)\n</v>
+        <v> todos los contratistas disponibles:\n\nNuestro equipo de investigación en &lt;EM4&gt;{0} está trabajando incansablemente para resolver la actual "Crisis de Regeneración" y abordar el problema de las impresiones inestables. Su trabajo ha producido resultados prometedores, pero la falta de un recurso clave está impidiendo su capacidad para realizar más experimentos.\n\nHemos recibido información de nuestro proveedor de que el aumento de la demanda combinado con menores rendimientos de minería significa que no recibiremos nuestro envío programado hasta dentro de unos meses. Nuestro equipo de investigación no puede esperar tanto, y esperamos que puedan ayudar.\n\nEl recurso es difícil de conseguir, pero tenemos información fidedigna de que las antiguas instalaciones mineras de Hathor se construyeron en áreas con una alta concentración del mineral. Dado que Hathor dejó de operar poco después de establecer sus operaciones en el sistema, hay una buena posibilidad de que activar uno de estos láseres mineros pueda proporcionarte lo que necesitamos.\n\nJuntos podemos hacer del universo un lugar mejor para todos.\n\nNarina Lerrem\nGerente sénior\nSubcontratación de investigación clínica\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 150\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Pistola láser de pulso\n- Pistola de pulso "Lista negra"\n- Pistola de pulso "Rouge"\n- Subfusil de energía de cuarzo\n- Subfusil de energía de cuarzo "Caída muerta"\n- Subfusil de energía de cuarzo "Operación negra"\n- Subfusil de energía de cuarzo "Lumen"\n- Batería de subfusil de energía de cuarzo (45 cap)\n- Batería de pistola láser de pulso (60 cap)\n</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>RED WIND LINEHAUL\n'YOUR GOODS IN GOOD HANDS'\n----------------------------  \n\nNeed a pilot for a straightforward haul going from the freight elevator at &lt;EM4&gt;{0} to &lt;EM4&gt;{1} Should be easy enough as long as you got a ship that can handle containers up to &lt;EM4&gt;{2} in size. \n\nCredits don't come much easier than this. Just be careful as the route's not exactly in the safest of sectors. And don't forget to pack a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; to bring along.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100 / 250 / 1,000</v>
+        <v>RED WIND LINEHAUL\n'SUS MERCANCÍAS EN BUENAS MANOS'\n---------------------------- \n\nSe necesita un piloto para un transporte directo desde el montacargas en &lt;EM4&gt;{0} hasta &lt;EM4&gt;{1}. Debería ser bastante fácil siempre que tengas una nave que pueda manejar contenedores de hasta &lt;EM4&gt;{2} de tamaño. \n\nLos créditos no se consiguen más fácilmente que esto. Solo ten cuidado, ya que la ruta no está precisamente en los sectores más seguros. Y no olvides llevar contigo un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt;.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100 / 250 / 1000</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>RED WIND LINEHAUL\n'YOUR GOODS IN GOOD HANDS'\n----------------------------  \n\nNeed a pilot for a waste material transfer going from the freight elevator at &lt;EM4&gt;{0} to &lt;EM4&gt;{1} Should be easy enough as long as you got a ship that can handle containers up to &lt;EM4&gt;{2} in size. Wouldn't bring your cleanest ship either.\n\nOn the bright side though, most likely outlaws will leave you alone when they see what you're carrying. And don't forget to pack a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; to bring along.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 250 / 1,000</v>
+        <v>RED WIND LINEHAUL\n'SUS MERCANCÍAS EN BUENAS MANOS'\n---------------------------- \n\nSe necesita un piloto para una transferencia de material de desecho desde el montacargas en &lt;EM4&gt;{0} hasta &lt;EM4&gt;{1}. Debería ser bastante fácil siempre que tengas una nave que pueda manejar contenedores de hasta &lt;EM4&gt;{2} de tamaño. Tampoco traerías tu nave más limpia.\n\nPor otro lado, lo más probable es que los forajidos te dejen en paz cuando vean lo que transportas. Y no olvides empacar un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt; para llevar contigo.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 250 / 1000</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>RED WIND LINEHAUL\n'YOUR GOODS IN GOOD HANDS'\n----------------------------\n\nJust got off a comm with a client. They got cargo (&lt;EM4&gt;{0} or smaller) at a few different locations ready to be taken over to a freight elevator at &lt;EM4&gt;{1} UP LOCATIONS (ANY ORDER)  \n{2}  \n\nI'd recommend taking a few minutes to plan your route before taking off. Might save you a bit of fuel. And don't forget to pack a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; to bring along.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 250 / 500 / 1,000 / 2,000 / 4,000</v>
+        <v>RED WIND LINEHAUL\n'SUS MERCANCÍAS EN BUENAS MANOS'\n----------------------------\n\nAcabo de terminar una comunicación con un cliente. Tienen carga (&lt;EM4&gt;{0} o más pequeña) en varias ubicaciones, lista para ser transportada a un montacargas en &lt;EM4&gt;{1} UBICACIONES ARRIBA (CUALQUIER ORDEN) \n{2} \n\nRecomiendo tomarse unos minutos para planificar la ruta antes de partir. Podría ahorrarle algo de combustible. Y no olvide llevar un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt;.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 250 / 500 / 1000 / 2000 / 4000</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>RED WIND LINEHAUL\n'YOUR GOODS IN GOOD HANDS'\n----------------------------\n\nGot a bunch of comms this morning. Seems one of the local trash collectors' ship is busted and we're gonna be picking up the slack.\n\nI got a bunch of trash (&lt;EM4&gt;{0} or smaller) at a few different locations ready to be taken over to a freight elevator at &lt;EM4&gt;{1} UP LOCATIONS (ANY ORDER)  \n{2} don't forget to pack a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; to bring along.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 250 / 500 / 2,000 / 4,000</v>
+        <v>RED WIND LINEHAUL\n'SUS MERCANCÍAS EN BUENAS MANOS'\n----------------------------\n\nHe recibido varias comunicaciones esta mañana. Parece que la nave de uno de los recolectores de basura locales está averiada y vamos a encargarnos del trabajo.\n\nTengo un montón de basura (&lt;EM4&gt;{0} o más pequeña) en varias ubicaciones, lista para ser llevada a un montacargas en &lt;EM4&gt;{1} UBICACIONES ARRIBA (CUALQUIER ORDEN) \n{2} No olvides empacar un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt; para llevar contigo.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 250 / 500 / 2000 / 4000</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>RED WIND LINEHAUL\n'YOUR GOODS IN GOOD HANDS'\n----------------------------   \n\nOne of the folks over at &lt;EM4&gt;{0} just hit me up about a pile of cargo, &lt;EM4&gt;{1} or smaller, that needs to be hauled out to a few different spots.   \n\nDROP OFF LOCATIONS (ANY ORDER)  \n{2}  \n\nI'm trusting you to set your own route here, so don't mess it up. And try to stay away from anywhere too dangerous. And don't forget to pack a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; to bring along.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100 / 250 / 500</v>
+        <v>RED WIND LINEHAUL\n'SUS MERCANCÍAS EN BUENAS MANOS'\n---------------------------- \n\nUna persona de &lt;EM4&gt;{0} me contactó recientemente sobre un montón de carga, &lt;EM4&gt;{1} o más pequeña, que necesita ser transportada a varios lugares. \n\nUBICACIONES DE ENTREGA (EN CUALQUIER ORDEN) \n{2} \n\nConfío en que establezcas tu propia ruta, así que no la arruines. Y trata de mantenerte alejado de cualquier lugar demasiado peligroso. Y no olvides empacar un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt; para llevar contigo.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100 / 250 / 500</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>RED WIND LINEHAUL\n'YOUR GOODS IN GOOD HANDS'\n----------------------------   \n\nThey're doing a clean out at &lt;EM4&gt;{0} and have a bunch of &lt;EM4&gt;{1} or smaller waste containers that needs to be hauled out to a few different spots. (Don't ask me why. They're paying us is all I know.)\n\nDROP OFF LOCATIONS (ANY ORDER)  \n{2} don't forget to pack a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; to bring along.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 500 / 1,000 / 2,000 / 4,000</v>
+        <v>RED WIND LINEHAUL\n'SUS MERCANCÍAS EN BUENAS MANOS'\n---------------------------- \n\nEstán haciendo una limpieza en &lt;EM4&gt;{0} y tienen un montón de contenedores de basura &lt;EM4&gt;{1} o más pequeños que necesitan ser transportados a varios lugares. (No me pregunten por qué. Solo sé que nos están pagando).\n\nPUNTOS DE ENTREGA (EN CUALQUIER ORDEN) \n{2} No olvides empacar un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt; para llevar contigo.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 500 / 1000 / 2000 / 4000</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>RED WIND LINEHAUL\n'YOUR GOODS IN GOOD HANDS'\n----------------------------\n\nPutting out a call for a highly skilled pilot who can recover our client’s cargo. Please only accept this contract if you have experience dealing with extremely hostile situations involving multiple combatants. Additional crew members and a &lt;EM4&gt;heavy-duty tractor beam&lt;/EM4&gt; are highly recommended.\n\nRECOVERY LOCATION\n     · &lt;EM4&gt;{0} OFF LOCATION\n     · Freight elevator at &lt;EM4&gt;{1} cargo should be in the bay of the abandoned ship. The client has already expressed frustration regarding the cargo’s delay so please work quickly and efficiently.\n\nBE RESILIENT – Life is hard and sometimes you have to roll with the punches. Keep going and don’t let it bring you down.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>RED WIND LINEHAUL\n'SUS MERCANCÍAS EN BUENAS MANOS'\n----------------------------\n\nSe solicita un piloto altamente capacitado para recuperar la carga de nuestro cliente. Solo acepte este contrato si tiene experiencia en situaciones extremadamente hostiles con múltiples combatientes. Se recomienda encarecidamente contar con tripulación adicional y un &lt;EM4&gt;rayo tractor de alta resistencia&lt;/EM4&gt;.\n\nUBICACIÓN DE RECUPERACIÓN\n · &lt;EM4&gt;{0} UBICACIÓN FUERA DE LA UBICACIÓN\n · El elevador de carga en &lt;EM4&gt;{1} debe estar en la bahía del barco abandonado. El cliente ya ha expresado su frustración por el retraso de la carga, así que trabaje con rapidez y eficiencia.\n\nSEA RESILIENTE: la vida es dura y a veces hay que adaptarse a las circunstancias. Siga adelante y no deje que le afecte.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for rare materials. We appreciate your help in this matter.\n\nThere are only a few known locations where these materials can be sourced, mainly from now defunct Hathor Group sites on &lt;EM4&gt;Daymar and Aberdeen&lt;/EM4&gt;. Our suggestion would be to head to the Platform Alignment Facilities (PAF) and attempt to reactivate their Orbital Laser Platform (OLP) to access the materials below the planet's surface.\n\nReminder, since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{1} you’re ready to sell us the required materials, deposit them in the freight elevator located at &lt;EM4&gt;{2} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de materiales raros. Agradecemos su ayuda en este asunto.\n\nSolo se conocen algunas ubicaciones donde se pueden obtener estos materiales, principalmente de los sitios ahora desaparecidos del Grupo Hathor en &lt;EM4&gt;Daymar y Aberdeen&lt;/EM4&gt;. Nuestra sugerencia sería dirigirse a las Instalaciones de Alineación de Plataformas (PAF) e intentar reactivar su Plataforma Láser Orbital (OLP) para acceder a los materiales debajo de la superficie del planeta.\n\nRecordatorio, dado que esta es una orden de compra y no un contrato de minería, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{1}. Cuando esté listo para vendernos los materiales requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{2}. Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for rare materials. We appreciate your help in this matter.\n\nThere are only a few known locations where these materials can be sourced, mainly from now defunct Hathor Group sites on &lt;EM4&gt;Daymar and Aberdeen&lt;/EM4&gt;. Our suggestion would be to head to the Platform Alignment Facilities (PAF) and attempt to reactivate their Orbital Laser Platform (OLP) to access the materials below the planet's surface.\n\nReminder, since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{1} you’re ready to sell us the required materials, deposit them in the freight elevator located at &lt;EM4&gt;{2} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de materiales raros. Agradecemos su ayuda en este asunto.\n\nSolo se conocen algunas ubicaciones donde se pueden obtener estos materiales, principalmente de los sitios ahora desaparecidos del Grupo Hathor en &lt;EM4&gt;Daymar y Aberdeen&lt;/EM4&gt;. Nuestra sugerencia sería dirigirse a las Instalaciones de Alineación de Plataformas (PAF) e intentar reactivar su Plataforma Láser Orbital (OLP) para acceder a los materiales debajo de la superficie del planeta.\n\nRecordatorio, dado que esta es una orden de compra y no un contrato de minería, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{1}. Cuando esté listo para vendernos los materiales requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{2}. Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for rare materials. We appreciate your help in this matter.\n\nThere are only a few known locations where these materials can be sourced, mainly from now defunct Hathor Group sites on &lt;EM4&gt;Daymar and Aberdeen&lt;/EM4&gt;. Our suggestion would be to head to the Platform Alignment Facilities (PAF) and attempt to reactivate their Orbital Laser Platform (OLP) to access the materials below the planet's surface.\n\nReminder, since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{1} you’re ready to sell us the required materials, deposit them in the freight elevator located at &lt;EM4&gt;{2} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de materiales raros. Agradecemos su ayuda en este asunto.\n\nSolo se conocen algunas ubicaciones donde se pueden obtener estos materiales, principalmente de los sitios ahora desaparecidos del Grupo Hathor en &lt;EM4&gt;Daymar y Aberdeen&lt;/EM4&gt;. Nuestra sugerencia sería dirigirse a las Instalaciones de Alineación de Plataformas (PAF) e intentar reactivar su Plataforma Láser Orbital (OLP) para acceder a los materiales debajo de la superficie del planeta.\n\nRecordatorio, dado que esta es una orden de compra y no un contrato de minería, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{1}. Cuando esté listo para vendernos los materiales requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{2}. Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTECH PREVIEW TESTING:\nComplete this mission to get blueprints for Volt weapons. For this test, these blueprints have some slots that accepting different materials for varying stat adjustments.\n\n{1} For a comprehensive list of where to find these minerals, consult &lt;EM4&gt;Mining Fundamentals #2: Where to Mine&lt;/EM4&gt; in your mobiGlas Journal. While you're there, feel free to read the first part &lt;EM4&gt;Mining Fundamentals #1: Basic Overview&lt;/EM4&gt; if you want a refresher on how to get the materials.\n\nSince this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{2} you’re ready to sell us the required materials, deposit them in the freight elevator located at &lt;EM4&gt;{3} Awarded:&lt;/EM4&gt; 100\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Patch City, Patch City Clinic, Checkmate Clinic&lt;/EM4&gt;\n- Arclight "Herrero" Pistol\n- Arclight "Desert Shadow" Pistol\n- Pembroke Exploration Suit\n- Pembroke Helmet\n- Novikov Exploration Suit\n- Novikov Helmet\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Aberdeen, Arial, Ita&lt;/EM4&gt;\n- Arclight "Midnight" Pistol\n- Strata Arms\n- Strata Core\n- Strata Legs\n- Strata Helmet Shooting Star\n- Arclight Pistol Battery (30 cap)\n</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nPRUEBA DE VISTA PREVIA TECNOLÓGICA:\nCompleta esta misión para obtener planos de armas Volt. Para esta prueba, estos planos tienen algunas ranuras que aceptan diferentes materiales para ajustes de estadísticas variables.\n\n{1} Para obtener una lista completa de dónde encontrar estos minerales, consulta &lt;EM4&gt;Fundamentos de minería n.° 2: Dónde minar&lt;/EM4&gt; en tu diario mobiGlas. Mientras estés allí, no dudes en leer la primera parte &lt;EM4&gt;Fundamentos de minería n.° 1: Descripción general básica&lt;/EM4&gt; si quieres repasar cómo obtener los materiales.\n\nDado que se trata de una orden de compra y no de un contrato de minería, se espera que proporciones tu propio equipo, como un &lt;EM4&gt;{2}. Cuando estés listo para vendernos los materiales requeridos, deposítalos en el montacargas ubicado en &lt;EM4&gt;{3}. Otorgado:&lt;/EM4&gt; 100\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Patch City, Patch City Clinic, Checkmate Clinic&lt;/EM4&gt;\n- Pistola Arclight "Herrero"\n- Pistola Arclight "Desert Shadow"\n- Traje de exploración Pembroke\n- Casco Pembroke\n- Traje de exploración Novikov\n- Casco Novikov\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Aberdeen, Arial, Ita&lt;/EM4&gt;\n- Pistola Arclight "Midnight"\n- Brazos Strata\n- Núcleo Strata\n- Piernas Strata\n- Casco Strata Shooting Star\n- Batería para pistola Arclight (30 cápsulas)\n</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for a variety of refined materials. We appreciate your help in this matter.\n\n{1} Many of these ores are extremely rare and difficult to find, detectable only when a rock has been cracked open.\n\nReminder, all the &lt;EM4&gt;materials must be refined before delivery&lt;/EM4&gt;, and since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{2} you’re ready to sell us the required refined materials, deposit them in the freight elevator located at &lt;EM4&gt;{3} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Multiple Blueprint Pools&lt;/EM4&gt;\n&lt;EM4&gt;Pool 1&lt;/EM4&gt;\n- Arclight "Stormfall" Pistol\n- Arclight Pistol\n- Venture Arms Base\n- Venture Core Base\n- Venture Legs Base\n- Horizon Helmet Base\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;Pool 2&lt;/EM4&gt;\n- Arbor MHV Mining Laser (Mining Laser)\n- S00 Hofstede (Mining Laser)\n- Lawson Mining Laser (Mining Laser)\n- S0 Helix (Mining Laser)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Pitman Mining Laser (Mining Laser)\n- Hofstede-S1 Mining Laser (Mining Laser)\n- Klein-S1 Mining Laser (Mining Laser)\n- Helix I Mining Laser (Mining Laser)\n- Impact I Mining Laser (Mining Laser)\n- Arbor MH1 Mining Laser (Mining Laser)\n- Lancet MH1 Mining Laser (Mining Laser)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Arbor MH2 Mining Laser (Mining Laser)\n- Lancet MH2 Mining Laser (Mining Laser)\n- Hofstede-S2 Mining Laser (Mining Laser)\n- Klein-S2 Mining Laser (Mining Laser)\n- Helix II Mining Laser (Mining Laser)\n- Impact II Mining Laser (Mining Laser)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de una variedad de materiales refinados. Agradecemos su ayuda en este asunto.\n\n{1} Muchos de estos minerales son extremadamente raros y difíciles de encontrar, detectables solo cuando una roca se ha abierto.\n\nRecordatorio: todos los &lt;EM4&gt;materiales deben refinarse antes de la entrega&lt;/EM4&gt;, y dado que se trata de una orden de compra y no de un contrato de minería, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{2} cuando esté listo para vendernos los materiales refinados requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{3} Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Múltiples grupos de planos&lt;/EM4&gt;\n&lt;EM4&gt;Grupo 1&lt;/EM4&gt;\n- Pistola Arclight "Stormfall"\n- Pistola Arclight\n- Base de brazos Venture\n- Base de núcleo Venture\n- Base de piernas Venture\n- Base de casco Horizon\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;Grupo 2&lt;/EM4&gt;\n- Láser minero Arbor MHV (Láser minero)\n- S00 Hofstede (Láser minero)\n- Láser minero Lawson (Láser minero)\n- S0 Helix (Láser minero)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Láser minero Pitman (Láser minero)\n- Láser minero Hofstede-S1 (Láser minero)\n- Láser minero Klein-S1 (Láser minero)\n- Láser minero Helix I (Láser minero)\n- Láser minero Impact I (Láser minero)\n- Láser minero Arbor MH1 (Láser minero)\n- Láser minero Lancet MH1 (Láser minero)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Láser de minería Arbor MH2 (Láser de minería)\n- Láser de minería Lancet MH2 (Láser de minería)\n- Láser de minería Hofstede-S2 (Láser de minería)\n- Láser de minería Klein-S2 (Láser de minería)\n- Láser de minería Helix II (Láser de minería)\n- Láser de minería Impact II (Láser de minería)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for a variety of refined materials. We appreciate your help in this matter.\n\n{1} all the &lt;EM4&gt;materials must be refined before delivery&lt;/EM4&gt;, and since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{2} you’re ready to sell us the required refined materials, deposit them in the freight elevator located at &lt;EM4&gt;{3} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Multiple Blueprint Pools&lt;/EM4&gt;\n&lt;EM4&gt;Pool 1&lt;/EM4&gt;\n- Arclight "Stormfall" Pistol\n- Arclight Pistol\n- Venture Arms Base\n- Venture Core Base\n- Venture Legs Base\n- Horizon Helmet Base\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;Pool 2&lt;/EM4&gt;\n- Arbor MHV Mining Laser (Mining Laser)\n- S00 Hofstede (Mining Laser)\n- Lawson Mining Laser (Mining Laser)\n- S0 Helix (Mining Laser)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Pitman Mining Laser (Mining Laser)\n- Hofstede-S1 Mining Laser (Mining Laser)\n- Klein-S1 Mining Laser (Mining Laser)\n- Helix I Mining Laser (Mining Laser)\n- Impact I Mining Laser (Mining Laser)\n- Arbor MH1 Mining Laser (Mining Laser)\n- Lancet MH1 Mining Laser (Mining Laser)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Arbor MH2 Mining Laser (Mining Laser)\n- Lancet MH2 Mining Laser (Mining Laser)\n- Hofstede-S2 Mining Laser (Mining Laser)\n- Klein-S2 Mining Laser (Mining Laser)\n- Helix II Mining Laser (Mining Laser)\n- Impact II Mining Laser (Mining Laser)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de una variedad de materiales refinados. Agradecemos su ayuda en este asunto.\n\n{1} Todos los &lt;EM4&gt;materiales deben ser refinados antes de la entrega&lt;/EM4&gt;, y dado que se trata de una orden de compra y no de un contrato de minería, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{2} Cuando esté listo para vendernos los materiales refinados requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{3} Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Múltiples grupos de planos&lt;/EM4&gt;\n&lt;EM4&gt;Grupo 1&lt;/EM4&gt;\n- Pistola Arclight "Stormfall"\n- Pistola Arclight\n- Base de brazos Venture\n- Base de núcleo Venture\n- Base de piernas Venture\n- Base de casco Horizon\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;Grupo 2&lt;/EM4&gt;\n- Láser de minería Arbor MHV (Láser de minería)\n- S00 Hofstede (Minería Láser)\n- Lawson Mining Laser (Láser de Minería)\n- S0 Helix (Láser de Minería)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Pitman Mining Laser (Láser de Minería)\n- Hofstede-S1 Mining Laser (Láser de Minería)\n- Klein-S1 Mining Laser (Láser de Minería)\n- Helix I Mining Laser (Láser de Minería)\n- Impact I Mining Laser (Láser de Minería)\n- Arbor MH1 Mining Laser (Láser de Minería)\n- Lancet MH1 Mining Laser (Láser de Minería)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Arbor Láser minero MH2 (Láser minero)\n- Láser minero Lancet MH2 (Láser minero)\n- Láser minero Hofstede-S2 (Láser minero)\n- Láser minero Klein-S2 (Láser minero)\n- Láser minero Helix II (Láser minero)\n- Láser minero Impact II (Láser minero)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for a variety of refined materials. We appreciate your help in this matter.\n\n{1} Many of these ores are extremely rare and difficult to find, detectable only when a rock has been cracked open.\n\nReminder, all the &lt;EM4&gt;materials must be refined before delivery&lt;/EM4&gt;, and since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{2} you’re ready to sell us the required refined materials, deposit them in the freight elevator located at &lt;EM4&gt;{3} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Multiple Blueprint Pools&lt;/EM4&gt;\n&lt;EM4&gt;Pool 1&lt;/EM4&gt;\n- Arclight "Stormfall" Pistol\n- Arclight Pistol\n- Venture Arms Base\n- Venture Core Base\n- Venture Legs Base\n- Horizon Helmet Base\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;Pool 2&lt;/EM4&gt;\n- Arbor MHV Mining Laser (Mining Laser)\n- S00 Hofstede (Mining Laser)\n- Lawson Mining Laser (Mining Laser)\n- S0 Helix (Mining Laser)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Pitman Mining Laser (Mining Laser)\n- Hofstede-S1 Mining Laser (Mining Laser)\n- Klein-S1 Mining Laser (Mining Laser)\n- Helix I Mining Laser (Mining Laser)\n- Impact I Mining Laser (Mining Laser)\n- Arbor MH1 Mining Laser (Mining Laser)\n- Lancet MH1 Mining Laser (Mining Laser)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Arbor MH2 Mining Laser (Mining Laser)\n- Lancet MH2 Mining Laser (Mining Laser)\n- Hofstede-S2 Mining Laser (Mining Laser)\n- Klein-S2 Mining Laser (Mining Laser)\n- Helix II Mining Laser (Mining Laser)\n- Impact II Mining Laser (Mining Laser)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de una variedad de materiales refinados. Agradecemos su ayuda en este asunto.\n\n{1} Muchos de estos minerales son extremadamente raros y difíciles de encontrar, detectables solo cuando una roca se ha abierto.\n\nRecordatorio: todos los &lt;EM4&gt;materiales deben refinarse antes de la entrega&lt;/EM4&gt;, y dado que se trata de una orden de compra y no de un contrato de minería, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{2} cuando esté listo para vendernos los materiales refinados requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{3} Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Múltiples grupos de planos&lt;/EM4&gt;\n&lt;EM4&gt;Grupo 1&lt;/EM4&gt;\n- Pistola Arclight "Stormfall"\n- Pistola Arclight\n- Base de brazos Venture\n- Base de núcleo Venture\n- Base de piernas Venture\n- Base de casco Horizon\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;Grupo 2&lt;/EM4&gt;\n- Láser minero Arbor MHV (Láser minero)\n- S00 Hofstede (Láser minero)\n- Láser minero Lawson (Láser minero)\n- S0 Helix (Láser minero)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Láser minero Pitman (Láser minero)\n- Láser minero Hofstede-S1 (Láser minero)\n- Láser minero Klein-S1 (Láser minero)\n- Láser minero Helix I (Láser minero)\n- Láser minero Impact I (Láser minero)\n- Láser minero Arbor MH1 (Láser minero)\n- Láser minero Lancet MH1 (Láser minero)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Láser de minería Arbor MH2 (Láser de minería)\n- Láser de minería Lancet MH2 (Láser de minería)\n- Láser de minería Hofstede-S2 (Láser de minería)\n- Láser de minería Klein-S2 (Láser de minería)\n- Láser de minería Helix II (Láser de minería)\n- Láser de minería Impact II (Láser de minería)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for a variety of refined materials. We appreciate your help in this matter.\n\n{1} Many of these ores are extremely rare and difficult to find, detectable only when a rock has been cracked open.\n\nReminder, all the &lt;EM4&gt;materials must be refined before delivery&lt;/EM4&gt;, and since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{2} you’re ready to sell us the required refined materials, deposit them in the freight elevator located at &lt;EM4&gt;{3} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Multiple Blueprint Pools&lt;/EM4&gt;\n&lt;EM4&gt;Pool 1&lt;/EM4&gt;\n- Arclight "Stormfall" Pistol\n- Arclight Pistol\n- Venture Arms Base\n- Venture Core Base\n- Venture Legs Base\n- Horizon Helmet Base\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;Pool 2&lt;/EM4&gt;\n- Arbor MHV Mining Laser (Mining Laser)\n- S00 Hofstede (Mining Laser)\n- Lawson Mining Laser (Mining Laser)\n- S0 Helix (Mining Laser)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Pitman Mining Laser (Mining Laser)\n- Hofstede-S1 Mining Laser (Mining Laser)\n- Klein-S1 Mining Laser (Mining Laser)\n- Helix I Mining Laser (Mining Laser)\n- Impact I Mining Laser (Mining Laser)\n- Arbor MH1 Mining Laser (Mining Laser)\n- Lancet MH1 Mining Laser (Mining Laser)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Arbor MH2 Mining Laser (Mining Laser)\n- Lancet MH2 Mining Laser (Mining Laser)\n- Hofstede-S2 Mining Laser (Mining Laser)\n- Klein-S2 Mining Laser (Mining Laser)\n- Helix II Mining Laser (Mining Laser)\n- Impact II Mining Laser (Mining Laser)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de una variedad de materiales refinados. Agradecemos su ayuda en este asunto.\n\n{1} Muchos de estos minerales son extremadamente raros y difíciles de encontrar, detectables solo cuando una roca se ha abierto.\n\nRecordatorio: todos los &lt;EM4&gt;materiales deben refinarse antes de la entrega&lt;/EM4&gt;, y dado que se trata de una orden de compra y no de un contrato de minería, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{2} cuando esté listo para vendernos los materiales refinados requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{3} Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Múltiples grupos de planos&lt;/EM4&gt;\n&lt;EM4&gt;Grupo 1&lt;/EM4&gt;\n- Pistola Arclight "Stormfall"\n- Pistola Arclight\n- Base de brazos Venture\n- Base de núcleo Venture\n- Base de piernas Venture\n- Base de casco Horizon\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;Grupo 2&lt;/EM4&gt;\n- Láser minero Arbor MHV (Láser minero)\n- S00 Hofstede (Láser minero)\n- Láser minero Lawson (Láser minero)\n- S0 Helix (Láser minero)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Láser minero Pitman (Láser minero)\n- Láser minero Hofstede-S1 (Láser minero)\n- Láser minero Klein-S1 (Láser minero)\n- Láser minero Helix I (Láser minero)\n- Láser minero Impact I (Láser minero)\n- Láser minero Arbor MH1 (Láser minero)\n- Láser minero Lancet MH1 (Láser minero)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Láser de minería Arbor MH2 (Láser de minería)\n- Láser de minería Lancet MH2 (Láser de minería)\n- Láser de minería Hofstede-S2 (Láser de minería)\n- Láser de minería Klein-S2 (Láser de minería)\n- Láser de minería Helix II (Láser de minería)\n- Láser de minería Impact II (Láser de minería)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for a variety of refined materials. We appreciate your help in this matter.\n\n{1} Many of these ores are extremely rare and difficult to find, detectable only when a rock has been cracked open.\n\nReminder, all the &lt;EM4&gt;materials must be refined before delivery&lt;/EM4&gt;, and since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{2} you’re ready to sell us the required refined materials, deposit them in the freight elevator located at &lt;EM4&gt;{3} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Multiple Blueprint Pools&lt;/EM4&gt;\n&lt;EM4&gt;Pool 1&lt;/EM4&gt;\n- Arclight "Stormfall" Pistol\n- Arclight Pistol\n- Venture Arms Base\n- Venture Core Base\n- Venture Legs Base\n- Horizon Helmet Base\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;Pool 2&lt;/EM4&gt;\n- Arbor MHV Mining Laser (Mining Laser)\n- S00 Hofstede (Mining Laser)\n- Lawson Mining Laser (Mining Laser)\n- S0 Helix (Mining Laser)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Pitman Mining Laser (Mining Laser)\n- Hofstede-S1 Mining Laser (Mining Laser)\n- Klein-S1 Mining Laser (Mining Laser)\n- Helix I Mining Laser (Mining Laser)\n- Impact I Mining Laser (Mining Laser)\n- Arbor MH1 Mining Laser (Mining Laser)\n- Lancet MH1 Mining Laser (Mining Laser)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Arbor MH2 Mining Laser (Mining Laser)\n- Lancet MH2 Mining Laser (Mining Laser)\n- Hofstede-S2 Mining Laser (Mining Laser)\n- Klein-S2 Mining Laser (Mining Laser)\n- Helix II Mining Laser (Mining Laser)\n- Impact II Mining Laser (Mining Laser)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de una variedad de materiales refinados. Agradecemos su ayuda en este asunto.\n\n{1} Muchos de estos minerales son extremadamente raros y difíciles de encontrar, detectables solo cuando una roca se ha abierto.\n\nRecordatorio: todos los &lt;EM4&gt;materiales deben refinarse antes de la entrega&lt;/EM4&gt;, y dado que se trata de una orden de compra y no de un contrato de minería, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{2} cuando esté listo para vendernos los materiales refinados requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{3} Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Múltiples grupos de planos&lt;/EM4&gt;\n&lt;EM4&gt;Grupo 1&lt;/EM4&gt;\n- Pistola Arclight "Stormfall"\n- Pistola Arclight\n- Base de brazos Venture\n- Base de núcleo Venture\n- Base de piernas Venture\n- Base de casco Horizon\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;Grupo 2&lt;/EM4&gt;\n- Láser minero Arbor MHV (Láser minero)\n- S00 Hofstede (Láser minero)\n- Láser minero Lawson (Láser minero)\n- S0 Helix (Láser minero)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Láser minero Pitman (Láser minero)\n- Láser minero Hofstede-S1 (Láser minero)\n- Láser minero Klein-S1 (Láser minero)\n- Láser minero Helix I (Láser minero)\n- Láser minero Impact I (Láser minero)\n- Láser minero Arbor MH1 (Láser minero)\n- Láser minero Lancet MH1 (Láser minero)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Láser de minería Arbor MH2 (Láser de minería)\n- Láser de minería Lancet MH2 (Láser de minería)\n- Láser de minería Hofstede-S2 (Láser de minería)\n- Láser de minería Klein-S2 (Láser de minería)\n- Láser de minería Helix II (Láser de minería)\n- Láser de minería Impact II (Láser de minería)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for a variety of refined materials. This purchase order is more complex than typical, requiring multiple mining methods, but since you've proven your skill thus far, we think you and your team are up for the challenge.\n\nReminder, &lt;EM4&gt;materials must be refined before delivery&lt;/EM4&gt;, and since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{1} you’re ready to sell us the required materials, deposit them in the freight elevator located at &lt;EM4&gt;{2} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de una variedad de materiales refinados. Esta orden de compra es más compleja de lo habitual, ya que requiere múltiples métodos de minería, pero como has demostrado tu habilidad hasta ahora, creemos que tú y tu equipo están preparados para el desafío.\n\nRecordatorio: los &lt;EM4&gt;materiales deben refinarse antes de la entrega&lt;/EM4&gt;, y dado que se trata de una orden de compra y no de un contrato de minería, se espera que proporciones tu propio equipo, como un &lt;EM4&gt;{1}. Cuando estés listo para vendernos los materiales requeridos, deposítalos en el montacargas ubicado en &lt;EM4&gt;{2}. Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for a variety of refined materials. We appreciate your help in this matter.\n\n{1} Many of these ores are extremely rare and difficult to find, detectable only when a rock has been cracked open.\n\nReminder, all the &lt;EM4&gt;materials must be refined before delivery&lt;/EM4&gt;, and since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{2} you’re ready to sell us the required refined materials, deposit them in the freight elevator located at &lt;EM4&gt;{3} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Monox, Pyro V, Pyro IV&lt;/EM4&gt;\n- Arclight "Stormfall" Pistol\n- Arclight Pistol\n- Venture Arms Base\n- Venture Core Base\n- Venture Legs Base\n- Horizon Helmet Base\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Magda, Aberdeen, Arial&lt;/EM4&gt;\n- Arclight "Nightstalker" Pistol\n- Aril Arms\n- Aril Core\n- Aril Legs\n- Aril Helmet\n- Arclight "Warhawk" Pistol\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Pyro, Pyro V, Magda&lt;/EM4&gt;\n- Arbor MHV Mining Laser (Mining Laser)\n- S00 Hofstede (Mining Laser)\n- Lawson Mining Laser (Mining Laser)\n- S0 Helix (Mining Laser)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: Arial, Pyro IV, Magda&lt;/EM4&gt;\n- Pitman Mining Laser (Mining Laser)\n- Hofstede-S1 Mining Laser (Mining Laser)\n- Klein-S1 Mining Laser (Mining Laser)\n- Helix I Mining Laser (Mining Laser)\n- Impact I Mining Laser (Mining Laser)\n- Arbor MH1 Mining Laser (Mining Laser)\n- Lancet MH1 Mining Laser (Mining Laser)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: Pyro V, Pyro I, Arial&lt;/EM4&gt;\n- Arbor MH2 Mining Laser (Mining Laser)\n- Lancet MH2 Mining Laser (Mining Laser)\n- Hofstede-S2 Mining Laser (Mining Laser)\n- Klein-S2 Mining Laser (Mining Laser)\n- Helix II Mining Laser (Mining Laser)\n- Impact II Mining Laser (Mining Laser)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de una variedad de materiales refinados. Agradecemos su ayuda en este asunto.\n\n{1} Muchos de estos minerales son extremadamente raros y difíciles de encontrar, detectables solo cuando una roca se ha abierto.\n\nRecordatorio: todos los &lt;EM4&gt;materiales deben refinarse antes de la entrega&lt;/EM4&gt;, y dado que se trata de una orden de compra y no de un contrato de minería, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{2} cuando esté listo para vendernos los materiales refinados requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{3} Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Monox, Pyro V, Pyro IV&lt;/EM4&gt;\n- Pistola Arclight "Stormfall"\n- Pistola Arclight\n- Base de brazos Venture\n- Base de núcleo Venture\n- Base de piernas Venture\n- Base de casco Horizon\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Magda, Aberdeen, Arial&lt;/EM4&gt;\n- Pistola Arclight "Nightstalker"\n- Brazos Aril\n- Núcleo Aril\n- Piernas Aril\n- Casco Aril\n- Pistola Arclight "Warhawk"\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Pyro, Pyro V, Magda&lt;/EM4&gt;\n- Láser minero Arbor MHV (Láser minero)\n- S00 Hofstede (Láser minero)\n- Láser minero Lawson (Láser minero)\n- S0 Helix (Láser minero)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Arial, Pyro IV, Magda&lt;/EM4&gt;\n- Láser minero Pitman (Láser minero)\n- Láser minero Hofstede-S1 (Láser minero)\n- Láser minero Klein-S1 (Láser minero)\n- Láser minero Helix I (Láser minero)\n- Láser minero Impact I (Láser minero)\n- Láser minero Arbor MH1 (Láser minero)\n- Láser minero Lancet MH1 (Láser minero)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Pyro V, Pyro I, Arial&lt;/EM4&gt;\n- Láser minero Arbor MH2 (Láser minero)\n- Láser minero Lancet MH2 (Láser minero)\n- Láser minero Hofstede-S2 (Láser minero)\n- Láser minero Klein-S2 (Láser minero) Láser)\n- Láser de minería Helix II (Láser de minería)\n- Láser de minería Impact II (Láser de minería)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for a variety of refined materials. We appreciate your help in this matter.\n\n{1} Many of these ores are extremely rare and difficult to find, detectable only when a rock has been cracked open.\n\nReminder, all the &lt;EM4&gt;materials must be refined before delivery&lt;/EM4&gt;, and since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{2} you’re ready to sell us the required refined materials, deposit them in the freight elevator located at &lt;EM4&gt;{3} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Stanton, Pyro&lt;/EM4&gt;\n- Arclight "Stormfall" Pistol\n- Arclight Pistol\n- Venture Arms Base\n- Venture Core Base\n- Venture Legs Base\n- Horizon Helmet Base\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Stanton System, Hurston, Stanton&lt;/EM4&gt;\n- Arclight "Nightstalker" Pistol\n- Aril Arms\n- Aril Core\n- Aril Legs\n- Aril Helmet\n- Arclight "Warhawk" Pistol\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Crusader, microTech, ArcCorp&lt;/EM4&gt;\n- Arbor MHV Mining Laser (Mining Laser)\n- S00 Hofstede (Mining Laser)\n- Lawson Mining Laser (Mining Laser)\n- S0 Helix (Mining Laser)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: ArcCorp, Crusader, Pyro&lt;/EM4&gt;\n- Pitman Mining Laser (Mining Laser)\n- Hofstede-S1 Mining Laser (Mining Laser)\n- Klein-S1 Mining Laser (Mining Laser)\n- Helix I Mining Laser (Mining Laser)\n- Impact I Mining Laser (Mining Laser)\n- Arbor MH1 Mining Laser (Mining Laser)\n- Lancet MH1 Mining Laser (Mining Laser)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: Hurston, Stanton, Stanton System&lt;/EM4&gt;\n- Arbor MH2 Mining Laser (Mining Laser)\n- Lancet MH2 Mining Laser (Mining Laser)\n- Hofstede-S2 Mining Laser (Mining Laser)\n- Klein-S2 Mining Laser (Mining Laser)\n- Helix II Mining Laser (Mining Laser)\n- Impact II Mining Laser (Mining Laser)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de una variedad de materiales refinados. Agradecemos su ayuda en este asunto.\n\n{1} Muchos de estos minerales son extremadamente raros y difíciles de encontrar, detectables solo cuando una roca se ha abierto.\n\nRecordatorio: todos los &lt;EM4&gt;materiales deben refinarse antes de la entrega&lt;/EM4&gt;, y dado que se trata de una orden de compra y no de un contrato de minería, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{2} cuando esté listo para vendernos los materiales refinados requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{3} Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Stanton, Pyro&lt;/EM4&gt;\n- Pistola Arclight "Stormfall"\n- Pistola Arclight\n- Base de brazos Venture\n- Base de núcleo Venture\n- Base de piernas Venture\n- Base de casco Horizon\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Stanton System, Hurston, Stanton&lt;/EM4&gt;\n- Pistola Arclight "Nightstalker"\n- Brazos Aril\n- Núcleo Aril\n- Piernas Aril\n- Casco Aril\n- Pistola Arclight "Warhawk"\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Crusader, microTech, ArcCorp&lt;/EM4&gt;\n- Láser minero Arbor MHV (Láser minero)\n- S00 Hofstede (Láser minero)\n- Láser minero Lawson (Láser minero)\n- S0 Helix (Láser minero)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: ArcCorp, Cruzado, Pyro&lt;/EM4&gt;\n- Láser minero Pitman (Láser minero)\n- Láser minero Hofstede-S1 (Láser minero)\n- Láser minero Klein-S1 (Láser minero)\n- Láser minero Helix I (Láser minero)\n- Láser minero Impact I (Láser minero)\n- Láser minero Arbor MH1 (Láser minero)\n- Láser minero Lancet MH1 (Láser minero)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Hurston, Stanton, Sistema Stanton&lt;/EM4&gt;\n- Láser minero Arbor MH2 (Láser minero)\n- Láser minero Lancet MH2 (Láser minero)\n- Láser minero Hofstede-S2 (Láser minero)\n- Láser minero Klein-S2 (Láser minero) Láser)\n- Láser de minería Helix II (Láser de minería)\n- Láser de minería Impact II (Láser de minería)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for a variety of refined materials. We appreciate your help in this matter.\n\n{1} all the &lt;EM4&gt;materials must be refined before delivery&lt;/EM4&gt;, and since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{2} you’re ready to sell us the required refined materials, deposit them in the freight elevator located at &lt;EM4&gt;{3} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Multiple Blueprint Pools&lt;/EM4&gt;\n&lt;EM4&gt;Pool 1&lt;/EM4&gt;\n- Arclight "Nightstalker" Pistol\n- Aril Arms\n- Aril Core\n- Aril Legs\n- Aril Helmet\n- Arclight "Warhawk" Pistol\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;Pool 2&lt;/EM4&gt;\n- Arbor MHV Mining Laser (Mining Laser)\n- S00 Hofstede (Mining Laser)\n- Lawson Mining Laser (Mining Laser)\n- S0 Helix (Mining Laser)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Pitman Mining Laser (Mining Laser)\n- Hofstede-S1 Mining Laser (Mining Laser)\n- Klein-S1 Mining Laser (Mining Laser)\n- Helix I Mining Laser (Mining Laser)\n- Impact I Mining Laser (Mining Laser)\n- Arbor MH1 Mining Laser (Mining Laser)\n- Lancet MH1 Mining Laser (Mining Laser)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Arbor MH2 Mining Laser (Mining Laser)\n- Lancet MH2 Mining Laser (Mining Laser)\n- Hofstede-S2 Mining Laser (Mining Laser)\n- Klein-S2 Mining Laser (Mining Laser)\n- Helix II Mining Laser (Mining Laser)\n- Impact II Mining Laser (Mining Laser)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de una variedad de materiales refinados. Agradecemos su ayuda en este asunto.\n\n{1} Todos los &lt;EM4&gt;materiales deben ser refinados antes de la entrega&lt;/EM4&gt;, y dado que se trata de una orden de compra y no de un contrato de minería, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{2} Cuando esté listo para vendernos los materiales refinados requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{3} Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Múltiples grupos de planos&lt;/EM4&gt;\n&lt;EM4&gt;Grupo 1&lt;/EM4&gt;\n- Pistola Arclight "Nightstalker"\n- Brazos Aril\n- Núcleo Aril\n- Piernas Aril\n- Casco Aril\n- Pistola Arclight "Warhawk"\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;Grupo 2&lt;/EM4&gt;\n- Láser de minería Arbor MHV (Láser de minería)\n- S00 Hofstede (Láser de minería)\n- Lawson Mining Laser (Láser de minería)\n- S0 Helix (Láser de minería)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Pitman Mining Laser (Láser de minería)\n- Hofstede-S1 Mining Laser (Láser de minería)\n- Klein-S1 Mining Laser (Láser de minería)\n- Helix I Mining Laser (Láser de minería)\n- Impact I Mining Laser (Láser de minería)\n- Arbor MH1 Mining Laser (Láser de minería)\n- Lancet MH1 Mining Laser (Láser de minería)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Láser minero Arbor MH2 (Láser minero)\n- Láser minero Lancet MH2 (Láser minero)\n- Láser minero Hofstede-S2 (Láser minero)\n- Láser minero Klein-S2 (Láser minero)\n- Láser minero Helix II (Láser minero)\n- Láser minero Impact II (Láser minero)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for a variety of refined materials. We appreciate your help in this matter.\n\n{1} Many of these ores are extremely rare and difficult to find, detectable only when a rock has been cracked open.\n\nReminder, all the &lt;EM4&gt;materials must be refined before delivery&lt;/EM4&gt;, and since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{2} you’re ready to sell us the required refined materials, deposit them in the freight elevator located at &lt;EM4&gt;{3} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Multiple Blueprint Pools&lt;/EM4&gt;\n&lt;EM4&gt;Pool 1&lt;/EM4&gt;\n- Arclight "Nightstalker" Pistol\n- Aril Arms\n- Aril Core\n- Aril Legs\n- Aril Helmet\n- Arclight "Warhawk" Pistol\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;Pool 2&lt;/EM4&gt;\n- Arbor MHV Mining Laser (Mining Laser)\n- S00 Hofstede (Mining Laser)\n- Lawson Mining Laser (Mining Laser)\n- S0 Helix (Mining Laser)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Pitman Mining Laser (Mining Laser)\n- Hofstede-S1 Mining Laser (Mining Laser)\n- Klein-S1 Mining Laser (Mining Laser)\n- Helix I Mining Laser (Mining Laser)\n- Impact I Mining Laser (Mining Laser)\n- Arbor MH1 Mining Laser (Mining Laser)\n- Lancet MH1 Mining Laser (Mining Laser)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Arbor MH2 Mining Laser (Mining Laser)\n- Lancet MH2 Mining Laser (Mining Laser)\n- Hofstede-S2 Mining Laser (Mining Laser)\n- Klein-S2 Mining Laser (Mining Laser)\n- Helix II Mining Laser (Mining Laser)\n- Impact II Mining Laser (Mining Laser)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de una variedad de materiales refinados. Agradecemos su ayuda en este asunto.\n\n{1} Muchos de estos minerales son extremadamente raros y difíciles de encontrar, detectables solo cuando una roca se ha abierto.\n\nRecordatorio: todos los &lt;EM4&gt;materiales deben refinarse antes de la entrega&lt;/EM4&gt;, y dado que se trata de una orden de compra y no de un contrato de minería, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{2} cuando esté listo para vendernos los materiales refinados requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{3} Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Múltiples grupos de planos&lt;/EM4&gt;\n&lt;EM4&gt;Grupo 1&lt;/EM4&gt;\n- Pistola Arclight "Nightstalker"\n- Brazos Aril\n- Núcleo Aril\n- Piernas Aril\n- Casco Aril\n- Pistola Arclight "Warhawk"\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;Grupo 2&lt;/EM4&gt;\n- Láser minero Arbor MHV (Láser minero)\n- S00 Hofstede (Láser minero)\n- Láser minero Lawson (Láser minero)\n- S0 Helix (Láser minero)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Láser minero Pitman (Láser minero)\n- Láser minero Hofstede-S1 (Láser minero)\n- Láser minero Klein-S1 (Láser minero)\n- Láser minero Helix I (Láser minero)\n- Láser minero Impact I (Láser minero)\n- Láser minero Arbor MH1 (Láser minero)\n- Láser minero Lancet MH1 (Láser minero)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Láser de minería Arbor MH2 (Láser de minería)\n- Láser de minería Lancet MH2 (Láser de minería)\n- Láser de minería Hofstede-S2 (Láser de minería)\n- Láser de minería Klein-S2 (Láser de minería)\n- Láser de minería Helix II (Láser de minería)\n- Láser de minería Impact II (Láser de minería)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for a variety of refined materials. We appreciate your help in this matter.\n\n{1} Many of these ores are extremely rare and difficult to find, detectable only when a rock has been cracked open.\n\nReminder, all the &lt;EM4&gt;materials must be refined before delivery&lt;/EM4&gt;, and since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{2} you’re ready to sell us the required refined materials, deposit them in the freight elevator located at &lt;EM4&gt;{3} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Nyx II, nyx, Nyx&lt;/EM4&gt;\n- Arclight "Stormfall" Pistol\n- Arclight Pistol\n- Venture Arms Base\n- Venture Core Base\n- Venture Legs Base\n- Horizon Helmet Base\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Crusader, Daymar, Cellin&lt;/EM4&gt;\n- Arclight "Nightstalker" Pistol\n- Aril Arms\n- Aril Core\n- Aril Legs\n- Aril Helmet\n- Arclight "Warhawk" Pistol\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Nyx System, Crusader, Daymar&lt;/EM4&gt;\n- Arbor MHV Mining Laser (Mining Laser)\n- S00 Hofstede (Mining Laser)\n- Lawson Mining Laser (Mining Laser)\n- S0 Helix (Mining Laser)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: Nyx III, Nyx II, Nyx System&lt;/EM4&gt;\n- Pitman Mining Laser (Mining Laser)\n- Hofstede-S1 Mining Laser (Mining Laser)\n- Klein-S1 Mining Laser (Mining Laser)\n- Helix I Mining Laser (Mining Laser)\n- Impact I Mining Laser (Mining Laser)\n- Arbor MH1 Mining Laser (Mining Laser)\n- Lancet MH1 Mining Laser (Mining Laser)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;[Regional Variants] example locations: Nyx II, Nyx System, Daymar&lt;/EM4&gt;\n- Arbor MH2 Mining Laser (Mining Laser)\n- Lancet MH2 Mining Laser (Mining Laser)\n- Hofstede-S2 Mining Laser (Mining Laser)\n- Klein-S2 Mining Laser (Mining Laser)\n- Helix II Mining Laser (Mining Laser)\n- Impact II Mining Laser (Mining Laser)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de una variedad de materiales refinados. Agradecemos su ayuda en este asunto.\n\n{1} Muchos de estos minerales son extremadamente raros y difíciles de encontrar, detectables solo cuando una roca se ha agrietado.\n\nRecordatorio: todos los &lt;EM4&gt;materiales deben refinarse antes de la entrega&lt;/EM4&gt;, y dado que se trata de una orden de compra y no de un contrato minero, se espera que proporcione su propio equipo, como un &lt;EM4&gt;{2}. Cuando esté listo para vendernos los materiales refinados requeridos, deposítelos en el montacargas ubicado en &lt;EM4&gt;{3}. Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx II, nyx, Nyx&lt;/EM4&gt;\n- Pistola Arclight "Stormfall"\n- Pistola Arclight\n- Base de brazos Venture\n- Base de núcleo Venture\n- Base de piernas Venture\n- Base de casco Horizon\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Crusader, Daymar, Cellin&lt;/EM4&gt;\n- Pistola Arclight "Nightstalker"\n- Brazos Aril\n- Núcleo Aril\n- Piernas Aril\n- Casco Aril\n- Pistola Arclight "Warhawk"\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx System, Crusader, Daymar&lt;/EM4&gt;\n- Láser minero Arbor MHV (Láser minero)\n- S00 Hofstede (Láser minero)\n- Láser minero Lawson (Láser minero)\n- S0 Helix (Láser minero)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nyx III, Nyx II, Nyx System&lt;/EM4&gt;\n- Pitman Mining Laser (Láser de Minería)\n- Hofstede-S1 Mining Laser (Láser de Minería)\n- Klein-S1 Mining Laser (Láser de Minería)\n- Helix I Mining Laser (Láser de Minería)\n- Impact I Mining Laser (Láser de Minería)\n- Arbor MH1 Mining Laser (Láser de Minería)\n- Lancet MH1 Mining Laser (Láser de Minería)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;[Variantes Regionales] ejemplos de ubicaciones: Nyx II, Nyx System, Daymar&lt;/EM4&gt;\n- Arbor MH2 Mining Laser (Láser de Minería)\n- Lancet MH2 Mining Laser (Láser de Minería)\n- Hofstede-S2 Mining Laser (Láser de Minería)\n- Klein-S2 Mining Laser (Láser de Minería) Láser)\n- Láser de minería Helix II (Láser de minería)\n- Láser de minería Impact II (Láser de minería)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>POSTING: Purchase Order\nLOCATION: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTERMS*: \nShubin Interstellar is currently looking to fulfil another purchase order for a variety of refined materials. This purchase order is more complex than typical, requiring multiple mining methods, but since you've proven your skill thus far, we think you and your team are up for the challenge.\n\nReminder, &lt;EM4&gt;materials must be refined before delivery&lt;/EM4&gt;, and since this is a purchase order and not a mining contract, you are expected to provide your own equipment, such as a &lt;EM4&gt;{1} you’re ready to sell us the required materials, deposit them in the freight elevator located at &lt;EM4&gt;{2} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Multiple Blueprint Pools&lt;/EM4&gt;\n&lt;EM4&gt;Pool 1&lt;/EM4&gt;\n- Arclight "Stormfall" Pistol\n- Arclight Pistol\n- Venture Arms Base\n- Venture Core Base\n- Venture Legs Base\n- Horizon Helmet Base\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;Pool 2&lt;/EM4&gt;\n- Arclight "Nightstalker" Pistol\n- Aril Arms\n- Aril Core\n- Aril Legs\n- Aril Helmet\n- Arclight "Warhawk" Pistol\n- Arclight Pistol Battery (30 cap)\n\n&lt;EM4&gt;Pool 3&lt;/EM4&gt;\n- Arbor MHV Mining Laser (Mining Laser)\n- S00 Hofstede (Mining Laser)\n- Lawson Mining Laser (Mining Laser)\n- S0 Helix (Mining Laser)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Pool 4&lt;/EM4&gt;\n- Pitman Mining Laser (Mining Laser)\n- Hofstede-S1 Mining Laser (Mining Laser)\n- Klein-S1 Mining Laser (Mining Laser)\n- Helix I Mining Laser (Mining Laser)\n- Impact I Mining Laser (Mining Laser)\n- Arbor MH1 Mining Laser (Mining Laser)\n- Lancet MH1 Mining Laser (Mining Laser)\n- BroadSpec-Go (Radar)\n- BroadSpec (Radar)\n- BroadSpec-Max (Radar)\n\n&lt;EM4&gt;Pool 5&lt;/EM4&gt;\n- Arbor MH2 Mining Laser (Mining Laser)\n- Lancet MH2 Mining Laser (Mining Laser)\n- Hofstede-S2 Mining Laser (Mining Laser)\n- Klein-S2 Mining Laser (Mining Laser)\n- Helix II Mining Laser (Mining Laser)\n- Impact II Mining Laser (Mining Laser)\n- FullSpec-Go (Radar)\n- FullSpec (Radar)\n- FullSpec-Max (Radar)\n</v>
+        <v>PUBLICACIÓN: Orden de compra\nUBICACIÓN: &lt;EM4&gt;{0} &lt;/EM4&gt;\n\nTÉRMINOS*: \nShubin Interstellar está buscando actualmente cumplir otra orden de compra de una variedad de materiales refinados. Esta orden de compra es más compleja de lo habitual, ya que requiere múltiples métodos de minería, pero dado que has demostrado tu habilidad hasta ahora, creemos que tú y tu equipo están preparados para el desafío.\n\nRecordatorio: los materiales deben refinarse antes de la entrega, y dado que se trata de una orden de compra y no de un contrato de minería, se espera que proporciones tu propio equipo, como un {1}. Cuando estés listo para vendernos los materiales requeridos, deposítalos en el montacargas ubicado en {2}. Otorgado (por dificultad): 50 / 200\n&lt;Múltiples grupos de planos&lt;/EM4&gt;\n&lt;Grupo 1&lt;/EM4&gt;\n- Pistola Arclight "Stormfall"\n- Pistola Arclight\n- Base de brazos Venture\n- Base de núcleo Venture\n- Base de piernas Venture\n- Base de casco Horizon\n- Batería de pistola Arclight (30 cap)\n\n&lt;Grupo 2&lt;/EM4&gt;\n- Pistola Arclight "Nightstalker"\n- Brazos Aril\n- Núcleo Aril\n- Piernas Aril\n- Casco Aril\n- Pistola Arclight "Warhawk"\n- Batería de pistola Arclight (30 cap)\n\n&lt;EM4&gt;Piscina 3&lt;/EM4&gt;\n- Láser de minería Arbor MHV (Láser de minería)\n- S00 Hofstede (Láser de minería)\n- Láser de minería Lawson (Láser de minería)\n- S0 Helix (Láser de minería)\n- Surveyor-Go (Radar)\n- Surveyor-Lite (Radar)\n- Surveyor (Radar)\n- Surveyor-Max (Radar)\n\n&lt;EM4&gt;Piscina 4&lt;/EM4&gt;\n- Láser de minería Pitman (Láser de minería)\n- Láser de minería Hofstede-S1 (Láser de minería)\n- Láser de minería Klein-S1 (Láser de minería)\n- Minería Helix I Láser (láser de minería)\n- Impact I Láser de minería (láser de minería)\n- Arbor MH1 Láser de minería (láser de minería)\n- Lancet MH1 Láser de minería (láser de minería)\n- BroadSpec-Go (radar)\n- BroadSpec (radar)\n- BroadSpec-Max (radar)\n\n&lt;EM4&gt;Pool 5&lt;/EM4&gt;\n- Arbor MH2 Láser de minería (láser de minería)\n- Lancet MH2 Láser de minería (láser de minería)\n- Hofstede-S2 Láser de minería (láser de minería)\n- Klein-S2 Láser de minería (láser de minería)\n- Helix II Láser de minería (láser de minería)\n- Impact II Láser de minería (láser de minería)\n- FullSpec-Go (radar)\n- FullSpec (radar)\n- FullSpec-Max (radar)\n</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>Hey there,\n\nIf you're fitted for refueling, you might like this one. \n\nA beacon has just gone live at &lt;EM4&gt;{0} from a client whose &lt;EM4&gt;{1} is running on empty, so make sure your fuel pods are topped off.\n\nThe client vessel will pay you at the rate of &lt;EM4&gt;{2} aUEC per SCU of Hydrogen&lt;/EM4&gt; and  &lt;EM4&gt;{3} aUEC per SCU of Quantum &lt;/EM4&gt;, and as a United Wayfarers Club contractor, you will also qualify for the UWC service fee listed above upon completion.\n\nLooks like a zero-drama one and done, but it never hurts to keep your scanners live.\nLet me know if you're interested and let's get these good people on their way.\n\nWaiting to hear from you,\n\nDina Deloit\nDispatch Hub\nUnited Wayfarers Club\n"We’ve got your back"\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 200\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- bp_craft_nozzle_fuelgiver_grin_nozzlefast (Fuel Nozzle)\n- Marlin (Fuel Nozzle)\n- Lindstrom (Fuel Nozzle)\n- bp_craft_nozzle_fuelgiver_grin_nozzleverysecure (Fuel Nozzle)\n- bp_craft_nozzle_fuelgiver_misc_nozzlestandard (Fuel Nozzle)\n- Bendix (Fuel Nozzle)\n- Torrez (Fuel Nozzle)\n- Ezra (Fuel Nozzle)\n</v>
+        <v>Hola,\n\nSi estás equipado para repostar, puede que te guste este. \n\nUna baliza acaba de activarse en &lt;EM4&gt;{0} de un cliente cuyo &lt;EM4&gt;{1} se está quedando sin combustible, así que asegúrese de que sus depósitos de combustible estén llenos.\n\nLa embarcación del cliente le pagará a una tasa de &lt;EM4&gt;{2} aUEC por SCU de hidrógeno&lt;/EM4&gt; y &lt;EM4&gt;{3} aUEC por SCU de Quantum&lt;/EM4&gt;, y como contratista del United Wayfarers Club, también podrá optar a la tarifa de servicio del UWC mencionada anteriormente al finalizar.\n\nParece un trabajo sencillo y sin complicaciones, pero nunca está de más mantener los escáneres activos.\nAvíseme si está interesado y pongamos en marcha a estas buenas personas.\n\nEspero su respuesta,\n\nDina Deloit\nCentro de Despacho\nUnited Wayfarers Club\n"Le respaldamos"\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 200\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- bp_craft_nozzle_fuelgiver_grin_nozzlefast (Boquilla de combustible)\n- Marlin (Boquilla de combustible)\n- Lindstrom (Boquilla de combustible)\n- bp_craft_nozzle_fuelgiver_grin_nozzleverysecure (Boquilla de combustible)\n- bp_craft_nozzle_fuelgiver_misc_nozzlestandard (Boquilla de combustible)\n- Bendix (Boquilla de combustible)\n- Torrez (Boquilla de combustible)\n- Ezra (Boquilla de combustible)\n</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>Hey again,\n\nI've got a beacon at &lt;EM4&gt;{0} and this one's a big one. An entire little fleet of ships all burned out of fuel at the same time. Impressive coordination and lack of planning at the same time. \n\nThe client vessel will pay you at the rate of &lt;EM4&gt;{1} aUEC per SCU of Hydrogen&lt;/EM4&gt; and  &lt;EM4&gt;{2} aUEC per SCU of Quantum &lt;/EM4&gt;, and as a United Wayfarers Club contractor, you will also qualify for the UWC service fee listed above upon completion.\n\nHopefully since the area they're in is pretty safe, there shouldn't be too much trouble lurking, but these days you never know. Wouldn't hurt to get them back flying again as quick as you're able.\n\nHappy trails,\n\nDina Deloit\nDispatch Hub\nUnited Wayfarers Club\n"We’ve got your back"\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 150 / 200\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- bp_craft_nozzle_fuelgiver_grin_nozzlefast (Fuel Nozzle)\n- Marlin (Fuel Nozzle)\n- Lindstrom (Fuel Nozzle)\n- bp_craft_nozzle_fuelgiver_grin_nozzleverysecure (Fuel Nozzle)\n- bp_craft_nozzle_fuelgiver_misc_nozzlestandard (Fuel Nozzle)\n- Bendix (Fuel Nozzle)\n- Torrez (Fuel Nozzle)\n- Ezra (Fuel Nozzle)\n</v>
+        <v>Hola de nuevo,\n\nTengo una baliza en &lt;EM4&gt;{0} y esta es una grande. Toda una pequeña flota de barcos se quedaron sin combustible al mismo tiempo. Impresionante coordinación y falta de planificación al mismo tiempo. \n\nEl buque cliente te pagará a una tasa de &lt;EM4&gt;{1} aUEC por SCU de hidrógeno&lt;/EM4&gt; y &lt;EM4&gt;{2} aUEC por SCU de Quantum&lt;/EM4&gt;, y como contratista del United Wayfarers Club, también calificarás para la tarifa de servicio de UWC mencionada anteriormente al finalizar.\n\nEsperemos que, dado que el área en la que están es bastante segura, no haya demasiados problemas al acecho, pero en estos días nunca se sabe. No estaría mal que volvieran a volar lo antes posible.\n\nQue tengas un buen viaje,\n\nDina Deloit\nCentro de Despacho\nClub United Wayfarers\n"Te respaldamos"\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 150 / 200\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- bp_craft_nozzle_fuelgiver_grin_nozzlefast (Boquilla de combustible)\n- Marlin (Boquilla de combustible)\n- Lindstrom (Boquilla de combustible)\n- bp_craft_nozzle_fuelgiver_grin_nozzleverysecure (Boquilla de combustible)\n- bp_craft_nozzle_fuelgiver_misc_nozzlestandard (Boquilla de combustible)\n- Bendix (Boquilla de combustible)\n- Torrez (Boquilla de combustible)\n- Ezra (Boquilla de combustible)</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>--------------------------------------------------------\n----------------- BOUNTY CONTRACT -----------------\n--------------------------------------------------------\n\nBOUNTY HUNTERS GUILD\nPROCESSING &amp; DISTRIBUTION\n\nThe Bounty Hunters Guild has authorized an official bounty.\n\nNAME: {0} \nSYSTEM: {1} ASSESSMENT: {2} KNOWN LOCATION:  {3} AFFILIATIONS: &lt;None&gt;\nNOTES: They have several known associates with criminal records so they may not be alone so arm up and exercise caution when engaging.\n\n\nBOUNTY HUNTERS GUILD\nIn Pursuit of Justice\n\nThe Bounty Hunters Guild is a security service sanctioned by the Mercenary Guild and authorized to operate in both the UEE and beyond in accordance with Xenotrade Authority Acts.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 500 / 1,000 / 2,000 / 8,000 / 16,000</v>
+        <v>--------------------------------------------------------\n----------------- CONTRATO DE RECOMPENSA -----------------\n--------------------------------------------------------\n\nGREMIO DE CAZADORES DE RECOMPENSAS\nPROCESAMIENTO Y DISTRIBUCIÓN\n\nEl Gremio de Cazadores de Recompensas ha autorizado una recompensa oficial.\n\nNOMBRE: {0} \nSISTEMA: {1} EVALUACIÓN: {2} UBICACIÓN CONOCIDA: {3} AFILIACIONES: &lt;Ninguna&gt;\nNOTAS: Tienen varios asociados conocidos con antecedentes penales, por lo que podrían no estar solos; así que ármense y tengan precaución al enfrentarse a ellos.\n\n\nGREMIO DE CAZADORES DE RECOMPENSAS\nEn busca de la justicia\n\nEl Gremio de Cazadores de Recompensas es un servicio de seguridad sancionado por el Gremio de Mercenarios y autorizado para operar tanto en la UEE como más allá, de acuerdo con las Leyes de la Autoridad de Xenotrade.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 500 / 1000 / 2.000 / 8.000 / 16.000</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>We need any available security personnel to report to {0} A group of armed individuals have attacked one of our outpost clusters and we're in desperate need of help. Although the group seems to be unaffiliated with any of the known gangs, we've received word that their leader is {1} a local outlaw with a vicious reputation.\n\nPlease head out as soon as you can and secure the area by taking out the outlaws and {2} Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna "Brimstone" Rifle\n- Artimex Core Lodestone\n- Artimex Arms Lodestone\n- Artimex Legs Lodestone\n- Artimex Helmet Lodestone\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Necesitamos que todo el personal de seguridad disponible se presente en {0}. Un grupo de individuos armados ha atacado uno de nuestros grupos de puestos avanzados y necesitamos ayuda desesperadamente. Aunque el grupo parece no estar afiliado a ninguna de las bandas conocidas, hemos recibido información de que su líder es {1}, un forajido local con una reputación terrible.\n\nPor favor, salgan lo antes posible y aseguren la zona eliminando a los forajidos y a {2} Endicott.\nDespachador principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna "Brimstone"\n- Piedra imán Artimex Core\n- Piedra imán Artimex Arms\n- Piedra imán Artimex Legs\n- Piedra imán Artimex Helmet\n- Batería de rifle Karna (35 cap)\n</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>We are currently looking for any qualified and available security operatives to head out to {0} and reclaim a CFP installation that had been taken by Headhunters. \n\nThe group that's currently occupying the outpost is being led by {1} a Headhunter of some note who's had a history of aggression against locals and CFP volunteers.\n\nWe need all Headhunters secured and {2} taken out.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna "Brimstone" Rifle\n- Artimex Core Lodestone\n- Artimex Arms Lodestone\n- Artimex Legs Lodestone\n- Artimex Helmet Lodestone\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Actualmente estamos buscando agentes de seguridad cualificados y disponibles para dirigirse a {0} y recuperar una instalación de CFP que había sido tomada por Headhunters. \n\nEl grupo que actualmente ocupa el puesto avanzado está liderado por {1}, un Headhunter de cierta importancia con un historial de agresiones contra los lugareños y los voluntarios de CFP.\n\nNecesitamos asegurar a todos los Headhunters y eliminar a {2}.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna "Brimstone"\n- Piedra imán Artimex Core\n- Piedra imán Artimex Arms\n- Piedra imán Artimex Legs\n- Piedra imán Artimex Helmet\n- Batería de rifle Karna (capacidad 35)\n</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>We just received a frantic comm from {0} and are looking for any available combat specialists to help repel a Headhunter attack. There are still hostiles on site and there are reports of several casualties so we need this handled quickly.\n\nI will provide all relevant data upon acceptance. Thank you for your assistance.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna "Fate" Rifle\n- Artimex Core (Modified)\n- Artimex Arms (Modified)\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Acabamos de recibir una comunicación frenética de {0} y estamos buscando especialistas en combate disponibles para ayudar a repeler un ataque de Headhunter. Todavía hay hostiles en el lugar y hay informes de varias bajas, por lo que necesitamos que esto se resuelva rápidamente.\n\nProporcionaré todos los datos relevantes una vez aceptada la solicitud. Gracias por su ayuda.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Fusil Karna "Fate"\n- Núcleo Artimex (modificado)\n- Brazos Artimex (modificados)\n- Batería de fusil Karna (capacidad de 35)\n</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>Several CFP clusters near {0} just got hit by a group of outlaws led by {1} We're looking for any available combat specialists to help retake the outposts.\n\nI can provide the locations upon acceptance but we need to clear out the main outpost and satellite installations from all hostile forces and take out {2} as it's unlikely that they will not cease their hostilities if they escape.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna "Brimstone" Rifle\n- Artimex Core Lodestone\n- Artimex Arms Lodestone\n- Artimex Legs Lodestone\n- Artimex Helmet Lodestone\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Varios grupos de CFP cerca de {0} acaban de ser atacados por un grupo de forajidos liderados por {1}. Buscamos especialistas en combate disponibles para ayudar a retomar los puestos de avanzada.\n\nPuedo proporcionar las ubicaciones una vez aceptada la solicitud, pero necesitamos despejar el puesto de avanzada principal y las instalaciones satélite de todas las fuerzas hostiles y eliminar a {2}, ya que es poco probable que no cesen sus hostilidades si escapan.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna "Brimstone"\n- Piedra imán de núcleo Artimex\n- Piedra imán de brazos Artimex\n- Piedra imán de piernas Artimex\n- Piedra imán de casco Artimex\n- Batería de rifle Karna (35 de capacidad)\n</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>Citizens for Prosperity is looking for any available security operatives to retake several former CFP installations near {0} from Headhunter control. These clusters were violently taken from us by {1} and resulted in the deaths of many volunteers.\n\nBringing these outposts back under our control will help provide more stability to the system. Reports indicate that {2} tends to hide behind their rank and file, so they will likely appear once you've cleared out most of the hostiles.\n\nXenoThreat are trained and motivated so they will not give up easily.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna "Brimstone" Rifle\n- Artimex Core Lodestone\n- Artimex Arms Lodestone\n- Artimex Legs Lodestone\n- Artimex Helmet Lodestone\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Ciudadanos por la Prosperidad busca agentes de seguridad disponibles para recuperar varias antiguas instalaciones de CFP cerca de {0} que estaban bajo el control de Headhunter. Estos grupos nos fueron arrebatados violentamente por {1}, lo que provocó la muerte de muchos voluntarios.\n\nRecuperar el control de estos puestos avanzados contribuirá a brindar mayor estabilidad al sistema. Los informes indican que {2} tiende a esconderse detrás de sus filas, por lo que probablemente aparecerán una vez que hayas eliminado a la mayoría de los hostiles.\n\nLos XenoThreat están entrenados y motivados, por lo que no se rendirán fácilmente.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna "Brimstone"\n- Piedra imán de núcleo Artimex\n- Piedra imán de brazos Artimex\n- Piedra imán de piernas Artimex\n- Piedra imán de casco Artimex\n- Batería de rifle Karna (35 cap)\n</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>Looking for any available security personnel to reclaim several clusters previously lost to XenoThreat aggressors. Located near {0} they had been seized in brutal attacks led by {1} a notorious XenoThreat lieutenant.\n\nWe're looking to take these clusters back so we can reestablish operations and continue our good work. You'll need to clear all the hostiles still on-site as well as {2} a reminder, that XenoThreat are highly trained and quick to fight, so prepare accordingly.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 400\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna "Brimstone" Rifle\n- Artimex Core Lodestone\n- Artimex Arms Lodestone\n- Artimex Legs Lodestone\n- Artimex Helmet Lodestone\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Buscamos personal de seguridad disponible para recuperar varios clústeres que fueron arrebatados por agresores de XenoThreat. Ubicados cerca de {0}, fueron tomados en brutales ataques liderados por {1}, un notorio lugarteniente de XenoThreat.\n\nQueremos recuperar estos clústeres para restablecer las operaciones y continuar con nuestro buen trabajo. Deberás eliminar a todos los enemigos que aún se encuentren en el lugar, así como {2} un recordatorio: los XenoThreat están altamente entrenados y son rápidos para luchar, así que prepárate en consecuencia.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 400\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna "Brimstone"\n- Piedra imán de núcleo Artimex\n- Piedra imán de brazos Artimex\n- Piedra imán de piernas Artimex\n- Piedra imán de casco Artimex\n- Batería de rifle Karna (35 cap)\n</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>The outlaw presence here has become much bolder of late and a lot of people are getting hurt. We've recently lost several clusters around {0} While we don't like to have to resort to violence, the board has acknowledged that these locations are crucial to establishing stability in the system and authorized the use of a security detail to retake them.\n\nWe're also aware that the embedded hostiles are being led by {1} who's had a history of attacking CFP interests. The board would like {2} dealt with to prevent future attacks.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna "Fate" Rifle\n- Artimex Core (Modified)\n- Artimex Arms (Modified)\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>La presencia de delincuentes aquí se ha vuelto mucho más audaz últimamente y muchas personas están resultando heridas. Recientemente hemos perdido varios grupos alrededor de {0}. Si bien no nos gusta tener que recurrir a la violencia, la junta ha reconocido que estas ubicaciones son cruciales para establecer la estabilidad en el sistema y ha autorizado el uso de un equipo de seguridad para recuperarlas.\n\nTambién sabemos que los hostiles infiltrados están siendo liderados por {1}, quien tiene un historial de ataques a los intereses de CFP. La junta desea que se resuelva {2} para prevenir futuros ataques.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna "Destino"\n- Núcleo Artimex (modificado)\n- Brazos Artimex (modificados)\n- Batería de rifle Karna (capacidad de 35)\n</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>Citizens for Prosperity's board just authorized funds to hire security personnel to retake several clusters near {0} that have since fallen into the hands of the Headhunters. While we tried to just accept the loss, it's become apparent that they are crucial to our ongoing operations in the system.\n\nYou'll need to clear out each of the locations that will be provided but more importantly, you'll also need to take out {1} who's in charge of the hostiles on site.\n\nThese Headhunters are heavily embedded and have a history of violence, so you should prepare accordingly. \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna "Fate" Rifle\n- Artimex Core (Modified)\n- Artimex Arms (Modified)\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>La junta de Ciudadanos por la Prosperidad acaba de autorizar fondos para contratar personal de seguridad para recuperar varios grupos cerca de {0} que han caído en manos de los Cazadores de Cabezas. Aunque intentamos aceptar la pérdida, se ha hecho evidente que son cruciales para nuestras operaciones en curso en el sistema.\n\nDeberás despejar cada una de las ubicaciones que se te proporcionarán, pero más importante aún, también deberás eliminar a {1}, quien está a cargo de los hostiles en el lugar.\n\nEstos Cazadores de Cabezas están muy bien infiltrados y tienen un historial de violencia, así que debes prepararte en consecuencia. \n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Fusil Karna "Destino"\n- Núcleo Artimex (modificado)\n- Armas Artimex (modificadas)\n- Batería de fusil Karna (capacidad de 35)\n</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>Although Citizens for Prosperity is committed to change through non-violent means, it's become apparent that exceptions might have to be made. CFP safe zones near {0} were recently and violently taken by XenoThreat forces under the command of {1} looking for any available combat operatives to help take these outposts back. This will undoubtedly be a difficult endeavor as XenoThreat are highly trained and eager to fight, so you should prepare accordingly.\n\nAside from clearing each cluster of XenoThreat forces, you will need to take out {2} who's loss will certainly make the system safer.\n\nGood luck,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 400\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna "Fate" Rifle\n- Artimex Core (Modified)\n- Artimex Arms (Modified)\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Aunque Citizens for Prosperity está comprometida con el cambio por medios no violentos, se ha hecho evidente que podrían ser necesarias excepciones. Las zonas seguras de CFP cerca de {0} fueron tomadas recientemente y de forma violenta por fuerzas de XenoThreat bajo el mando de {1}, que buscaban operativos de combate disponibles para ayudar a recuperar estos puestos avanzados. Esta será sin duda una tarea difícil, ya que los XenoThreat están altamente entrenados y ansiosos por luchar, así que debes prepararte en consecuencia.\n\nAdemás de eliminar cada grupo de fuerzas XenoThreat, tendrás que eliminar a {2} cuya pérdida sin duda hará que el sistema sea más seguro.\n\nBuena suerte,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 400\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna "Fate"\n- Núcleo Artimex (modificado)\n- Brazos Artimex (modificados)\n- Batería de rifle Karna (capacidad de 35)\n</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>Reports indicate that {0} has come under attack from a group of armed individuals led by a notorious outlaw named {1} There have been multiple reported deaths and injuries, so Citizens for Prosperity has been looking for qualified combat operatives to provide some support. \n\nThough we don't advocate conflict resolution through violence, we believe that the group will disperse if {2} is not there to lead them.\n\nHead over as soon as you can. Lives are on the line.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 75</v>
+        <v>Los informes indican que {0} ha sido atacado por un grupo de individuos armados liderados por un conocido forajido llamado {1}. Se han reportado múltiples muertes y heridos, por lo que Ciudadanos por la Prosperidad ha estado buscando operativos de combate calificados para brindar apoyo. \n\nAunque no abogamos por la resolución de conflictos mediante la violencia, creemos que el grupo se dispersará si {2} no está allí para liderarlos.\n\nDirígete lo antes posible. Hay vidas en peligro.\n\nLima Endicott\nOficial de Despacho Principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 75</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>Hi, we need to move some cargo across the system and were wondering if you could help. I know this is outside your usual purview, but I'm low on options. This would also be a great way to show your committed to Citizens for Prosperity's greater mission here.\n\nIf you head to &lt;EM4&gt;{0} there should be some cargo accessible via a freight elevator that we'll need you to take to another freight elevator at &lt;EM4&gt;{1} thing to call out is that your ship must be able to handle &lt;EM4&gt;{2} cargo containers&lt;/EM4&gt;. To make your life easier, be sure you have a &lt;EM4&gt;handheld tractor beam&lt;/EM4&gt; with you. Otherwise, it should be a simple run. \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>Hola, necesitamos mover algo de carga a través del sistema y nos preguntábamos si podrías ayudarnos. Sé que esto está fuera de tu ámbito habitual, pero tengo pocas opciones. Esta también sería una excelente manera de demostrar tu compromiso con la misión principal de Ciudadanos por la Prosperidad.\n\nSi te diriges a &lt;EM4&gt;{0}, debería haber algo de carga accesible a través de un montacargas que deberás llevar a otro montacargas en &lt;EM4&gt;{1}. Es importante que tu nave pueda manejar &lt;EM4&gt;{2} contenedores de carga&lt;/EM4&gt;. Para facilitarte la vida, asegúrate de tener un &lt;EM4&gt;rayo tractor portátil&lt;/EM4&gt; contigo. De lo contrario, debería ser un viaje sencillo. \n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>We've been having escalating issues with the outlaws at {0} and can no longer stand by and watch as their aggressive actions hurt our community. \n\nWe are wary of launching a full scale assault, but believe that if their fuel stores are wiped out, it would deter them from further hostile actions. \n\nIf you're able, I'd appreciate you handling the destruction of the fuel personally. A ship capable of launching missiles would probably make the most sense, but I leave that up to you.\n\nThanks,\n \nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Orbituary Clinic, RAB-CHARLIE, Bloom&lt;/EM4&gt;\n- FS-9 LMG\n- BR-2 Shotgun\n- Gallant Rifle\n- ADP Arms Woodland\n- ADP Core\n- ADP Legs Woodland\n- Balor HCH Helmet\n- ADP-mk4 Arms Woodland\n- ADP-mk4 Legs Woodland\n- ADP-mk4 Core Woodland\n- ADP-mk4 Helmet Woodland\n- FS-9 Magazine (75 cap)\n- BR-2 Shotgun Magazine (12 cap)\n- Gallant Rifle Battery (45 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Gaslight Clinic, Ruin Station, Fuego&lt;/EM4&gt;\n- P6-LR Sniper Rifle\n- A03 Sniper Rifle\n- CBH-3 Helmet Base\n- PAB-1 Arms Woodland\n- PAB-1 Core Woodland\n- PAB-1 Legs Woodland\n- TrueDef-Pro Arms Base\n- TrueDef-Pro Core Base\n- Argus Helmet Base\n- TrueDef-Pro Legs Base\n- A03 Sniper Rifle Magazine (15 cap)\n- P6-LR Magazine (8 cap)\n</v>
+        <v>Hemos estado teniendo problemas cada vez mayores con los forajidos en {0} y ya no podemos quedarnos de brazos cruzados mientras sus acciones agresivas perjudican a nuestra comunidad. \n\nSomos cautelosos a la hora de lanzar un ataque a gran escala, pero creemos que si se agotan sus reservas de combustible, se disuadirán de realizar más acciones hostiles. \n\nSi le es posible, le agradecería que se encargara personalmente de la destrucción del combustible. Un barco capaz de lanzar misiles probablemente sería lo más lógico, pero te lo dejo a ti.\n\nGracias,\n \nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Clínica Orbituaria, RAB-CHARLIE, Bloom&lt;/EM4&gt;\n- FS-9 LMG\n- Escopeta BR-2\n- Fusil Gallant\n- Brazos ADP Woodland\n- Núcleo ADP\n- Piernas ADP Woodland\n- Casco Balor HCH\n- Brazos ADP-mk4 Woodland\n- Piernas ADP-mk4 Woodland\n- Núcleo ADP-mk4 Woodland\n- Casco ADP-mk4 Woodland\n- Cargador FS-9 (75 cap)\n- Cargador de escopeta BR-2 (12 cap)\n- Batería de rifle Gallant (45 cap)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Clínica Gaslight, Estación Ruin, Fuego&lt;/EM4&gt;\n- Rifle de francotirador P6-LR\n- Rifle de francotirador A03\n- Base de casco CBH-3\n- Brazos PAB-1 Woodland\n- Núcleo PAB-1 Woodland\n- Piernas PAB-1 Woodland\n- Base de brazos TrueDef-Pro\n- Base de núcleo TrueDef-Pro\n- Base de casco Argus\n- Base de piernas TrueDef-Pro\n- Cargador de rifle de francotirador A03 (15 cap)\n- Cargador P6-LR (8 cap)\n</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>We learned that {0} is under threat of attack by outlaws and has asked for assistance. We need someone to protect them and drive away the outlaws. \n\nMake sure you stay close after their initial attack. Too often, outlaws win fights just by sending more bodies than anyone can reasonably defend against, so make sure you fight off any reinforcements before leaving the area. \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 75 / 200\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Cluster JWY-925, RAB-CHARLIE, RAB-MAT&lt;/EM4&gt;\n- Karna "Fate" Rifle\n- Artimex Core (Modified)\n- Artimex Arms (Modified)\n- Karna Rifle Battery (35 cap)\n\n&lt;EM4&gt;outpost_regionab&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Arms\n- Artimex Core\n- Artimex Legs\n- Artimex Helmet\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Nos enteramos de que {0} está bajo amenaza de ataque por parte de forajidos y ha pedido ayuda. Necesitamos a alguien que lo proteja y ahuyente a los forajidos. \n\nAsegúrate de permanecer cerca después de su ataque inicial. Con demasiada frecuencia, los forajidos ganan las peleas simplemente enviando más hombres de los que nadie puede defender razonablemente, así que asegúrate de repeler cualquier refuerzo antes de abandonar la zona. \n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 75 / 200\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Cluster JWY-925, RAB-CHARLIE, RAB-MAT&lt;/EM4&gt;\n- Rifle Karna "Fate"\n- Núcleo Artimex (modificado)\n- Brazos Artimex (modificados)\n- Batería de rifle Karna (capacidad 35)\n\n&lt;EM4&gt;outpost_regionab&lt;/EM4&gt;\n- Rifle Karna\n- Brazos Artimex\n- Núcleo Artimex\n- Piernas Artimex\n- Casco Artimex\n- Batería de rifle Karna (capacidad 35)\n</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>We’ve learned that XenoThreat is about to launch an attack on {0} If they are successful, the number of casualties is expected to be high. I’m hoping that with your aid in defending them, we can make sure that doesn’t happen.\n \nWe know from past encounters that XenoThreat sends several raiding parties to carry out their attacks, so make sure you don’t leave the outpost until you’ve fought off all the reinforcements. \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna "Fate" Rifle\n- Artimex Core (Modified)\n- Artimex Arms (Modified)\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Hemos descubierto que XenoThreat está a punto de lanzar un ataque contra {0}. Si tienen éxito, se espera que el número de bajas sea elevado. Espero que con vuestra ayuda para defenderlos, podamos asegurarnos de que eso no ocurra.\n \nSabemos por encuentros anteriores que XenoThreat envía varios grupos de asalto para llevar a cabo sus ataques, así que aseguraos de no abandonar el puesto de avanzada hasta que hayáis repelido a todos los refuerzos. \n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Fusil Karna "Destino"\n- Núcleo Artimex (modificado)\n- Brazos Artimex (modificados)\n- Batería de fusil Karna (capacidad 35)\n</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>Urgent!\n\nXenoThreat is targeting {0} to send a message to other settlers about what happens if they accept our support. \n\nIf you’re able to fend off the attackers, I’m sure they’ll send additional forces, so you’ll need to dig in for multiple assaults. Since XenoThreat has a lot of resources at their disposal, you should think about recruiting others to help you keep everyone safe.\n\nWe’re all counting on you.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Arms\n- Artimex Core\n- Artimex Legs\n- Artimex Helmet\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>¡Urgente!\n\nXenoThreat tiene como objetivo {0} para enviar un mensaje a otros colonos sobre lo que sucederá si aceptan nuestro apoyo.\n\nSi logras repeler a los atacantes, estoy seguro de que enviarán fuerzas adicionales, así que tendrás que prepararte para múltiples asaltos. Dado que XenoThreat tiene muchos recursos a su disposición, deberías considerar reclutar a otros para que te ayuden a mantener a todos a salvo.\n\nTodos contamos contigo.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna\n- Brazos Artimex\n- Núcleo Artimex\n- Piernas Artimex\n- Casco Artimex\n- Batería de rifle Karna (35 cap)\n</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>Urgent!\n\nXenoThreat is mobilizing for a massive incursion to wipe {0} off the map. You’re their only hope of enduring this assault and protecting them from XenoThreat’s cruelty.\n\nI know I’m asking you to put yourself in the line of fire, but this system won’t change unless people like you are brave enough to take on these dangers. No amount of credits could measure up to how much good you’d be doing by stepping in.\n\nIf you’re willing and able to take on this mission, make sure to take some allies with you. XenoThreat will certainly send in stronger reinforcements once they realize they’re taking losses.\n\nWe believe in you.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Arms\n- Artimex Core\n- Artimex Legs\n- Artimex Helmet\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>¡Urgente!\n\nXenoThreat se está movilizando para una incursión masiva con el objetivo de borrar a {0} del mapa. Eres su única esperanza para resistir este ataque y protegerlos de la crueldad de XenoThreat.\n\nSé que te estoy pidiendo que te pongas en la línea de fuego, pero este sistema no cambiará a menos que personas como tú sean lo suficientemente valientes como para afrontar estos peligros. Ninguna cantidad de créditos podría compensar el bien que harías al intervenir.\n\nSi estás dispuesto y eres capaz de asumir esta misión, asegúrate de llevar algunos aliados contigo. XenoThreat sin duda enviará refuerzos más fuertes una vez que se den cuenta de que están sufriendo bajas.\n\nCreemos en ti.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna\n- Brazos Artimex\n- Núcleo Artimex\n- Piernas Artimex\n- Casco Artimex\n- Batería para rifle Karna (35 cap)\n</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>We just received reports of a massive attack against {0} by a large group of armed individuals led by {1} a notorious outlaw who has been threatening Citizens for Prosperity personnel for months. Details are still yet to be confirmed but we know there have been multiple casualties.\n\nCitizens for Prosperity is looking for any qualified security personnel to go and retake the outposts from these hostile elements. Our understanding is that {2} tends to hide behind their soldiers, but will emerge if you take enough of the rank-and-file out.\n\nWhile we don't like to resort to violence, management can see no other way of resolving this situation and continuing our good work in the system.\n\nGood luck,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 800\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Core Canuto\n- Artimex Arms Canuto\n- Artimex Legs Canuto\n- Artimex Helmet Canuto\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Acabamos de recibir informes de un ataque masivo contra {0} por parte de un numeroso grupo de individuos armados liderados por {1}, un conocido delincuente que lleva meses amenazando al personal de Ciudadanos por la Prosperidad. Aún no se han confirmado los detalles, pero sabemos que ha habido varias víctimas.\n\nCiudadanos por la Prosperidad busca personal de seguridad cualificado para recuperar los puestos de avanzada de manos de estos elementos hostiles. Entendemos que {2} tiende a esconderse detrás de sus soldados, pero emergerá si eliminas a suficientes soldados rasos.\n\nSi bien no nos gusta recurrir a la violencia, la gerencia no ve otra forma de resolver esta situación y continuar nuestro buen trabajo en el sistema.\n\nBuena suerte,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 800\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna\n- Núcleo Artimex Canuto\n- Brazos Artimex Canuto\n- Piernas Artimex Canuto\n- Casco Artimex Canuto\n- Batería de rifle Karna (35 cap)\n</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>We received a distress call from {0} saying that they're being robbed by a small group of outlaws. {1} Though remote, this outpost is a crucial piece of CFP's infrastructure in the area so we need to take it back.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Arms\n- Artimex Core\n- Artimex Legs\n- Artimex Helmet\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Recibimos una llamada de auxilio de {0} diciendo que están siendo asaltados por un pequeño grupo de forajidos. {1} Aunque remoto, este puesto de avanzada es una pieza crucial de la infraestructura de CFP en la zona, así que necesitamos recuperarlo.\n\nLima Endicott\nOperadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna\n- Brazos Artimex\n- Núcleo Artimex\n- Piernas Artimex\n- Casco Artimex\n- Batería de rifle Karna (capacidad 35)\n</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>A distress call just came in from {0} claiming that a large Headhunter force has just attacked our outpost there. There have been multiple deaths and injuries from those who managed to flee the scene. We're looking for any available security personnel to head there and retake the outpost.\n\nWitness accounts identified the attackers as elite Headhunter enforcers, so watch yourself out there and bring help if you can. \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Arms\n- Artimex Core\n- Artimex Legs\n- Artimex Helmet\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Acabamos de recibir una llamada de auxilio de {0} informando que una gran fuerza de Headhunters ha atacado nuestro puesto avanzado. Se han registrado múltiples muertos y heridos entre quienes lograron huir. Buscamos personal de seguridad disponible para que se dirija allí y retome el puesto avanzado.\n\nLos testimonios identificaron a los atacantes como agentes de élite de Headhunters, así que tengan cuidado y traigan ayuda si pueden. \n\nLima Endicott\nOficial de despacho principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna\n- Brazos Artimex\n- Núcleo Artimex\n- Piernas Artimex\n- Casco Artimex\n- Batería de rifle Karna (capacidad 35)\n</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>Headhunters have launched an unprovoked attack against {0} Although we don't support the use of violence, Citizens for Prosperity won't let innocent people die. We need qualified security personnel to retake the outpost.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Arms\n- Artimex Core\n- Artimex Legs\n- Artimex Helmet\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Los cazadores de cabezas han lanzado un ataque no provocado contra {0}. Aunque no apoyamos el uso de la violencia, Ciudadanos por la Prosperidad no permitirá que mueran personas inocentes. Necesitamos personal de seguridad cualificado para retomar el puesto de avanzada.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna\n- Brazos Artimex\n- Núcleo Artimex\n- Piernas Artimex\n- Casco Artimex\n- Batería de rifle Karna (35 cap)\n</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>We've received a distress call from {0} A group of unknown assailants have launched an attack. There have been multiple deaths reported and we need to reclaim the outpost.\n\nI know this is far from your current position, but we're desperate to secure the area and get the outpost back and running again.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: RAB-ULTRA, RAB-LYNX, Terminus&lt;/EM4&gt;\n- Karna "Brimstone" Rifle\n- Artimex Core Lodestone\n- Artimex Arms Lodestone\n- Artimex Legs Lodestone\n- Artimex Helmet Lodestone\n- Karna Rifle Battery (35 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Pyro I, RAB-MAT, Cluster BGR-560&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Arms\n- Artimex Core\n- Artimex Legs\n- Artimex Helmet\n- Karna Rifle Battery (35 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-XENO, Fuego, RAB-POINT&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Core Canuto\n- Artimex Arms Canuto\n- Artimex Legs Canuto\n- Artimex Helmet Canuto\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Hemos recibido una llamada de auxilio de {0}. Un grupo de asaltantes desconocidos ha lanzado un ataque. Se han reportado múltiples muertes y necesitamos recuperar el puesto avanzado.\n\nSé que esto está lejos de tu posición actual, pero estamos desesperados por asegurar el área y hacer que el puesto avanzado vuelva a funcionar.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-ULTRA, RAB-LYNX, Terminus&lt;/EM4&gt;\n- Rifle Karna "Brimstone"\n- Piedra imán Artimex Core\n- Piedra imán Artimex Arms\n- Piedra imán Artimex Legs\n- Piedra imán Artimex Helmet\n- Batería de rifle Karna (35 cap)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Pyro I, RAB-MAT, Cluster BGR-560&lt;/EM4&gt;\n- Rifle Karna\n- Brazos Artimex\n- Núcleo Artimex\n- Piernas Artimex\n- Casco Artimex\n- Batería de rifle Karna (35 cap)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-XENO, Fuego, RAB-POINT&lt;/EM4&gt;\n- Rifle Karna\n- Núcleo Artimex Canuto\n- Brazos Artimex Canuto\n- Piernas Artimex Canuto\n- Casco Artimex Canuto\n- Batería de rifle Karna (35 cap)\n</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>One of our pilots had just picked up a shipment of supplies near {0} when they were attacked by some vicious shipjackers. \n\nWe just received their distress beacon and I'm hoping you can go provide them combat support.\n\nAny assistance you could give would make all the difference.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 150\n\n&lt;EM4&gt;Potential Blueprints (Nyx Only)&lt;/EM4&gt;\n- R97 Shotgun\n- Monde Arms\n- Monde Core\n- Monde Legs\n- Monde Helmet\n- Monde Arms Hiro\n- Monde Core Hiro\n- Monde Legs Hiro\n- Monde Helmet Hiro\n- R97 Shotgun Magazine (18 cap)\n</v>
+        <v>Uno de nuestros pilotos acababa de recoger un cargamento de suministros cerca de {0} cuando fueron atacados por unos despiadados secuestradores de naves. \n\nAcabamos de recibir su baliza de socorro y espero que puedas ir a brindarles apoyo en combate.\n\nCualquier ayuda que puedas brindar marcaría la diferencia.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 150\n\n&lt;EM4&gt;Planos potenciales (solo Nyx)&lt;/EM4&gt;\n- Escopeta R97\n- Monde Arms\n- Monde Core\n- Monde Legs\n- Monde Helmet\n- Monde Arms Hiro\n- Monde Core Hiro\n- Monde Legs Hiro\n- Monde Helmet Hiro\n- Cargador de escopeta R97 (capacidad de 18)\n</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>A Citizens for Prosperity affiliated ship was attempting to deliver some supplies to {0} when they were attacked by the recipients who didn't want to pay for their purchase and chose violence instead.\n\nI'll instruct our traders to be more careful about who they deal with in the future, but for now, I would really appreciate you lending them a hand in fighting off these attackers. \n\nAppreciated,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 150 / 200\n\n&lt;EM4&gt;Potential Blueprints (Nyx Only)&lt;/EM4&gt;\n- R97 Shotgun\n- Monde Arms\n- Monde Core\n- Monde Legs\n- Monde Helmet\n- Monde Arms Hiro\n- Monde Core Hiro\n- Monde Legs Hiro\n- Monde Helmet Hiro\n- R97 Shotgun Magazine (18 cap)\n</v>
+        <v>Un barco afiliado a Ciudadanos por la Prosperidad intentaba entregar suministros a {0} cuando fue atacado por los destinatarios, quienes no quisieron pagar su compra y optaron por la violencia.\n\nInstruiré a nuestros comerciantes para que tengan más cuidado con quién tratan en el futuro, pero por ahora, les agradecería mucho que les echaran una mano para repeler a estos atacantes. \n\nAgradecido,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 150 / 200\n\n&lt;EM4&gt;Planos potenciales (solo Nyx)&lt;/EM4&gt;\n- Escopeta R97\n- Monde Arms\n- Monde Core\n- Monde Legs\n- Monde Helmet\n- Monde Arms Hiro\n- Monde Core Hiro\n- Monde Legs Hiro\n- Monde Helmet Hiro\n- Cargador de escopeta R97 (capacidad de 18)\n</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>Despite our efforts to promote non-violence, local outlaw groups continue to attack our organization. XenoThreat recently assaulted {0} and chased out our volunteers that had been working there.\n\nWe're looking to enlist combat personnel to retake the outpost. Ideally we could work something out to encourage them to move on, but XenoThreat quickly resorts to violence to solve all their issues so there will undoubtedly be a fight.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Core Canuto\n- Artimex Arms Canuto\n- Artimex Legs Canuto\n- Artimex Helmet Canuto\n- Karna Rifle Battery (35 cap)\n</v>
+        <v> pesar de nuestros esfuerzos por promover la no violencia, los grupos locales de delincuentes siguen atacando a nuestra organización. XenoThreat agredió recientemente a {0} y expulsó a nuestros voluntarios que trabajaban allí.\n\nBuscamos reclutar personal de combate para retomar el puesto de avanzada. Idealmente, podríamos llegar a un acuerdo para animarlos a marcharse, pero XenoThreat recurre rápidamente a la violencia para resolver todos sus problemas, así que sin duda habrá una pelea.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna\n- Núcleo Artimex Canuto\n- Brazos Artimex Canuto\n- Piernas Artimex Canuto\n- Casco Artimex Canuto\n- Batería de rifle Karna (35 cap)\n</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>Citizens for Prosperity is looking for any available combat operators to {0} A group of outlaws have launched an unprovoked attack and our security personnel are desperately in need of support.\n\nPlease dispatch to {1} with all urgency and good luck.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Core Canuto\n- Artimex Arms Canuto\n- Artimex Legs Canuto\n- Artimex Helmet Canuto\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Ciudadanos por la Prosperidad busca operadores de combate disponibles para {0} Un grupo de forajidos ha lanzado un ataque no provocado y nuestro personal de seguridad necesita apoyo urgentemente.\n\nPor favor, envíenlos a {1} con toda urgencia y buena suerte.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna\n- Núcleo Artimex Canuto\n- Brazos Artimex Canuto\n- Piernas Artimex Canuto\n- Casco Artimex Canuto\n- Batería de rifle Karna (35 cap)\n</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>XenoThreat forces launched an unprovoked attack near {0} We're looking for any available combat operators to go and provide support. \n\nIf you haven't dealt with them before, it's important to know that XenoThreat are trained fighters so this will not be an easy fight, but it's a necessary one.\n\nGood luck,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200 / 400\n\n&lt;EM4&gt;Potential Blueprints (Pyro IV/V Area Only)&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Core Canuto\n- Artimex Arms Canuto\n- Artimex Legs Canuto\n- Artimex Helmet Canuto\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Las fuerzas de XenoThreat lanzaron un ataque no provocado cerca de {0}. Buscamos operadores de combate disponibles para brindar apoyo. \n\nSi no los has enfrentado antes, es importante saber que XenoThreat son combatientes entrenados, por lo que esta no será una lucha fácil, pero es necesaria.\n\nBuena suerte,\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200 / 400\n\n&lt;EM4&gt;Planos potenciales (solo área Pyro IV/V)&lt;/EM4&gt;\n- Rifle Karna\n- Núcleo Artimex Canuto\n- Brazos Artimex Canuto\n- Piernas Artimex Canuto\n- Casco Artimex Canuto\n- Batería de rifle Karna (35 cap)\n</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>We received an emergency comm from {0} reporting that they are currently under attack by a group of Headhunters. We know our presence in the system has upset the Headhunters, but it hardly excuses this unprovoked attack.\n\nIf available, please gather your gear and head out. Just understand that Headhunters are experienced fighters and will not back down easily.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100 / 200\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Vatra, Pyro IV, RAB-ECHO&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Core Canuto\n- Artimex Arms Canuto\n- Artimex Legs Canuto\n- Artimex Helmet Canuto\n- Karna Rifle Battery (35 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-ION, Terminus, Cluster DLO-486&lt;/EM4&gt;\n- Karna "Rager" Rifle\n- Artimex Core Wildwood\n- Artimex Arms Wildwood\n- Artimex Legs Wildwood\n- Artimex Helmet Wildwood\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Hemos recibido una comunicación de emergencia de {0} informando que están siendo atacados por un grupo de Headhunters. Sabemos que nuestra presencia en el sistema ha molestado a los Headhunters, pero eso no justifica este ataque no provocado.\n\nSi es posible, por favor, reúnan su equipo y salgan. Solo entiende que los Headhunters son luchadores experimentados y no retrocederán fácilmente.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100 / 200\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Vatra, Pyro IV, RAB-ECHO&lt;/EM4&gt;\n- Rifle Karna\n- Núcleo Artimex Canuto\n- Brazos Artimex Canuto\n- Piernas Artimex Canuto\n- Casco Artimex Canuto\n- Batería de rifle Karna (35 cap)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-ION, Terminus, Cluster DLO-486&lt;/EM4&gt;\n- Rifle Karna "Rager"\n- Núcleo Artimex Wildwood\n- Brazos Artimex Wildwood\n- Piernas Artimex Wildwood\n- Casco Artimex Wildwood\n- Batería para rifle Karna (35 cápsulas)\n</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>Citizens for Prosperity is looking for security personnel to take a former CFP outpost that's currently serving as a hideout for Headhunters to launch attacks throughout the system. \n\nLocated near {0} reclaiming this outpost will allow CFP to provide greater support to local efforts to build stability.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Karna Rifle\n- Artimex Arms\n- Artimex Core\n- Artimex Legs\n- Artimex Helmet\n- Karna Rifle Battery (35 cap)\n</v>
+        <v>Ciudadanos por la Prosperidad busca personal de seguridad para hacerse cargo de un antiguo puesto avanzado de CFP que actualmente sirve de escondite para que los Cazadores de Cabezas lancen ataques por todo el sistema. \n\nUbicado cerca de {0}, recuperar este puesto avanzado permitirá a CFP brindar mayor apoyo a los esfuerzos locales para construir estabilidad.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle Karna\n- Brazos Artimex\n- Núcleo Artimex\n- Piernas Artimex\n- Casco Artimex\n- Batería de rifle Karna (35 cap)\n</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>Welcome to the system, not sure if you're familiar with our organization but Citizens for Prosperity are a non-profit organization dedicated to bringing security and civilization to unclaimed systems.\n\nIf you're looking for work in the system and would like to help achieve our goal, we need a package picked up from &lt;EM4&gt;{0} and taken to &lt;EM4&gt;{1} complete, we can offer you a variety of new job opportunities in this system and beyond.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50</v>
+        <v>Bienvenido al sistema. No sé si conoce nuestra organización, pero Ciudadanos por la Prosperidad es una organización sin fines de lucro dedicada a brindar seguridad y civilización a sistemas no reclamados.\n\nSi busca trabajo en el sistema y desea ayudarnos a lograr nuestro objetivo, necesitamos que recoja un paquete de &lt;EM4&gt;{0} y lo lleve a &lt;EM4&gt;{1} completo. Podemos ofrecerle diversas oportunidades laborales en este sistema y más allá.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>Hi,\n\nOne of our outposts at &lt;EM4&gt;{0} is in need of some light repairs. The folks onsite have estimated that you’ll need &lt;EM4&gt;three fuses&lt;/EM4&gt;, a &lt;EM4&gt;salvaging tool&lt;/EM4&gt;, and &lt;EM4&gt;enough RMC canisters to fix up to three or so pipes.&lt;/EM4&gt;\n\nIf you need more information on maintenance work, see &lt;EM4&gt;“Cornerstone Developments' Guide to Maintenance”&lt;/EM4&gt; entry in your mobiGlas Journal.\n\nThanks again for your help,\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50</v>
+        <v>Hola,\n\nUno de nuestros puestos avanzados en &lt;EM4&gt;{0} necesita algunas reparaciones menores. El personal en el lugar ha estimado que necesitará &lt;EM4&gt;tres fusibles&lt;/EM4&gt;, una &lt;EM4&gt;herramienta de recuperación&lt;/EM4&gt; y &lt;EM4&gt;suficientes cartuchos RMC para reparar hasta tres tuberías aproximadamente.&lt;/EM4&gt;\n\nSi necesita más información sobre trabajos de mantenimiento, consulte la entrada &lt;EM4&gt;“Guía de mantenimiento de Cornerstone Developments”&lt;/EM4&gt; en su diario de mobiGlas.\n\nGracias nuevamente por su ayuda,\n\nLima Endicott\nDespachadora principal\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>We need some help. The CFP facility at &lt;EM4&gt;{0} suffered severe damage during a recent electrical storm and we're looking for anyone who can help with repairs.\n\nSurveying the site, you'll have to bring &lt;EM4&gt;six fuses&lt;/EM4&gt;, a &lt;EM4&gt;salvaging tool&lt;/EM4&gt;, and &lt;EM4&gt;enough RMC canisters to take care of eight or so pipes&lt;/EM4&gt;. That should be enough to repair the damage and get the outpost back in operation.\n\nIf you need more information on maintenance work, see &lt;EM4&gt;“Cornerstone Developments' Guide to Maintenance”&lt;/EM4&gt; entry in your mobiGlas Journal.\n\nDo you think you can help?\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 400</v>
+        <v>Necesitamos ayuda. Las instalaciones de CFP en &lt;EM4&gt;{0} sufrieron graves daños durante una reciente tormenta eléctrica y buscamos a alguien que pueda ayudar con las reparaciones.\n\nPara inspeccionar el sitio, deberá traer &lt;EM4&gt;seis fusibles&lt;/EM4&gt;, una &lt;EM4&gt;herramienta de recuperación&lt;/EM4&gt; y &lt;EM4&gt;suficientes botes de RMC para reparar unas ocho tuberías&lt;/EM4&gt;. Eso debería ser suficiente para reparar los daños y poner el puesto de avanzada de nuevo en funcionamiento.\n\nSi necesita más información sobre trabajos de mantenimiento, consulte la entrada &lt;EM4&gt;“Guía de mantenimiento de Cornerstone Developments”&lt;/EM4&gt; en su diario de mobiGlas.\n\n¿Cree que puede ayudar?\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 400</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>An upstanding member of the Citizens for Prosperity community, Doctor {0} was recently abducted by XenoThreat while distributing vital medical supplies to one of our settlements.\n\nThe kidnappers were last seen entering their base at {1} but we are uncertain whether they will remain there for long. XenoThreat maintains multiple outposts throughout this system and has been known to swap locations at a moment's notice. \n\nConsidering the danger and the distance you may have to travel, CFP is prepared to offer a substantial reward for determining what happened to Dr. {2} Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 400</v>
+        <v>El doctor {0}, un miembro ejemplar de la comunidad Ciudadanos por la Prosperidad, fue secuestrado recientemente por XenoThreat mientras distribuía suministros médicos vitales a uno de nuestros asentamientos.\n\nLos secuestradores fueron vistos por última vez entrando en su base en {1}, pero no estamos seguros de si permanecerán allí mucho tiempo. XenoThreat mantiene múltiples puestos avanzados en todo este sistema y se sabe que cambia de ubicación en cualquier momento.\n\nConsiderando el peligro y la distancia que podría tener que recorrer, CFP está dispuesto a ofrecer una recompensa sustancial por determinar qué le sucedió al Dr. {2} Endicott.\nDespachador principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 400</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>Two of our volunteers vanished while on a recent foraging expedition. It has been over two standard days since their disappearance, and their families have begun to fear the worst and are willing to offer a reward if someone can help trace their whereabouts.\n\nThey were last seen in the vicinity of {0} It is possible that they may have been injured and sought shelter in an abandoned building or a cave. The area is full of potential hiding spots, so your search will need to be thorough. \n\nThank you for taking this on. \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 800</v>
+        <v>Dos de nuestros voluntarios desaparecieron durante una reciente expedición de recolección. Han transcurrido más de dos días desde su desaparición, y sus familias temen lo peor y ofrecen una recompensa a quien pueda ayudar a localizarlos.\n\nFueron vistos por última vez en las cercanías de {0}. Es posible que se hayan lesionado y hayan buscado refugio en un edificio abandonado o una cueva. La zona está llena de posibles escondites, por lo que la búsqueda deberá ser exhaustiva.\n\nGracias por su colaboración.\n\nLima Endicott\nOficial de Despacho\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 800</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>{0} a member of the Citizens for Prosperity family, vanished two standard days ago while attempting to find a buyer for some old farming equipment. CFP regrets to report that we have just discovered the wreckage of a vehicle registered under the name of the missing person in an area known to be frequented by pirates. \n\nWe found evidence at the crash site that the victim survived and is most likely being held at {1} We are offering a reward to anyone who can track down {2} on our behalf. \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100</v>
+        <v>{0}, miembro de la familia Ciudadanos por la Prosperidad, desapareció hace dos días estándar mientras intentaba encontrar un comprador para algunos equipos agrícolas viejos. CFP lamenta informar que acabamos de descubrir los restos de un vehículo registrado a nombre de la persona desaparecida en un área conocida por ser frecuentada por piratas. \n\nEncontramos evidencia en el lugar del accidente de que la víctima sobrevivió y probablemente se encuentra retenida en {1}. Ofrecemos una recompensa a cualquiera que pueda localizar a {2} en nuestro nombre. \n\nLima Endicott\nOficial de Despacho Principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>Junior surveyor {0} fell out of contact with their team while identifying potentially viable mineral seams in a cave near {1} Wild animals have been known to frequent this location, which has led Citizens for Prosperity to believe that the surveyor may have been attacked while on the job and is currently stranded. \n\nWe need someone to find them and render aid if at all possible. If it's too late and they're beyond help, it will at least comfort the rest of the team to know what happened to their friend. \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50</v>
+        <v>El topógrafo junior {0} perdió el contacto con su equipo mientras identificaba vetas minerales potencialmente viables en una cueva cerca de {1}. Se sabe que animales salvajes frecuentan este lugar, lo que ha llevado a Ciudadanos por la Prosperidad a creer que el topógrafo pudo haber sido atacado mientras trabajaba y actualmente se encuentra atrapado. \n\nNecesitamos que alguien lo encuentre y le preste ayuda si es posible. Si es demasiado tarde y no hay nada que hacer por él, al menos reconfortará al resto del equipo saber qué le sucedió a su amigo. \n\nLima Endicott\nOficial de Despacho Principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>Citizens for Pyro is concerned about one of our local contractors, {0} They finished up a trade at {1} and haven’t been seen since. We’re hearing reports that outlaws have been frequenting the area, so I suspect that the worst might have happened.\n\nEither way, {2} has done good work for us in the past and I’d hate for them to wind up as just another one of the system's missing. If you’re willing to find them for me, I’ll see that you get a reward.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100</v>
+        <v>Citizens for Pyro está preocupado por uno de nuestros contratistas locales, {0}. Terminó un trabajo en {1} y no se le ha visto desde entonces. Estamos recibiendo informes de que forajidos han estado frecuentando la zona, así que sospecho que podría haber ocurrido lo peor.\n\nDe cualquier manera, {2} ha hecho un buen trabajo para nosotros en el pasado y me daría mucha pena que terminara siendo uno más de los desaparecidos del sistema. Si estás dispuesto a encontrarlo por mí, me aseguraré de que recibas una recompensa.\n\nLima Endicott\nDespachadora principal\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>During what should have been a routine cargo run, hauler and long-time friend of Citizens for Prosperity {0} was ambushed and abducted by XenoThreat. The coded distress signal we received from the victim just before their comms went dark gave us just enough information to pinpoint their most likely location: {1} needs someone to slip into the outpost, confirm the whereabouts of {2} and relay this information back to us so we know exactly where to send our rescue team. Or, in the worst possible scenario, deliver news to the hauler's family that their loved one didn't survive. \n\nWe understand how dangerous it is to approach a XenoThreat stronghold, and are prepared to offer a sizeable reward for putting yourself at risk.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 400</v>
+        <v>Durante lo que debería haber sido un viaje de carga rutinario, el transportista y viejo amigo de Ciudadanos por la Prosperidad {0} fue emboscado y secuestrado por XenoThreat. La señal de socorro codificada que recibimos de la víctima justo antes de que sus comunicaciones se cortaran nos dio la información suficiente para determinar su ubicación más probable: {1} necesita que alguien se infiltre en el puesto de avanzada, confirme el paradero de {2} y nos transmita esta información para que sepamos exactamente dónde enviar a nuestro equipo de rescate. O, en el peor de los casos, que le comunique a la familia del transportista que su ser querido no sobrevivió. \n\nEntendemos lo peligroso que es acercarse a una fortaleza de XenoThreat y estamos dispuestos a ofrecer una recompensa considerable por ponerse en riesgo.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 400</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>{0} a mechanic who has performed countless services for our community, was abducted by a group of outlaws three standard days ago. CFP has received a ransom comm, but we refuse to negotiate with the types of people who actively work to destroy the peace in this system. If we open that door even once, we will never be safe. \n\nThe outlaws known to have abducted {1}  were last seen entering {2} CFP needs someone to infiltrate the base and confirm our missing person's whereabouts.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v>{0} Un mecánico que ha prestado innumerables servicios a nuestra comunidad, fue secuestrado por un grupo de forajidos hace tres días estándar. CFP ha recibido una comunicación de rescate, pero nos negamos a negociar con el tipo de personas que trabajan activamente para destruir la paz en este sistema. Si abrimos esa puerta aunque sea una sola vez, nunca estaremos a salvo. \n\nLos forajidos que se sabe que secuestraron a {1} fueron vistos por última vez entrando en {2}. CFP necesita que alguien se infiltre en la base y confirme el paradero de nuestra persona desaparecida.\n\nLima Endicott\nOperadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>We've received disturbing news: {0} the scout that was reported missing last week has been seen in Headhunter custody. According to the witness, they were spotted being loaded into a transport headed to {1} this time yesterday. \n\nIf anyone out there can confirm their whereabouts, there's a reward in store. Citizens for Prosperity maintains hope that they are alive and well. If not, their families deserve to know their fates either way. \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100</v>
+        <v>Hemos recibido noticias inquietantes: {0} el explorador que fue reportado como desaparecido la semana pasada ha sido visto bajo custodia de Headhunter. Según el testigo, fue visto siendo subido a un transporte con destino a {1} ayer a esta misma hora. \n\nSi alguien puede confirmar su paradero, hay una recompensa. Ciudadanos por la Prosperidad mantiene la esperanza de que esté vivo y bien. De no ser así, sus familias merecen saber su destino. \n\nLima Endicott\nOficial de Despacho Principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>Last night, the homesteader {0} was abducted by Headhunters for unknown reasons. Citizens for Prosperity has not received a ransom note, nor has the victim's family. However, we have just received word from an informant that the abducted party was most likely taken to {1} \n\nWe need someone to determine the validity of this information, and to report back to CFP. A reward will be provided whether your findings are good or bad. \n\nYou may need to utilize a ground vehicle to help you search the area. \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100</v>
+        <v>Anoche, el colono {0} fue secuestrado por cazadores de cabezas por razones desconocidas. Ciudadanos por la Prosperidad no ha recibido ninguna nota de rescate, ni tampoco la familia de la víctima. Sin embargo, acabamos de recibir información de un informante de que la persona secuestrada probablemente fue llevada a {1}. \n\nNecesitamos que alguien determine la veracidad de esta información y que se la comunique a Ciudadanos por la Prosperidad. Se ofrecerá una recompensa independientemente de si sus hallazgos son positivos o negativos. \n\nEs posible que necesite utilizar un vehículo terrestre para ayudarle a registrar la zona. \n\nLima Endicott\nOficial de Despacho Principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>A small group of Citizens for Prosperity members were supposed to be delivering sensitive data back to our headquarters in Stanton, but they never arrived. \n\nWe now believe that they were captured by XenoThreat before they could leave the system. I'd like you to investigate {0} to discover what happened to the missing crew and then destroy any servers they could be using to store the stolen data.\n\nYour help is very appreciated,\n \nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 1,500</v>
+        <v>Un pequeño grupo de miembros de Ciudadanos por la Prosperidad debía entregar datos confidenciales a nuestra sede en Stanton, pero nunca llegaron. \n\nAhora creemos que fueron capturados por XenoThreat antes de que pudieran abandonar el sistema. Me gustaría que investigaras {0} para descubrir qué les sucedió a los desaparecidos y luego destruyeras cualquier servidor que pudieran estar utilizando para almacenar los datos robados.\n\nAgradecemos mucho tu ayuda.\n \nLima Endicott\nOperadora principal\nCiudadanos por la Prosperidad\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 1500</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>I just have received confirmation that {0} a Citizens for Prosperity courier, was captured by the Headhunters while transporting some critical data. \n\nWe need you to investigate {1} to discover what happened to {2} and then destroy any Headhunter servers that may contain stolen data.\n\nWe're counting on you,\n \nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 1,500</v>
+        <v>Acabo de recibir confirmación de que {0}, un mensajero de Ciudadanos por la Prosperidad, fue capturado por los Cazadores de Cabezas mientras transportaba datos críticos. \n\nNecesitamos que investigues {1} para descubrir qué le sucedió a {2} y luego destruyas cualquier servidor de los Cazadores de Cabezas que pueda contener datos robados.\n\nContamos contigo,\n \nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 1500</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>The family of {0} a Citizens for Prosperity courier, has been in contact with me with the terrible news that they never arrived back home. We learned that {1} was captured by XenoThreat while transporting some critical data. \n\nWe need you to search {2} and see if you can learn what has become of {3} and then destroy any XenoThreat servers that may contain stolen data.\n\nThank you,\n \nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 1,500</v>
+        <v> La familia de {0}, mensajero de Ciudadanos por la Prosperidad, se ha puesto en contacto conmigo con la terrible noticia de que no han regresado a casa. Nos enteramos de que {1} fue capturado por XenoThreat mientras transportaba datos críticos. \n\nNecesitamos que busques a {2} y averigües qué le ha sucedido a {3}, y que destruyas cualquier servidor de XenoThreat que pueda contener datos robados.\n\nGracias,\n \nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 1500</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>One of our most trusted datarunners, {0} has found themselves the victim of a XenoThreat assault. Now both they and the data they were ferrying have been captured and taken to {1} \n\nI am charging you with heading there to ascertain what happened to {2} and to destroy data servers which may be housing the stolen information.\n\nEven if the worst has happened, I think they would want us to make sure they data they were charged with protecting isn't used for nefarious gains.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 1,500</v>
+        <v>Uno de nuestros agentes de datos más confiables, {0}, ha sido víctima de un ataque de XenoThreat. Ahora, tanto él como los datos que transportaba han sido capturados y llevados a {1}. \n\nTe encargo que vayas allí para averiguar qué le sucedió a {2} y destruir los servidores de datos que podrían contener la información robada.\n\nIncluso si ha ocurrido lo peor, creo que querrían que nos aseguráramos de que los datos que tenían la responsabilidad de proteger no se utilicen para fines maliciosos.\n\nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 1500</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>We have gotten word that the outlaws at {0} have begun recruiting with the hopes of launching a raid against Citizens for Prosperity. \n\nIn order to deescalate the situation before it gets out of hand, we would like you to disable their power generators and halt their expansion. \n\nPull this off and it could save a lot of lives.\n \nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 150\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- FS-9 LMG\n- BR-2 Shotgun\n- Gallant Rifle\n- ADP Arms Woodland\n- ADP Core\n- ADP Legs Woodland\n- Balor HCH Helmet\n- ADP-mk4 Arms Woodland\n- ADP-mk4 Legs Woodland\n- ADP-mk4 Core Woodland\n- ADP-mk4 Helmet Woodland\n- FS-9 Magazine (75 cap)\n- BR-2 Shotgun Magazine (12 cap)\n- Gallant Rifle Battery (45 cap)\n</v>
+        <v>Hemos recibido información de que los forajidos de {0} han comenzado a reclutar con la intención de lanzar un ataque contra Ciudadanos por la Prosperidad. \n\nPara calmar la situación antes de que se salga de control, les pedimos que desactiven sus generadores de energía y detengan su expansión. \n\nSi lo logramos, podríamos salvar muchas vidas.\n \nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 150\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Ametralladora ligera FS-9\n- Escopeta BR-2\n- Fusil Gallant\n- Armas ADP Woodland\n- Núcleo ADP\n- Piernas ADP Woodland\n- Casco Balor HCH\n- Armas ADP-mk4 Woodland\n- Piernas ADP-mk4 Woodland\n- Núcleo ADP-mk4 Woodland\n- Casco ADP-mk4 Woodland\n- Cargador FS-9 (75 cap)\n- Cargador de escopeta BR-2 (12 cap)\n- Batería de fusil Gallant (45 cap)\n</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>Following a series of raids against Citizens for Prosperity aligned settlements, we believe we have traced those responsible back to {0} them directly will pose too great of a risk and most likely encourage aggressive reprisals. Instead, we believe that if their power generators were to be disable it could force them to settle somewhere else.\n\nDo you think you could handle it for us?\n \nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: RAB-ULTRA, Cluster NBD-102, RAB-WHISKEY&lt;/EM4&gt;\n- FS-9 LMG\n- BR-2 Shotgun\n- Gallant Rifle\n- ADP Arms Woodland\n- ADP Core\n- ADP Legs Woodland\n- Balor HCH Helmet\n- ADP-mk4 Arms Woodland\n- ADP-mk4 Legs Woodland\n- ADP-mk4 Core Woodland\n- ADP-mk4 Helmet Woodland\n- FS-9 Magazine (75 cap)\n- BR-2 Shotgun Magazine (12 cap)\n- Gallant Rifle Battery (45 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Cluster YKA-011, Ruin Station, Cluster KKE-717&lt;/EM4&gt;\n- P6-LR Sniper Rifle\n- A03 Sniper Rifle\n- CBH-3 Helmet Base\n- PAB-1 Arms Woodland\n- PAB-1 Core Woodland\n- PAB-1 Legs Woodland\n- TrueDef-Pro Arms Base\n- TrueDef-Pro Core Base\n- Argus Helmet Base\n- TrueDef-Pro Legs Base\n- A03 Sniper Rifle Magazine (15 cap)\n- P6-LR Magazine (8 cap)\n</v>
+        <v>Después de una serie de incursiones contra asentamientos alineados con Ciudadanos por la Prosperidad, creemos haber rastreado a los responsables hasta {0} ellos directamente representarán un riesgo demasiado grande y muy probablemente alentarán represalias agresivas. En cambio, creemos que si sus generadores de energía se desactivaran, podrían verse obligados a establecerse en otro lugar.\n\n¿Crees que podrías encargarte de ello por nosotros?\n \nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-ULTRA, Cluster NBD-102, RAB-WHISKEY&lt;/EM4&gt;\n- FS-9 LMG\n- Escopeta BR-2\n- Rifle Gallant\n- Brazos ADP Woodland\n- Núcleo ADP\n- Piernas ADP Woodland\n- Casco Balor HCH\n- Brazos ADP-mk4 Woodland\n- Piernas ADP-mk4 Woodland\n- Núcleo ADP-mk4 Woodland\n- Casco ADP-mk4 Woodland\n- Cargador FS-9 (75 cap)\n- Cargador de escopeta BR-2 (12 cap)\n- Batería de rifle Gallant (45 cap)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Cluster YKA-011, Ruin Station, Cluster KKE-717&lt;/EM4&gt;\n- Rifle de francotirador P6-LR\n- Rifle de francotirador A03\n- Base de casco CBH-3\n- Brazos PAB-1 Woodland\n- Núcleo PAB-1 Woodland\n- Piernas PAB-1 Woodland\n- Base de brazos TrueDef-Pro\n- Base de núcleo TrueDef-Pro\n- Base de casco Argus\n- Base de piernas TrueDef-Pro\n- Cargador de rifle de francotirador A03 (15 cap)\n- Cargador P6-LR (8 cap)\n</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>We're just putting the full picture together now, but so far we've learned that a Headhunter by the name of {0} recently stole some sensitive data that if exposed will be detrimental to Citizens for Prosperity's cause. \n\nWe need to ensure that all traces of the stolen data are eradicated. This means taking out all the Headhunter servers at {1} as well as tracking down {2} to stop them from further disseminating the information.\n\nYour help is much appreciated,\n \nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 1,500\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- P6-LR Sniper Rifle\n- A03 Sniper Rifle\n- CBH-3 Helmet Base\n- PAB-1 Arms Woodland\n- PAB-1 Core Woodland\n- PAB-1 Legs Woodland\n- TrueDef-Pro Arms Base\n- TrueDef-Pro Core Base\n- Argus Helmet Base\n- TrueDef-Pro Legs Base\n- A03 Sniper Rifle Magazine (15 cap)\n- P6-LR Magazine (8 cap)\n</v>
+        <v>Estamos reconstruyendo la situación por completo, pero hasta ahora sabemos que un reclutador llamado {0} robó recientemente datos confidenciales que, de ser expuestos, perjudicarían la causa de Ciudadanos por la Prosperidad. \n\nDebemos asegurarnos de que se eliminen todos los rastros de los datos robados. Esto significa eliminar todos los servidores Headhunter en {1} y localizar {2} para impedir que sigan difundiendo la información.\n\nAgradecemos mucho su ayuda,\n \nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 1500\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle de francotirador P6-LR\n- Rifle de francotirador A03\n- Base de casco CBH-3\n- Brazos PAB-1 Woodland\n- Núcleo PAB-1 Woodland\n- Piernas PAB-1 Woodland\n- Base de brazos TrueDef-Pro\n- Base de núcleo TrueDef-Pro\n- Base de casco Argus\n- Base de piernas TrueDef-Pro\n- Cargador de rifle de francotirador A03 (capacidad de 15)\n- Cargador P6-LR (8 cápsulas)</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>We got a bit of a problem that I'm hoping you can solve for me. One of our informers has revealed that XenoThreat has been amassing data on Citizens for Prosperity operations throughout the system. \n\nThis information, if used correctly, could put our people at serious risk. The best solution is for you to completely destroy the servers where the data is being stored at {0} their trove of information wiped out, it should give our people a fighting chance.\n \nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 75\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: RAB-WHISKEY, Cluster JWY-925, Cluster BGR-560&lt;/EM4&gt;\n- FS-9 LMG\n- BR-2 Shotgun\n- Gallant Rifle\n- ADP Arms Woodland\n- ADP Core\n- ADP Legs Woodland\n- Balor HCH Helmet\n- ADP-mk4 Arms Woodland\n- ADP-mk4 Legs Woodland\n- ADP-mk4 Core Woodland\n- ADP-mk4 Helmet Woodland\n- FS-9 Magazine (75 cap)\n- BR-2 Shotgun Magazine (12 cap)\n- Gallant Rifle Battery (45 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Cluster LHB-976, Ruin Clinic, Ruin Station&lt;/EM4&gt;\n- P6-LR Sniper Rifle\n- A03 Sniper Rifle\n- CBH-3 Helmet Base\n- PAB-1 Arms Woodland\n- PAB-1 Core Woodland\n- PAB-1 Legs Woodland\n- TrueDef-Pro Arms Base\n- TrueDef-Pro Core Base\n- Argus Helmet Base\n- TrueDef-Pro Legs Base\n- A03 Sniper Rifle Magazine (15 cap)\n- P6-LR Magazine (8 cap)\n</v>
+        <v>Tenemos un pequeño problema que espero que puedas resolver. Uno de nuestros informantes ha revelado que XenoThreat ha estado recopilando datos sobre las operaciones de Ciudadanos por la Prosperidad en todo el sistema. Esta información, si se utiliza correctamente, podría poner a nuestra gente en grave riesgo. La mejor solución es que destruyas por completo los servidores donde se almacenan los datos en {0}, borrando así su tesoro de información. Esto debería darles a nuestra gente una oportunidad de luchar.\n \nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 75\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-WHISKEY, Cluster JWY-925, Cluster BGR-560&lt;/EM4&gt;\n- FS-9 LMG\n- Escopeta BR-2\n- Rifle Gallant\n- Brazos ADP Woodland\n- Núcleo ADP\n- Piernas ADP Woodland\n- Casco Balor HCH\n- Brazos ADP-mk4 Woodland\n- Piernas ADP-mk4 Woodland\n- Núcleo ADP-mk4 Woodland\n- Casco ADP-mk4 Woodland\n- Cargador FS-9 (75 cap)\n- Cargador de escopeta BR-2 (12 cap)\n- Batería de rifle Gallant (45 cap)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Cluster LHB-976, Ruin Clinic, Ruin Station&lt;/EM4&gt;\n- Rifle de francotirador P6-LR\n- Rifle de francotirador A03\n- Base de casco CBH-3\n- Brazos PAB-1 Woodland\n- Núcleo PAB-1 Woodland\n- Piernas PAB-1 Woodland\n- Base de brazos TrueDef-Pro\n- Base de núcleo TrueDef-Pro\n- Base de casco Argus\n- Base de piernas TrueDef-Pro\n- Cargador de rifle de francotirador A03 (15 cap)\n- Cargador P6-LR (8 cap)\n</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>The Headhunters recently attacked one of our transports and were sadly able to get their hands on some secure data. Although the encryption on it is strong, its only a matter of time before they'll be able to access it.\n\nBefore that happens, we need you to go to {0} and destroy all traces of the information from their servers.\n\nYou'd really be helping Citizens for Prosperity out if you can pull this off.\n \nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 75 / 150\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: RAB-YORK, Cluster CAJ-445, Cluster BGR-560&lt;/EM4&gt;\n- FS-9 LMG\n- BR-2 Shotgun\n- Gallant Rifle\n- ADP Arms Woodland\n- ADP Core\n- ADP Legs Woodland\n- Balor HCH Helmet\n- ADP-mk4 Arms Woodland\n- ADP-mk4 Legs Woodland\n- ADP-mk4 Core Woodland\n- ADP-mk4 Helmet Woodland\n- FS-9 Magazine (75 cap)\n- BR-2 Shotgun Magazine (12 cap)\n- Gallant Rifle Battery (45 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-POINT, Cluster MNK-833, Vatra&lt;/EM4&gt;\n- P6-LR Sniper Rifle\n- A03 Sniper Rifle\n- CBH-3 Helmet Base\n- PAB-1 Arms Woodland\n- PAB-1 Core Woodland\n- PAB-1 Legs Woodland\n- TrueDef-Pro Arms Base\n- TrueDef-Pro Core Base\n- Argus Helmet Base\n- TrueDef-Pro Legs Base\n- A03 Sniper Rifle Magazine (15 cap)\n- P6-LR Magazine (8 cap)\n</v>
+        <v>Los Headhunters atacaron recientemente uno de nuestros transportes y, lamentablemente, lograron hacerse con algunos datos confidenciales. Aunque el cifrado es fuerte, es solo cuestión de tiempo antes de que puedan acceder a él.\n\nAntes de que eso suceda, necesitamos que vayas a {0} y destruyas todos los rastros de la información de sus servidores.\n\nRealmente estarías ayudando a Ciudadanos por la Prosperidad si puedes lograr esto.\n \nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 75 / 150\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-YORK, Cluster CAJ-445, Cluster BGR-560&lt;/EM4&gt;\n- FS-9 LMG\n- Escopeta BR-2\n- Rifle Gallant\n- Armas ADP Woodland\n- Núcleo ADP\n- Piernas ADP Woodland\n- Casco Balor HCH\n- Brazos ADP-mk4 Woodland\n- Piernas ADP-mk4 Woodland\n- Núcleo ADP-mk4 Woodland\n- Casco ADP-mk4 Woodland\n- Cargador FS-9 (75 cap)\n- Cargador de escopeta BR-2 (12 cap)\n- Batería de rifle Gallant (45 cap)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-POINT, Cluster MNK-833, Vatra&lt;/EM4&gt;\n- Rifle de francotirador P6-LR\n- Rifle de francotirador A03\n- Base de casco CBH-3\n- Brazos PAB-1 Woodland\n- Núcleo PAB-1 Woodland\n- Piernas PAB-1 Woodland\n- Base de brazos TrueDef-Pro\n- Base de núcleo TrueDef-Pro\n- Base de casco Argus\n- Base de piernas TrueDef-Pro\n- Cargador de rifle de francotirador A03 (15 - Cargador P6-LR (8 cápsulas)</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>One of the Citizens for Prosperity members who have been serving as a XenoThreat informer has let us know that the data servers located at {0} our housing a trove of information vital to the gang's operation. \n\nIf you were able to destroy these servers on our behalf it would be a huge win for the security of the entire system.\n \nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- FS-9 LMG\n- BR-2 Shotgun\n- Gallant Rifle\n- ADP Arms Woodland\n- ADP Core\n- ADP Legs Woodland\n- Balor HCH Helmet\n- ADP-mk4 Arms Woodland\n- ADP-mk4 Legs Woodland\n- ADP-mk4 Core Woodland\n- ADP-mk4 Helmet Woodland\n- FS-9 Magazine (75 cap)\n- BR-2 Shotgun Magazine (12 cap)\n- Gallant Rifle Battery (45 cap)\n</v>
+        <v>Uno de los miembros de Citizens for Prosperity que ha estado sirviendo como informante de XenoThreat nos ha hecho saber que los servidores de datos ubicados en {0} albergan un tesoro de información vital para la operación de la banda. \n\nSi pudieras destruir estos servidores en nuestro nombre, sería una gran victoria para la seguridad de todo el sistema.\n \nLima Endicott\nDespachadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 300\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- FS-9 LMG\n- Escopeta BR-2\n- Fusil Gallant\n- Brazos ADP Woodland\n- Núcleo ADP\n- Piernas ADP Woodland\n- Casco Balor HCH\n- Brazos ADP-mk4 Woodland\n- Piernas ADP-mk4 Woodland\n- Núcleo ADP-mk4 Woodland\n- Casco ADP-mk4 Woodland\n- Cargador FS-9 (75 cap)\n- Cargador de escopeta BR-2 (12 cap)\n- Batería de fusil Gallant (45 tapa)\n</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>We’ve been trying to get in contact with community member {0} but haven’t heard from them in a few days. From what Citizens for Prosperity has been able to find out, they were scouting out near {1} which is a known outlaw hotspot.\n\nWe need someone to go there for us and try to locate them, or worst case scenario, their remains. \n\nIf you are able to find them, there’s a reward on offer.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100</v>
+        <v>Hemos intentado contactar con el miembro de la comunidad {0}, pero no hemos tenido noticias suyas en varios días. Según la información que ha podido recabar Ciudadanos por la Prosperidad, se encontraban explorando cerca de {1}, un conocido punto conflictivo de delincuentes.\n\nNecesitamos que alguien vaya allí por nosotros e intente localizarlos, o en el peor de los casos, sus restos.\n\nSi logras encontrarlos, hay una recompensa.\n\nLima Endicott\nOficial de Despacho\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>Unfortunately, one of our community partners, {0} has been missing for a few days. Their family contacted Citizens for Prosperity for help and I told them we would do what we could. That said, with so much time passed, I’m not too hopeful.\n\nWhatever their current state is, we're looking for someone to be our eyes on the ground for this one. There’s a strong chance that they were headed to {1} an area known to be very dangerous.\n\nIf you can track them down and confirm their status, one way or another, I’ll see that you’re properly compensated.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100 / 200 / 400</v>
+        <v>Lamentablemente, uno de nuestros socios comunitarios, {0}, lleva desaparecido varios días. Su familia contactó con Citizens for Prosperity para pedir ayuda y les dije que haríamos lo posible. Dicho esto, con tanto tiempo transcurrido, no tengo muchas esperanzas.\n\nSea cual sea su situación actual, buscamos a alguien que nos ayude a localizarlo. Hay muchas probabilidades de que se dirigiera a {1}, una zona conocida por ser muy peligrosa.\n\nSi logra localizarlo y confirmar su paradero, de una forma u otra, me aseguraré de que reciba la compensación adecuada.\n\nLima Endicott\nOperadora principal\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100 / 200 / 400</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>{0} is a local who only has done a few jobs for Citizen for Prosperity, but they had promise. That is, until they went missing while exploring {1} last week. Unfortunately, we didn’t hear about it until today. Chances of survival at this point are pretty slim, but we still think its worth confirming what happened to them.\n \nCFP could use help on this if anyone is interested. And besides being a good deed, the payment should make it worth the effort. \n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50 / 100</v>
+        <v>{0} es un residente local que solo ha realizado algunos trabajos para Citizen for Prosperity, pero tenía potencial. Eso fue hasta que desapareció mientras exploraba {1} la semana pasada. Desafortunadamente, no nos enteramos hasta hoy. Las probabilidades de supervivencia en este punto son bastante escasas, pero aún creemos que vale la pena confirmar qué le sucedió.\n \nCFP podría necesitar ayuda con esto si alguien está interesado. Y además de ser una buena acción, el pago debería compensar el esfuerzo. \n\nLima Endicott\nDespachadora principal\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50 / 100</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>One of our people, {0} was supposed to be doing some preliminary scouting work over at {1} but they never reported in. We’re hoping that they just ran into some bad luck, but too often out here even the smallest misstep can prove fatal.\n\nI’d appreciate someone heading that way and seeing if they can be located. It’d be great if you find them alive, but if not, some closure is the least we can do for their family.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50 / 100 / 150</v>
+        <v>Uno de los nuestros, {0}, debía realizar un trabajo de reconocimiento preliminar en {1}, pero nunca se presentó. Esperamos que simplemente haya tenido mala suerte, pero aquí, incluso el más mínimo error puede resultar fatal.\n\nAgradecería que alguien se dirigiera hacia allí e intentara localizarlo. Sería estupendo encontrarlo con vida, pero si no, brindarles un cierre es lo mínimo que podemos hacer por su familia.\n\nLima Endicott\nOficial de Despacho Principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50 / 100 / 150</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>Two locals we work with were out salvaging at {0} when they had some issues with faulty equipment. One managed to escape, but their partner, {1} was unfortunately left behind.\n\nWith the state they were last reported to be in, I’m guessing they didn’t make it, but I’d like to know for sure. If you’re willing, I could use your help in finding their remains.\n\nIf you can track them down, I’ll see that you’re properly compensated for the effort.\n\nLima Endicott\nLead Dispatcher\nCitizens for Prosperity\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100</v>
+        <v>Dos personas de la zona con las que trabajamos estaban realizando labores de salvamento en {0} cuando tuvieron problemas con un equipo defectuoso. Uno logró escapar, pero su compañero, {1}, lamentablemente se quedó atrás.\n\nPor el estado en que se les reportó la última vez, supongo que no sobrevivieron, pero me gustaría estar seguro. Si está dispuesto, agradecería su ayuda para encontrar sus restos.\n\nSi logra localizarlos, me aseguraré de que reciba la compensación adecuada por su esfuerzo.\n\nLima Endicott\nOperadora principal\nCiudadanos por la Prosperidad\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>Been getting word that CFP security have been getting a little more aggressive and started pushing people out of the homes they've built out of the scrap in the system and they want payback, so they came to us.\n\nHead out to {0} and clear out the CFP there. Should be pretty cut and dry with a nice payday.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 75 / 300\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Atzkav Sniper Rifle\n- Atzkav "Igniter" Sniper Rifle\n- Atzkav "Mirage" Sniper Rifle\n- Calico Arms Tactical\n- Calico Core Tactical\n- Calico Legs Tactical\n- Calico Helmet Tactical\n- Atzkav Sniper Rifle Battery (8 cap)\n</v>
+        <v>Hemos recibido información de que la seguridad de CFP se ha vuelto un poco más agresiva y ha comenzado a expulsar a la gente de las casas que han construido con la chatarra del sistema y quieren venganza, así que vinieron a nosotros.\n\nDirígete a {0} y elimina a los de CFP de allí. Debería ser bastante sencillo y con una buena paga.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 75 / 300\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle de francotirador Atzkav\n- Rifle de francotirador Atzkav "Igniter"\n- Rifle de francotirador Atzkav "Mirage"\n- Armas tácticas Calico\n- Núcleo táctico Calico\n- Piernas tácticas Calico\n- Casco táctico Calico\n- Batería de rifle de francotirador Atzkav (8 de capacidad)\n</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>These XenoThreat assholes are like aloprats. Every time you thing you wipe them out, they just pop back up again. They seem to be back to their usual shit and trying to put together something big. No idea what, but we've been cleared to stop it before it starts.\n\nA group of XenoThreat biggies are supposedly meeting at {0} to plan or just rage or whatever it is they do, but we're gonna bust it up. Or you are.\n\nHead over there and wipe out everyone you find. Sure enough I'm sure the biggies will jump into the fight. That's what they always do.\n\nThis'll be a tough one. As much as I hate XenoThreat, they're damn good in a fight, so watch yourself and bring help if you can.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 400\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Cluster NBD-102, Starlight Service Station, RAB-ROTH&lt;/EM4&gt;\n- Atzkav Sniper Rifle\n- Atzkav "Igniter" Sniper Rifle\n- Atzkav "Mirage" Sniper Rifle\n- Calico Arms Tactical\n- Calico Core Tactical\n- Calico Legs Tactical\n- Calico Helmet Tactical\n- Atzkav Sniper Rifle Battery (8 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-OVER, Ruin Clinic, Cluster YKA-011&lt;/EM4&gt;\n- Yubarev Pistol\n- Yubarev "Mirage" Pistol\n- Yubarev "Igniter" Pistol\n- DustUp Arms Tactical\n- DustUp Core Tactical\n- DustUp Legs Tactical\n- DustUp Helmet Tactical\n- Yubarev Pistol Battery (10 cap)\n</v>
+        <v>Estos cabrones de XenoThreat son como aloprats. Cada vez que crees que los has eliminado, vuelven a aparecer. Parece que han vuelto a sus andadas y están intentando organizar algo grande. No tengo ni idea de qué, pero nos han dado permiso para detenerlo antes de que empiece.\n\nSe supone que un grupo de los grandes de XenoThreat se reúne en {0} para planear o simplemente desahogarse o lo que sea que hagan, pero vamos a acabar con ellos. O lo harás tú.\n\nVe allí y elimina a todos los que encuentres. Seguro que los grandes se meterán en la pelea. Eso es lo que siempre hacen.\n\nEsto va a ser duro. Por mucho que odie a XenoThreat, son muy buenos en combate, así que ten cuidado y trae ayuda si puedes.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 400\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Cluster NBD-102, Estación de servicio Starlight, RAB-ROTH&lt;/EM4&gt;\n- Rifle de francotirador Atzkav\n- Rifle de francotirador Atzkav "Igniter"\n- Rifle de francotirador Atzkav "Mirage"\n- Armas tácticas Calico\n- Núcleo táctico Calico\n- Piernas tácticas Calico\n- Casco táctico Calico\n- Batería de rifle de francotirador Atzkav (8 de capacidad)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-OVER, Clínica Ruin, Cluster YKA-011&lt;/EM4&gt;\n- Yubarev Pistola\n- Pistola Yubarev "Mirage"\n- Pistola Yubarev "Igniter"\n- Armas tácticas DustUp\n- Armazón táctico DustUp\n- Piernas tácticas DustUp\n- Casco táctico DustUp\n- Batería para pistola Yubarev (10 cápsulas)\n</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>Got word of crew that's been pulling jobs and building a rep for themselves. Since they've said they don't want anything to do with Headhunters, we're looking to break 'em apart before they become a problem. Their leader is some punk named {0} and we figure if they met the wrong end of a bullet, the rest of them would break apart.\n\nWe're told you can find {1} around {2} Head over and take care of it.\n\nThey shouldn't pose much of a problem to a pro like you.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 50\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: RAB-MAT, Starlight Service Station, RAB-YORK&lt;/EM4&gt;\n- Scalpel Sniper Rifle\n- Coda Pistol\n- Coda "Nighthawk" Pistol\n- Coda "Big Boss" Pistol\n- Morozov-SH Arms\n- Morozov-SH Core\n- Morozov-SH Legs\n- Morozov-SH Helmet\n- Scalpel Sniper Rifle Magazine (12 cap)\n- Coda Pistol Magazine (6 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-ZETA, Gaslight, RAB-ROTH&lt;/EM4&gt;\n- Devastator Shotgun\n- Devastator "Warhawk" Shotgun\n- Devastator "Midnight" Shotgun\n- Morozov-SH Core Thule\n- Morozov-SH Arms Thule\n- Morozov-SH Legs Thule\n- Morozov-SH Helmet Thule\n- Devastator Shotgun Battery (12 cap)\n</v>
+        <v>Nos enteramos de que hay un grupo de personas que se dedican a conseguir trabajos y a labrarse una mala reputación. Como han dicho que no quieren tener nada que ver con los cazatalentos, estamos intentando separarlos antes de que se conviertan en un problema. Su líder es un punk llamado {0} y suponemos que si les llega un disparo, el resto se desintegraría.\n\nNos han dicho que puedes encontrar a {1} cerca de {2}. Ve y encárgate de ello.\n\nNo deberían suponer un gran problema para un profesional como tú.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 50\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-MAT, Estación de servicio Starlight, RAB-YORK&lt;/EM4&gt;\n- Rifle de francotirador Scalpel\n- Pistola Coda\n- Pistola Coda "Nighthawk"\n- Pistola Coda "Big Boss"\n- Brazos Morozov-SH\n- Núcleo Morozov-SH\n- Piernas Morozov-SH\n- Casco Morozov-SH\n- Cargador de rifle de francotirador Scalpel (12 cap)\n- Revista Coda Pistol (6 cap)\n\n&lt;EM4&gt;[Variantes regionales] ubicaciones de ejemplo: RAB-ZETA, Gaslight, RAB-ROTH&lt;/EM4&gt;\n- Escopeta Devastator\n- Escopeta Devastator "Warhawk"\n- Escopeta Devastator "Midnight"\n- Morozov-SH Core Thule\n- Morozov-SH Arms Thule\n- Morozov-SH Piernas Thule\n- Casco Morozov-SH Thule\n- Batería de escopeta Devastator (12 cap)\n</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>Need an available trigger to take down a target in a CFP outpost. They're a real piece of work named {0} Old school merc filled with lead-pipe cruelty. \n\nHeard they're posted over at {1} Swing by and take them out. Try not to cause too much damage. They're the target, not anyone else.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 75 / 100\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Cluster NBD-102, RAB-FOXTROT, Orbituary&lt;/EM4&gt;\n- Scalpel Sniper Rifle\n- Coda Pistol\n- Coda "Nighthawk" Pistol\n- Coda "Big Boss" Pistol\n- Morozov-SH Arms\n- Morozov-SH Core\n- Morozov-SH Legs\n- Morozov-SH Helmet\n- Scalpel Sniper Rifle Magazine (12 cap)\n- Coda Pistol Magazine (6 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Pyro V, Pyro IV, RAB-FOXTROT&lt;/EM4&gt;\n- Devastator Shotgun\n- Devastator "Warhawk" Shotgun\n- Devastator "Midnight" Shotgun\n- Morozov-SH Core Thule\n- Morozov-SH Arms Thule\n- Morozov-SH Legs Thule\n- Morozov-SH Helmet Thule\n- Devastator Shotgun Battery (12 cap)\n</v>
+        <v>Necesitas un detonante disponible para eliminar a un objetivo en un puesto avanzado de CFP. Son un verdadero desastre llamado {0} Mercenario de la vieja escuela lleno de crueldad extrema. \n\nEscuché que están en {1} Pásate y elimínalos. Intenta no causarles demasiado daño. Son el objetivo, no nadie más.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 75 / 100\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Cluster NBD-102, RAB-FOXTROT, Orbituary&lt;/EM4&gt;\n- Rifle de francotirador Scalpel\n- Pistola Coda\n- Pistola Coda "Nighthawk"\n- Pistola Coda "Big Boss"\n- Brazos Morozov-SH\n- Núcleo Morozov-SH\n- Piernas Morozov-SH\n- Casco Morozov-SH\n- Cargador de rifle de francotirador Scalpel (12 cap)\n- Cargador de pistola Coda (6 cap)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Pyro V, Pyro IV, RAB-FOXTROT&lt;/EM4&gt;\n- Escopeta Devastator\n- Escopeta Devastator "Warhawk"\n- Escopeta Devastator "Midnight"\n- Morozov-SH Core Thule\n- Morozov-SH Arms Thule\n- Morozov-SH Legs Thule\n- Morozov-SH Casco Thule\n- Escopeta Devastator Batería (12 cápsulas)\n</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>Got a crew that's been hitting Headhunter ships lately. Their leader's a real piece of work named {0} We've tracked them to  {1} so we're looking for someone to put them down for good.\n\nThis group likes to fight, but shouldn't be a problem for someone like you. \n\nGet over there and get it done.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Scalpel Sniper Rifle\n- Coda Pistol\n- Coda "Nighthawk" Pistol\n- Coda "Big Boss" Pistol\n- Morozov-SH Arms\n- Morozov-SH Core\n- Morozov-SH Legs\n- Morozov-SH Helmet\n- Scalpel Sniper Rifle Magazine (12 cap)\n- Coda Pistol Magazine (6 cap)\n</v>
+        <v>Tenemos una tripulación que últimamente ha estado atacando naves de Headhunters. Su líder es un verdadero personaje llamado {0}. Los hemos rastreado hasta {1}, así que estamos buscando a alguien que los elimine de una vez por todas.\n\nA este grupo le gusta pelear, pero no debería ser un problema para alguien como tú. \n\nVe allí y hazlo.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle de francotirador Scalpel\n- Pistola Coda\n- Pistola Coda "Nighthawk"\n- Pistola Coda "Big Boss"\n- Brazos Morozov-SH\n- Núcleo Morozov-SH\n- Piernas Morozov-SH\n- Casco Morozov-SH\n- Cargador de rifle de francotirador Scalpel (12 cap)\n- Cargador de pistola Coda (6 cap)</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>Headhunters just rallied up a crew to go hit {0} and wipe out the XenoThreat there, but I'm looking to add some extra insurance. \n\nSee there's this heavy hitter there named {1} who's up in the XenoThreat command structure and we want them taken out. Every other one you kill is gravy, but they're your prime target.\n\n-Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 75\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Scalpel Sniper Rifle\n- Coda Pistol\n- Coda "Nighthawk" Pistol\n- Coda "Big Boss" Pistol\n- Morozov-SH Arms\n- Morozov-SH Core\n- Morozov-SH Legs\n- Morozov-SH Helmet\n- Scalpel Sniper Rifle Magazine (12 cap)\n- Coda Pistol Magazine (6 cap)\n</v>
+        <v>Los Headhunters acaban de reunir un equipo para atacar {0} y eliminar a la XenoThreat de allí, pero quiero añadir un seguro adicional. \n\nMira, hay un pez gordo allí llamado {1} que está en la estructura de mando de la XenoThreat y queremos eliminarlo. Todos los demás que mates son un extra, pero son tu objetivo principal.\n\n-Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 75\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Rifle de francotirador Scalpel\n- Pistola Coda\n- Pistola Coda "Nighthawk"\n- Pistola Coda "Big Boss"\n- Brazos Morozov-SH\n- Núcleo Morozov-SH\n- Piernas Morozov-SH\n- Casco Morozov-SH\n- Cargador de rifle de francotirador Scalpel (12 cap)\n- Cargador de pistola Coda (6 cap)\n</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>It seems like I can't go a day without waking up to one of my people bitchin' and moanin' about how hard Citizens for Prosperity is making their life. \n\nEventually we're going wipe those do-gooders out of the system, but for now I'll settle for some peace and quiet. \n\nGo to {0} and destroy the fuel stores CFP have got there. That should at least keep them out of our business for a bit.\n\n-Stows out\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100 / 200</v>
+        <v>Parece que no puedo pasar un día sin despertarme con alguno de los míos quejándose de lo difícil que Ciudadanos por la Prosperidad les está haciendo la vida. \n\nAl final, eliminaremos a esos bienhechores del sistema, pero por ahora me conformaré con un poco de paz y tranquilidad. \n\nVe a {0} y destruye las reservas de combustible que CFP tiene allí. Eso al menos debería mantenerlos fuera de nuestros asuntos por un tiempo.\n\n-Stows fuera\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100 / 200</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>It seems that XenoThreat has gotten the same intel we did and are looking to pull off the same job as us. \n\nI want you to knock the competition out of the picture. Go to {0} and take out the fuel tanks they got there.\n\nThen my people can finish up without worrying about XenoThreat crashing the party.\n\n-Stows out\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100</v>
+        <v> Parece que XenoThreat ha obtenido la misma información que nosotros y pretende llevar a cabo el mismo plan. \n\nQuiero que elimines a la competencia. Ve a {0} y destruye los tanques de combustible que tienen allí.\n\nAsí mi gente podrá terminar sin preocuparse de que XenoThreat arruine la fiesta.\n\n-Stows out\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>I'm getting pretty bloody sick of Citizens for Prosperity sticking their noses where they don't belong. \n\nStarted thinking that it might be pretty nice to ground their fleet for a little bit. We blow up their fuel tanks at {0} and those little pissheads won't be going nowhere quick.\n\nSound like your kinda thing?\n\n-Stows out\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100 / 200</v>
+        <v>Estoy harto de que Ciudadanos por la Prosperidad se meta en asuntos que no le incumben. \n\nEmpecé a pensar que sería buena idea dejar su flota en tierra un tiempo. Les volamos los tanques de combustible a {0} y esos mocosos no se irán a ninguna parte rápidamente.\n\n¿Te parece bien?\n\n-Stows out\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100 / 200</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>Those XenoThreat punks launched an attack against {0} so we're looking for people to go fend them off. \n\nGet out there and waste every XenoThreat you see.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Yubarev Pistol\n- Yubarev "Mirage" Pistol\n- Yubarev "Igniter" Pistol\n- DustUp Arms Tactical\n- DustUp Core Tactical\n- DustUp Legs Tactical\n- DustUp Helmet Tactical\n- Yubarev Pistol Battery (10 cap)\n</v>
+        <v> Esos punks de XenoThreat lanzaron un ataque contra {0}, así que estamos buscando gente para que los detenga. \n\nSalgan y acaben con cada XenoThreat que vean.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Pistola Yubarev\n- Pistola Yubarev "Mirage"\n- Pistola Yubarev "Igniter"\n- Armas tácticas DustUp\n- Núcleo táctico DustUp\n- Piernas tácticas DustUp\n- Casco táctico DustUp\n- Batería de pistola Yubarev (10 cápsulas)\n</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>One of our Judges caught wind of XenoThreat trying to move in on our territory. Seems like they’re trying to take over {0} We don’t want to let those psychos get any more of a foothold in system than they already have, so we’re putting some creds on the line to get ‘em to back off.\n\nWe want you to come down on them hard. Don’t let up till the whole place is a graveyard. We’ll send your payment once the bodies are ready to bury.\n\n- Stows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Atzkav Sniper Rifle\n- Atzkav "Igniter" Sniper Rifle\n- Atzkav "Mirage" Sniper Rifle\n- Calico Arms Tactical\n- Calico Core Tactical\n- Calico Legs Tactical\n- Calico Helmet Tactical\n- Atzkav Sniper Rifle Battery (8 cap)\n</v>
+        <v>Uno de nuestros jueces se enteró de que XenoThreat está intentando invadir nuestro territorio. Parece que están intentando tomar el control de {0}. No queremos dejar que esos psicópatas se afiancen más en el sistema de lo que ya lo han hecho, así que estamos poniendo algunos créditos en juego para que se retiren.\n\nQueremos que actúes con dureza contra ellos. No ceses hasta que todo el lugar sea un cementerio. Enviaremos su pago una vez que los cuerpos estén listos para ser enterrados.\n\n- Se esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Fusil de francotirador Atzkav\n- Fusil de francotirador Atzkav "Igniter"\n- Fusil de francotirador Atzkav "Mirage"\n- Armas tácticas Calico\n- Núcleo táctico Calico\n- Piernas tácticas Calico\n- Casco táctico Calico\n- Batería de fusil de francotirador Atzkav (8 unidades)\n</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>So here's the deal, we got some small time dirtbags who think they're hotshots running out of a base near {0} I don't know what toxic shit they're drinking but they thought it'd be a good idea to step to some Headhunter Clips. Killed one, injured three more. So I'm looking to send someone there to blast their ambition right out of their skulls.\n\nHead over and get it done. You'll get a nice bump of creds for it.\n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 50\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Monox, RAB-YORK, Checkmate&lt;/EM4&gt;\n- Atzkav Sniper Rifle\n- Atzkav "Igniter" Sniper Rifle\n- Atzkav "Mirage" Sniper Rifle\n- Calico Arms Tactical\n- Calico Core Tactical\n- Calico Legs Tactical\n- Calico Helmet Tactical\n- Atzkav Sniper Rifle Battery (8 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Cluster YKA-011, RAB-ECHO, Cluster MNK-833&lt;/EM4&gt;\n- Yubarev Pistol\n- Yubarev "Mirage" Pistol\n- Yubarev "Igniter" Pistol\n- DustUp Arms Tactical\n- DustUp Core Tactical\n- DustUp Legs Tactical\n- DustUp Helmet Tactical\n- Yubarev Pistol Battery (10 cap)\n</v>
+        <v>Así que aquí está el trato, tenemos a unos mocosos de poca monta que se creen muy listos huyendo de una base cerca de {0}. No sé qué mierda tóxica están bebiendo, pero pensaron que sería una buena idea enfrentarse a unos Headhunter Clips. Maté a uno, herí a tres más. Así que estoy buscando enviar a alguien allí para volarles la ambición de raíz.\n\nVe y hazlo. Obtendrás un buen aumento de créditos por ello.\n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 50\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Monox, RAB-YORK, Checkmate&lt;/EM4&gt;\n- Fusil de francotirador Atzkav\n- Fusil de francotirador Atzkav "Igniter"\n- Fusil de francotirador Atzkav "Mirage"\n- Armas tácticas Calico\n- Núcleo táctico Calico\n- Piernas tácticas Calico\n- Casco táctico Calico\n- Batería de fusil de francotirador Atzkav (8 cap)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Cluster YKA-011, RAB-ECHO, Cluster MNK-833&lt;/EM4&gt;\n- Pistola Yubarev\n- Pistola Yubarev "Mirage"\n- Yubarev Pistola "Igniter" - Armas tácticas DustUp - Núcleo táctico DustUp - Piernas tácticas DustUp - Casco táctico DustUp - Batería para pistola Yubarev (10 cápsulas)</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>Here's the deal. Some of those mercs that CFP hired as security went and shot up some Headhunters that were just moving through the system. They weren't even doing anything, just flying.\n\nAnyway, we tracked them back to {0} and want to dish out some payback. Grab your gear and be our weapon, we'll make it worth your while.\n\n- Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Yubarev Pistol\n- Yubarev "Mirage" Pistol\n- Yubarev "Igniter" Pistol\n- DustUp Arms Tactical\n- DustUp Core Tactical\n- DustUp Legs Tactical\n- DustUp Helmet Tactical\n- Yubarev Pistol Battery (10 cap)\n</v>
+        <v>Aquí está el trato. Algunos de esos mercenarios que CFP contrató como seguridad fueron y dispararon a unos Headhunters que simplemente estaban pasando por el sistema. Ni siquiera estaban haciendo nada, solo volando.\n\nDe todos modos, los rastreamos hasta {0} y queremos vengarnos. Toma tu equipo y sé nuestra arma, te lo haremos merecer.\n\n- Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Pistola Yubarev\n- Pistola Yubarev "Mirage"\n- Pistola Yubarev "Igniter"\n- Armas tácticas DustUp\n- Núcleo táctico DustUp\n- Piernas tácticas DustUp\n- Casco táctico DustUp\n- Batería de pistola Yubarev (10 cápsulas)\n</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>Some assholes are refusing to pay us what we’re owed. Problem is, these idiots are bragging about it. Had they kept it quiet, we could’ve taken care of this more surgically, but now we need to send a message.\n\nThe fools are operating from {0} We need them all gone. Make it as loud as you can. We’ll send your payment once everyone’s taken care of.\n\n- Stows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50 / 300\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Yubarev Pistol\n- Yubarev "Mirage" Pistol\n- Yubarev "Igniter" Pistol\n- DustUp Arms Tactical\n- DustUp Core Tactical\n- DustUp Legs Tactical\n- DustUp Helmet Tactical\n- Yubarev Pistol Battery (10 cap)\n</v>
+        <v>Algunos imbéciles se niegan a pagarnos lo que nos deben. El problema es que estos idiotas se jactan de ello. Si se hubieran callado, podríamos haber resuelto esto de forma más precisa, pero ahora necesitamos enviar un mensaje.\n\nLos tontos están operando desde {0}. Necesitamos que se vayan todos. Háganlo lo más fuerte posible. Enviaremos su pago una vez que todos se hayan encargado.\n\n- Se esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50 / 300\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Pistola Yubarev\n- Pistola Yubarev "Mirage"\n- Pistola Yubarev "Igniter"\n- Armas tácticas DustUp\n- Núcleo táctico DustUp\n- Piernas tácticas DustUp\n- Casco táctico DustUp\n- Batería para pistola Yubarev (10 cápsulas)\n</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>It's sad to say but we lost one of our outposts to XenoThreat. Appalling if you ask me, but that's why we're looking for someone who's got the time and ammunition to take it back.\n\nIf that's you, head over to {0} and take it back.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100\n\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n- Yubarev Pistol\n- Yubarev "Mirage" Pistol\n- Yubarev "Igniter" Pistol\n- DustUp Arms Tactical\n- DustUp Core Tactical\n- DustUp Legs Tactical\n- DustUp Helmet Tactical\n- Yubarev Pistol Battery (10 cap)\n</v>
+        <v>Es triste decirlo, pero perdimos uno de nuestros puestos avanzados a manos de XenoThreat. Espantoso, si me preguntan, pero por eso estamos buscando a alguien que tenga el tiempo y la munición para recuperarlo.\n\nSi eres tú, dirígete a {0} y recupéralo.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100\n\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n- Pistola Yubarev\n- Pistola Yubarev "Mirage"\n- Pistola Yubarev "Igniter"\n- Armas tácticas DustUp\n- Núcleo táctico DustUp\n- Piernas tácticas DustUp\n- Casco táctico DustUp\n- Batería para pistola Yubarev (10 cápsulas)\n</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>So here's the deal, Headhunters are looking to expand their talent pool and have a few openings for anyone who's got the stones.\n\nThere's a real piece of work named {0} who thinks they've been really clever pinching cargo off of haulers moving through the system. We asked for a cut of their profits as a licensing tax to continue operating. When {1} responded, they were very disrespectful.\n\nWe've tracked their ship to {2} and need them taken out. You should know, they're being smart and sticking close to some allies so they won't be alone.\n\nDo this and we'll consider you for future Headhunter work.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 50\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Patch City, RAB-IGNITION, Checkmate Clinic&lt;/EM4&gt;\n- 9-Series Longsword Cannon\n- 10-Series Greatsword Cannon\n- 11-Series Broadsword Cannon\n- Sledge I Mass Driver Cannon\n- Strife Mass Driver Cannon\n- Sledge II Mass Driver Cannon\n- Sledge III Mass Driver Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Starlight Clinic, RAB-GULF, Cluster JWY-925&lt;/EM4&gt;\n- HeatSafe (Cooler)\n- HeatSink (Cooler)\n- Dominance-1 Scattergun\n- Dominance-2 Scattergun\n- Dominance-3 Scattergun\n\n&lt;EM4&gt;[Regional Variants] example locations: Vatra, Cluster GRP-839, RAB-ROTH&lt;/EM4&gt;\n- VaporBlock (Cooler)\n- IceBox (Cooler)\n- NN-13 Cannon\n- NN-14 Cannon\n- NN-15 Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-MAT, Ruin Station, Cluster HJS-232&lt;/EM4&gt;\n- SnowBlind (Cooler)\n- NightFall (Cooler)\n- M6A Cannon\n- M7A Cannon\n- M8A Cannon\n- Singe Cannon (S1)\n- Singe Cannon (S2)\n- Singe Cannon (S3)\n</v>
+        <v>Así que aquí está el trato, Headhunters está buscando ampliar su grupo de talentos y tiene algunas vacantes para cualquiera que tenga agallas.\n\nHay un verdadero sinvergüenza llamado {0} que se cree muy listo robando carga de los transportistas que se mueven por el sistema. Pedimos una parte de sus ganancias como impuesto de licencia para continuar operando. Cuando {1} respondió, fue muy irrespetuoso.\n\nHemos rastreado su nave hasta {2} y necesitamos eliminarlo. Debes saber que están siendo inteligentes y manteniéndose cerca de algunos aliados para no estar solos.\n\nHaz esto y te consideraremos para futuros trabajos de Headhunter.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 50\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Patch City, RAB-IGNITION, Checkmate Clinic&lt;/EM4&gt;\n- Cañón de espada larga serie 9\n- Cañón de espada grande serie 10\n- Cañón de espada ancha serie 11\n- Cañón de impulsor de masa Sledge I\n- Cañón de impulsor de masa Strife\n- Cañón de impulsor de masa Sledge II\n- Cañón de impulsor de masa Sledge III\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Starlight Clinic, RAB-GULF, Cluster JWY-925&lt;/EM4&gt;\n- HeatSafe (enfriador)\n- HeatSink (enfriador)\n- Escopeta Dominance-1\n- Escopeta Dominance-2\n- Escopeta Dominance-3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Vatra, Cluster GRP-839, RAB-ROTH&lt;/EM4&gt;\n- VaporBlock (enfriador)\n- IceBox (enfriador)\n- Cañón NN-13\n- Cañón NN-14\n- Cañón NN-15\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-MAT, Ruin Station, Cluster HJS-232&lt;/EM4&gt;\n- SnowBlind (enfriador)\n- NightFall (enfriador)\n- Cañón M6A\n- Cañón M7A\n- Cañón M8A\n- Cañón individual (S1)\n- Cañón individual (S2)\n- Cañón único (S3)\n</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>There's a nest that needs to be taken out around {0} that has been taken over by some squatters. We don't care about most of them, but word's gotten back to us that they're sheltering {1} who has a long history of stealing Headhunter loot. Time's come to take them out.\n\nWord is that {2} is in a ship, but may rely on the base's defenses to protect them, so be careful. You kill 'em, you get paid. \n\nYou know, the usual.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 50\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: RAB-KILO, Patch City, RAB-FOXTROT&lt;/EM4&gt;\n- 9-Series Longsword Cannon\n- 10-Series Greatsword Cannon\n- 11-Series Broadsword Cannon\n- Sledge I Mass Driver Cannon\n- Strife Mass Driver Cannon\n- Sledge II Mass Driver Cannon\n- Sledge III Mass Driver Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-YORK, Cluster CAJ-445, Rat's Nest Clinic&lt;/EM4&gt;\n- HeatSafe (Cooler)\n- HeatSink (Cooler)\n- Dominance-1 Scattergun\n- Dominance-2 Scattergun\n- Dominance-3 Scattergun\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-QUAGMIRE, RAB-ZETA, RAB-POINT&lt;/EM4&gt;\n- VaporBlock (Cooler)\n- IceBox (Cooler)\n- NN-13 Cannon\n- NN-14 Cannon\n- NN-15 Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Cluster DLO-486, Ruin Clinic, RAB-ION&lt;/EM4&gt;\n- SnowBlind (Cooler)\n- NightFall (Cooler)\n- M6A Cannon\n- M7A Cannon\n- M8A Cannon\n- Singe Cannon (S1)\n- Singe Cannon (S2)\n- Singe Cannon (S3)\n</v>
+        <v>Hay un nido que hay que eliminar cerca de {0} que ha sido ocupado por unos intrusos. No nos importan la mayoría, pero nos ha llegado información de que están dando refugio a {1}, que tiene un largo historial de robar el botín de los Cazadores de Cabezas. Ha llegado el momento de eliminarlos.\n\nSe rumorea que {2} está en una nave, pero puede que confíe en las defensas de la base para protegerse, así que ten cuidado. Si los matas, te pagan. \n\nYa sabes, lo de siempre.\n\nSe oculta.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 50\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-KILO, Patch City, RAB-FOXTROT&lt;/EM4&gt;\n- Cañón de espada larga serie 9\n- Cañón de espada grande serie 10\n- Cañón de espada ancha serie 11\n- Cañón de impulsor de masa Sledge I\n- Cañón de impulsor de masa Strife\n- Cañón de impulsor de masa Sledge II\n- Cañón de impulsor de masa Sledge III\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-YORK, Cluster CAJ-445, Clínica Rat's Nest&lt;/EM4&gt;\n- HeatSafe (enfriador)\n- HeatSink (enfriador)\n- Dominance-1 Escopeta\n- Escopeta Dominance-2\n- Escopeta Dominance-3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-QUAGMIRE, RAB-ZETA, RAB-POINT&lt;/EM4&gt;\n- VaporBlock (refrigerador)\n- IceBox (refrigerador)\n- Cañón NN-13\n- Cañón NN-14\n- Cañón NN-15\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Cluster DLO-486, Ruin Clinic, RAB-ION&lt;/EM4&gt;\n- SnowBlind (refrigerador)\n- NightFall (refrigerador)\n- Cañón M6A\n- Cañón M7A\n- Cañón M8A\n- Cañón individual (S1)\n- Cañón individual (S2)\n- Cañón individual (S3)\n</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>Need another CFP ship taken out. It belongs to {0} who's been  driving locals out of their homes if they don't accept Citizens for Prosperity help. They're a real piece of work and we've been given the go-ahead to take them down.\n\nTheir ship was spotted around {1} so head out there and do the deed.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 600\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Monox, Pyro I, RAB-TUNG&lt;/EM4&gt;\n- 9-Series Longsword Cannon\n- 10-Series Greatsword Cannon\n- 11-Series Broadsword Cannon\n- Sledge I Mass Driver Cannon\n- Strife Mass Driver Cannon\n- Sledge II Mass Driver Cannon\n- Sledge III Mass Driver Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Orbituary Clinic, RAB-CHARLIE, Cluster CAJ-445&lt;/EM4&gt;\n- HeatSafe (Cooler)\n- HeatSink (Cooler)\n- Dominance-1 Scattergun\n- Dominance-2 Scattergun\n- Dominance-3 Scattergun\n\n&lt;EM4&gt;[Regional Variants] example locations: Cluster GRP-839, RAB-DELTA, RAB-POINT&lt;/EM4&gt;\n- VaporBlock (Cooler)\n- IceBox (Cooler)\n- NN-13 Cannon\n- NN-14 Cannon\n- NN-15 Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Cluster DLO-486, RAB-ULTRA, RAB-LYNX&lt;/EM4&gt;\n- SnowBlind (Cooler)\n- NightFall (Cooler)\n- M6A Cannon\n- M7A Cannon\n- M8A Cannon\n- Singe Cannon (S1)\n- Singe Cannon (S2)\n- Singe Cannon (S3)\n</v>
+        <v>Hay que sacar otro barco de Ciudadanos por la Prosperidad. Pertenece a {0}, que ha estado expulsando a los lugareños de sus casas si no aceptan la ayuda de Ciudadanos por la Prosperidad. Son un verdadero problema y nos han dado luz verde para acabar con ellos.\n\nSu nave fue avistada alrededor de {1}, así que diríjanse allí y hagan el trabajo.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 600\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Monox, Pyro I, RAB-TUNG&lt;/EM4&gt;\n- Cañón de espada larga serie 9\n- Cañón de espada grande serie 10\n- Cañón de espada ancha serie 11\n- Cañón de impulsor de masa Sledge I\n- Cañón de impulsor de masa Strife\n- Cañón de impulsor de masa Sledge II\n- Cañón de impulsor de masa Sledge III\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Clínica Orbital, RAB-CHARLIE, Cluster CAJ-445&lt;/EM4&gt;\n- HeatSafe (enfriador)\n- HeatSink (enfriador)\n- Escopeta Dominance-1\n- Escopeta Dominance-2\n- Escopeta Dominance-3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Cluster GRP-839, RAB-DELTA, RAB-POINT&lt;/EM4&gt;\n- VaporBlock (enfriador)\n- IceBox (enfriador)\n- Cañón NN-13\n- Cañón NN-14\n- Cañón NN-15\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Cluster DLO-486, RAB-ULTRA, RAB-LYNX&lt;/EM4&gt;\n- SnowBlind (enfriador)\n- NightFall (enfriador)\n- Cañón M6A\n- Cañón M7A\n- M8A Cañón\n- Cañón único (T1)\n- Cañón único (T2)\n- Cañón único (T3)\n</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>CFP Security forces have been attacking locals and we're looking to balance the scales. Caught wind of one in particular named {0} who's been causing some damage and we need them taken out.\n\nYou can find them flying around {1} Go introduce yourself.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 300\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Pyro I, RAB-NOVEMBER, RAB-KILO&lt;/EM4&gt;\n- 9-Series Longsword Cannon\n- 10-Series Greatsword Cannon\n- 11-Series Broadsword Cannon\n- Sledge I Mass Driver Cannon\n- Strife Mass Driver Cannon\n- Sledge II Mass Driver Cannon\n- Sledge III Mass Driver Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Cluster JWY-925, Rat's Nest Clinic, RAB-MAT&lt;/EM4&gt;\n- HeatSafe (Cooler)\n- HeatSink (Cooler)\n- Dominance-1 Scattergun\n- Dominance-2 Scattergun\n- Dominance-3 Scattergun\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-ECHO, RAB-DELTA, RAB-OVER&lt;/EM4&gt;\n- VaporBlock (Cooler)\n- IceBox (Cooler)\n- NN-13 Cannon\n- NN-14 Cannon\n- NN-15 Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-MAT, RAB-COOK, Cluster DLO-486&lt;/EM4&gt;\n- SnowBlind (Cooler)\n- NightFall (Cooler)\n- M6A Cannon\n- M7A Cannon\n- M8A Cannon\n- Singe Cannon (S1)\n- Singe Cannon (S2)\n- Singe Cannon (S3)\n</v>
+        <v>Las fuerzas de seguridad de CFP han estado atacando a los residentes locales y estamos buscando restablecer el equilibrio. Nos enteramos de uno en particular llamado {0} que ha estado causando algunos daños y necesitamos eliminarlo.\n\nPuedes encontrarlo volando alrededor de {1} Ve a presentarte.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 300\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Pyro I, RAB-NOVIEMBRE, RAB-KILO&lt;/EM4&gt;\n- Cañón de espada larga serie 9\n- Cañón de espada grande serie 10\n- Cañón de espada ancha serie 11\n- Cañón de impulsor de masa Sledge I\n- Cañón de impulsor de masa Strife\n- Cañón de impulsor de masa Sledge II\n- Cañón de impulsor de masa Sledge III\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Cluster JWY-925, Clínica Nido de Ratas, RAB-MAT&lt;/EM4&gt;\n- HeatSafe (Enfriador)\n- HeatSink (Enfriador)\n- Escopeta Dominance-1\n- Escopeta Dominance-2\n- Escopeta Dominance-3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-ECHO, RAB-DELTA, RAB-OVER&lt;/EM4&gt;\n- VaporBlock (Enfriador)\n- IceBox (Enfriador)\n- Cañón NN-13\n- Cañón NN-14\n- Cañón NN-15\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-MAT, RAB-COOK, Cluster DLO-486&lt;/EM4&gt;\n- SnowBlind (Enfriador)\n- NightFall (Enfriador)\n- Cañón M6A\n- Cañón M7A\n- Cañón M8A\n- Cañón individual (S1)\n- Cañón único (S2)\n- Cañón único (S3)\n</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>Got a platinum target that needs to get taken down. {0} is a heavy hitter who's one of the people running security for Citizens for Prosperity. Although {1} might have forgotten, the Headhunters remember their work with a merc company a few years ago that lead to the deaths of five brothers and sisters. We want blood for blood.\n\nThey've been spotted poking around {2} so you should still be able to find them there.\n\nThey're a mean bastard, so bring some friends but make sure they end up dead.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 1,200\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: RAB-KILO, Patch City, Pyro I&lt;/EM4&gt;\n- 9-Series Longsword Cannon\n- 10-Series Greatsword Cannon\n- 11-Series Broadsword Cannon\n- Sledge I Mass Driver Cannon\n- Strife Mass Driver Cannon\n- Sledge II Mass Driver Cannon\n- Sledge III Mass Driver Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Rat's Nest, Orbituary, RAB-CHARLIE&lt;/EM4&gt;\n- HeatSafe (Cooler)\n- HeatSink (Cooler)\n- Dominance-1 Scattergun\n- Dominance-2 Scattergun\n- Dominance-3 Scattergun\n\n&lt;EM4&gt;[Regional Variants] example locations: Vatra, RAB-DELTA, Adir&lt;/EM4&gt;\n- VaporBlock (Cooler)\n- IceBox (Cooler)\n- NN-13 Cannon\n- NN-14 Cannon\n- NN-15 Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Cluster LHB-976, Ruin Station, Cluster EMM-567&lt;/EM4&gt;\n- SnowBlind (Cooler)\n- NightFall (Cooler)\n- M6A Cannon\n- M7A Cannon\n- M8A Cannon\n- Singe Cannon (S1)\n- Singe Cannon (S2)\n- Singe Cannon (S3)\n</v>
+        <v>Tenemos un objetivo de platino que hay que eliminar. {0} es un pez gordo que trabaja en la seguridad de Ciudadanos por la Prosperidad. Aunque {1} lo haya olvidado, los Cazadores de Cabezas recuerdan su colaboración con una compañía de mercenarios hace unos años, que provocó la muerte de cinco hermanos. Queremos sangre por sangre.\n\nSe les ha visto merodeando por {2} así que aún deberías poder encontrarlos allí.\n\nSon unos bastardos malvados, así que trae algunos amigos, pero asegúrate de que terminen muertos.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 1200\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-KILO, Patch City, Pyro I&lt;/EM4&gt;\n- Cañón de espada larga serie 9\n- Cañón de espada grande serie 10\n- Cañón de espada ancha serie 11\n- Cañón de impulsor de masa Sledge I\n- Cañón de impulsor de masa Strife\n- Cañón de impulsor de masa Sledge II\n- Cañón de impulsor de masa Sledge III\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Nido de ratas, Orbituario, RAB-CHARLIE&lt;/EM4&gt;\n- HeatSafe (Enfriador)\n- HeatSink (Enfriador)\n- Escopeta Dominance-1\n- Escopeta Dominance-2\n- Escopeta Dominance-3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Vatra, RAB-DELTA, Adir&lt;/EM4&gt;\n- VaporBlock (Enfriador)\n- IceBox (Enfriador)\n- Cañón NN-13\n- Cañón NN-14\n- Cañón NN-15\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Cluster LHB-976, Ruin Station, Cluster EMM-567&lt;/EM4&gt;\n- SnowBlind (Enfriador)\n- NightFall (Enfriador)\n- Cañón M6A\n- Cañón M7A\n- Cañón M8A\n- Cañón individual (S1)\n- Cañón único (S2)\n- Cañón único (S3)\n</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>We got a greenlight to finally take out {0} They've been a pain in our ass ever since they came to the system a few years ago and it's finally time to take them out once and for all. \n\nWe've gotten word that {1} was spotted flying near {2} and the Judge wants this handled now.\n\nTake 'em out.\n\n- Stows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 600\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Cluster NBD-102, RAB-IGNITION, RAB-FOXTROT&lt;/EM4&gt;\n- 9-Series Longsword Cannon\n- 10-Series Greatsword Cannon\n- 11-Series Broadsword Cannon\n- Sledge I Mass Driver Cannon\n- Strife Mass Driver Cannon\n- Sledge II Mass Driver Cannon\n- Sledge III Mass Driver Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Starlight Service Station, RAB-GULF, Starlight Clinic&lt;/EM4&gt;\n- HeatSafe (Cooler)\n- HeatSink (Cooler)\n- Dominance-1 Scattergun\n- Dominance-2 Scattergun\n- Dominance-3 Scattergun\n\n&lt;EM4&gt;[Regional Variants] example locations: Vatra, Ignis, RAB-DELTA&lt;/EM4&gt;\n- VaporBlock (Cooler)\n- IceBox (Cooler)\n- NN-13 Cannon\n- NN-14 Cannon\n- NN-15 Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-LYNX, Cluster MNK-833, Cluster HJS-232&lt;/EM4&gt;\n- SnowBlind (Cooler)\n- NightFall (Cooler)\n- M6A Cannon\n- M7A Cannon\n- M8A Cannon\n- Singe Cannon (S1)\n- Singe Cannon (S2)\n- Singe Cannon (S3)\n</v>
+        <v>Tenemos luz verde para finalmente eliminar a {0} Han sido una molestia desde que llegaron al sistema hace unos años y finalmente es hora de eliminarlos de una vez por todas. \n\nHemos recibido información de que {1} fue visto volando cerca de {2} y el Juez quiere que esto se resuelva ahora.\n\nElimínenlos.\n\n- Se esconde.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 600\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Cluster NBD-102, RAB-IGNITION, RAB-FOXTROT&lt;/EM4&gt;\n- Cañón de espada larga serie 9\n- Cañón de espada grande serie 10\n- Cañón de espada ancha serie 11\n- Cañón de impulsor de masa Sledge I\n- Cañón de impulsor de masa Strife\n- Cañón de impulsor de masa Sledge II\n- Cañón de impulsor de masa Sledge III\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Estación de servicio Starlight, RAB-GULF, Starlight Clínica&lt;/EM4&gt;\n- HeatSafe (Enfriador)\n- HeatSink (Enfriador)\n- Escopeta Dominance-1\n- Escopeta Dominance-2\n- Escopeta Dominance-3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Vatra, Ignis, RAB-DELTA&lt;/EM4&gt;\n- VaporBlock (Enfriador)\n- IceBox (Enfriador)\n- Cañón NN-13\n- Cañón NN-14\n- Cañón NN-15\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-LYNX, Cluster MNK-833, Cluster HJS-232&lt;/EM4&gt;\n- SnowBlind (Enfriador)\n- NightFall (Enfriador)\n- Cañón M6A\n- Cañón M7A\n- Cañón M8A\n- Cañón único (S1)\n- Cañón único (S2)\n- Cañón único (S3)\n</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>Got another scumbag who needs their ticket punched. {0} is just a low level thug who doesn't seem to learn. We've warned them to either throw in with us or move system, but they don't seem to be listening so we're out of patience.\n\nHead to {1} and you should find {2} flying around. \n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 75\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: RAB-TUNG, Patch City Clinic, RAB-NOVEMBER&lt;/EM4&gt;\n- 9-Series Longsword Cannon\n- 10-Series Greatsword Cannon\n- 11-Series Broadsword Cannon\n- Sledge I Mass Driver Cannon\n- Strife Mass Driver Cannon\n- Sledge II Mass Driver Cannon\n- Sledge III Mass Driver Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-GULF, Cluster CAJ-445, Orbituary Clinic&lt;/EM4&gt;\n- HeatSafe (Cooler)\n- HeatSink (Cooler)\n- Dominance-1 Scattergun\n- Dominance-2 Scattergun\n- Dominance-3 Scattergun\n\n&lt;EM4&gt;[Regional Variants] example locations: Fuego, RAB-ROTH, Cluster KKE-717&lt;/EM4&gt;\n- VaporBlock (Cooler)\n- IceBox (Cooler)\n- NN-13 Cannon\n- NN-14 Cannon\n- NN-15 Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Terminus, RAB-MAT, Cluster DLO-486&lt;/EM4&gt;\n- SnowBlind (Cooler)\n- NightFall (Cooler)\n- M6A Cannon\n- M7A Cannon\n- M8A Cannon\n- Singe Cannon (S1)\n- Singe Cannon (S2)\n- Singe Cannon (S3)\n</v>
+        <v>Tenemos a otro canalla que necesita su merecido. {0} es solo un matón de poca monta que parece no aprender. Les hemos advertido que se unan a nosotros o cambien de sistema, pero no parecen escuchar, así que se nos acabó la paciencia.\n\nDirígete a {1} y deberías encontrar a {2} volando por ahí. \n\nSe oculta.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 75\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-TUNG, Clínica Patch City, RAB-NOVIEMBRE&lt;/EM4&gt;\n- Cañón de espada larga serie 9\n- Cañón de espada grande serie 10\n- Cañón de espada ancha serie 11\n- Cañón de impulsor de masa Sledge I\n- Cañón de impulsor de masa Strife\n- Cañón de impulsor de masa Sledge II\n- Cañón de impulsor de masa Sledge III\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-GULF, Cluster CAJ-445, Clínica Orbituaria&lt;/EM4&gt;\n- HeatSafe (enfriador)\n- HeatSink (enfriador)\n- Escopeta Dominance-1\n- Dominance-2 Escopeta\n- Escopeta Dominance-3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Fuego, RAB-ROTH, Cluster KKE-717&lt;/EM4&gt;\n- VaporBlock (refrigerador)\n- IceBox (refrigerador)\n- Cañón NN-13\n- Cañón NN-14\n- Cañón NN-15\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Terminus, RAB-MAT, Cluster DLO-486&lt;/EM4&gt;\n- SnowBlind (refrigerador)\n- NightFall (refrigerador)\n- Cañón M6A\n- Cañón M7A\n- Cañón M8A\n- Cañón individual (S1)\n- Cañón individual (S2)\n- Cañón individual (S3)\n</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>Another gang tried to make a move and carve out some territory for themselves. They failed but Headhunters don't forget. We've taken out most of them but one of the last members named {0} has been spotted flying around {1} are they're getting desperate, so don't underestimate them in the fight.\n\nYou'll get paid when it's done.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 300\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: RAB-TUNG, Monox, RAB-IGNITION&lt;/EM4&gt;\n- 9-Series Longsword Cannon\n- 10-Series Greatsword Cannon\n- 11-Series Broadsword Cannon\n- Sledge I Mass Driver Cannon\n- Strife Mass Driver Cannon\n- Sledge II Mass Driver Cannon\n- Sledge III Mass Driver Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Orbituary Clinic, Cluster JWY-925, Rat's Nest&lt;/EM4&gt;\n- HeatSafe (Cooler)\n- HeatSink (Cooler)\n- Dominance-1 Scattergun\n- Dominance-2 Scattergun\n- Dominance-3 Scattergun\n\n&lt;EM4&gt;[Regional Variants] example locations: Pyro IV, Cluster FSN-704, RAB-ECHO&lt;/EM4&gt;\n- VaporBlock (Cooler)\n- IceBox (Cooler)\n- NN-13 Cannon\n- NN-14 Cannon\n- NN-15 Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-ION, Cluster HJS-232, RAB-LYNX&lt;/EM4&gt;\n- SnowBlind (Cooler)\n- NightFall (Cooler)\n- M6A Cannon\n- M7A Cannon\n- M8A Cannon\n- Singe Cannon (S1)\n- Singe Cannon (S2)\n- Singe Cannon (S3)\n</v>
+        <v>Otra banda intentó tomar el control y hacerse con parte del territorio. Fracasaron, pero los Headhunters no olvidan. Hemos eliminado a la mayoría, pero uno de los últimos miembros llamado {0} ha sido visto volando alrededor de {1} y se están desesperando, así que no los subestimes en la lucha.\n\nTe pagarán cuando termine.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 300\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-TUNG, Monox, RAB-IGNITION&lt;/EM4&gt;\n- Cañón de espada larga serie 9\n- Cañón de espada grande serie 10\n- Cañón de espada ancha serie 11\n- Cañón de impulsor de masa Sledge I\n- Cañón de impulsor de masa Strife\n- Cañón de impulsor de masa Sledge II\n- Cañón de impulsor de masa Sledge III\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Clínica Orbituaria, Cluster JWY-925, Nido de ratas&lt;/EM4&gt;\n- HeatSafe (enfriador)\n- HeatSink (enfriador)\n- Escopeta Dominance-1\n- Escopeta Dominance-2\n- Escopeta Dominance-3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Pyro IV, Cluster FSN-704, RAB-ECHO&lt;/EM4&gt;\n- VaporBlock (enfriador)\n- IceBox (enfriador)\n- Cañón NN-13\n- Cañón NN-14\n- Cañón NN-15\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-ION, Cluster HJS-232, RAB-LYNX&lt;/EM4&gt;\n- SnowBlind (enfriador)\n- NightFall (enfriador)\n- Cañón M6A\n- Cañón M7A\n- M8A Cañón\n- Cañón único (T1)\n- Cañón único (T2)\n- Cañón único (T3)\n</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>Got a small fry who thinks they can hit the Headhunters and get away with it. So {0} tried to knock over one of our stashes and think they can get away with it. \n\nLast we heard they were spotted around {1} We need someone to head over and send a very clear message who is the reigning power in the system.\n\nDo it quick and clean.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 50\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: RAB-ROTH, Cluster NBD-102, RAB-IGNITION&lt;/EM4&gt;\n- 9-Series Longsword Cannon\n- 10-Series Greatsword Cannon\n- 11-Series Broadsword Cannon\n- Sledge I Mass Driver Cannon\n- Strife Mass Driver Cannon\n- Sledge II Mass Driver Cannon\n- Sledge III Mass Driver Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Orbituary, RAB-YORK, RAB-ULTRA&lt;/EM4&gt;\n- HeatSafe (Cooler)\n- HeatSink (Cooler)\n- Dominance-1 Scattergun\n- Dominance-2 Scattergun\n- Dominance-3 Scattergun\n\n&lt;EM4&gt;[Regional Variants] example locations: Cluster YKA-011, RAB-DELTA, RAB-POINT&lt;/EM4&gt;\n- VaporBlock (Cooler)\n- IceBox (Cooler)\n- NN-13 Cannon\n- NN-14 Cannon\n- NN-15 Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Ruin Station, RAB-LYNX, RAB-ION&lt;/EM4&gt;\n- SnowBlind (Cooler)\n- NightFall (Cooler)\n- M6A Cannon\n- M7A Cannon\n- M8A Cannon\n- Singe Cannon (S1)\n- Singe Cannon (S2)\n- Singe Cannon (S3)\n</v>
+        <v>Tenemos a un mocoso que cree que puede atacar a los Headhunters y salirse con la suya. Así que {0} intentó derribar uno de nuestros alijos y cree que puede salirse con la suya. \n\nLa última vez que supimos de ellos, fueron vistos alrededor de {1}. Necesitamos que alguien vaya y envíe un mensaje muy claro sobre quién es el poder reinante en el sistema.\n\nHágalo rápido y limpio.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 50\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-ROTH, Cluster NBD-102, RAB-IGNITION&lt;/EM4&gt;\n- Cañón de espada larga serie 9\n- Cañón de espada grande serie 10\n- Cañón de espada ancha serie 11\n- Cañón de impulsor de masa Sledge I\n- Cañón de impulsor de masa Strife\n- Cañón de impulsor de masa Sledge II\n- Cañón de impulsor de masa Sledge III\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Orbituary, RAB-YORK, RAB-ULTRA&lt;/EM4&gt;\n- HeatSafe (Enfriador)\n- HeatSink (Enfriador)\n- Escopeta Dominance-1\n- Escopeta Dominance-2\n- Escopeta Dominance-3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Cluster YKA-011, RAB-DELTA, RAB-POINT&lt;/EM4&gt;\n- VaporBlock (Enfriador)\n- IceBox (Enfriador)\n- Cañón NN-13\n- Cañón NN-14\n- Cañón NN-15\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Ruin Station, RAB-LYNX, RAB-ION&lt;/EM4&gt;\n- SnowBlind (Enfriador)\n- NightFall (Enfriador)\n- Cañón M6A\n- Cañón M7A\n- Cañón M8A\n- Cañón individual (S1)\n- Cañón único (S2)\n- Cañón único (S3)\n</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>You know us. You know what we do. System’s getting a little crowded, so we’re looking for some good soldiers to help keep our place here.\n\nIf you’re up for it and don’t mind getting your hands dirty, we’ve got something to prove you’ve got the stuff we’re looking for.\n\n{0} was a former member who sold us out to XenoThreat and got some of their brothers and sisters killed. Now they think they can just live their life without consequence.\n\nYou take them out. You get boosted in. Sounds like a fair trade.\n\nThey’ve been spotted around {1} so get there and take care of it.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 50\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: RAB-NOVEMBER, RAB-BRAVO, Patch City&lt;/EM4&gt;\n- 9-Series Longsword Cannon\n- 10-Series Greatsword Cannon\n- 11-Series Broadsword Cannon\n- Sledge I Mass Driver Cannon\n- Strife Mass Driver Cannon\n- Sledge II Mass Driver Cannon\n- Sledge III Mass Driver Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-MAT, Starlight Clinic, Orbituary Clinic&lt;/EM4&gt;\n- HeatSafe (Cooler)\n- HeatSink (Cooler)\n- Dominance-1 Scattergun\n- Dominance-2 Scattergun\n- Dominance-3 Scattergun\n\n&lt;EM4&gt;[Regional Variants] example locations: Vuur, Vatra, Cluster YKA-011&lt;/EM4&gt;\n- VaporBlock (Cooler)\n- IceBox (Cooler)\n- NN-13 Cannon\n- NN-14 Cannon\n- NN-15 Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Cluster DLO-486, RAB-ULTRA, Ruin Station&lt;/EM4&gt;\n- SnowBlind (Cooler)\n- NightFall (Cooler)\n- M6A Cannon\n- M7A Cannon\n- M8A Cannon\n- Singe Cannon (S1)\n- Singe Cannon (S2)\n- Singe Cannon (S3)\n</v>
+        <v>Ya nos conoces. Ya sabes lo que hacemos. El sistema se está llenando un poco, así que buscamos buenos soldados para ayudarnos a mantener nuestro lugar aquí.\n\nSi estás dispuesto y no te importa ensuciarte las manos, tenemos algo para demostrar que tienes lo que buscamos.\n\n{0} era un antiguo miembro que nos vendió a XenoThreat y provocó la muerte de algunos de sus hermanos y hermanas. Ahora creen que pueden vivir su vida sin consecuencias.\n\nAcaba con ellos. Te impulsan. Parece un trato justo.\n\nSe les ha visto alrededor de {1}, así que ve allí y encárgate de ello.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 50\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-NOVIEMBRE, RAB-BRAVO, Patch City&lt;/EM4&gt;\n- Cañón de espada larga serie 9\n- Cañón de espada grande serie 10\n- Cañón de espada ancha serie 11\n- Cañón de impulso de masa Sledge I\n- Cañón de impulso de masa Strife\n- Cañón de impulso de masa Sledge II\n- Cañón de impulso de masa Sledge III\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-MAT, Clínica Starlight, Clínica Orbituary&lt;/EM4&gt;\n- HeatSafe (enfriador)\n- Disipador de calor (enfriador)\n- Escopeta Dominance-1\n- Escopeta Dominance-2\n- Escopeta Dominance-3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Vuur, Vatra, Cluster YKA-011&lt;/EM4&gt;\n- Bloque de vapor (enfriador)\n- Caja de hielo (enfriador)\n- Cañón NN-13\n- Cañón NN-14\n- Cañón NN-15\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Cluster DLO-486, RAB-ULTRA, Estación de ruinas&lt;/EM4&gt;\n- Ceguera de nieve (enfriador)\n- Anochecer (enfriador)\n- Cañón M6A\n- Cañón M7A\n- Cañón M8A\n- Cañón individual (S1)\n- Cañón individual (S2)\n- Cañón individual (S3)\n</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>Need you to move quick on this one. There's a XenoThreat lieutenant named {0} who's popped up for air. Judge thinks this is a big chance to mess with XenoThreat's command by taking them out. I heard {1} was spotted flying around {2} so get there quick before they disappear again.\n\nI'd bring some support, I doubt they'll go down without a fight. \n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 3,200\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Checkmate, Checkmate Clinic, Monox&lt;/EM4&gt;\n- 9-Series Longsword Cannon\n- 10-Series Greatsword Cannon\n- 11-Series Broadsword Cannon\n- Sledge I Mass Driver Cannon\n- Strife Mass Driver Cannon\n- Sledge II Mass Driver Cannon\n- Sledge III Mass Driver Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Bloom, RAB-MAT, Cluster JWY-925&lt;/EM4&gt;\n- HeatSafe (Cooler)\n- HeatSink (Cooler)\n- Dominance-1 Scattergun\n- Dominance-2 Scattergun\n- Dominance-3 Scattergun\n\n&lt;EM4&gt;[Regional Variants] example locations: Ignis, Cluster YKA-011, Cluster RSC-340&lt;/EM4&gt;\n- VaporBlock (Cooler)\n- IceBox (Cooler)\n- NN-13 Cannon\n- NN-14 Cannon\n- NN-15 Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-ION, Cluster LHB-976, RAB-LYNX&lt;/EM4&gt;\n- SnowBlind (Cooler)\n- NightFall (Cooler)\n- M6A Cannon\n- M7A Cannon\n- M8A Cannon\n- Singe Cannon (S1)\n- Singe Cannon (S2)\n- Singe Cannon (S3)\n</v>
+        <v>Necesito que te muevas rápido en esto. Hay un teniente de XenoThreat llamado {0} que ha aparecido para tomar aire. Judge cree que esta es una gran oportunidad para interferir con el mando de XenoThreat eliminándolos. Escuché que {1} fue visto volando alrededor de {2}, así que llega rápido antes de que desaparezcan de nuevo.\n\nYo traería refuerzos, dudo que caigan sin luchar. \n\nSe guarda.\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 3200\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Checkmate, Checkmate Clinic, Monox&lt;/EM4&gt;\n- Cañón de espada larga serie 9\n- Cañón de espada grande serie 10\n- Cañón de espada ancha serie 11\n- Cañón de impulsor de masa Sledge I\n- Cañón de impulsor de masa Strife\n- Cañón de impulsor de masa Sledge II\n- Cañón de impulsor de masa Sledge III\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Bloom, RAB-MAT, Cluster JWY-925&lt;/EM4&gt;\n- HeatSafe (enfriador)\n- HeatSink (enfriador)\n- Escopeta Dominance-1\n- Escopeta Dominance-2\n- Escopeta Dominance-3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Ignis, Cluster YKA-011, Cluster RSC-340&lt;/EM4&gt;\n- VaporBlock (enfriador)\n- IceBox (enfriador)\n- Cañón NN-13\n- Cañón NN-14\n- Cañón NN-15\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-ION, Cluster LHB-976, RAB-LYNX&lt;/EM4&gt;\n- SnowBlind (enfriador)\n- NightFall (enfriador)\n- Cañón M6A\n- Cañón M7A\n- Cañón M8A\n- Cañón individual (S1)\n- Cañón individual (S2)\n- Cañón individual (S3)\n</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>The storms over at &lt;EM4&gt;{0} are getting to be a real pain in the ass. One of our outposts got absolutely reamed yesterday and needs some serious repairs so we're looking for help.\n\nFigure you'd need to bring &lt;EM4&gt;about six fuses&lt;/EM4&gt;, a &lt;EM4&gt;salvaging tool&lt;/EM4&gt;, and &lt;EM4&gt;enough RMC canisters to deal with at most eight busted pipes&lt;/EM4&gt;. We think that’ll cover, but you'll get exact numbers on site.\n\nHell with this place.\n\nHopefully you know what you're doing, but just in case, that &lt;EM4&gt;“Guide to Maintenance”&lt;/EM4&gt; in your mobiGlas Journal might be worth a look.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 400</v>
+        <v>Las tormentas en &lt;EM4&gt;{0} se están volviendo un verdadero fastidio. Uno de nuestros puestos avanzados fue arrasado ayer y necesita reparaciones importantes, así que estamos buscando ayuda.\n\nCalcula que necesitarás traer &lt;EM4&gt;unos seis fusibles&lt;/EM4&gt;, una &lt;EM4&gt;herramienta de salvamento&lt;/EM4&gt; y &lt;EM4&gt;suficientes botes de RMC para reparar como máximo ocho tuberías rotas&lt;/EM4&gt;. Creemos que con eso será suficiente, pero te daremos las cifras exactas en el lugar.\n\n¡Al diablo con este lugar!\n\nEsperemos que sepas lo que estás haciendo, pero por si acaso, esa &lt;EM4&gt;“Guía de mantenimiento”&lt;/EM4&gt; en tu Diario mobiGlas podría ser útil.\n\nSe detiene.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 400</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>Need somebody handy with tools to pop over to &lt;EM4&gt;{0} and help out with some repairs. Our last repair guy knocked out most of the fixes but there's still some stuff that could use looking at.\n\nI think if you've got &lt;EM4&gt;six fuses&lt;/EM4&gt;, a &lt;EM4&gt;salvaging tool&lt;/EM4&gt;, and &lt;EM4&gt;enough RMC canisters to patch up around five pipes&lt;/EM4&gt;, you should be covered.\n\nHopefully you know what you're doing, but just in case, the &lt;EM4&gt;“Guide to Maintenance”&lt;/EM4&gt; in your mobiGlas Journal might be worth a look.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 100</v>
+        <v>Necesito a alguien con herramientas para que venga a &lt;EM4&gt;{0} y ayude con algunas reparaciones. Nuestro último técnico solucionó la mayoría de los problemas, pero aún hay algunas cosas que necesitan revisión.\n\nCreo que si tienes &lt;EM4&gt;seis fusibles&lt;/EM4&gt;, una &lt;EM4&gt;herramienta de recuperación&lt;/EM4&gt; y &lt;EM4&gt;suficientes botes de RMC para reparar unas cinco tuberías&lt;/EM4&gt;, deberías estar cubierto.\n\nEspero que sepas lo que estás haciendo, pero por si acaso, la &lt;EM4&gt;“Guía de mantenimiento”&lt;/EM4&gt; en tu Diario mobiGlas podría ser útil.\n\nSe detiene.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 100</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>Hey if you’re reading this, we need a hand. An outpost of ours down at &lt;EM4&gt;{0} got hit by a nasty storm and suffered some damage. None of our usual techs are available (or alive) to swing by so we wanna hire someone to go fix some fuses (no idea how many but &lt;EM4&gt;no more than three&lt;/EM4&gt; I think). If you can bring a &lt;EM4&gt;salvaging tool&lt;/EM4&gt; with &lt;EM4&gt;enough RMC canisters to sort out around three pipes&lt;/EM4&gt;, we should be good.\n\nHopefully you know what you're doing, but just in case, the &lt;EM4&gt;“Guide to Maintenance”&lt;/EM4&gt; in your mobiGlas Journal might be worth a look.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50</v>
+        <v>Hola, si estás leyendo esto, necesitamos ayuda. Un puesto avanzado nuestro en &lt;EM4&gt;{0} fue azotado por una fuerte tormenta y sufrió algunos daños. Ninguno de nuestros técnicos habituales está disponible (o vivo) para venir, así que queremos contratar a alguien para que vaya a arreglar algunos fusibles (no tengo idea de cuántos, pero &lt;EM4&gt;no más de tres&lt;/EM4&gt; creo). Si puedes traer una &lt;EM4&gt;herramienta de recuperación&lt;/EM4&gt; con &lt;EM4&gt;suficientes cartuchos RMC para arreglar unas tres tuberías&lt;/EM4&gt;, deberíamos estar bien.\n\nEspero que sepas lo que estás haciendo, pero por si acaso, la &lt;EM4&gt;“Guía de mantenimiento”&lt;/EM4&gt; en tu diario de mobiGlas podría ser útil.\n\nSalido.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>I'm a bit at the end of my rope. I had sent {0} a pretty dependable Headhunter, out to destroy the XenoThreat data servers at {1} was a while ago and I still haven't heard from them and the servers are still sitting there intact. \n\nDo me a favor, huh? Go on over and see if you can figure out what happened to {2} and help finish destroying the servers.\n\n-Stows out\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 400 / 600</v>
+        <v>Estoy un poco al límite. Hace tiempo envié a {0}, un Headhunter bastante confiable, a destruir los servidores de datos de XenoThreat en {1}, y todavía no he tenido noticias suyas, y los servidores siguen ahí intactos. \n\n¿Me harías un favor? Ve a ver si puedes averiguar qué le pasó a {2} y ayuda a terminar de destruir los servidores.\n\n-Stows out\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 400 / 600</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v>A lotta wannabe gangs have stepped to the Headhunters over the years thinking that they could force their way into the system. We're still here. They aren't. But it seems the survivors of these groups have decided to band together and try again. Guess some people never learn.\n\nLatest group hit a couple of our convoys while on supply runs. Shouldn't be a surprise that the Judge wants to stomp them out quick. We've learned they're out near {0} and likely rearming for another attack. \n\nWe want you to go there and make them wish they died with their old gang.\n\nStows out\n\n&lt;EM4&gt;Reputation Awarded:&lt;/EM4&gt; 300\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: Checkmate Clinic, RAB-ROTH, Checkmate&lt;/EM4&gt;\n- 9-Series Longsword Cannon\n- 10-Series Greatsword Cannon\n- 11-Series Broadsword Cannon\n- Sledge I Mass Driver Cannon\n- Strife Mass Driver Cannon\n- Sledge II Mass Driver Cannon\n- Sledge III Mass Driver Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-CHARLIE, Cluster BGR-560, Cluster CAJ-445&lt;/EM4&gt;\n- HeatSafe (Cooler)\n- HeatSink (Cooler)\n- Dominance-1 Scattergun\n- Dominance-2 Scattergun\n- Dominance-3 Scattergun\n\n&lt;EM4&gt;[Regional Variants] example locations: RAB-LAMDA, Pyro IV, RAB-ZETA&lt;/EM4&gt;\n- VaporBlock (Cooler)\n- IceBox (Cooler)\n- NN-13 Cannon\n- NN-14 Cannon\n- NN-15 Cannon\n\n&lt;EM4&gt;[Regional Variants] example locations: Ruin Clinic, Cluster LHB-976, Terminus&lt;/EM4&gt;\n- SnowBlind (Cooler)\n- NightFall (Cooler)\n- M6A Cannon\n- M7A Cannon\n- M8A Cannon\n- Singe Cannon (S1)\n- Singe Cannon (S2)\n- Singe Cannon (S3)\n</v>
+        <v>Muchos aspirantes a pandilleros se han acercado a los Headhunters a lo largo de los años pensando que podrían entrar por la fuerza en el sistema. Nosotros seguimos aquí. Ellos no. Pero parece que los supervivientes de estos grupos han decidido unirse e intentarlo de nuevo. Supongo que hay gente que nunca aprende.\n\nEl último grupo atacó a un par de nuestros convoyes mientras realizaban misiones de suministro. No debería sorprender que el Juez quiera acabar con ellos rápidamente. Hemos descubierto que están cerca de {0} y probablemente se estén rearmando para otro ataque. \n\nQueremos que vayas allí y les hagas desear haber muerto con su antigua pandilla.\n\nEsconde\n\n&lt;EM4&gt;Reputación otorgada:&lt;/EM4&gt; 300\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: Clínica Checkmate, RAB-ROTH, Checkmate&lt;/EM4&gt;\n- Cañón de espada larga serie 9\n- Cañón de espada grande serie 10\n- Cañón de espada ancha serie 11\n- Cañón de impulsor de masa Sledge I\n- Cañón de impulsor de masa Strife\n- Cañón de impulsor de masa Sledge II\n- Cañón de impulsor de masa Sledge III\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: RAB-CHARLIE, Cluster BGR-560, Cluster CAJ-445&lt;/EM4&gt;\n- HeatSafe (enfriador)\n- HeatSink (enfriador)\n- Escopeta Dominance-1\n- Escopeta Dominance-2\n- Escopeta Dominance-3\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: RAB-LAMDA, Pyro IV, RAB-ZETA&lt;/EM4&gt;\n- VaporBlock (refrigerador)\n- IceBox (refrigerador)\n- Cañón NN-13\n- Cañón NN-14\n- Cañón NN-15\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Clínica Ruin, Cluster LHB-976, Terminus&lt;/EM4&gt;\n- SnowBlind (refrigerador)\n- NightFall (refrigerador)\n- Cañón M6A\n- Cañón M7A\n- Cañón M8A\n- Cañón Singe (S1)\n- Cañón Singe (S2)\n- Cañón Singe (S3)\n</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v>We got big plans about to go down but unfortunately Citizens for Prosperity have people nearby at  {0} I can't afford to have those bastards cockin' things up for us, I want you to go there and take out their power generators.\n\nShould keep them sidelined until we're done with our business. \n\n-Stows out\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 75</v>
+        <v>Tenemos grandes planes a punto de llevarse a cabo, pero desafortunadamente Ciudadanos por la Prosperidad tiene gente cerca en {0}. No puedo permitir que esos bastardos nos arruinen las cosas, quiero que vayas allí y destruyas sus generadores de energía.\n\nDeberíamos mantenerlos fuera de juego hasta que terminemos con nuestro asunto.\n\n-Se esconde\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 75</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v>Something just fell into my lap that is way too good to pass up. XenoThreat's intelligence gathering is a bit of legend in the circles I run in and it turns out that they're storing a whole heap of their best intel at {0} be a shame if someone, say like you, were to go there and blow it all up, huh? \n\n-Stows out\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 75 / 1,500</v>
+        <v> Me acaba de caer del cielo una oportunidad demasiado buena para dejarla pasar. La recopilación de inteligencia de XenoThreat es casi legendaria en los círculos en los que me muevo, y resulta que están almacenando un montón de su mejor inteligencia en {0}. Sería una lástima que alguien, digamos como tú, fuera allí y lo hiciera explotar todo, ¿eh? \n\n-Se guarda\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 75 / 1500</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v>Turns out those Citizens for Prosperity bastards have been gathering intel on us. They're going to try to cut us off from several revenue streams and bleed us dry. Can't let that happen. \n\nHead to {0} and destroy their data storage. \n\nThat should teach them not to stick their noses where they don't belong.\n\n-Stows out\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 75 / 200</v>
+        <v>Resulta que esos bastardos de Ciudadanos por la Prosperidad han estado recopilando información sobre nosotros. Van a intentar cortarnos varias fuentes de ingresos y exprimirnos hasta la última gota. No podemos permitir que eso suceda. \n\nDirígete a {0} y destruye su almacenamiento de datos. \n\nEso les enseñará a no meter las narices donde no les incumbe.\n\n-Se esconde\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 75 / 200</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>So, I sent one of our people, a new recruit by the name {0} to do a hand-off over at {1} but now the bastard’s gone missing.\n\nI’m thinking they either ran off with Headhunter credits and they’re good as dead, or they were robbed and now they’re lying there actually good as dead. Either way, I’d like for you to go have a look and see if you can find them.\n\nIf you settle the matter, I’ll give you what their cut would have been.\n\n-Stows\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50</v>
+        <v> Así que envié a uno de los nuestros, un nuevo recluta llamado {0}, a hacer el traspaso en {1}, pero ahora el muy cabrón ha desaparecido.\n\nCreo que o bien se fugaron con créditos de Cazador de Cabezas y están prácticamente muertos, o bien les robaron y ahora están ahí tirados, prácticamente muertos. En cualquier caso, me gustaría que fueras a echar un vistazo y vieras si puedes encontrarlos.\n\nSi resuelves el asunto, te daré lo que les habría correspondido.\n\n-Stows\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>A few days back I dispatched {0} to scope out a cave system for potential use as a storehouse. Haven't heard from them since. \n\nMy gut tells me they ran into trouble. The local wildlife isn't known for being friendly, and {1} isn't exactly known for being cautious. If you're in need of some creds, I'm offering some up for anyone who can get in there and figure out what happened. \n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 25 / 50 / 200</v>
+        <v>Hace unos días envié a {0} a explorar un sistema de cuevas para usarlo como posible almacén. No he vuelto a saber de ellos. \n\nMi intuición me dice que tuvieron problemas. La fauna local no se caracteriza por ser amigable, y {1} no se caracteriza precisamente por ser precavido. Si necesitas créditos, ofrezco algunos a quien pueda entrar y averiguar qué pasó. \n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 25 / 50 / 200</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>Last night, some no-name drifters threw down with our enforcers and ran when things got too hot. Didn't find out 'til they were long gone, but they made off with one of our Prospects when they split. Goes by the name of {0} \n\nLast we saw, they were headed in the direction {1} We need someone to head there and track down our missing Prospect. \n\nIf you take any of them down while you're at it, all the better.\n\nStows out.\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 200</v>
+        <v> Anoche, unos vagabundos sin nombre se enfrentaron a nuestros ejecutores y huyeron cuando la situación se puso tensa. No nos enteramos hasta que ya se habían ido, pero se llevaron a uno de nuestros prospectos cuando se separaron. Se hace llamar {0}. \n\nLa última vez que los vimos, se dirigían hacia {1}. Necesitamos que alguien vaya allí y localice a nuestro prospecto desaparecido. \n\nSi eliminas a alguno de ellos en el proceso, mejor aún.\n\nSe esconde.\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 50 / 200</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v>Seems there’s a new upstart in the sector who hasn’t been paying the right dues to the right people. To teach them a little lesson, my client wants you to go down to {0} and destroy all the drugs on site.\n\nThe low-level lugs they got on site will probably make a stink about it and try to stop you. Handle them however you want but getting rid of the product is the most important thing.\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 1,000</v>
+        <v>Parece que hay un nuevo advenedizo en el sector que no ha estado pagando lo que le corresponde a la gente adecuada. Para darles una lección, mi cliente quiere que vayas a {0} y destruyas todas las drogas que hay allí.\n\nLos tipos de bajo nivel que tienen allí probablemente armarán un escándalo e intentarán detenerte. Trátalos como quieras, pero lo más importante es deshacerte del producto.\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 1000</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
-        <v>A client of mine‘s trying to negotiate a deal, but isn’t having much luck. The other party feels like they got all the leverage because they’re sitting comfortably on a pile of inventory. To help move the negotiations along, I’m gonna need you to head down to {0} and destroy all the drugs on site. \n\nNow, I should probably tell you that the site’s being protected by some very serious people, so getting to the stash is going to be a bit tricky, but I trust you’ll find a way. \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 4,000</v>
+        <v>Un cliente mío está intentando negociar un acuerdo, pero no está teniendo mucha suerte. La otra parte cree tener toda la ventaja porque tiene un gran inventario a su disposición. Para ayudar a que las negociaciones avancen, necesito que vayas a {0} y destruyas todas las drogas del lugar. \n\nAhora bien, debo decirte que el lugar está protegido por gente muy peligrosa, así que llegar al alijo va a ser un poco complicado, pero confío en que encontrarás la manera. \n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 4000</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
-        <v>One of my clients has been unhappy to learn that someone's been muscling in on their territory. Now rather than going down the more traditional route of killing some people and starting a whole thing, they’ve opted to send a different kind of message instead.\n\nYou’re gonna go down to {0} and destroy all the drugs on site. \n\nOf course, if someone does wanna pick a fight with you, feel free to defend yourself, but getting rid of the product is the most important thing.\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 2,000</v>
+        <v>Uno de mis clientes se ha mostrado disgustado al enterarse de que alguien está invadiendo su territorio. Ahora, en lugar de seguir la ruta más tradicional de matar a algunas personas y armar un escándalo, ha optado por enviar un mensaje diferente.\n\nVas a bajar a {0} y destruir todas las drogas del lugar.\n\nPor supuesto, si alguien quiere pelear contigo, siéntete libre de defenderte, pero lo más importante es deshacerte del producto.\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 2000</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
-        <v>Everybody holds grudges, right? I mean, when you get popped pulling a crime, I get that you’re a little sour, but that’s pretty much the game, right?\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 2,000</v>
+        <v> Todo el mundo guarda rencor, ¿no? O sea, cuando te pillan cometiendo un delito, entiendo que te moleste un poco, pero así son las cosas, ¿no?\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 2000</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v>A client is getting out produced by a new competitor and is looking to throw a wrench into the works.\n\nYou’re going to head to {0} and kill all the civies who work there. \n\nDo what you want with the gun-toting goons guarding the workers, but remember that they aren’t the priority.  \n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 1,000</v>
+        <v>Un cliente está siendo superado en producción por un nuevo competidor y busca sabotear el negocio.\n\nVas a dirigirte a {0} y matar a todos los civiles que trabajan allí.\n\nHaz lo que quieras con los matones armados que custodian a los trabajadores, pero recuerda que no son la prioridad.\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 1000</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v>This is a bit aggressive for my taste, but credits are credits, right?\n\nGot a client who's looking for a highly motivated individual to head over to {0} and kill everyone who’s there. \n\nBasically, start shooting and don’t stop. You'll get paid once the site's clear.\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 1,000</v>
+        <v> Esto es un poco agresivo para mi gusto, pero los créditos son créditos, ¿no?\n\nTengo un cliente que busca a una persona muy motivada para ir a {0} y matar a todos los que estén allí. \n\nBásicamente, empieza a disparar y no pares. Te pagarán una vez que el sitio esté despejado.\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 1000</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
-        <v>{0} Awarded:&lt;/EM4&gt; 100\n&lt;EM4&gt;Potential Blueprints&lt;/EM4&gt;\n&lt;EM4&gt;[Regional Variants] example locations: nyx, Nyx III, Nyx I&lt;/EM4&gt;\n- Custodian SMG\n- Custodian "Midnight" SMG\n- Custodian "Scorched" SMG\n- Arden-SL Arms\n- Arden-SL Core\n- Arden-SL Legs\n- Arden-SL Helmet\n- Custodian SMG Magazine (60 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: microTech, Stanton, ArcCorp&lt;/EM4&gt;\n- Lumin V SMG\n- Inquisitor Core Black\n- Inquisitor Arms Black\n- Inquisitor Legs Black\n- Morningstar Helmet Icefall\n- Inquisitor Core Grey\n- Inquisitor Arms Grey\n- Inquisitor Legs Grey\n- Lumin V SMG Battery (45 cap)\n\n&lt;EM4&gt;[Regional Variants] example locations: Nyx II, Nyx System, Nyx III&lt;/EM4&gt;\n- R97 "Kismet" Shotgun\n- R97 "Righteous" Shotgun\n- Monde Arms Delta Camo\n- Monde Legs Delta Camo\n- Monde Core Delta Camo\n- Monde Helmet Delta Camo\n- Monde Helmet Hemlock Camo\n- Monde Legs Hemlock Camo\n- Monde Core Hemlock Camo\n- Monde Arms Hemlock Camo\n- R97 Shotgun Magazine (18 cap)\n</v>
+        <v>{0} Otorgado:&lt;/EM4&gt; 100\n&lt;EM4&gt;Planos potenciales&lt;/EM4&gt;\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: nyx, Nyx III, Nyx I&lt;/EM4&gt;\n- Subfusil Custodian\n- Subfusil Custodian "Midnight"\n- Subfusil Custodian "Scorched"\n- Brazos Arden-SL\n- Núcleo Arden-SL\n- Piernas Arden-SL\n- Casco Arden-SL\n- Cargador de subfusil Custodian (capacidad de 60)\n\n&lt;EM4&gt;[Variantes regionales] ejemplos de ubicaciones: microTech, Stanton, ArcCorp&lt;/EM4&gt;\n- Subfusil Lumin V\n- Núcleo Inquisitor negro\n- Brazos Inquisitor negros\n- Piernas Inquisitor negras\n- Casco Morningstar Icefall\n- Núcleo Inquisitor gris\n- Brazos Inquisitor grises\n- Piernas Inquisitor grises\n- Subfusil Lumin V Batería (capacidad 45)\n\n&lt;EM4&gt;[Variantes regionales] Ubicaciones de ejemplo: Nyx II, Nyx System, Nyx III&lt;/EM4&gt;\n- Escopeta R97 "Kismet"\n- Escopeta R97 "Righteous"\n- Arms Delta Camo\n- Piernas Monde Delta Camo\n- Núcleo Monde Delta Camo\n- Casco Monde Delta Camo\n- Casco Monde Hemlock Camo\n- Piernas Monde Hemlock Camo\n- Núcleo Monde Hemlock Camo\n- Arms Monde Hemlock Camo\n- Cargador de escopeta R97 (capacidad 18)\n</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v>Firstly, allow me to introduce myself. To put it rather dramatically, I deal in lives. \n\nPeople hire me when some soul needs to be extinguished, and I in return employ the perfect person to serve as the extinguishant. This provides security to all parties involved as none know the identity of the other. An ideal situation as far as these things go.\n\nI was recently made aware that you may possess skills that would make you of service to me and decided that it would be worthwhile to pursue the validity of this claim. \n \nIf you have any interest in forging a working relationship, I will need a demonstration of said skills. \n\nSeek out and discreetly kill {0} over at {1} so successfully and you will be rewarded. Not only that, but you will have proven yourself worthy of further consideration.\n\nSincerely,\nVaughn\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 100 / 500</v>
+        <v>En primer lugar, permítame presentarme. Para decirlo de forma un tanto dramática, me dedico a la vida. \n\nLa gente me contrata cuando hay que extinguir un alma, y yo, a cambio, empleo a la persona perfecta para que cumpla esa función. Esto proporciona seguridad a todas las partes involucradas, ya que nadie conoce la identidad de la otra. Una situación ideal en estos asuntos.\n\nRecientemente me enteré de que usted podría poseer habilidades que me serían útiles y decidí que valdría la pena investigar la veracidad de esta afirmación. \n \nSi tiene algún interés en establecer una relación laboral, necesitaré una demostración de dichas habilidades. \n\nBusque y elimine discretamente a {0} en {1} con éxito y será recompensado. No solo eso, sino que habrá demostrado ser digno de mayor consideración.\n\nAtentamente,\nVaughn\n\n\n&lt;EM4&gt;Reputación otorgada (por dificultad):&lt;/EM4&gt; 100 / 500</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
-        <v>It is not often in life that we get another chance to make a first impression, but I am going to provide to you with just that.\n\nTo say I was disappointed in how things last transpired on your last assassination attempt would be a severe understatement. However, here is your chance to prove yourself capable of more. \n\nKill {0} over at {1} and I will consider the slate wiped clean. \n\nSincerely,\nVaughn\n\n\n&lt;EM4&gt;Reputation Awarded (by difficulty):&lt;/EM4&gt; 50 / 500</v>
+        <v>No es frecuente en la vida tener otra oportunidad para causar una buena primera impresión, pero te la voy a brindar. Decir que me decepcionó cómo se desarrollaron las cosas en tu último intento de asesinato sería quedarse corto. Sin embargo, aquí tienes la oportunidad de demostrar que eres capaz de más. Mata a {0} en {1} y consideraré que has borrado el pasado. Atentamente, Vaughn. Reputación otorgada (por dificultad): 50/500</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
-        <v>{0} Awarded (by difficulty):&lt;/EM4&gt; 100 / 1,000</v>
+        <v> {0} Otorgado (por dificultad):&lt;/EM4&gt; 100 / 1.000</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v>{0} Awarded (by difficulty):&lt;/EM4&gt; 200 / 4,000</v>
+        <v> {0} Otorgado (por dificultad):&lt;/EM4&gt; 200 / 4.000</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
-        <v>{0} Awarded (by difficulty):&lt;/EM4&gt; 150 / 2,000</v>
+        <v> {0} Otorgado (por dificultad):&lt;/EM4&gt; 150 / 2.000</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
-        <v>{0} Awarded (by difficulty):&lt;/EM4&gt; 300 / 16,000</v>
+        <v> {0} Otorgado (por dificultad):&lt;/EM4&gt; 300 / 16.000</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
-        <v>{0} Awarded (by difficulty):&lt;/EM4&gt; 50 / 500</v>
+        <v> {0} Otorgado (por dificultad):&lt;/EM4&gt; 50 / 500</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v>{0} Awarded (by difficulty):&lt;/EM4&gt; 50 / 200 / 8,000</v>
+        <v> {0} Otorgado (por dificultad):&lt;/EM4&gt; 50 / 200 / 8.000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>